<commit_message>
log: Wk 3 Sun 5/17 Lower B done + Wk 4 Mon 5/18 AM check
- Close 5/17 Lower B: filled session log, totals (12 WS/152 reps/2420 kg/
  RPE 8.07), Trap DL e1RM 48→54 (+6/7d, cut working), next bumps.
- Hip Thrust reframed: MACHINE load scale, correctly loaded, no setup
  fix needed (clears 5/10 + 5/17-AM plate-check item).
- 5/18 Upper A AM check logged: full green, GO; flags Tue Lower A.
- build_log.py: +5/17 Lower B sets, +5/17 BW 76.2 AM + run (avg HR 160),
  5/16 note corrected (slow cut, not illness). xlsx re-synced.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -8841,17 +8841,35 @@
       </c>
     </row>
     <row r="166" ht="18" customHeight="1">
-      <c r="A166" s="15" t="n"/>
+      <c r="A166" s="15" t="n">
+        <v>46159</v>
+      </c>
       <c r="B166" s="16">
         <f>IF(A166="","",IFERROR(INT((A166-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C166" s="16" t="n"/>
-      <c r="D166" s="17" t="n"/>
-      <c r="E166" s="16" t="n"/>
-      <c r="F166" s="16" t="n"/>
-      <c r="G166" s="18" t="n"/>
-      <c r="H166" s="16" t="n"/>
+      <c r="C166" s="16" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D166" s="17" t="inlineStr">
+        <is>
+          <t>Trap Bar Deadlift</t>
+        </is>
+      </c>
+      <c r="E166" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F166" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G166" s="18" t="n">
+        <v>45</v>
+      </c>
+      <c r="H166" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I166" s="19">
         <f>IF(OR(F166="",G166=""),"",F166*G166)</f>
         <v/>
@@ -8860,20 +8878,42 @@
         <f>IF(OR(F166="",G166=""),"",ROUND(G166*(1+F166/30),1))</f>
         <v/>
       </c>
-      <c r="K166" s="20" t="n"/>
+      <c r="K166" s="20" t="inlineStr">
+        <is>
+          <t>RIR2; under-loaded</t>
+        </is>
+      </c>
     </row>
     <row r="167" ht="18" customHeight="1">
-      <c r="A167" s="21" t="n"/>
+      <c r="A167" s="21" t="n">
+        <v>46159</v>
+      </c>
       <c r="B167" s="22">
         <f>IF(A167="","",IFERROR(INT((A167-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C167" s="22" t="n"/>
-      <c r="D167" s="23" t="n"/>
-      <c r="E167" s="22" t="n"/>
-      <c r="F167" s="22" t="n"/>
-      <c r="G167" s="24" t="n"/>
-      <c r="H167" s="22" t="n"/>
+      <c r="C167" s="22" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D167" s="23" t="inlineStr">
+        <is>
+          <t>Trap Bar Deadlift</t>
+        </is>
+      </c>
+      <c r="E167" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F167" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="G167" s="24" t="n">
+        <v>45</v>
+      </c>
+      <c r="H167" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I167" s="25">
         <f>IF(OR(F167="",G167=""),"",F167*G167)</f>
         <v/>
@@ -8882,20 +8922,42 @@
         <f>IF(OR(F167="",G167=""),"",ROUND(G167*(1+F167/30),1))</f>
         <v/>
       </c>
-      <c r="K167" s="26" t="n"/>
+      <c r="K167" s="26" t="inlineStr">
+        <is>
+          <t>RIR3; bump 50 next; e1RM 54.0</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="18" customHeight="1">
-      <c r="A168" s="15" t="n"/>
+      <c r="A168" s="15" t="n">
+        <v>46159</v>
+      </c>
       <c r="B168" s="16">
         <f>IF(A168="","",IFERROR(INT((A168-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C168" s="16" t="n"/>
-      <c r="D168" s="17" t="n"/>
-      <c r="E168" s="16" t="n"/>
-      <c r="F168" s="16" t="n"/>
-      <c r="G168" s="18" t="n"/>
-      <c r="H168" s="16" t="n"/>
+      <c r="C168" s="16" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D168" s="17" t="inlineStr">
+        <is>
+          <t>Bulgarian Split Squat</t>
+        </is>
+      </c>
+      <c r="E168" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F168" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G168" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="H168" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I168" s="19">
         <f>IF(OR(F168="",G168=""),"",F168*G168)</f>
         <v/>
@@ -8904,20 +8966,42 @@
         <f>IF(OR(F168="",G168=""),"",ROUND(G168*(1+F168/30),1))</f>
         <v/>
       </c>
-      <c r="K168" s="20" t="n"/>
+      <c r="K168" s="20" t="inlineStr">
+        <is>
+          <t>5/DB=10kg total; 10L+10R; RIR2</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="18" customHeight="1">
-      <c r="A169" s="21" t="n"/>
+      <c r="A169" s="21" t="n">
+        <v>46159</v>
+      </c>
       <c r="B169" s="22">
         <f>IF(A169="","",IFERROR(INT((A169-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C169" s="22" t="n"/>
-      <c r="D169" s="23" t="n"/>
-      <c r="E169" s="22" t="n"/>
-      <c r="F169" s="22" t="n"/>
-      <c r="G169" s="24" t="n"/>
-      <c r="H169" s="22" t="n"/>
+      <c r="C169" s="22" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D169" s="23" t="inlineStr">
+        <is>
+          <t>Bulgarian Split Squat</t>
+        </is>
+      </c>
+      <c r="E169" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F169" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="G169" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="H169" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I169" s="25">
         <f>IF(OR(F169="",G169=""),"",F169*G169)</f>
         <v/>
@@ -8926,20 +9010,42 @@
         <f>IF(OR(F169="",G169=""),"",ROUND(G169*(1+F169/30),1))</f>
         <v/>
       </c>
-      <c r="K169" s="26" t="n"/>
+      <c r="K169" s="26" t="inlineStr">
+        <is>
+          <t>10L+10R; top×all; bump 7.5/DB next</t>
+        </is>
+      </c>
     </row>
     <row r="170" ht="18" customHeight="1">
-      <c r="A170" s="15" t="n"/>
+      <c r="A170" s="15" t="n">
+        <v>46159</v>
+      </c>
       <c r="B170" s="16">
         <f>IF(A170="","",IFERROR(INT((A170-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C170" s="16" t="n"/>
-      <c r="D170" s="17" t="n"/>
-      <c r="E170" s="16" t="n"/>
-      <c r="F170" s="16" t="n"/>
-      <c r="G170" s="18" t="n"/>
-      <c r="H170" s="16" t="n"/>
+      <c r="C170" s="16" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D170" s="17" t="inlineStr">
+        <is>
+          <t>Hip Thrust</t>
+        </is>
+      </c>
+      <c r="E170" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F170" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G170" s="18" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H170" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="I170" s="19">
         <f>IF(OR(F170="",G170=""),"",F170*G170)</f>
         <v/>
@@ -8948,20 +9054,42 @@
         <f>IF(OR(F170="",G170=""),"",ROUND(G170*(1+F170/30),1))</f>
         <v/>
       </c>
-      <c r="K170" s="20" t="n"/>
+      <c r="K170" s="20" t="inlineStr">
+        <is>
+          <t>MACHINE load scale; RIR0</t>
+        </is>
+      </c>
     </row>
     <row r="171" ht="18" customHeight="1">
-      <c r="A171" s="21" t="n"/>
+      <c r="A171" s="21" t="n">
+        <v>46159</v>
+      </c>
       <c r="B171" s="22">
         <f>IF(A171="","",IFERROR(INT((A171-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C171" s="22" t="n"/>
-      <c r="D171" s="23" t="n"/>
-      <c r="E171" s="22" t="n"/>
-      <c r="F171" s="22" t="n"/>
-      <c r="G171" s="24" t="n"/>
-      <c r="H171" s="22" t="n"/>
+      <c r="C171" s="22" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D171" s="23" t="inlineStr">
+        <is>
+          <t>Hip Thrust</t>
+        </is>
+      </c>
+      <c r="E171" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F171" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G171" s="24" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H171" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="I171" s="25">
         <f>IF(OR(F171="",G171=""),"",F171*G171)</f>
         <v/>
@@ -8970,20 +9098,42 @@
         <f>IF(OR(F171="",G171=""),"",ROUND(G171*(1+F171/30),1))</f>
         <v/>
       </c>
-      <c r="K171" s="26" t="n"/>
+      <c r="K171" s="26" t="inlineStr">
+        <is>
+          <t>MACHINE; correctly loaded; hold 12.5</t>
+        </is>
+      </c>
     </row>
     <row r="172" ht="18" customHeight="1">
-      <c r="A172" s="15" t="n"/>
+      <c r="A172" s="15" t="n">
+        <v>46159</v>
+      </c>
       <c r="B172" s="16">
         <f>IF(A172="","",IFERROR(INT((A172-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C172" s="16" t="n"/>
-      <c r="D172" s="17" t="n"/>
-      <c r="E172" s="16" t="n"/>
-      <c r="F172" s="16" t="n"/>
-      <c r="G172" s="18" t="n"/>
-      <c r="H172" s="16" t="n"/>
+      <c r="C172" s="16" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D172" s="17" t="inlineStr">
+        <is>
+          <t>Walking Lunge</t>
+        </is>
+      </c>
+      <c r="E172" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F172" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G172" s="18" t="n">
+        <v>14</v>
+      </c>
+      <c r="H172" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I172" s="19">
         <f>IF(OR(F172="",G172=""),"",F172*G172)</f>
         <v/>
@@ -8992,20 +9142,42 @@
         <f>IF(OR(F172="",G172=""),"",ROUND(G172*(1+F172/30),1))</f>
         <v/>
       </c>
-      <c r="K172" s="20" t="n"/>
+      <c r="K172" s="20" t="inlineStr">
+        <is>
+          <t>7/DB=14kg total; 10L+10R</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="18" customHeight="1">
-      <c r="A173" s="21" t="n"/>
+      <c r="A173" s="21" t="n">
+        <v>46159</v>
+      </c>
       <c r="B173" s="22">
         <f>IF(A173="","",IFERROR(INT((A173-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C173" s="22" t="n"/>
-      <c r="D173" s="23" t="n"/>
-      <c r="E173" s="22" t="n"/>
-      <c r="F173" s="22" t="n"/>
-      <c r="G173" s="24" t="n"/>
-      <c r="H173" s="22" t="n"/>
+      <c r="C173" s="22" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D173" s="23" t="inlineStr">
+        <is>
+          <t>Walking Lunge</t>
+        </is>
+      </c>
+      <c r="E173" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F173" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="G173" s="24" t="n">
+        <v>14</v>
+      </c>
+      <c r="H173" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I173" s="25">
         <f>IF(OR(F173="",G173=""),"",F173*G173)</f>
         <v/>
@@ -9014,20 +9186,42 @@
         <f>IF(OR(F173="",G173=""),"",ROUND(G173*(1+F173/30),1))</f>
         <v/>
       </c>
-      <c r="K173" s="26" t="n"/>
+      <c r="K173" s="26" t="inlineStr">
+        <is>
+          <t>top×all; bump 9/DB next</t>
+        </is>
+      </c>
     </row>
     <row r="174" ht="18" customHeight="1">
-      <c r="A174" s="15" t="n"/>
+      <c r="A174" s="15" t="n">
+        <v>46159</v>
+      </c>
       <c r="B174" s="16">
         <f>IF(A174="","",IFERROR(INT((A174-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C174" s="16" t="n"/>
-      <c r="D174" s="17" t="n"/>
-      <c r="E174" s="16" t="n"/>
-      <c r="F174" s="16" t="n"/>
-      <c r="G174" s="18" t="n"/>
-      <c r="H174" s="16" t="n"/>
+      <c r="C174" s="16" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D174" s="17" t="inlineStr">
+        <is>
+          <t>Seated Calf Raise</t>
+        </is>
+      </c>
+      <c r="E174" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F174" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G174" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="H174" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I174" s="19">
         <f>IF(OR(F174="",G174=""),"",F174*G174)</f>
         <v/>
@@ -9036,20 +9230,42 @@
         <f>IF(OR(F174="",G174=""),"",ROUND(G174*(1+F174/30),1))</f>
         <v/>
       </c>
-      <c r="K174" s="20" t="n"/>
+      <c r="K174" s="20" t="inlineStr">
+        <is>
+          <t>soleus bias</t>
+        </is>
+      </c>
     </row>
     <row r="175" ht="18" customHeight="1">
-      <c r="A175" s="21" t="n"/>
+      <c r="A175" s="21" t="n">
+        <v>46159</v>
+      </c>
       <c r="B175" s="22">
         <f>IF(A175="","",IFERROR(INT((A175-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C175" s="22" t="n"/>
-      <c r="D175" s="23" t="n"/>
-      <c r="E175" s="22" t="n"/>
-      <c r="F175" s="22" t="n"/>
-      <c r="G175" s="24" t="n"/>
-      <c r="H175" s="22" t="n"/>
+      <c r="C175" s="22" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D175" s="23" t="inlineStr">
+        <is>
+          <t>Seated Calf Raise</t>
+        </is>
+      </c>
+      <c r="E175" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F175" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G175" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="H175" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I175" s="25">
         <f>IF(OR(F175="",G175=""),"",F175*G175)</f>
         <v/>
@@ -9058,20 +9274,42 @@
         <f>IF(OR(F175="",G175=""),"",ROUND(G175*(1+F175/30),1))</f>
         <v/>
       </c>
-      <c r="K175" s="26" t="n"/>
+      <c r="K175" s="26" t="inlineStr">
+        <is>
+          <t>RPE6 under-loaded; bump 35 next</t>
+        </is>
+      </c>
     </row>
     <row r="176" ht="18" customHeight="1">
-      <c r="A176" s="15" t="n"/>
+      <c r="A176" s="15" t="n">
+        <v>46159</v>
+      </c>
       <c r="B176" s="16">
         <f>IF(A176="","",IFERROR(INT((A176-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C176" s="16" t="n"/>
-      <c r="D176" s="17" t="n"/>
-      <c r="E176" s="16" t="n"/>
-      <c r="F176" s="16" t="n"/>
-      <c r="G176" s="18" t="n"/>
-      <c r="H176" s="16" t="n"/>
+      <c r="C176" s="16" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D176" s="17" t="inlineStr">
+        <is>
+          <t>Ab Roller</t>
+        </is>
+      </c>
+      <c r="E176" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F176" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G176" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H176" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="I176" s="19">
         <f>IF(OR(F176="",G176=""),"",F176*G176)</f>
         <v/>
@@ -9080,20 +9318,42 @@
         <f>IF(OR(F176="",G176=""),"",ROUND(G176*(1+F176/30),1))</f>
         <v/>
       </c>
-      <c r="K176" s="20" t="n"/>
+      <c r="K176" s="20" t="inlineStr">
+        <is>
+          <t>BW knee rollout</t>
+        </is>
+      </c>
     </row>
     <row r="177" ht="18" customHeight="1">
-      <c r="A177" s="21" t="n"/>
+      <c r="A177" s="21" t="n">
+        <v>46159</v>
+      </c>
       <c r="B177" s="22">
         <f>IF(A177="","",IFERROR(INT((A177-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C177" s="22" t="n"/>
-      <c r="D177" s="23" t="n"/>
-      <c r="E177" s="22" t="n"/>
-      <c r="F177" s="22" t="n"/>
-      <c r="G177" s="24" t="n"/>
-      <c r="H177" s="22" t="n"/>
+      <c r="C177" s="22" t="inlineStr">
+        <is>
+          <t>Lower B</t>
+        </is>
+      </c>
+      <c r="D177" s="23" t="inlineStr">
+        <is>
+          <t>Ab Roller</t>
+        </is>
+      </c>
+      <c r="E177" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F177" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G177" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H177" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="I177" s="25">
         <f>IF(OR(F177="",G177=""),"",F177*G177)</f>
         <v/>
@@ -9102,7 +9362,11 @@
         <f>IF(OR(F177="",G177=""),"",ROUND(G177*(1+F177/30),1))</f>
         <v/>
       </c>
-      <c r="K177" s="26" t="n"/>
+      <c r="K177" s="26" t="inlineStr">
+        <is>
+          <t>BW; hold, target 2×12</t>
+        </is>
+      </c>
     </row>
     <row r="178" ht="18" customHeight="1">
       <c r="A178" s="15" t="n"/>
@@ -22957,22 +23221,42 @@
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="21" t="n"/>
+      <c r="A3" s="21" t="n">
+        <v>46159</v>
+      </c>
       <c r="B3" s="22">
         <f>IF(A3="","",IFERROR(INT((A3-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C3" s="28" t="n"/>
-      <c r="D3" s="24" t="n"/>
+      <c r="C3" s="28" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="D3" s="24" t="n">
+        <v>35</v>
+      </c>
       <c r="E3" s="22">
         <f>IF(OR(C3="",D3=""),"",TEXT(D3/C3/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F3" s="22" t="n"/>
-      <c r="G3" s="22" t="n"/>
-      <c r="H3" s="22" t="n"/>
-      <c r="I3" s="22" t="n"/>
-      <c r="J3" s="26" t="n"/>
+      <c r="F3" s="22" t="n">
+        <v>160</v>
+      </c>
+      <c r="G3" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="I3" s="22" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J3" s="26" t="inlineStr">
+        <is>
+          <t>Sun Z2 chill 6:43/km; avg HR 160; max not recorded; aerobic base held</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="15" t="n"/>
@@ -25954,23 +26238,33 @@
       <c r="H11" s="24" t="n"/>
       <c r="I11" s="26" t="inlineStr">
         <is>
-          <t>Wk 3 Sat AM (-1kg vs Fri, illness Thu/Fri)</t>
+          <t>Wk 3 Sat AM (-1kg vs Fri; slow cut, NOT illness)</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="15" t="n"/>
+      <c r="A12" s="15" t="n">
+        <v>46159</v>
+      </c>
       <c r="B12" s="16">
         <f>IF(A12="","",IFERROR(INT((A12-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C12" s="18" t="n"/>
-      <c r="D12" s="18" t="n"/>
+      <c r="C12" s="18" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="D12" s="18" t="n">
+        <v>8</v>
+      </c>
       <c r="E12" s="18" t="n"/>
       <c r="F12" s="18" t="n"/>
       <c r="G12" s="18" t="n"/>
       <c r="H12" s="18" t="n"/>
-      <c r="I12" s="20" t="n"/>
+      <c r="I12" s="20" t="inlineStr">
+        <is>
+          <t>Wk 3 Sun AM (cut on-plan; AM slope toward ~73)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="21" t="n"/>

</xml_diff>

<commit_message>
log: Wk 4 Mon 5/18 Upper A done + xlsx sync
Bench 37.5 5×8 (RPE→10, S5 6r), e1RM 44.3→47.5 (+3.2/7d) —
strength rising through deficit, guardrail green. Incline DB /
Face Pull / Pushdown top-range × all → bump. Lat PD 42.5 RPE7
too light → start 45. Totals 29 WS / 306 reps / 6632 kg / RPE 8.2.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -9369,17 +9369,35 @@
       </c>
     </row>
     <row r="178" ht="18" customHeight="1">
-      <c r="A178" s="15" t="n"/>
+      <c r="A178" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B178" s="16">
         <f>IF(A178="","",IFERROR(INT((A178-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C178" s="16" t="n"/>
-      <c r="D178" s="17" t="n"/>
-      <c r="E178" s="16" t="n"/>
-      <c r="F178" s="16" t="n"/>
-      <c r="G178" s="18" t="n"/>
-      <c r="H178" s="16" t="n"/>
+      <c r="C178" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D178" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E178" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F178" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G178" s="18" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H178" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I178" s="19">
         <f>IF(OR(F178="",G178=""),"",F178*G178)</f>
         <v/>
@@ -9388,20 +9406,38 @@
         <f>IF(OR(F178="",G178=""),"",ROUND(G178*(1+F178/30),1))</f>
         <v/>
       </c>
-      <c r="K178" s="20" t="n"/>
+      <c r="K178" s="20" t="inlineStr"/>
     </row>
     <row r="179" ht="18" customHeight="1">
-      <c r="A179" s="21" t="n"/>
+      <c r="A179" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B179" s="22">
         <f>IF(A179="","",IFERROR(INT((A179-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C179" s="22" t="n"/>
-      <c r="D179" s="23" t="n"/>
-      <c r="E179" s="22" t="n"/>
-      <c r="F179" s="22" t="n"/>
-      <c r="G179" s="24" t="n"/>
-      <c r="H179" s="22" t="n"/>
+      <c r="C179" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D179" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E179" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F179" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G179" s="24" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H179" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I179" s="25">
         <f>IF(OR(F179="",G179=""),"",F179*G179)</f>
         <v/>
@@ -9410,20 +9446,38 @@
         <f>IF(OR(F179="",G179=""),"",ROUND(G179*(1+F179/30),1))</f>
         <v/>
       </c>
-      <c r="K179" s="26" t="n"/>
+      <c r="K179" s="26" t="inlineStr"/>
     </row>
     <row r="180" ht="18" customHeight="1">
-      <c r="A180" s="15" t="n"/>
+      <c r="A180" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B180" s="16">
         <f>IF(A180="","",IFERROR(INT((A180-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C180" s="16" t="n"/>
-      <c r="D180" s="17" t="n"/>
-      <c r="E180" s="16" t="n"/>
-      <c r="F180" s="16" t="n"/>
-      <c r="G180" s="18" t="n"/>
-      <c r="H180" s="16" t="n"/>
+      <c r="C180" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D180" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E180" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F180" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G180" s="18" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H180" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="I180" s="19">
         <f>IF(OR(F180="",G180=""),"",F180*G180)</f>
         <v/>
@@ -9432,20 +9486,38 @@
         <f>IF(OR(F180="",G180=""),"",ROUND(G180*(1+F180/30),1))</f>
         <v/>
       </c>
-      <c r="K180" s="20" t="n"/>
+      <c r="K180" s="20" t="inlineStr"/>
     </row>
     <row r="181" ht="18" customHeight="1">
-      <c r="A181" s="21" t="n"/>
+      <c r="A181" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B181" s="22">
         <f>IF(A181="","",IFERROR(INT((A181-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C181" s="22" t="n"/>
-      <c r="D181" s="23" t="n"/>
-      <c r="E181" s="22" t="n"/>
-      <c r="F181" s="22" t="n"/>
-      <c r="G181" s="24" t="n"/>
-      <c r="H181" s="22" t="n"/>
+      <c r="C181" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D181" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E181" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F181" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G181" s="24" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H181" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="I181" s="25">
         <f>IF(OR(F181="",G181=""),"",F181*G181)</f>
         <v/>
@@ -9454,20 +9526,42 @@
         <f>IF(OR(F181="",G181=""),"",ROUND(G181*(1+F181/30),1))</f>
         <v/>
       </c>
-      <c r="K181" s="26" t="n"/>
+      <c r="K181" s="26" t="inlineStr">
+        <is>
+          <t>S4 failure RIR0</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="18" customHeight="1">
-      <c r="A182" s="15" t="n"/>
+      <c r="A182" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B182" s="16">
         <f>IF(A182="","",IFERROR(INT((A182-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C182" s="16" t="n"/>
-      <c r="D182" s="17" t="n"/>
-      <c r="E182" s="16" t="n"/>
-      <c r="F182" s="16" t="n"/>
-      <c r="G182" s="18" t="n"/>
-      <c r="H182" s="16" t="n"/>
+      <c r="C182" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D182" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E182" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="F182" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G182" s="18" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H182" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="I182" s="19">
         <f>IF(OR(F182="",G182=""),"",F182*G182)</f>
         <v/>
@@ -9476,20 +9570,42 @@
         <f>IF(OR(F182="",G182=""),"",ROUND(G182*(1+F182/30),1))</f>
         <v/>
       </c>
-      <c r="K182" s="20" t="n"/>
+      <c r="K182" s="20" t="inlineStr">
+        <is>
+          <t>fell to 6r; hold 37.5, clean 5×8 next; e1RM 47.5</t>
+        </is>
+      </c>
     </row>
     <row r="183" ht="18" customHeight="1">
-      <c r="A183" s="21" t="n"/>
+      <c r="A183" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B183" s="22">
         <f>IF(A183="","",IFERROR(INT((A183-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C183" s="22" t="n"/>
-      <c r="D183" s="23" t="n"/>
-      <c r="E183" s="22" t="n"/>
-      <c r="F183" s="22" t="n"/>
-      <c r="G183" s="24" t="n"/>
-      <c r="H183" s="22" t="n"/>
+      <c r="C183" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D183" s="23" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E183" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F183" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G183" s="24" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H183" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I183" s="25">
         <f>IF(OR(F183="",G183=""),"",F183*G183)</f>
         <v/>
@@ -9498,20 +9614,38 @@
         <f>IF(OR(F183="",G183=""),"",ROUND(G183*(1+F183/30),1))</f>
         <v/>
       </c>
-      <c r="K183" s="26" t="n"/>
+      <c r="K183" s="26" t="inlineStr"/>
     </row>
     <row r="184" ht="18" customHeight="1">
-      <c r="A184" s="15" t="n"/>
+      <c r="A184" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B184" s="16">
         <f>IF(A184="","",IFERROR(INT((A184-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C184" s="16" t="n"/>
-      <c r="D184" s="17" t="n"/>
-      <c r="E184" s="16" t="n"/>
-      <c r="F184" s="16" t="n"/>
-      <c r="G184" s="18" t="n"/>
-      <c r="H184" s="16" t="n"/>
+      <c r="C184" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D184" s="17" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E184" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F184" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G184" s="18" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H184" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I184" s="19">
         <f>IF(OR(F184="",G184=""),"",F184*G184)</f>
         <v/>
@@ -9520,20 +9654,38 @@
         <f>IF(OR(F184="",G184=""),"",ROUND(G184*(1+F184/30),1))</f>
         <v/>
       </c>
-      <c r="K184" s="20" t="n"/>
+      <c r="K184" s="20" t="inlineStr"/>
     </row>
     <row r="185" ht="18" customHeight="1">
-      <c r="A185" s="21" t="n"/>
+      <c r="A185" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B185" s="22">
         <f>IF(A185="","",IFERROR(INT((A185-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C185" s="22" t="n"/>
-      <c r="D185" s="23" t="n"/>
-      <c r="E185" s="22" t="n"/>
-      <c r="F185" s="22" t="n"/>
-      <c r="G185" s="24" t="n"/>
-      <c r="H185" s="22" t="n"/>
+      <c r="C185" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D185" s="23" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E185" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F185" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G185" s="24" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H185" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I185" s="25">
         <f>IF(OR(F185="",G185=""),"",F185*G185)</f>
         <v/>
@@ -9542,20 +9694,38 @@
         <f>IF(OR(F185="",G185=""),"",ROUND(G185*(1+F185/30),1))</f>
         <v/>
       </c>
-      <c r="K185" s="26" t="n"/>
+      <c r="K185" s="26" t="inlineStr"/>
     </row>
     <row r="186" ht="18" customHeight="1">
-      <c r="A186" s="15" t="n"/>
+      <c r="A186" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B186" s="16">
         <f>IF(A186="","",IFERROR(INT((A186-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C186" s="16" t="n"/>
-      <c r="D186" s="17" t="n"/>
-      <c r="E186" s="16" t="n"/>
-      <c r="F186" s="16" t="n"/>
-      <c r="G186" s="18" t="n"/>
-      <c r="H186" s="16" t="n"/>
+      <c r="C186" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D186" s="17" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E186" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F186" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G186" s="18" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H186" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="I186" s="19">
         <f>IF(OR(F186="",G186=""),"",F186*G186)</f>
         <v/>
@@ -9564,20 +9734,38 @@
         <f>IF(OR(F186="",G186=""),"",ROUND(G186*(1+F186/30),1))</f>
         <v/>
       </c>
-      <c r="K186" s="20" t="n"/>
+      <c r="K186" s="20" t="inlineStr"/>
     </row>
     <row r="187" ht="18" customHeight="1">
-      <c r="A187" s="21" t="n"/>
+      <c r="A187" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B187" s="22">
         <f>IF(A187="","",IFERROR(INT((A187-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C187" s="22" t="n"/>
-      <c r="D187" s="23" t="n"/>
-      <c r="E187" s="22" t="n"/>
-      <c r="F187" s="22" t="n"/>
-      <c r="G187" s="24" t="n"/>
-      <c r="H187" s="22" t="n"/>
+      <c r="C187" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D187" s="23" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E187" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="F187" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="G187" s="24" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="H187" s="22" t="n">
+        <v>9</v>
+      </c>
       <c r="I187" s="25">
         <f>IF(OR(F187="",G187=""),"",F187*G187)</f>
         <v/>
@@ -9586,20 +9774,42 @@
         <f>IF(OR(F187="",G187=""),"",ROUND(G187*(1+F187/30),1))</f>
         <v/>
       </c>
-      <c r="K187" s="26" t="n"/>
+      <c r="K187" s="26" t="inlineStr">
+        <is>
+          <t>S5 7r; hold 37.5, clean 5×8 next</t>
+        </is>
+      </c>
     </row>
     <row r="188" ht="18" customHeight="1">
-      <c r="A188" s="15" t="n"/>
+      <c r="A188" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B188" s="16">
         <f>IF(A188="","",IFERROR(INT((A188-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C188" s="16" t="n"/>
-      <c r="D188" s="17" t="n"/>
-      <c r="E188" s="16" t="n"/>
-      <c r="F188" s="16" t="n"/>
-      <c r="G188" s="18" t="n"/>
-      <c r="H188" s="16" t="n"/>
+      <c r="C188" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D188" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E188" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F188" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G188" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="H188" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I188" s="19">
         <f>IF(OR(F188="",G188=""),"",F188*G188)</f>
         <v/>
@@ -9608,20 +9818,42 @@
         <f>IF(OR(F188="",G188=""),"",ROUND(G188*(1+F188/30),1))</f>
         <v/>
       </c>
-      <c r="K188" s="20" t="n"/>
+      <c r="K188" s="20" t="inlineStr">
+        <is>
+          <t>ran 15 vs start 14</t>
+        </is>
+      </c>
     </row>
     <row r="189" ht="18" customHeight="1">
-      <c r="A189" s="21" t="n"/>
+      <c r="A189" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B189" s="22">
         <f>IF(A189="","",IFERROR(INT((A189-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C189" s="22" t="n"/>
-      <c r="D189" s="23" t="n"/>
-      <c r="E189" s="22" t="n"/>
-      <c r="F189" s="22" t="n"/>
-      <c r="G189" s="24" t="n"/>
-      <c r="H189" s="22" t="n"/>
+      <c r="C189" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D189" s="23" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E189" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F189" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G189" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="H189" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I189" s="25">
         <f>IF(OR(F189="",G189=""),"",F189*G189)</f>
         <v/>
@@ -9630,20 +9862,38 @@
         <f>IF(OR(F189="",G189=""),"",ROUND(G189*(1+F189/30),1))</f>
         <v/>
       </c>
-      <c r="K189" s="26" t="n"/>
+      <c r="K189" s="26" t="inlineStr"/>
     </row>
     <row r="190" ht="18" customHeight="1">
-      <c r="A190" s="15" t="n"/>
+      <c r="A190" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B190" s="16">
         <f>IF(A190="","",IFERROR(INT((A190-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C190" s="16" t="n"/>
-      <c r="D190" s="17" t="n"/>
-      <c r="E190" s="16" t="n"/>
-      <c r="F190" s="16" t="n"/>
-      <c r="G190" s="18" t="n"/>
-      <c r="H190" s="16" t="n"/>
+      <c r="C190" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D190" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E190" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F190" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G190" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="H190" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="I190" s="19">
         <f>IF(OR(F190="",G190=""),"",F190*G190)</f>
         <v/>
@@ -9652,20 +9902,42 @@
         <f>IF(OR(F190="",G190=""),"",ROUND(G190*(1+F190/30),1))</f>
         <v/>
       </c>
-      <c r="K190" s="20" t="n"/>
+      <c r="K190" s="20" t="inlineStr">
+        <is>
+          <t>top×3, bump 16 next</t>
+        </is>
+      </c>
     </row>
     <row r="191" ht="18" customHeight="1">
-      <c r="A191" s="21" t="n"/>
+      <c r="A191" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B191" s="22">
         <f>IF(A191="","",IFERROR(INT((A191-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C191" s="22" t="n"/>
-      <c r="D191" s="23" t="n"/>
-      <c r="E191" s="22" t="n"/>
-      <c r="F191" s="22" t="n"/>
-      <c r="G191" s="24" t="n"/>
-      <c r="H191" s="22" t="n"/>
+      <c r="C191" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D191" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E191" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F191" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G191" s="24" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="H191" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I191" s="25">
         <f>IF(OR(F191="",G191=""),"",F191*G191)</f>
         <v/>
@@ -9674,20 +9946,42 @@
         <f>IF(OR(F191="",G191=""),"",ROUND(G191*(1+F191/30),1))</f>
         <v/>
       </c>
-      <c r="K191" s="26" t="n"/>
+      <c r="K191" s="26" t="inlineStr">
+        <is>
+          <t>RIR3 too light</t>
+        </is>
+      </c>
     </row>
     <row r="192" ht="18" customHeight="1">
-      <c r="A192" s="15" t="n"/>
+      <c r="A192" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B192" s="16">
         <f>IF(A192="","",IFERROR(INT((A192-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C192" s="16" t="n"/>
-      <c r="D192" s="17" t="n"/>
-      <c r="E192" s="16" t="n"/>
-      <c r="F192" s="16" t="n"/>
-      <c r="G192" s="18" t="n"/>
-      <c r="H192" s="16" t="n"/>
+      <c r="C192" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D192" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E192" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F192" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G192" s="18" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="H192" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I192" s="19">
         <f>IF(OR(F192="",G192=""),"",F192*G192)</f>
         <v/>
@@ -9696,20 +9990,42 @@
         <f>IF(OR(F192="",G192=""),"",ROUND(G192*(1+F192/30),1))</f>
         <v/>
       </c>
-      <c r="K192" s="20" t="n"/>
+      <c r="K192" s="20" t="inlineStr">
+        <is>
+          <t>RIR3</t>
+        </is>
+      </c>
     </row>
     <row r="193" ht="18" customHeight="1">
-      <c r="A193" s="21" t="n"/>
+      <c r="A193" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B193" s="22">
         <f>IF(A193="","",IFERROR(INT((A193-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C193" s="22" t="n"/>
-      <c r="D193" s="23" t="n"/>
-      <c r="E193" s="22" t="n"/>
-      <c r="F193" s="22" t="n"/>
-      <c r="G193" s="24" t="n"/>
-      <c r="H193" s="22" t="n"/>
+      <c r="C193" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D193" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E193" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F193" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G193" s="24" t="n">
+        <v>42.5</v>
+      </c>
+      <c r="H193" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I193" s="25">
         <f>IF(OR(F193="",G193=""),"",F193*G193)</f>
         <v/>
@@ -9718,20 +10034,42 @@
         <f>IF(OR(F193="",G193=""),"",ROUND(G193*(1+F193/30),1))</f>
         <v/>
       </c>
-      <c r="K193" s="26" t="n"/>
+      <c r="K193" s="26" t="inlineStr">
+        <is>
+          <t>RIR3</t>
+        </is>
+      </c>
     </row>
     <row r="194" ht="18" customHeight="1">
-      <c r="A194" s="15" t="n"/>
+      <c r="A194" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B194" s="16">
         <f>IF(A194="","",IFERROR(INT((A194-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C194" s="16" t="n"/>
-      <c r="D194" s="17" t="n"/>
-      <c r="E194" s="16" t="n"/>
-      <c r="F194" s="16" t="n"/>
-      <c r="G194" s="18" t="n"/>
-      <c r="H194" s="16" t="n"/>
+      <c r="C194" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D194" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E194" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F194" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G194" s="18" t="n">
+        <v>45</v>
+      </c>
+      <c r="H194" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="I194" s="19">
         <f>IF(OR(F194="",G194=""),"",F194*G194)</f>
         <v/>
@@ -9740,20 +10078,42 @@
         <f>IF(OR(F194="",G194=""),"",ROUND(G194*(1+F194/30),1))</f>
         <v/>
       </c>
-      <c r="K194" s="20" t="n"/>
+      <c r="K194" s="20" t="inlineStr">
+        <is>
+          <t>self-bump S4; start 45 next</t>
+        </is>
+      </c>
     </row>
     <row r="195" ht="18" customHeight="1">
-      <c r="A195" s="21" t="n"/>
+      <c r="A195" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B195" s="22">
         <f>IF(A195="","",IFERROR(INT((A195-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C195" s="22" t="n"/>
-      <c r="D195" s="23" t="n"/>
-      <c r="E195" s="22" t="n"/>
-      <c r="F195" s="22" t="n"/>
-      <c r="G195" s="24" t="n"/>
-      <c r="H195" s="22" t="n"/>
+      <c r="C195" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D195" s="23" t="inlineStr">
+        <is>
+          <t>Pec Deck</t>
+        </is>
+      </c>
+      <c r="E195" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F195" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G195" s="24" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H195" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I195" s="25">
         <f>IF(OR(F195="",G195=""),"",F195*G195)</f>
         <v/>
@@ -9762,20 +10122,38 @@
         <f>IF(OR(F195="",G195=""),"",ROUND(G195*(1+F195/30),1))</f>
         <v/>
       </c>
-      <c r="K195" s="26" t="n"/>
+      <c r="K195" s="26" t="inlineStr"/>
     </row>
     <row r="196" ht="18" customHeight="1">
-      <c r="A196" s="15" t="n"/>
+      <c r="A196" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B196" s="16">
         <f>IF(A196="","",IFERROR(INT((A196-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C196" s="16" t="n"/>
-      <c r="D196" s="17" t="n"/>
-      <c r="E196" s="16" t="n"/>
-      <c r="F196" s="16" t="n"/>
-      <c r="G196" s="18" t="n"/>
-      <c r="H196" s="16" t="n"/>
+      <c r="C196" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D196" s="17" t="inlineStr">
+        <is>
+          <t>Pec Deck</t>
+        </is>
+      </c>
+      <c r="E196" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F196" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G196" s="18" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H196" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I196" s="19">
         <f>IF(OR(F196="",G196=""),"",F196*G196)</f>
         <v/>
@@ -9784,20 +10162,38 @@
         <f>IF(OR(F196="",G196=""),"",ROUND(G196*(1+F196/30),1))</f>
         <v/>
       </c>
-      <c r="K196" s="20" t="n"/>
+      <c r="K196" s="20" t="inlineStr"/>
     </row>
     <row r="197" ht="18" customHeight="1">
-      <c r="A197" s="21" t="n"/>
+      <c r="A197" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B197" s="22">
         <f>IF(A197="","",IFERROR(INT((A197-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C197" s="22" t="n"/>
-      <c r="D197" s="23" t="n"/>
-      <c r="E197" s="22" t="n"/>
-      <c r="F197" s="22" t="n"/>
-      <c r="G197" s="24" t="n"/>
-      <c r="H197" s="22" t="n"/>
+      <c r="C197" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D197" s="23" t="inlineStr">
+        <is>
+          <t>Pec Deck</t>
+        </is>
+      </c>
+      <c r="E197" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F197" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G197" s="24" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H197" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="I197" s="25">
         <f>IF(OR(F197="",G197=""),"",F197*G197)</f>
         <v/>
@@ -9806,20 +10202,42 @@
         <f>IF(OR(F197="",G197=""),"",ROUND(G197*(1+F197/30),1))</f>
         <v/>
       </c>
-      <c r="K197" s="26" t="n"/>
+      <c r="K197" s="26" t="inlineStr">
+        <is>
+          <t>muscular failure; hold 7.5 chase 15×3</t>
+        </is>
+      </c>
     </row>
     <row r="198" ht="18" customHeight="1">
-      <c r="A198" s="15" t="n"/>
+      <c r="A198" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B198" s="16">
         <f>IF(A198="","",IFERROR(INT((A198-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C198" s="16" t="n"/>
-      <c r="D198" s="17" t="n"/>
-      <c r="E198" s="16" t="n"/>
-      <c r="F198" s="16" t="n"/>
-      <c r="G198" s="18" t="n"/>
-      <c r="H198" s="16" t="n"/>
+      <c r="C198" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D198" s="17" t="inlineStr">
+        <is>
+          <t>Face Pull</t>
+        </is>
+      </c>
+      <c r="E198" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F198" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G198" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="H198" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I198" s="19">
         <f>IF(OR(F198="",G198=""),"",F198*G198)</f>
         <v/>
@@ -9828,20 +10246,38 @@
         <f>IF(OR(F198="",G198=""),"",ROUND(G198*(1+F198/30),1))</f>
         <v/>
       </c>
-      <c r="K198" s="20" t="n"/>
+      <c r="K198" s="20" t="inlineStr"/>
     </row>
     <row r="199" ht="18" customHeight="1">
-      <c r="A199" s="21" t="n"/>
+      <c r="A199" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B199" s="22">
         <f>IF(A199="","",IFERROR(INT((A199-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C199" s="22" t="n"/>
-      <c r="D199" s="23" t="n"/>
-      <c r="E199" s="22" t="n"/>
-      <c r="F199" s="22" t="n"/>
-      <c r="G199" s="24" t="n"/>
-      <c r="H199" s="22" t="n"/>
+      <c r="C199" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D199" s="23" t="inlineStr">
+        <is>
+          <t>Face Pull</t>
+        </is>
+      </c>
+      <c r="E199" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F199" s="22" t="n">
+        <v>20</v>
+      </c>
+      <c r="G199" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="H199" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I199" s="25">
         <f>IF(OR(F199="",G199=""),"",F199*G199)</f>
         <v/>
@@ -9850,20 +10286,38 @@
         <f>IF(OR(F199="",G199=""),"",ROUND(G199*(1+F199/30),1))</f>
         <v/>
       </c>
-      <c r="K199" s="26" t="n"/>
+      <c r="K199" s="26" t="inlineStr"/>
     </row>
     <row r="200" ht="18" customHeight="1">
-      <c r="A200" s="15" t="n"/>
+      <c r="A200" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B200" s="16">
         <f>IF(A200="","",IFERROR(INT((A200-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C200" s="16" t="n"/>
-      <c r="D200" s="17" t="n"/>
-      <c r="E200" s="16" t="n"/>
-      <c r="F200" s="16" t="n"/>
-      <c r="G200" s="18" t="n"/>
-      <c r="H200" s="16" t="n"/>
+      <c r="C200" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D200" s="17" t="inlineStr">
+        <is>
+          <t>Face Pull</t>
+        </is>
+      </c>
+      <c r="E200" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F200" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="G200" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="H200" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I200" s="19">
         <f>IF(OR(F200="",G200=""),"",F200*G200)</f>
         <v/>
@@ -9872,20 +10326,42 @@
         <f>IF(OR(F200="",G200=""),"",ROUND(G200*(1+F200/30),1))</f>
         <v/>
       </c>
-      <c r="K200" s="20" t="n"/>
+      <c r="K200" s="20" t="inlineStr">
+        <is>
+          <t>top×3 RPE8, bump 16 next</t>
+        </is>
+      </c>
     </row>
     <row r="201" ht="18" customHeight="1">
-      <c r="A201" s="21" t="n"/>
+      <c r="A201" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B201" s="22">
         <f>IF(A201="","",IFERROR(INT((A201-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C201" s="22" t="n"/>
-      <c r="D201" s="23" t="n"/>
-      <c r="E201" s="22" t="n"/>
-      <c r="F201" s="22" t="n"/>
-      <c r="G201" s="24" t="n"/>
-      <c r="H201" s="22" t="n"/>
+      <c r="C201" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D201" s="23" t="inlineStr">
+        <is>
+          <t>Triceps Pushdown</t>
+        </is>
+      </c>
+      <c r="E201" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F201" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G201" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="H201" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I201" s="25">
         <f>IF(OR(F201="",G201=""),"",F201*G201)</f>
         <v/>
@@ -9894,20 +10370,38 @@
         <f>IF(OR(F201="",G201=""),"",ROUND(G201*(1+F201/30),1))</f>
         <v/>
       </c>
-      <c r="K201" s="26" t="n"/>
+      <c r="K201" s="26" t="inlineStr"/>
     </row>
     <row r="202" ht="18" customHeight="1">
-      <c r="A202" s="15" t="n"/>
+      <c r="A202" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B202" s="16">
         <f>IF(A202="","",IFERROR(INT((A202-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C202" s="16" t="n"/>
-      <c r="D202" s="17" t="n"/>
-      <c r="E202" s="16" t="n"/>
-      <c r="F202" s="16" t="n"/>
-      <c r="G202" s="18" t="n"/>
-      <c r="H202" s="16" t="n"/>
+      <c r="C202" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D202" s="17" t="inlineStr">
+        <is>
+          <t>Triceps Pushdown</t>
+        </is>
+      </c>
+      <c r="E202" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F202" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G202" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="H202" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I202" s="19">
         <f>IF(OR(F202="",G202=""),"",F202*G202)</f>
         <v/>
@@ -9916,20 +10410,38 @@
         <f>IF(OR(F202="",G202=""),"",ROUND(G202*(1+F202/30),1))</f>
         <v/>
       </c>
-      <c r="K202" s="20" t="n"/>
+      <c r="K202" s="20" t="inlineStr"/>
     </row>
     <row r="203" ht="18" customHeight="1">
-      <c r="A203" s="21" t="n"/>
+      <c r="A203" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B203" s="22">
         <f>IF(A203="","",IFERROR(INT((A203-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C203" s="22" t="n"/>
-      <c r="D203" s="23" t="n"/>
-      <c r="E203" s="22" t="n"/>
-      <c r="F203" s="22" t="n"/>
-      <c r="G203" s="24" t="n"/>
-      <c r="H203" s="22" t="n"/>
+      <c r="C203" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D203" s="23" t="inlineStr">
+        <is>
+          <t>Triceps Pushdown</t>
+        </is>
+      </c>
+      <c r="E203" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F203" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G203" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="H203" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I203" s="25">
         <f>IF(OR(F203="",G203=""),"",F203*G203)</f>
         <v/>
@@ -9938,20 +10450,42 @@
         <f>IF(OR(F203="",G203=""),"",ROUND(G203*(1+F203/30),1))</f>
         <v/>
       </c>
-      <c r="K203" s="26" t="n"/>
+      <c r="K203" s="26" t="inlineStr">
+        <is>
+          <t>target clean×3, bump 17 next</t>
+        </is>
+      </c>
     </row>
     <row r="204" ht="18" customHeight="1">
-      <c r="A204" s="15" t="n"/>
+      <c r="A204" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B204" s="16">
         <f>IF(A204="","",IFERROR(INT((A204-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C204" s="16" t="n"/>
-      <c r="D204" s="17" t="n"/>
-      <c r="E204" s="16" t="n"/>
-      <c r="F204" s="16" t="n"/>
-      <c r="G204" s="18" t="n"/>
-      <c r="H204" s="16" t="n"/>
+      <c r="C204" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D204" s="17" t="inlineStr">
+        <is>
+          <t>DB Curl</t>
+        </is>
+      </c>
+      <c r="E204" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F204" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G204" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="H204" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I204" s="19">
         <f>IF(OR(F204="",G204=""),"",F204*G204)</f>
         <v/>
@@ -9960,20 +10494,38 @@
         <f>IF(OR(F204="",G204=""),"",ROUND(G204*(1+F204/30),1))</f>
         <v/>
       </c>
-      <c r="K204" s="20" t="n"/>
+      <c r="K204" s="20" t="inlineStr"/>
     </row>
     <row r="205" ht="18" customHeight="1">
-      <c r="A205" s="21" t="n"/>
+      <c r="A205" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B205" s="22">
         <f>IF(A205="","",IFERROR(INT((A205-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C205" s="22" t="n"/>
-      <c r="D205" s="23" t="n"/>
-      <c r="E205" s="22" t="n"/>
-      <c r="F205" s="22" t="n"/>
-      <c r="G205" s="24" t="n"/>
-      <c r="H205" s="22" t="n"/>
+      <c r="C205" s="22" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D205" s="23" t="inlineStr">
+        <is>
+          <t>DB Curl</t>
+        </is>
+      </c>
+      <c r="E205" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F205" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G205" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="H205" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I205" s="25">
         <f>IF(OR(F205="",G205=""),"",F205*G205)</f>
         <v/>
@@ -9982,20 +10534,38 @@
         <f>IF(OR(F205="",G205=""),"",ROUND(G205*(1+F205/30),1))</f>
         <v/>
       </c>
-      <c r="K205" s="26" t="n"/>
+      <c r="K205" s="26" t="inlineStr"/>
     </row>
     <row r="206" ht="18" customHeight="1">
-      <c r="A206" s="15" t="n"/>
+      <c r="A206" s="15" t="n">
+        <v>46160</v>
+      </c>
       <c r="B206" s="16">
         <f>IF(A206="","",IFERROR(INT((A206-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C206" s="16" t="n"/>
-      <c r="D206" s="17" t="n"/>
-      <c r="E206" s="16" t="n"/>
-      <c r="F206" s="16" t="n"/>
-      <c r="G206" s="18" t="n"/>
-      <c r="H206" s="16" t="n"/>
+      <c r="C206" s="16" t="inlineStr">
+        <is>
+          <t>Upper A</t>
+        </is>
+      </c>
+      <c r="D206" s="17" t="inlineStr">
+        <is>
+          <t>DB Curl</t>
+        </is>
+      </c>
+      <c r="E206" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F206" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G206" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="H206" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I206" s="19">
         <f>IF(OR(F206="",G206=""),"",F206*G206)</f>
         <v/>
@@ -10004,7 +10574,11 @@
         <f>IF(OR(F206="",G206=""),"",ROUND(G206*(1+F206/30),1))</f>
         <v/>
       </c>
-      <c r="K206" s="20" t="n"/>
+      <c r="K206" s="20" t="inlineStr">
+        <is>
+          <t>S3 10r; hold 8 chase 12×3</t>
+        </is>
+      </c>
     </row>
     <row r="207" ht="18" customHeight="1">
       <c r="A207" s="21" t="n"/>
@@ -26267,18 +26841,28 @@
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="21" t="n"/>
+      <c r="A13" s="21" t="n">
+        <v>46160</v>
+      </c>
       <c r="B13" s="22">
         <f>IF(A13="","",IFERROR(INT((A13-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C13" s="24" t="n"/>
-      <c r="D13" s="24" t="n"/>
+      <c r="C13" s="24" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="D13" s="24" t="n">
+        <v>8</v>
+      </c>
       <c r="E13" s="24" t="n"/>
       <c r="F13" s="24" t="n"/>
       <c r="G13" s="24" t="n"/>
       <c r="H13" s="24" t="n"/>
-      <c r="I13" s="26" t="n"/>
+      <c r="I13" s="26" t="inlineStr">
+        <is>
+          <t>Wk 4 Mon AM (flat vs Sun; post-Lower-B water noise, not stall)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="15" t="n"/>

</xml_diff>

<commit_message>
log: Build W1 Mon 6/8 PM — Push DONE (19 sets/208 reps/1209.5kg, RPE6.8)
First lift in 2+ wks. Shoulder gate CLEAN. Bench -> Standing chest press
(locked sub, user pref). Loads under START = layoff + new machine, not
flagged. Macros maintenance (cut paused). xlsx rebuilt w/ 19 sets + BW 77.1.
Tue 6/9 run pre-staged (6k easy Z2, run-gate + cadence 165+).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -10581,17 +10581,35 @@
       </c>
     </row>
     <row r="207" ht="18" customHeight="1">
-      <c r="A207" s="21" t="n"/>
+      <c r="A207" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B207" s="22">
         <f>IF(A207="","",IFERROR(INT((A207-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C207" s="22" t="n"/>
-      <c r="D207" s="23" t="n"/>
-      <c r="E207" s="22" t="n"/>
-      <c r="F207" s="22" t="n"/>
-      <c r="G207" s="24" t="n"/>
-      <c r="H207" s="22" t="n"/>
+      <c r="C207" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D207" s="23" t="inlineStr">
+        <is>
+          <t>Standing Chest Press</t>
+        </is>
+      </c>
+      <c r="E207" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F207" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G207" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="H207" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="I207" s="25">
         <f>IF(OR(F207="",G207=""),"",F207*G207)</f>
         <v/>
@@ -10600,20 +10618,42 @@
         <f>IF(OR(F207="",G207=""),"",ROUND(G207*(1+F207/30),1))</f>
         <v/>
       </c>
-      <c r="K207" s="26" t="n"/>
+      <c r="K207" s="26" t="inlineStr">
+        <is>
+          <t>new locked sub vs bench (user pref + shoulder)</t>
+        </is>
+      </c>
     </row>
     <row r="208" ht="18" customHeight="1">
-      <c r="A208" s="15" t="n"/>
+      <c r="A208" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B208" s="16">
         <f>IF(A208="","",IFERROR(INT((A208-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C208" s="16" t="n"/>
-      <c r="D208" s="17" t="n"/>
-      <c r="E208" s="16" t="n"/>
-      <c r="F208" s="16" t="n"/>
-      <c r="G208" s="18" t="n"/>
-      <c r="H208" s="16" t="n"/>
+      <c r="C208" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D208" s="17" t="inlineStr">
+        <is>
+          <t>Standing Chest Press</t>
+        </is>
+      </c>
+      <c r="E208" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F208" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G208" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H208" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I208" s="19">
         <f>IF(OR(F208="",G208=""),"",F208*G208)</f>
         <v/>
@@ -10622,20 +10662,38 @@
         <f>IF(OR(F208="",G208=""),"",ROUND(G208*(1+F208/30),1))</f>
         <v/>
       </c>
-      <c r="K208" s="20" t="n"/>
+      <c r="K208" s="20" t="inlineStr"/>
     </row>
     <row r="209" ht="18" customHeight="1">
-      <c r="A209" s="21" t="n"/>
+      <c r="A209" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B209" s="22">
         <f>IF(A209="","",IFERROR(INT((A209-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C209" s="22" t="n"/>
-      <c r="D209" s="23" t="n"/>
-      <c r="E209" s="22" t="n"/>
-      <c r="F209" s="22" t="n"/>
-      <c r="G209" s="24" t="n"/>
-      <c r="H209" s="22" t="n"/>
+      <c r="C209" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D209" s="23" t="inlineStr">
+        <is>
+          <t>Standing Chest Press</t>
+        </is>
+      </c>
+      <c r="E209" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F209" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G209" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="H209" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I209" s="25">
         <f>IF(OR(F209="",G209=""),"",F209*G209)</f>
         <v/>
@@ -10644,20 +10702,38 @@
         <f>IF(OR(F209="",G209=""),"",ROUND(G209*(1+F209/30),1))</f>
         <v/>
       </c>
-      <c r="K209" s="26" t="n"/>
+      <c r="K209" s="26" t="inlineStr"/>
     </row>
     <row r="210" ht="18" customHeight="1">
-      <c r="A210" s="15" t="n"/>
+      <c r="A210" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B210" s="16">
         <f>IF(A210="","",IFERROR(INT((A210-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C210" s="16" t="n"/>
-      <c r="D210" s="17" t="n"/>
-      <c r="E210" s="16" t="n"/>
-      <c r="F210" s="16" t="n"/>
-      <c r="G210" s="18" t="n"/>
-      <c r="H210" s="16" t="n"/>
+      <c r="C210" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D210" s="17" t="inlineStr">
+        <is>
+          <t>Standing Chest Press</t>
+        </is>
+      </c>
+      <c r="E210" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F210" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G210" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H210" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I210" s="19">
         <f>IF(OR(F210="",G210=""),"",F210*G210)</f>
         <v/>
@@ -10666,20 +10742,42 @@
         <f>IF(OR(F210="",G210=""),"",ROUND(G210*(1+F210/30),1))</f>
         <v/>
       </c>
-      <c r="K210" s="20" t="n"/>
+      <c r="K210" s="20" t="inlineStr">
+        <is>
+          <t>RPE5-6 trivial; bump 7.5-10 next</t>
+        </is>
+      </c>
     </row>
     <row r="211" ht="18" customHeight="1">
-      <c r="A211" s="21" t="n"/>
+      <c r="A211" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B211" s="22">
         <f>IF(A211="","",IFERROR(INT((A211-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C211" s="22" t="n"/>
-      <c r="D211" s="23" t="n"/>
-      <c r="E211" s="22" t="n"/>
-      <c r="F211" s="22" t="n"/>
-      <c r="G211" s="24" t="n"/>
-      <c r="H211" s="22" t="n"/>
+      <c r="C211" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D211" s="23" t="inlineStr">
+        <is>
+          <t>DB Shoulder Press</t>
+        </is>
+      </c>
+      <c r="E211" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F211" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G211" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="H211" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="I211" s="25">
         <f>IF(OR(F211="",G211=""),"",F211*G211)</f>
         <v/>
@@ -10688,20 +10786,42 @@
         <f>IF(OR(F211="",G211=""),"",ROUND(G211*(1+F211/30),1))</f>
         <v/>
       </c>
-      <c r="K211" s="26" t="n"/>
+      <c r="K211" s="26" t="inlineStr">
+        <is>
+          <t>shoulder gate CLEAN (weak, no pain)</t>
+        </is>
+      </c>
     </row>
     <row r="212" ht="18" customHeight="1">
-      <c r="A212" s="15" t="n"/>
+      <c r="A212" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B212" s="16">
         <f>IF(A212="","",IFERROR(INT((A212-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C212" s="16" t="n"/>
-      <c r="D212" s="17" t="n"/>
-      <c r="E212" s="16" t="n"/>
-      <c r="F212" s="16" t="n"/>
-      <c r="G212" s="18" t="n"/>
-      <c r="H212" s="16" t="n"/>
+      <c r="C212" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D212" s="17" t="inlineStr">
+        <is>
+          <t>DB Shoulder Press</t>
+        </is>
+      </c>
+      <c r="E212" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F212" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G212" s="18" t="n">
+        <v>3</v>
+      </c>
+      <c r="H212" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="I212" s="19">
         <f>IF(OR(F212="",G212=""),"",F212*G212)</f>
         <v/>
@@ -10710,20 +10830,38 @@
         <f>IF(OR(F212="",G212=""),"",ROUND(G212*(1+F212/30),1))</f>
         <v/>
       </c>
-      <c r="K212" s="20" t="n"/>
+      <c r="K212" s="20" t="inlineStr"/>
     </row>
     <row r="213" ht="18" customHeight="1">
-      <c r="A213" s="21" t="n"/>
+      <c r="A213" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B213" s="22">
         <f>IF(A213="","",IFERROR(INT((A213-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C213" s="22" t="n"/>
-      <c r="D213" s="23" t="n"/>
-      <c r="E213" s="22" t="n"/>
-      <c r="F213" s="22" t="n"/>
-      <c r="G213" s="24" t="n"/>
-      <c r="H213" s="22" t="n"/>
+      <c r="C213" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D213" s="23" t="inlineStr">
+        <is>
+          <t>DB Shoulder Press</t>
+        </is>
+      </c>
+      <c r="E213" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F213" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G213" s="24" t="n">
+        <v>3</v>
+      </c>
+      <c r="H213" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="I213" s="25">
         <f>IF(OR(F213="",G213=""),"",F213*G213)</f>
         <v/>
@@ -10732,20 +10870,42 @@
         <f>IF(OR(F213="",G213=""),"",ROUND(G213*(1+F213/30),1))</f>
         <v/>
       </c>
-      <c r="K213" s="26" t="n"/>
+      <c r="K213" s="26" t="inlineStr">
+        <is>
+          <t>RPE5; bump 5/DB next, cap RPE7</t>
+        </is>
+      </c>
     </row>
     <row r="214" ht="18" customHeight="1">
-      <c r="A214" s="15" t="n"/>
+      <c r="A214" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B214" s="16">
         <f>IF(A214="","",IFERROR(INT((A214-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C214" s="16" t="n"/>
-      <c r="D214" s="17" t="n"/>
-      <c r="E214" s="16" t="n"/>
-      <c r="F214" s="16" t="n"/>
-      <c r="G214" s="18" t="n"/>
-      <c r="H214" s="16" t="n"/>
+      <c r="C214" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D214" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E214" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F214" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G214" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H214" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I214" s="19">
         <f>IF(OR(F214="",G214=""),"",F214*G214)</f>
         <v/>
@@ -10754,20 +10914,38 @@
         <f>IF(OR(F214="",G214=""),"",ROUND(G214*(1+F214/30),1))</f>
         <v/>
       </c>
-      <c r="K214" s="20" t="n"/>
+      <c r="K214" s="20" t="inlineStr"/>
     </row>
     <row r="215" ht="18" customHeight="1">
-      <c r="A215" s="21" t="n"/>
+      <c r="A215" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B215" s="22">
         <f>IF(A215="","",IFERROR(INT((A215-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C215" s="22" t="n"/>
-      <c r="D215" s="23" t="n"/>
-      <c r="E215" s="22" t="n"/>
-      <c r="F215" s="22" t="n"/>
-      <c r="G215" s="24" t="n"/>
-      <c r="H215" s="22" t="n"/>
+      <c r="C215" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D215" s="23" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E215" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F215" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G215" s="24" t="n">
+        <v>5</v>
+      </c>
+      <c r="H215" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I215" s="25">
         <f>IF(OR(F215="",G215=""),"",F215*G215)</f>
         <v/>
@@ -10776,20 +10954,38 @@
         <f>IF(OR(F215="",G215=""),"",ROUND(G215*(1+F215/30),1))</f>
         <v/>
       </c>
-      <c r="K215" s="26" t="n"/>
+      <c r="K215" s="26" t="inlineStr"/>
     </row>
     <row r="216" ht="18" customHeight="1">
-      <c r="A216" s="15" t="n"/>
+      <c r="A216" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B216" s="16">
         <f>IF(A216="","",IFERROR(INT((A216-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C216" s="16" t="n"/>
-      <c r="D216" s="17" t="n"/>
-      <c r="E216" s="16" t="n"/>
-      <c r="F216" s="16" t="n"/>
-      <c r="G216" s="18" t="n"/>
-      <c r="H216" s="16" t="n"/>
+      <c r="C216" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D216" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E216" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F216" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G216" s="18" t="n">
+        <v>5</v>
+      </c>
+      <c r="H216" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I216" s="19">
         <f>IF(OR(F216="",G216=""),"",F216*G216)</f>
         <v/>
@@ -10798,20 +10994,42 @@
         <f>IF(OR(F216="",G216=""),"",ROUND(G216*(1+F216/30),1))</f>
         <v/>
       </c>
-      <c r="K216" s="20" t="n"/>
+      <c r="K216" s="20" t="inlineStr">
+        <is>
+          <t>RPE7 top range; bump 6-7/DB next</t>
+        </is>
+      </c>
     </row>
     <row r="217" ht="18" customHeight="1">
-      <c r="A217" s="21" t="n"/>
+      <c r="A217" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B217" s="22">
         <f>IF(A217="","",IFERROR(INT((A217-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C217" s="22" t="n"/>
-      <c r="D217" s="23" t="n"/>
-      <c r="E217" s="22" t="n"/>
-      <c r="F217" s="22" t="n"/>
-      <c r="G217" s="24" t="n"/>
-      <c r="H217" s="22" t="n"/>
+      <c r="C217" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D217" s="23" t="inlineStr">
+        <is>
+          <t>Pec Deck</t>
+        </is>
+      </c>
+      <c r="E217" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F217" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="G217" s="24" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H217" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I217" s="25">
         <f>IF(OR(F217="",G217=""),"",F217*G217)</f>
         <v/>
@@ -10820,20 +11038,38 @@
         <f>IF(OR(F217="",G217=""),"",ROUND(G217*(1+F217/30),1))</f>
         <v/>
       </c>
-      <c r="K217" s="26" t="n"/>
+      <c r="K217" s="26" t="inlineStr"/>
     </row>
     <row r="218" ht="18" customHeight="1">
-      <c r="A218" s="15" t="n"/>
+      <c r="A218" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B218" s="16">
         <f>IF(A218="","",IFERROR(INT((A218-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C218" s="16" t="n"/>
-      <c r="D218" s="17" t="n"/>
-      <c r="E218" s="16" t="n"/>
-      <c r="F218" s="16" t="n"/>
-      <c r="G218" s="18" t="n"/>
-      <c r="H218" s="16" t="n"/>
+      <c r="C218" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D218" s="17" t="inlineStr">
+        <is>
+          <t>Pec Deck</t>
+        </is>
+      </c>
+      <c r="E218" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F218" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G218" s="18" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H218" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I218" s="19">
         <f>IF(OR(F218="",G218=""),"",F218*G218)</f>
         <v/>
@@ -10842,20 +11078,38 @@
         <f>IF(OR(F218="",G218=""),"",ROUND(G218*(1+F218/30),1))</f>
         <v/>
       </c>
-      <c r="K218" s="20" t="n"/>
+      <c r="K218" s="20" t="inlineStr"/>
     </row>
     <row r="219" ht="18" customHeight="1">
-      <c r="A219" s="21" t="n"/>
+      <c r="A219" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B219" s="22">
         <f>IF(A219="","",IFERROR(INT((A219-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C219" s="22" t="n"/>
-      <c r="D219" s="23" t="n"/>
-      <c r="E219" s="22" t="n"/>
-      <c r="F219" s="22" t="n"/>
-      <c r="G219" s="24" t="n"/>
-      <c r="H219" s="22" t="n"/>
+      <c r="C219" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D219" s="23" t="inlineStr">
+        <is>
+          <t>Pec Deck</t>
+        </is>
+      </c>
+      <c r="E219" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F219" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="G219" s="24" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H219" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I219" s="25">
         <f>IF(OR(F219="",G219=""),"",F219*G219)</f>
         <v/>
@@ -10864,20 +11118,42 @@
         <f>IF(OR(F219="",G219=""),"",ROUND(G219*(1+F219/30),1))</f>
         <v/>
       </c>
-      <c r="K219" s="26" t="n"/>
+      <c r="K219" s="26" t="inlineStr">
+        <is>
+          <t>reps fell 9-&gt;6-&gt;6; HOLD 2.5 rebuild 12+</t>
+        </is>
+      </c>
     </row>
     <row r="220" ht="18" customHeight="1">
-      <c r="A220" s="15" t="n"/>
+      <c r="A220" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B220" s="16">
         <f>IF(A220="","",IFERROR(INT((A220-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C220" s="16" t="n"/>
-      <c r="D220" s="17" t="n"/>
-      <c r="E220" s="16" t="n"/>
-      <c r="F220" s="16" t="n"/>
-      <c r="G220" s="18" t="n"/>
-      <c r="H220" s="16" t="n"/>
+      <c r="C220" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D220" s="17" t="inlineStr">
+        <is>
+          <t>Triceps Pushdown</t>
+        </is>
+      </c>
+      <c r="E220" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F220" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G220" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="H220" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I220" s="19">
         <f>IF(OR(F220="",G220=""),"",F220*G220)</f>
         <v/>
@@ -10886,20 +11162,38 @@
         <f>IF(OR(F220="",G220=""),"",ROUND(G220*(1+F220/30),1))</f>
         <v/>
       </c>
-      <c r="K220" s="20" t="n"/>
+      <c r="K220" s="20" t="inlineStr"/>
     </row>
     <row r="221" ht="18" customHeight="1">
-      <c r="A221" s="21" t="n"/>
+      <c r="A221" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B221" s="22">
         <f>IF(A221="","",IFERROR(INT((A221-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C221" s="22" t="n"/>
-      <c r="D221" s="23" t="n"/>
-      <c r="E221" s="22" t="n"/>
-      <c r="F221" s="22" t="n"/>
-      <c r="G221" s="24" t="n"/>
-      <c r="H221" s="22" t="n"/>
+      <c r="C221" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D221" s="23" t="inlineStr">
+        <is>
+          <t>Triceps Pushdown</t>
+        </is>
+      </c>
+      <c r="E221" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F221" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G221" s="24" t="n">
+        <v>15</v>
+      </c>
+      <c r="H221" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I221" s="25">
         <f>IF(OR(F221="",G221=""),"",F221*G221)</f>
         <v/>
@@ -10908,20 +11202,38 @@
         <f>IF(OR(F221="",G221=""),"",ROUND(G221*(1+F221/30),1))</f>
         <v/>
       </c>
-      <c r="K221" s="26" t="n"/>
+      <c r="K221" s="26" t="inlineStr"/>
     </row>
     <row r="222" ht="18" customHeight="1">
-      <c r="A222" s="15" t="n"/>
+      <c r="A222" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B222" s="16">
         <f>IF(A222="","",IFERROR(INT((A222-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C222" s="16" t="n"/>
-      <c r="D222" s="17" t="n"/>
-      <c r="E222" s="16" t="n"/>
-      <c r="F222" s="16" t="n"/>
-      <c r="G222" s="18" t="n"/>
-      <c r="H222" s="16" t="n"/>
+      <c r="C222" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D222" s="17" t="inlineStr">
+        <is>
+          <t>Triceps Pushdown</t>
+        </is>
+      </c>
+      <c r="E222" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F222" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G222" s="18" t="n">
+        <v>15</v>
+      </c>
+      <c r="H222" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="I222" s="19">
         <f>IF(OR(F222="",G222=""),"",F222*G222)</f>
         <v/>
@@ -10930,20 +11242,42 @@
         <f>IF(OR(F222="",G222=""),"",ROUND(G222*(1+F222/30),1))</f>
         <v/>
       </c>
-      <c r="K222" s="20" t="n"/>
+      <c r="K222" s="20" t="inlineStr">
+        <is>
+          <t>hit top @RPE8-9; bump 17.5 next</t>
+        </is>
+      </c>
     </row>
     <row r="223" ht="18" customHeight="1">
-      <c r="A223" s="21" t="n"/>
+      <c r="A223" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B223" s="22">
         <f>IF(A223="","",IFERROR(INT((A223-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C223" s="22" t="n"/>
-      <c r="D223" s="23" t="n"/>
-      <c r="E223" s="22" t="n"/>
-      <c r="F223" s="22" t="n"/>
-      <c r="G223" s="24" t="n"/>
-      <c r="H223" s="22" t="n"/>
+      <c r="C223" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D223" s="23" t="inlineStr">
+        <is>
+          <t>DB Lateral Raise</t>
+        </is>
+      </c>
+      <c r="E223" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F223" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G223" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H223" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I223" s="25">
         <f>IF(OR(F223="",G223=""),"",F223*G223)</f>
         <v/>
@@ -10952,20 +11286,38 @@
         <f>IF(OR(F223="",G223=""),"",ROUND(G223*(1+F223/30),1))</f>
         <v/>
       </c>
-      <c r="K223" s="26" t="n"/>
+      <c r="K223" s="26" t="inlineStr"/>
     </row>
     <row r="224" ht="18" customHeight="1">
-      <c r="A224" s="15" t="n"/>
+      <c r="A224" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B224" s="16">
         <f>IF(A224="","",IFERROR(INT((A224-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C224" s="16" t="n"/>
-      <c r="D224" s="17" t="n"/>
-      <c r="E224" s="16" t="n"/>
-      <c r="F224" s="16" t="n"/>
-      <c r="G224" s="18" t="n"/>
-      <c r="H224" s="16" t="n"/>
+      <c r="C224" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D224" s="17" t="inlineStr">
+        <is>
+          <t>DB Lateral Raise</t>
+        </is>
+      </c>
+      <c r="E224" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F224" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G224" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="H224" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I224" s="19">
         <f>IF(OR(F224="",G224=""),"",F224*G224)</f>
         <v/>
@@ -10974,20 +11326,38 @@
         <f>IF(OR(F224="",G224=""),"",ROUND(G224*(1+F224/30),1))</f>
         <v/>
       </c>
-      <c r="K224" s="20" t="n"/>
+      <c r="K224" s="20" t="inlineStr"/>
     </row>
     <row r="225" ht="18" customHeight="1">
-      <c r="A225" s="21" t="n"/>
+      <c r="A225" s="21" t="n">
+        <v>46181</v>
+      </c>
       <c r="B225" s="22">
         <f>IF(A225="","",IFERROR(INT((A225-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C225" s="22" t="n"/>
-      <c r="D225" s="23" t="n"/>
-      <c r="E225" s="22" t="n"/>
-      <c r="F225" s="22" t="n"/>
-      <c r="G225" s="24" t="n"/>
-      <c r="H225" s="22" t="n"/>
+      <c r="C225" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D225" s="23" t="inlineStr">
+        <is>
+          <t>DB Lateral Raise</t>
+        </is>
+      </c>
+      <c r="E225" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F225" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G225" s="24" t="n">
+        <v>2</v>
+      </c>
+      <c r="H225" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I225" s="25">
         <f>IF(OR(F225="",G225=""),"",F225*G225)</f>
         <v/>
@@ -10996,7 +11366,11 @@
         <f>IF(OR(F225="",G225=""),"",ROUND(G225*(1+F225/30),1))</f>
         <v/>
       </c>
-      <c r="K225" s="26" t="n"/>
+      <c r="K225" s="26" t="inlineStr">
+        <is>
+          <t>bottom range; HOLD 2 chase 15s then 3/DB</t>
+        </is>
+      </c>
     </row>
     <row r="226" ht="18" customHeight="1">
       <c r="A226" s="15" t="n"/>
@@ -26865,18 +27239,28 @@
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="15" t="n"/>
+      <c r="A14" s="15" t="n">
+        <v>46181</v>
+      </c>
       <c r="B14" s="16">
         <f>IF(A14="","",IFERROR(INT((A14-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C14" s="18" t="n"/>
-      <c r="D14" s="18" t="n"/>
+      <c r="C14" s="18" t="n">
+        <v>77.09999999999999</v>
+      </c>
+      <c r="D14" s="18" t="n">
+        <v>7</v>
+      </c>
       <c r="E14" s="18" t="n"/>
       <c r="F14" s="18" t="n"/>
       <c r="G14" s="18" t="n"/>
       <c r="H14" s="18" t="n"/>
-      <c r="I14" s="20" t="n"/>
+      <c r="I14" s="20" t="inlineStr">
+        <is>
+          <t>Build W1 Mon AM (cut PAUSED, maintenance — BW gain expected, NOT flagged)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="21" t="n"/>

</xml_diff>

<commit_message>
log: Build W1 Wed 6/10 PM — Pull DONE (19 sets/230 reps/3743.8kg, RPE7.1) + exercise locks
Pull #1 off 2+ wk layoff. Shoulder fully clean whole session. Pulldown
35 opener = RPE9 misfire, settled 30 for clean 12s. Exercise changes
locked per user: pulldown 4x10-12, plain cable row, single-arm DB row
in (reverse pec deck out), EZ bar curl in (preacher out). Progression
posture re-confirmed slow-steady (supersedes aggressive bumps). Also
backfills 6/9 run + 6/9-6/10 BW into xlsx.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -11373,17 +11373,35 @@
       </c>
     </row>
     <row r="226" ht="18" customHeight="1">
-      <c r="A226" s="15" t="n"/>
+      <c r="A226" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B226" s="16">
         <f>IF(A226="","",IFERROR(INT((A226-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C226" s="16" t="n"/>
-      <c r="D226" s="17" t="n"/>
-      <c r="E226" s="16" t="n"/>
-      <c r="F226" s="16" t="n"/>
-      <c r="G226" s="18" t="n"/>
-      <c r="H226" s="16" t="n"/>
+      <c r="C226" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D226" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E226" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F226" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G226" s="18" t="n">
+        <v>35</v>
+      </c>
+      <c r="H226" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="I226" s="19">
         <f>IF(OR(F226="",G226=""),"",F226*G226)</f>
         <v/>
@@ -11392,20 +11410,42 @@
         <f>IF(OR(F226="",G226=""),"",ROUND(G226*(1+F226/30),1))</f>
         <v/>
       </c>
-      <c r="K226" s="20" t="n"/>
+      <c r="K226" s="20" t="inlineStr">
+        <is>
+          <t>opener 35 RPE9 off layoff; dropped to 30</t>
+        </is>
+      </c>
     </row>
     <row r="227" ht="18" customHeight="1">
-      <c r="A227" s="21" t="n"/>
+      <c r="A227" s="21" t="n">
+        <v>46183</v>
+      </c>
       <c r="B227" s="22">
         <f>IF(A227="","",IFERROR(INT((A227-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C227" s="22" t="n"/>
-      <c r="D227" s="23" t="n"/>
-      <c r="E227" s="22" t="n"/>
-      <c r="F227" s="22" t="n"/>
-      <c r="G227" s="24" t="n"/>
-      <c r="H227" s="22" t="n"/>
+      <c r="C227" s="22" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D227" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E227" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F227" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G227" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="H227" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I227" s="25">
         <f>IF(OR(F227="",G227=""),"",F227*G227)</f>
         <v/>
@@ -11414,20 +11454,42 @@
         <f>IF(OR(F227="",G227=""),"",ROUND(G227*(1+F227/30),1))</f>
         <v/>
       </c>
-      <c r="K227" s="26" t="n"/>
+      <c r="K227" s="26" t="inlineStr">
+        <is>
+          <t>rep range locked 4x10-12 (user pref)</t>
+        </is>
+      </c>
     </row>
     <row r="228" ht="18" customHeight="1">
-      <c r="A228" s="15" t="n"/>
+      <c r="A228" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B228" s="16">
         <f>IF(A228="","",IFERROR(INT((A228-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C228" s="16" t="n"/>
-      <c r="D228" s="17" t="n"/>
-      <c r="E228" s="16" t="n"/>
-      <c r="F228" s="16" t="n"/>
-      <c r="G228" s="18" t="n"/>
-      <c r="H228" s="16" t="n"/>
+      <c r="C228" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D228" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E228" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F228" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G228" s="18" t="n">
+        <v>30</v>
+      </c>
+      <c r="H228" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I228" s="19">
         <f>IF(OR(F228="",G228=""),"",F228*G228)</f>
         <v/>
@@ -11436,20 +11498,38 @@
         <f>IF(OR(F228="",G228=""),"",ROUND(G228*(1+F228/30),1))</f>
         <v/>
       </c>
-      <c r="K228" s="20" t="n"/>
+      <c r="K228" s="20" t="inlineStr"/>
     </row>
     <row r="229" ht="18" customHeight="1">
-      <c r="A229" s="21" t="n"/>
+      <c r="A229" s="21" t="n">
+        <v>46183</v>
+      </c>
       <c r="B229" s="22">
         <f>IF(A229="","",IFERROR(INT((A229-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C229" s="22" t="n"/>
-      <c r="D229" s="23" t="n"/>
-      <c r="E229" s="22" t="n"/>
-      <c r="F229" s="22" t="n"/>
-      <c r="G229" s="24" t="n"/>
-      <c r="H229" s="22" t="n"/>
+      <c r="C229" s="22" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D229" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E229" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F229" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G229" s="24" t="n">
+        <v>30</v>
+      </c>
+      <c r="H229" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I229" s="25">
         <f>IF(OR(F229="",G229=""),"",F229*G229)</f>
         <v/>
@@ -11458,20 +11538,42 @@
         <f>IF(OR(F229="",G229=""),"",ROUND(G229*(1+F229/30),1))</f>
         <v/>
       </c>
-      <c r="K229" s="26" t="n"/>
+      <c r="K229" s="26" t="inlineStr">
+        <is>
+          <t>12s clean @30; 32.5 next, cap RPE8</t>
+        </is>
+      </c>
     </row>
     <row r="230" ht="18" customHeight="1">
-      <c r="A230" s="15" t="n"/>
+      <c r="A230" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B230" s="16">
         <f>IF(A230="","",IFERROR(INT((A230-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C230" s="16" t="n"/>
-      <c r="D230" s="17" t="n"/>
-      <c r="E230" s="16" t="n"/>
-      <c r="F230" s="16" t="n"/>
-      <c r="G230" s="18" t="n"/>
-      <c r="H230" s="16" t="n"/>
+      <c r="C230" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D230" s="17" t="inlineStr">
+        <is>
+          <t>Cable Row</t>
+        </is>
+      </c>
+      <c r="E230" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F230" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G230" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="H230" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I230" s="19">
         <f>IF(OR(F230="",G230=""),"",F230*G230)</f>
         <v/>
@@ -11480,20 +11582,42 @@
         <f>IF(OR(F230="",G230=""),"",ROUND(G230*(1+F230/30),1))</f>
         <v/>
       </c>
-      <c r="K230" s="20" t="n"/>
+      <c r="K230" s="20" t="inlineStr">
+        <is>
+          <t>locked: plain cable row (vs chest-supported)</t>
+        </is>
+      </c>
     </row>
     <row r="231" ht="18" customHeight="1">
-      <c r="A231" s="21" t="n"/>
+      <c r="A231" s="21" t="n">
+        <v>46183</v>
+      </c>
       <c r="B231" s="22">
         <f>IF(A231="","",IFERROR(INT((A231-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C231" s="22" t="n"/>
-      <c r="D231" s="23" t="n"/>
-      <c r="E231" s="22" t="n"/>
-      <c r="F231" s="22" t="n"/>
-      <c r="G231" s="24" t="n"/>
-      <c r="H231" s="22" t="n"/>
+      <c r="C231" s="22" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D231" s="23" t="inlineStr">
+        <is>
+          <t>Cable Row</t>
+        </is>
+      </c>
+      <c r="E231" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F231" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G231" s="24" t="n">
+        <v>25</v>
+      </c>
+      <c r="H231" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I231" s="25">
         <f>IF(OR(F231="",G231=""),"",F231*G231)</f>
         <v/>
@@ -11502,20 +11626,38 @@
         <f>IF(OR(F231="",G231=""),"",ROUND(G231*(1+F231/30),1))</f>
         <v/>
       </c>
-      <c r="K231" s="26" t="n"/>
+      <c r="K231" s="26" t="inlineStr"/>
     </row>
     <row r="232" ht="18" customHeight="1">
-      <c r="A232" s="15" t="n"/>
+      <c r="A232" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B232" s="16">
         <f>IF(A232="","",IFERROR(INT((A232-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C232" s="16" t="n"/>
-      <c r="D232" s="17" t="n"/>
-      <c r="E232" s="16" t="n"/>
-      <c r="F232" s="16" t="n"/>
-      <c r="G232" s="18" t="n"/>
-      <c r="H232" s="16" t="n"/>
+      <c r="C232" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D232" s="17" t="inlineStr">
+        <is>
+          <t>Cable Row</t>
+        </is>
+      </c>
+      <c r="E232" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F232" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G232" s="18" t="n">
+        <v>25</v>
+      </c>
+      <c r="H232" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I232" s="19">
         <f>IF(OR(F232="",G232=""),"",F232*G232)</f>
         <v/>
@@ -11524,20 +11666,42 @@
         <f>IF(OR(F232="",G232=""),"",ROUND(G232*(1+F232/30),1))</f>
         <v/>
       </c>
-      <c r="K232" s="20" t="n"/>
+      <c r="K232" s="20" t="inlineStr">
+        <is>
+          <t>3x12 @RPE6-7 under; 27.5 next</t>
+        </is>
+      </c>
     </row>
     <row r="233" ht="18" customHeight="1">
-      <c r="A233" s="21" t="n"/>
+      <c r="A233" s="21" t="n">
+        <v>46183</v>
+      </c>
       <c r="B233" s="22">
         <f>IF(A233="","",IFERROR(INT((A233-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C233" s="22" t="n"/>
-      <c r="D233" s="23" t="n"/>
-      <c r="E233" s="22" t="n"/>
-      <c r="F233" s="22" t="n"/>
-      <c r="G233" s="24" t="n"/>
-      <c r="H233" s="22" t="n"/>
+      <c r="C233" s="22" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D233" s="23" t="inlineStr">
+        <is>
+          <t>Single Arm DB Row</t>
+        </is>
+      </c>
+      <c r="E233" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F233" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G233" s="24" t="n">
+        <v>7</v>
+      </c>
+      <c r="H233" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="I233" s="25">
         <f>IF(OR(F233="",G233=""),"",F233*G233)</f>
         <v/>
@@ -11546,20 +11710,42 @@
         <f>IF(OR(F233="",G233=""),"",ROUND(G233*(1+F233/30),1))</f>
         <v/>
       </c>
-      <c r="K233" s="26" t="n"/>
+      <c r="K233" s="26" t="inlineStr">
+        <is>
+          <t>NEW locked (replaces Reverse Pec Deck); reps per side</t>
+        </is>
+      </c>
     </row>
     <row r="234" ht="18" customHeight="1">
-      <c r="A234" s="15" t="n"/>
+      <c r="A234" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B234" s="16">
         <f>IF(A234="","",IFERROR(INT((A234-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C234" s="16" t="n"/>
-      <c r="D234" s="17" t="n"/>
-      <c r="E234" s="16" t="n"/>
-      <c r="F234" s="16" t="n"/>
-      <c r="G234" s="18" t="n"/>
-      <c r="H234" s="16" t="n"/>
+      <c r="C234" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D234" s="17" t="inlineStr">
+        <is>
+          <t>Single Arm DB Row</t>
+        </is>
+      </c>
+      <c r="E234" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F234" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G234" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="H234" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I234" s="19">
         <f>IF(OR(F234="",G234=""),"",F234*G234)</f>
         <v/>
@@ -11568,20 +11754,38 @@
         <f>IF(OR(F234="",G234=""),"",ROUND(G234*(1+F234/30),1))</f>
         <v/>
       </c>
-      <c r="K234" s="20" t="n"/>
+      <c r="K234" s="20" t="inlineStr"/>
     </row>
     <row r="235" ht="18" customHeight="1">
-      <c r="A235" s="21" t="n"/>
+      <c r="A235" s="21" t="n">
+        <v>46183</v>
+      </c>
       <c r="B235" s="22">
         <f>IF(A235="","",IFERROR(INT((A235-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C235" s="22" t="n"/>
-      <c r="D235" s="23" t="n"/>
-      <c r="E235" s="22" t="n"/>
-      <c r="F235" s="22" t="n"/>
-      <c r="G235" s="24" t="n"/>
-      <c r="H235" s="22" t="n"/>
+      <c r="C235" s="22" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D235" s="23" t="inlineStr">
+        <is>
+          <t>Single Arm DB Row</t>
+        </is>
+      </c>
+      <c r="E235" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F235" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G235" s="24" t="n">
+        <v>8</v>
+      </c>
+      <c r="H235" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I235" s="25">
         <f>IF(OR(F235="",G235=""),"",F235*G235)</f>
         <v/>
@@ -11590,20 +11794,42 @@
         <f>IF(OR(F235="",G235=""),"",ROUND(G235*(1+F235/30),1))</f>
         <v/>
       </c>
-      <c r="K235" s="26" t="n"/>
+      <c r="K235" s="26" t="inlineStr">
+        <is>
+          <t>top range @RPE7; 9/DB next</t>
+        </is>
+      </c>
     </row>
     <row r="236" ht="18" customHeight="1">
-      <c r="A236" s="15" t="n"/>
+      <c r="A236" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B236" s="16">
         <f>IF(A236="","",IFERROR(INT((A236-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C236" s="16" t="n"/>
-      <c r="D236" s="17" t="n"/>
-      <c r="E236" s="16" t="n"/>
-      <c r="F236" s="16" t="n"/>
-      <c r="G236" s="18" t="n"/>
-      <c r="H236" s="16" t="n"/>
+      <c r="C236" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D236" s="17" t="inlineStr">
+        <is>
+          <t>Face Pull</t>
+        </is>
+      </c>
+      <c r="E236" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F236" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G236" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="H236" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I236" s="19">
         <f>IF(OR(F236="",G236=""),"",F236*G236)</f>
         <v/>
@@ -11612,20 +11838,38 @@
         <f>IF(OR(F236="",G236=""),"",ROUND(G236*(1+F236/30),1))</f>
         <v/>
       </c>
-      <c r="K236" s="20" t="n"/>
+      <c r="K236" s="20" t="inlineStr"/>
     </row>
     <row r="237" ht="18" customHeight="1">
-      <c r="A237" s="21" t="n"/>
+      <c r="A237" s="21" t="n">
+        <v>46183</v>
+      </c>
       <c r="B237" s="22">
         <f>IF(A237="","",IFERROR(INT((A237-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C237" s="22" t="n"/>
-      <c r="D237" s="23" t="n"/>
-      <c r="E237" s="22" t="n"/>
-      <c r="F237" s="22" t="n"/>
-      <c r="G237" s="24" t="n"/>
-      <c r="H237" s="22" t="n"/>
+      <c r="C237" s="22" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D237" s="23" t="inlineStr">
+        <is>
+          <t>Face Pull</t>
+        </is>
+      </c>
+      <c r="E237" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F237" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G237" s="24" t="n">
+        <v>10</v>
+      </c>
+      <c r="H237" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I237" s="25">
         <f>IF(OR(F237="",G237=""),"",F237*G237)</f>
         <v/>
@@ -11634,20 +11878,38 @@
         <f>IF(OR(F237="",G237=""),"",ROUND(G237*(1+F237/30),1))</f>
         <v/>
       </c>
-      <c r="K237" s="26" t="n"/>
+      <c r="K237" s="26" t="inlineStr"/>
     </row>
     <row r="238" ht="18" customHeight="1">
-      <c r="A238" s="15" t="n"/>
+      <c r="A238" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B238" s="16">
         <f>IF(A238="","",IFERROR(INT((A238-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C238" s="16" t="n"/>
-      <c r="D238" s="17" t="n"/>
-      <c r="E238" s="16" t="n"/>
-      <c r="F238" s="16" t="n"/>
-      <c r="G238" s="18" t="n"/>
-      <c r="H238" s="16" t="n"/>
+      <c r="C238" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D238" s="17" t="inlineStr">
+        <is>
+          <t>Face Pull</t>
+        </is>
+      </c>
+      <c r="E238" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F238" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G238" s="18" t="n">
+        <v>10</v>
+      </c>
+      <c r="H238" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I238" s="19">
         <f>IF(OR(F238="",G238=""),"",F238*G238)</f>
         <v/>
@@ -11656,20 +11918,42 @@
         <f>IF(OR(F238="",G238=""),"",ROUND(G238*(1+F238/30),1))</f>
         <v/>
       </c>
-      <c r="K238" s="20" t="n"/>
+      <c r="K238" s="20" t="inlineStr">
+        <is>
+          <t>HOLD 10, chase 16-18, 12.5 at 20s</t>
+        </is>
+      </c>
     </row>
     <row r="239" ht="18" customHeight="1">
-      <c r="A239" s="21" t="n"/>
+      <c r="A239" s="21" t="n">
+        <v>46183</v>
+      </c>
       <c r="B239" s="22">
         <f>IF(A239="","",IFERROR(INT((A239-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C239" s="22" t="n"/>
-      <c r="D239" s="23" t="n"/>
-      <c r="E239" s="22" t="n"/>
-      <c r="F239" s="22" t="n"/>
-      <c r="G239" s="24" t="n"/>
-      <c r="H239" s="22" t="n"/>
+      <c r="C239" s="22" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D239" s="23" t="inlineStr">
+        <is>
+          <t>EZ Bar Curl</t>
+        </is>
+      </c>
+      <c r="E239" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F239" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G239" s="24" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="H239" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I239" s="25">
         <f>IF(OR(F239="",G239=""),"",F239*G239)</f>
         <v/>
@@ -11678,20 +11962,42 @@
         <f>IF(OR(F239="",G239=""),"",ROUND(G239*(1+F239/30),1))</f>
         <v/>
       </c>
-      <c r="K239" s="26" t="n"/>
+      <c r="K239" s="26" t="inlineStr">
+        <is>
+          <t>NEW locked (replaces Preacher Curl)</t>
+        </is>
+      </c>
     </row>
     <row r="240" ht="18" customHeight="1">
-      <c r="A240" s="15" t="n"/>
+      <c r="A240" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B240" s="16">
         <f>IF(A240="","",IFERROR(INT((A240-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C240" s="16" t="n"/>
-      <c r="D240" s="17" t="n"/>
-      <c r="E240" s="16" t="n"/>
-      <c r="F240" s="16" t="n"/>
-      <c r="G240" s="18" t="n"/>
-      <c r="H240" s="16" t="n"/>
+      <c r="C240" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D240" s="17" t="inlineStr">
+        <is>
+          <t>EZ Bar Curl</t>
+        </is>
+      </c>
+      <c r="E240" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F240" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G240" s="18" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="H240" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I240" s="19">
         <f>IF(OR(F240="",G240=""),"",F240*G240)</f>
         <v/>
@@ -11700,20 +12006,38 @@
         <f>IF(OR(F240="",G240=""),"",ROUND(G240*(1+F240/30),1))</f>
         <v/>
       </c>
-      <c r="K240" s="20" t="n"/>
+      <c r="K240" s="20" t="inlineStr"/>
     </row>
     <row r="241" ht="18" customHeight="1">
-      <c r="A241" s="21" t="n"/>
+      <c r="A241" s="21" t="n">
+        <v>46183</v>
+      </c>
       <c r="B241" s="22">
         <f>IF(A241="","",IFERROR(INT((A241-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C241" s="22" t="n"/>
-      <c r="D241" s="23" t="n"/>
-      <c r="E241" s="22" t="n"/>
-      <c r="F241" s="22" t="n"/>
-      <c r="G241" s="24" t="n"/>
-      <c r="H241" s="22" t="n"/>
+      <c r="C241" s="22" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D241" s="23" t="inlineStr">
+        <is>
+          <t>EZ Bar Curl</t>
+        </is>
+      </c>
+      <c r="E241" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F241" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G241" s="24" t="n">
+        <v>13.6</v>
+      </c>
+      <c r="H241" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I241" s="25">
         <f>IF(OR(F241="",G241=""),"",F241*G241)</f>
         <v/>
@@ -11722,20 +12046,42 @@
         <f>IF(OR(F241="",G241=""),"",ROUND(G241*(1+F241/30),1))</f>
         <v/>
       </c>
-      <c r="K241" s="26" t="n"/>
+      <c r="K241" s="26" t="inlineStr">
+        <is>
+          <t>S3 fell to 8; HOLD 13.6 chase 3x10</t>
+        </is>
+      </c>
     </row>
     <row r="242" ht="18" customHeight="1">
-      <c r="A242" s="15" t="n"/>
+      <c r="A242" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B242" s="16">
         <f>IF(A242="","",IFERROR(INT((A242-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C242" s="16" t="n"/>
-      <c r="D242" s="17" t="n"/>
-      <c r="E242" s="16" t="n"/>
-      <c r="F242" s="16" t="n"/>
-      <c r="G242" s="18" t="n"/>
-      <c r="H242" s="16" t="n"/>
+      <c r="C242" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D242" s="17" t="inlineStr">
+        <is>
+          <t>DB Curl</t>
+        </is>
+      </c>
+      <c r="E242" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F242" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G242" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="H242" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I242" s="19">
         <f>IF(OR(F242="",G242=""),"",F242*G242)</f>
         <v/>
@@ -11744,20 +12090,38 @@
         <f>IF(OR(F242="",G242=""),"",ROUND(G242*(1+F242/30),1))</f>
         <v/>
       </c>
-      <c r="K242" s="20" t="n"/>
+      <c r="K242" s="20" t="inlineStr"/>
     </row>
     <row r="243" ht="18" customHeight="1">
-      <c r="A243" s="21" t="n"/>
+      <c r="A243" s="21" t="n">
+        <v>46183</v>
+      </c>
       <c r="B243" s="22">
         <f>IF(A243="","",IFERROR(INT((A243-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C243" s="22" t="n"/>
-      <c r="D243" s="23" t="n"/>
-      <c r="E243" s="22" t="n"/>
-      <c r="F243" s="22" t="n"/>
-      <c r="G243" s="24" t="n"/>
-      <c r="H243" s="22" t="n"/>
+      <c r="C243" s="22" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D243" s="23" t="inlineStr">
+        <is>
+          <t>DB Curl</t>
+        </is>
+      </c>
+      <c r="E243" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F243" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G243" s="24" t="n">
+        <v>6</v>
+      </c>
+      <c r="H243" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I243" s="25">
         <f>IF(OR(F243="",G243=""),"",F243*G243)</f>
         <v/>
@@ -11766,20 +12130,38 @@
         <f>IF(OR(F243="",G243=""),"",ROUND(G243*(1+F243/30),1))</f>
         <v/>
       </c>
-      <c r="K243" s="26" t="n"/>
+      <c r="K243" s="26" t="inlineStr"/>
     </row>
     <row r="244" ht="18" customHeight="1">
-      <c r="A244" s="15" t="n"/>
+      <c r="A244" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B244" s="16">
         <f>IF(A244="","",IFERROR(INT((A244-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C244" s="16" t="n"/>
-      <c r="D244" s="17" t="n"/>
-      <c r="E244" s="16" t="n"/>
-      <c r="F244" s="16" t="n"/>
-      <c r="G244" s="18" t="n"/>
-      <c r="H244" s="16" t="n"/>
+      <c r="C244" s="16" t="inlineStr">
+        <is>
+          <t>Pull</t>
+        </is>
+      </c>
+      <c r="D244" s="17" t="inlineStr">
+        <is>
+          <t>DB Curl</t>
+        </is>
+      </c>
+      <c r="E244" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F244" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G244" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="H244" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I244" s="19">
         <f>IF(OR(F244="",G244=""),"",F244*G244)</f>
         <v/>
@@ -11788,7 +12170,11 @@
         <f>IF(OR(F244="",G244=""),"",ROUND(G244*(1+F244/30),1))</f>
         <v/>
       </c>
-      <c r="K244" s="20" t="n"/>
+      <c r="K244" s="20" t="inlineStr">
+        <is>
+          <t>HOLD 6 chase 3x10 then 7</t>
+        </is>
+      </c>
     </row>
     <row r="245" ht="18" customHeight="1">
       <c r="A245" s="21" t="n"/>
@@ -24207,22 +24593,42 @@
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="15" t="n"/>
+      <c r="A4" s="15" t="n">
+        <v>46182</v>
+      </c>
       <c r="B4" s="16">
         <f>IF(A4="","",IFERROR(INT((A4-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C4" s="27" t="n"/>
-      <c r="D4" s="18" t="n"/>
+      <c r="C4" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D4" s="18" t="n">
+        <v>38.08</v>
+      </c>
       <c r="E4" s="16">
         <f>IF(OR(C4="",D4=""),"",TEXT(D4/C4/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F4" s="16" t="n"/>
-      <c r="G4" s="16" t="n"/>
-      <c r="H4" s="16" t="n"/>
-      <c r="I4" s="16" t="n"/>
-      <c r="J4" s="20" t="n"/>
+      <c r="F4" s="16" t="n">
+        <v>165</v>
+      </c>
+      <c r="G4" s="16" t="n">
+        <v>181</v>
+      </c>
+      <c r="H4" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J4" s="20" t="inlineStr">
+        <is>
+          <t>6:21/km; cadence 162 (+7 vs W0 155); Z3 49%+Z4 45% — too hot, cap HR ≤150 next; shin HELD, no pinpoint</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="21" t="n"/>
@@ -27263,32 +27669,52 @@
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="21" t="n"/>
+      <c r="A15" s="21" t="n">
+        <v>46182</v>
+      </c>
       <c r="B15" s="22">
         <f>IF(A15="","",IFERROR(INT((A15-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C15" s="24" t="n"/>
-      <c r="D15" s="24" t="n"/>
+      <c r="C15" s="24" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="D15" s="24" t="n">
+        <v>7.5</v>
+      </c>
       <c r="E15" s="24" t="n"/>
       <c r="F15" s="24" t="n"/>
       <c r="G15" s="24" t="n"/>
       <c r="H15" s="24" t="n"/>
-      <c r="I15" s="26" t="n"/>
+      <c r="I15" s="26" t="inlineStr">
+        <is>
+          <t>Build W1 Tue AM (run #1 back off layoff)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="15" t="n"/>
+      <c r="A16" s="15" t="n">
+        <v>46183</v>
+      </c>
       <c r="B16" s="16">
         <f>IF(A16="","",IFERROR(INT((A16-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
+      <c r="C16" s="18" t="n">
+        <v>75.90000000000001</v>
+      </c>
+      <c r="D16" s="18" t="n">
+        <v>9</v>
+      </c>
       <c r="E16" s="18" t="n"/>
       <c r="F16" s="18" t="n"/>
       <c r="G16" s="18" t="n"/>
       <c r="H16" s="18" t="n"/>
-      <c r="I16" s="20" t="n"/>
+      <c r="I16" s="20" t="inlineStr">
+        <is>
+          <t>Build W1 Wed AM (glycogen dip post hot run + 19k steps; cut paused, NOT flagged)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="21" t="n"/>

</xml_diff>

<commit_message>
log: Build W3 Mon 6/22 18k LONG #2 DONE — best long of build
18.0 km / 2:07:00 / 7:03 pace / avg HR 149 (under <=150 cap) / 95% Z2 /
cadence 164 / RPE 4. +4k/+29% jump absorbed at easiest RPE yet — aerobic
base ahead of distance ramp. Shin clean through all 18k (Thu k7 blip did
not recur), layoff fully closed. Fuel 100 g in-run ~47 g/hr, no GI. xlsx
Running Log synced (row 7). Open: cadence parked 164, 1 short of 165.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -25104,22 +25104,42 @@
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="37" t="n"/>
+      <c r="A7" s="37" t="n">
+        <v>46195</v>
+      </c>
       <c r="B7" s="22">
         <f>IF(A7="","",IFERROR(INT((A7-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C7" s="28" t="n"/>
-      <c r="D7" s="38" t="n"/>
+      <c r="C7" s="28" t="n">
+        <v>18</v>
+      </c>
+      <c r="D7" s="38" t="n">
+        <v>127</v>
+      </c>
       <c r="E7" s="22">
         <f>IF(OR(C7="",D7=""),"",TEXT(D7/C7/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F7" s="22" t="n"/>
-      <c r="G7" s="22" t="n"/>
-      <c r="H7" s="22" t="n"/>
-      <c r="I7" s="22" t="n"/>
-      <c r="J7" s="26" t="n"/>
+      <c r="F7" s="22" t="n">
+        <v>149</v>
+      </c>
+      <c r="G7" s="22" t="n">
+        <v>166</v>
+      </c>
+      <c r="H7" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="I7" s="22" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="J7" s="26" t="inlineStr">
+        <is>
+          <t>LONG #2 18k run/walk. 95% Z2, cad164, RPE4 'amazing'. 100g in-run ~47g/hr. Shin clean. Walk k5/9/13/16.</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Wk1 Wed 7/22 AM — GREEN, shin clean check #4, 6k staged
AM: sleep 8h q7 (bed 11:30pm, 2nd straight pre-midnight), BW 77.25
(3rd straight flat), RHR 44 (d-1), DOMS 3/3/3 -> 1/1/2 at 48h post
legs, no joint flags.

Shin clean for the 4th consecutive check. Bone has absorbed loaded
squats off a 62-day layoff plus 13 km of running inside 4 days with
zero signal.

Prescribed 6k easy Z2, HR <=150 cap, metronome 166 continuous (Tue's
6x2' ON/OFF drill retired). Fresh legs make today the continuous-
running test: target 0-1 walk breaks after 2 on Tue's DOMS 5k.

Backfilled training_log.xlsx Body Metrics row 23 (7/22 AM). Workbook
now current through today; Running Log row lands with the PM result.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -29124,18 +29124,28 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="37" t="n"/>
+      <c r="A23" s="37" t="n">
+        <v>46225</v>
+      </c>
       <c r="B23" s="22">
         <f>IF(A23="","",IFERROR(INT((A23-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C23" s="38" t="n"/>
-      <c r="D23" s="38" t="n"/>
+      <c r="C23" s="38" t="n">
+        <v>77.25</v>
+      </c>
+      <c r="D23" s="38" t="n">
+        <v>8</v>
+      </c>
       <c r="E23" s="38" t="n"/>
       <c r="F23" s="38" t="n"/>
       <c r="G23" s="38" t="n"/>
       <c r="H23" s="38" t="n"/>
-      <c r="I23" s="26" t="n"/>
+      <c r="I23" s="26" t="inlineStr">
+        <is>
+          <t>W1 Wed AM (RHR 44 d-1; BW flat 3rd straight day; shin clean check #4; DOMS 3/3/3 -&gt; 1/1/2 at 48h; bed 11:30pm = 2nd straight pre-midnight)</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Wk1 Wed 7/22 6k DONE — cadence PR 168, 0 walk breaks, shin clean
6.00 km / 40:27 / 6:44 km / avg HR 144 (block-low) / max 161 / 93% Z2
/ cadence 168 / RPE 6 / 0 walk breaks / outdoor / shin clean start,
middle and end.

Cleanest run of the block. Cadence 168 = new easy-run high and 3rd
straight run at 165+ (166/166/168) above the 166 metronome target —
turnover decoupling from pace, no longer a fluke. 0 walk breaks on
fresh legs closes the continuous-running watch (1 on the 8k, 2 on
Tue's DOMS 5k). Faster and -3 bpm vs Tue at 0 breaks = DOMS tax gone.
Shin clean during the run for the first time = check #5.

Protein 182 g (over floor), kcal 2612 ~ maintenance, no lift-day
blowout. Running Log row 14 appended; workbook current through today.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -26056,22 +26056,42 @@
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="35" t="n"/>
+      <c r="A14" s="35" t="n">
+        <v>46225</v>
+      </c>
       <c r="B14" s="16">
         <f>IF(A14="","",IFERROR(INT((A14-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C14" s="27" t="n"/>
-      <c r="D14" s="36" t="n"/>
+      <c r="C14" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D14" s="36" t="n">
+        <v>40.45</v>
+      </c>
       <c r="E14" s="16">
         <f>IF(OR(C14="",D14=""),"",TEXT(D14/C14/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F14" s="16" t="n"/>
-      <c r="G14" s="16" t="n"/>
-      <c r="H14" s="16" t="n"/>
-      <c r="I14" s="16" t="n"/>
-      <c r="J14" s="20" t="n"/>
+      <c r="F14" s="16" t="n">
+        <v>144</v>
+      </c>
+      <c r="G14" s="16" t="n">
+        <v>161</v>
+      </c>
+      <c r="H14" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I14" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J14" s="20" t="inlineStr">
+        <is>
+          <t>W1 Wed. 6:44/km; cadence 168 (PR, 3rd straight 165+ easy, above 166 target); 93%Z2; avg HR 144 = block-low; 0 walk breaks = first continuous run of block; shin clean start/mid/end; -3 bpm &amp; 0 breaks vs Tue at same pace = DOMS tax gone</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Wk1 Thu 7/23 Push DONE — shoulder gate clean, protein 213g 3rd straight, xlsx synced
21 sets / 218 reps / 1650.5 kg / avg RPE 7.2 off 36-day Push layoff.
Loads under seed = expected. Shoulder flag stays closed (weak, no pain).
Next Push W2 (7/30): DB Shoulder + Incline both -> 5/DB; rest HOLD.
xlsx: appended 7/23 Push to Lifting Log + BW 76.90 to Body Metrics
(DB tonnage per-DB convention verified, reconciles to 1650.5).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -14448,17 +14448,35 @@
       </c>
     </row>
     <row r="299" ht="18" customHeight="1">
-      <c r="A299" s="37" t="n"/>
+      <c r="A299" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B299" s="22">
         <f>IF(A299="","",IFERROR(INT((A299-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C299" s="22" t="n"/>
-      <c r="D299" s="23" t="n"/>
-      <c r="E299" s="22" t="n"/>
-      <c r="F299" s="22" t="n"/>
-      <c r="G299" s="38" t="n"/>
-      <c r="H299" s="22" t="n"/>
+      <c r="C299" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D299" s="23" t="inlineStr">
+        <is>
+          <t>Standing Chest Press</t>
+        </is>
+      </c>
+      <c r="E299" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F299" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G299" s="38" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="H299" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I299" s="25">
         <f>IF(OR(F299="",G299=""),"",F299*G299)</f>
         <v/>
@@ -14467,20 +14485,42 @@
         <f>IF(OR(F299="",G299=""),"",ROUND(G299*(1+F299/30),1))</f>
         <v/>
       </c>
-      <c r="K299" s="26" t="n"/>
+      <c r="K299" s="26" t="inlineStr">
+        <is>
+          <t>Push W1 maintenance, 36d layoff off 6/17; loads under seed = expected; shoulder gate clean (weak, no pain)</t>
+        </is>
+      </c>
     </row>
     <row r="300" ht="18" customHeight="1">
-      <c r="A300" s="35" t="n"/>
+      <c r="A300" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B300" s="16">
         <f>IF(A300="","",IFERROR(INT((A300-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C300" s="16" t="n"/>
-      <c r="D300" s="17" t="n"/>
-      <c r="E300" s="16" t="n"/>
-      <c r="F300" s="16" t="n"/>
-      <c r="G300" s="36" t="n"/>
-      <c r="H300" s="16" t="n"/>
+      <c r="C300" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D300" s="17" t="inlineStr">
+        <is>
+          <t>Standing Chest Press</t>
+        </is>
+      </c>
+      <c r="E300" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F300" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G300" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="H300" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I300" s="19">
         <f>IF(OR(F300="",G300=""),"",F300*G300)</f>
         <v/>
@@ -14492,17 +14532,35 @@
       <c r="K300" s="20" t="n"/>
     </row>
     <row r="301" ht="18" customHeight="1">
-      <c r="A301" s="37" t="n"/>
+      <c r="A301" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B301" s="22">
         <f>IF(A301="","",IFERROR(INT((A301-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C301" s="22" t="n"/>
-      <c r="D301" s="23" t="n"/>
-      <c r="E301" s="22" t="n"/>
-      <c r="F301" s="22" t="n"/>
-      <c r="G301" s="38" t="n"/>
-      <c r="H301" s="22" t="n"/>
+      <c r="C301" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D301" s="23" t="inlineStr">
+        <is>
+          <t>Standing Chest Press</t>
+        </is>
+      </c>
+      <c r="E301" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F301" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G301" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="H301" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I301" s="25">
         <f>IF(OR(F301="",G301=""),"",F301*G301)</f>
         <v/>
@@ -14514,17 +14572,35 @@
       <c r="K301" s="26" t="n"/>
     </row>
     <row r="302" ht="18" customHeight="1">
-      <c r="A302" s="35" t="n"/>
+      <c r="A302" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B302" s="16">
         <f>IF(A302="","",IFERROR(INT((A302-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C302" s="16" t="n"/>
-      <c r="D302" s="17" t="n"/>
-      <c r="E302" s="16" t="n"/>
-      <c r="F302" s="16" t="n"/>
-      <c r="G302" s="36" t="n"/>
-      <c r="H302" s="16" t="n"/>
+      <c r="C302" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D302" s="17" t="inlineStr">
+        <is>
+          <t>Standing Chest Press</t>
+        </is>
+      </c>
+      <c r="E302" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F302" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G302" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="H302" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I302" s="19">
         <f>IF(OR(F302="",G302=""),"",F302*G302)</f>
         <v/>
@@ -14536,17 +14612,35 @@
       <c r="K302" s="20" t="n"/>
     </row>
     <row r="303" ht="18" customHeight="1">
-      <c r="A303" s="37" t="n"/>
+      <c r="A303" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B303" s="22">
         <f>IF(A303="","",IFERROR(INT((A303-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C303" s="22" t="n"/>
-      <c r="D303" s="23" t="n"/>
-      <c r="E303" s="22" t="n"/>
-      <c r="F303" s="22" t="n"/>
-      <c r="G303" s="38" t="n"/>
-      <c r="H303" s="22" t="n"/>
+      <c r="C303" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D303" s="23" t="inlineStr">
+        <is>
+          <t>DB Shoulder Press</t>
+        </is>
+      </c>
+      <c r="E303" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F303" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G303" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="H303" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I303" s="25">
         <f>IF(OR(F303="",G303=""),"",F303*G303)</f>
         <v/>
@@ -14558,17 +14652,35 @@
       <c r="K303" s="26" t="n"/>
     </row>
     <row r="304" ht="18" customHeight="1">
-      <c r="A304" s="35" t="n"/>
+      <c r="A304" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B304" s="16">
         <f>IF(A304="","",IFERROR(INT((A304-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C304" s="16" t="n"/>
-      <c r="D304" s="17" t="n"/>
-      <c r="E304" s="16" t="n"/>
-      <c r="F304" s="16" t="n"/>
-      <c r="G304" s="36" t="n"/>
-      <c r="H304" s="16" t="n"/>
+      <c r="C304" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D304" s="17" t="inlineStr">
+        <is>
+          <t>DB Shoulder Press</t>
+        </is>
+      </c>
+      <c r="E304" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F304" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G304" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="H304" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I304" s="19">
         <f>IF(OR(F304="",G304=""),"",F304*G304)</f>
         <v/>
@@ -14580,17 +14692,35 @@
       <c r="K304" s="20" t="n"/>
     </row>
     <row r="305" ht="18" customHeight="1">
-      <c r="A305" s="37" t="n"/>
+      <c r="A305" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B305" s="22">
         <f>IF(A305="","",IFERROR(INT((A305-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C305" s="22" t="n"/>
-      <c r="D305" s="23" t="n"/>
-      <c r="E305" s="22" t="n"/>
-      <c r="F305" s="22" t="n"/>
-      <c r="G305" s="38" t="n"/>
-      <c r="H305" s="22" t="n"/>
+      <c r="C305" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D305" s="23" t="inlineStr">
+        <is>
+          <t>DB Shoulder Press</t>
+        </is>
+      </c>
+      <c r="E305" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F305" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G305" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="H305" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I305" s="25">
         <f>IF(OR(F305="",G305=""),"",F305*G305)</f>
         <v/>
@@ -14602,17 +14732,35 @@
       <c r="K305" s="26" t="n"/>
     </row>
     <row r="306" ht="18" customHeight="1">
-      <c r="A306" s="35" t="n"/>
+      <c r="A306" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B306" s="16">
         <f>IF(A306="","",IFERROR(INT((A306-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C306" s="16" t="n"/>
-      <c r="D306" s="17" t="n"/>
-      <c r="E306" s="16" t="n"/>
-      <c r="F306" s="16" t="n"/>
-      <c r="G306" s="36" t="n"/>
-      <c r="H306" s="16" t="n"/>
+      <c r="C306" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D306" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E306" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F306" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G306" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="H306" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I306" s="19">
         <f>IF(OR(F306="",G306=""),"",F306*G306)</f>
         <v/>
@@ -14624,17 +14772,35 @@
       <c r="K306" s="20" t="n"/>
     </row>
     <row r="307" ht="18" customHeight="1">
-      <c r="A307" s="37" t="n"/>
+      <c r="A307" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B307" s="22">
         <f>IF(A307="","",IFERROR(INT((A307-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C307" s="22" t="n"/>
-      <c r="D307" s="23" t="n"/>
-      <c r="E307" s="22" t="n"/>
-      <c r="F307" s="22" t="n"/>
-      <c r="G307" s="38" t="n"/>
-      <c r="H307" s="22" t="n"/>
+      <c r="C307" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D307" s="23" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E307" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F307" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G307" s="38" t="n">
+        <v>4</v>
+      </c>
+      <c r="H307" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I307" s="25">
         <f>IF(OR(F307="",G307=""),"",F307*G307)</f>
         <v/>
@@ -14646,17 +14812,35 @@
       <c r="K307" s="26" t="n"/>
     </row>
     <row r="308" ht="18" customHeight="1">
-      <c r="A308" s="35" t="n"/>
+      <c r="A308" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B308" s="16">
         <f>IF(A308="","",IFERROR(INT((A308-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C308" s="16" t="n"/>
-      <c r="D308" s="17" t="n"/>
-      <c r="E308" s="16" t="n"/>
-      <c r="F308" s="16" t="n"/>
-      <c r="G308" s="36" t="n"/>
-      <c r="H308" s="16" t="n"/>
+      <c r="C308" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D308" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E308" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F308" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G308" s="36" t="n">
+        <v>4</v>
+      </c>
+      <c r="H308" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I308" s="19">
         <f>IF(OR(F308="",G308=""),"",F308*G308)</f>
         <v/>
@@ -14668,17 +14852,35 @@
       <c r="K308" s="20" t="n"/>
     </row>
     <row r="309" ht="18" customHeight="1">
-      <c r="A309" s="37" t="n"/>
+      <c r="A309" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B309" s="22">
         <f>IF(A309="","",IFERROR(INT((A309-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C309" s="22" t="n"/>
-      <c r="D309" s="23" t="n"/>
-      <c r="E309" s="22" t="n"/>
-      <c r="F309" s="22" t="n"/>
-      <c r="G309" s="38" t="n"/>
-      <c r="H309" s="22" t="n"/>
+      <c r="C309" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D309" s="23" t="inlineStr">
+        <is>
+          <t>Pec Deck</t>
+        </is>
+      </c>
+      <c r="E309" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F309" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="G309" s="38" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H309" s="22" t="n">
+        <v>9</v>
+      </c>
       <c r="I309" s="25">
         <f>IF(OR(F309="",G309=""),"",F309*G309)</f>
         <v/>
@@ -14690,17 +14892,35 @@
       <c r="K309" s="26" t="n"/>
     </row>
     <row r="310" ht="18" customHeight="1">
-      <c r="A310" s="35" t="n"/>
+      <c r="A310" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B310" s="16">
         <f>IF(A310="","",IFERROR(INT((A310-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C310" s="16" t="n"/>
-      <c r="D310" s="17" t="n"/>
-      <c r="E310" s="16" t="n"/>
-      <c r="F310" s="16" t="n"/>
-      <c r="G310" s="36" t="n"/>
-      <c r="H310" s="16" t="n"/>
+      <c r="C310" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D310" s="17" t="inlineStr">
+        <is>
+          <t>Pec Deck</t>
+        </is>
+      </c>
+      <c r="E310" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F310" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="G310" s="36" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H310" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I310" s="19">
         <f>IF(OR(F310="",G310=""),"",F310*G310)</f>
         <v/>
@@ -14712,17 +14932,35 @@
       <c r="K310" s="20" t="n"/>
     </row>
     <row r="311" ht="18" customHeight="1">
-      <c r="A311" s="37" t="n"/>
+      <c r="A311" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B311" s="22">
         <f>IF(A311="","",IFERROR(INT((A311-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C311" s="22" t="n"/>
-      <c r="D311" s="23" t="n"/>
-      <c r="E311" s="22" t="n"/>
-      <c r="F311" s="22" t="n"/>
-      <c r="G311" s="38" t="n"/>
-      <c r="H311" s="22" t="n"/>
+      <c r="C311" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D311" s="23" t="inlineStr">
+        <is>
+          <t>Pec Deck</t>
+        </is>
+      </c>
+      <c r="E311" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F311" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="G311" s="38" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="H311" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I311" s="25">
         <f>IF(OR(F311="",G311=""),"",F311*G311)</f>
         <v/>
@@ -14734,17 +14972,35 @@
       <c r="K311" s="26" t="n"/>
     </row>
     <row r="312" ht="18" customHeight="1">
-      <c r="A312" s="35" t="n"/>
+      <c r="A312" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B312" s="16">
         <f>IF(A312="","",IFERROR(INT((A312-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C312" s="16" t="n"/>
-      <c r="D312" s="17" t="n"/>
-      <c r="E312" s="16" t="n"/>
-      <c r="F312" s="16" t="n"/>
-      <c r="G312" s="36" t="n"/>
-      <c r="H312" s="16" t="n"/>
+      <c r="C312" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D312" s="17" t="inlineStr">
+        <is>
+          <t>Triceps Pushdown</t>
+        </is>
+      </c>
+      <c r="E312" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F312" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G312" s="36" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H312" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I312" s="19">
         <f>IF(OR(F312="",G312=""),"",F312*G312)</f>
         <v/>
@@ -14756,17 +15012,35 @@
       <c r="K312" s="20" t="n"/>
     </row>
     <row r="313" ht="18" customHeight="1">
-      <c r="A313" s="37" t="n"/>
+      <c r="A313" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B313" s="22">
         <f>IF(A313="","",IFERROR(INT((A313-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C313" s="22" t="n"/>
-      <c r="D313" s="23" t="n"/>
-      <c r="E313" s="22" t="n"/>
-      <c r="F313" s="22" t="n"/>
-      <c r="G313" s="38" t="n"/>
-      <c r="H313" s="22" t="n"/>
+      <c r="C313" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D313" s="23" t="inlineStr">
+        <is>
+          <t>Triceps Pushdown</t>
+        </is>
+      </c>
+      <c r="E313" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F313" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="G313" s="38" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H313" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I313" s="25">
         <f>IF(OR(F313="",G313=""),"",F313*G313)</f>
         <v/>
@@ -14778,17 +15052,35 @@
       <c r="K313" s="26" t="n"/>
     </row>
     <row r="314" ht="18" customHeight="1">
-      <c r="A314" s="35" t="n"/>
+      <c r="A314" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B314" s="16">
         <f>IF(A314="","",IFERROR(INT((A314-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C314" s="16" t="n"/>
-      <c r="D314" s="17" t="n"/>
-      <c r="E314" s="16" t="n"/>
-      <c r="F314" s="16" t="n"/>
-      <c r="G314" s="36" t="n"/>
-      <c r="H314" s="16" t="n"/>
+      <c r="C314" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D314" s="17" t="inlineStr">
+        <is>
+          <t>Triceps Pushdown</t>
+        </is>
+      </c>
+      <c r="E314" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F314" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G314" s="36" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="H314" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I314" s="19">
         <f>IF(OR(F314="",G314=""),"",F314*G314)</f>
         <v/>
@@ -14800,17 +15092,35 @@
       <c r="K314" s="20" t="n"/>
     </row>
     <row r="315" ht="18" customHeight="1">
-      <c r="A315" s="37" t="n"/>
+      <c r="A315" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B315" s="22">
         <f>IF(A315="","",IFERROR(INT((A315-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C315" s="22" t="n"/>
-      <c r="D315" s="23" t="n"/>
-      <c r="E315" s="22" t="n"/>
-      <c r="F315" s="22" t="n"/>
-      <c r="G315" s="38" t="n"/>
-      <c r="H315" s="22" t="n"/>
+      <c r="C315" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D315" s="23" t="inlineStr">
+        <is>
+          <t>DB Lateral Raise</t>
+        </is>
+      </c>
+      <c r="E315" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F315" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G315" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H315" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I315" s="25">
         <f>IF(OR(F315="",G315=""),"",F315*G315)</f>
         <v/>
@@ -14822,17 +15132,35 @@
       <c r="K315" s="26" t="n"/>
     </row>
     <row r="316" ht="18" customHeight="1">
-      <c r="A316" s="35" t="n"/>
+      <c r="A316" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B316" s="16">
         <f>IF(A316="","",IFERROR(INT((A316-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C316" s="16" t="n"/>
-      <c r="D316" s="17" t="n"/>
-      <c r="E316" s="16" t="n"/>
-      <c r="F316" s="16" t="n"/>
-      <c r="G316" s="36" t="n"/>
-      <c r="H316" s="16" t="n"/>
+      <c r="C316" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D316" s="17" t="inlineStr">
+        <is>
+          <t>DB Lateral Raise</t>
+        </is>
+      </c>
+      <c r="E316" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F316" s="16" t="n">
+        <v>11</v>
+      </c>
+      <c r="G316" s="36" t="n">
+        <v>2</v>
+      </c>
+      <c r="H316" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I316" s="19">
         <f>IF(OR(F316="",G316=""),"",F316*G316)</f>
         <v/>
@@ -14844,17 +15172,35 @@
       <c r="K316" s="20" t="n"/>
     </row>
     <row r="317" ht="18" customHeight="1">
-      <c r="A317" s="37" t="n"/>
+      <c r="A317" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B317" s="22">
         <f>IF(A317="","",IFERROR(INT((A317-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C317" s="22" t="n"/>
-      <c r="D317" s="23" t="n"/>
-      <c r="E317" s="22" t="n"/>
-      <c r="F317" s="22" t="n"/>
-      <c r="G317" s="38" t="n"/>
-      <c r="H317" s="22" t="n"/>
+      <c r="C317" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D317" s="23" t="inlineStr">
+        <is>
+          <t>DB Lateral Raise</t>
+        </is>
+      </c>
+      <c r="E317" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F317" s="22" t="n">
+        <v>11</v>
+      </c>
+      <c r="G317" s="38" t="n">
+        <v>2</v>
+      </c>
+      <c r="H317" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I317" s="25">
         <f>IF(OR(F317="",G317=""),"",F317*G317)</f>
         <v/>
@@ -14866,17 +15212,35 @@
       <c r="K317" s="26" t="n"/>
     </row>
     <row r="318" ht="18" customHeight="1">
-      <c r="A318" s="35" t="n"/>
+      <c r="A318" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B318" s="16">
         <f>IF(A318="","",IFERROR(INT((A318-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C318" s="16" t="n"/>
-      <c r="D318" s="17" t="n"/>
-      <c r="E318" s="16" t="n"/>
-      <c r="F318" s="16" t="n"/>
-      <c r="G318" s="36" t="n"/>
-      <c r="H318" s="16" t="n"/>
+      <c r="C318" s="16" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D318" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E318" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F318" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G318" s="36" t="n">
+        <v>30</v>
+      </c>
+      <c r="H318" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I318" s="19">
         <f>IF(OR(F318="",G318=""),"",F318*G318)</f>
         <v/>
@@ -14888,17 +15252,35 @@
       <c r="K318" s="20" t="n"/>
     </row>
     <row r="319" ht="18" customHeight="1">
-      <c r="A319" s="37" t="n"/>
+      <c r="A319" s="37" t="n">
+        <v>46226</v>
+      </c>
       <c r="B319" s="22">
         <f>IF(A319="","",IFERROR(INT((A319-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C319" s="22" t="n"/>
-      <c r="D319" s="23" t="n"/>
-      <c r="E319" s="22" t="n"/>
-      <c r="F319" s="22" t="n"/>
-      <c r="G319" s="38" t="n"/>
-      <c r="H319" s="22" t="n"/>
+      <c r="C319" s="22" t="inlineStr">
+        <is>
+          <t>Push</t>
+        </is>
+      </c>
+      <c r="D319" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E319" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F319" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G319" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="H319" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I319" s="25">
         <f>IF(OR(F319="",G319=""),"",F319*G319)</f>
         <v/>
@@ -29168,18 +29550,28 @@
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="35" t="n"/>
+      <c r="A24" s="35" t="n">
+        <v>46226</v>
+      </c>
       <c r="B24" s="16">
         <f>IF(A24="","",IFERROR(INT((A24-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C24" s="36" t="n"/>
-      <c r="D24" s="36" t="n"/>
+      <c r="C24" s="36" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="D24" s="36" t="n">
+        <v>11</v>
+      </c>
       <c r="E24" s="36" t="n"/>
       <c r="F24" s="36" t="n"/>
       <c r="G24" s="36" t="n"/>
       <c r="H24" s="36" t="n"/>
-      <c r="I24" s="20" t="n"/>
+      <c r="I24" s="20" t="inlineStr">
+        <is>
+          <t>Peak readiness; RHR 45 (d0); shin clean 5th; 78.2 spike settling to ~77 on maintenance</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Wk1 Fri 7/24 REST — AM green, shin clean #6, Push DOMS on schedule, xlsx synced
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -29574,18 +29574,28 @@
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="37" t="n"/>
+      <c r="A25" s="37" t="n">
+        <v>46227</v>
+      </c>
       <c r="B25" s="22">
         <f>IF(A25="","",IFERROR(INT((A25-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C25" s="38" t="n"/>
-      <c r="D25" s="38" t="n"/>
+      <c r="C25" s="38" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="D25" s="38" t="n">
+        <v>9</v>
+      </c>
       <c r="E25" s="38" t="n"/>
       <c r="F25" s="38" t="n"/>
       <c r="G25" s="38" t="n"/>
       <c r="H25" s="38" t="n"/>
-      <c r="I25" s="26" t="n"/>
+      <c r="I25" s="26" t="inlineStr">
+        <is>
+          <t>W1 Fri REST AM (RHR 47 d+2 post-Push bump; shin clean check #6; Push DOMS 3 chest/shldr/tri on schedule; legs residual 1; bed 1:30am watch item; BW settled ~77)</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Wk1 Sat 7/25 AM — green, shin clean #7, RHR bump cleared, 5k staged, xlsx synced
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -29598,18 +29598,28 @@
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="35" t="n"/>
+      <c r="A26" s="35" t="n">
+        <v>46228</v>
+      </c>
       <c r="B26" s="16">
         <f>IF(A26="","",IFERROR(INT((A26-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C26" s="36" t="n"/>
-      <c r="D26" s="36" t="n"/>
+      <c r="C26" s="36" t="n">
+        <v>77.84999999999999</v>
+      </c>
+      <c r="D26" s="36" t="n">
+        <v>7.53</v>
+      </c>
       <c r="E26" s="36" t="n"/>
       <c r="F26" s="36" t="n"/>
       <c r="G26" s="36" t="n"/>
       <c r="H26" s="36" t="n"/>
-      <c r="I26" s="20" t="n"/>
+      <c r="I26" s="20" t="inlineStr">
+        <is>
+          <t>W1 Sat AM run day (RHR 43 d-1 post-Push bump cleared; shin clean check #7; Push DOMS 3-&gt;1 at 48h, legs 0; BW +0.65 single-day spike ignore, 7d ~77.4; bed 12:39am 2nd straight post-midnight, sleep 7:32 q6.5 week-low)</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Wk1 Sat 7/25 PM close — 5k done, cadence 167 4th straight, shin clean #8, felt-bad watch item
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -26476,22 +26476,42 @@
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="37" t="n"/>
+      <c r="A15" s="37" t="n">
+        <v>46228</v>
+      </c>
       <c r="B15" s="22">
         <f>IF(A15="","",IFERROR(INT((A15-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C15" s="28" t="n"/>
-      <c r="D15" s="38" t="n"/>
+      <c r="C15" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D15" s="38" t="n">
+        <v>34.27</v>
+      </c>
       <c r="E15" s="22">
         <f>IF(OR(C15="",D15=""),"",TEXT(D15/C15/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F15" s="22" t="n"/>
-      <c r="G15" s="22" t="n"/>
-      <c r="H15" s="22" t="n"/>
-      <c r="I15" s="22" t="n"/>
-      <c r="J15" s="26" t="n"/>
+      <c r="F15" s="22" t="n">
+        <v>148</v>
+      </c>
+      <c r="G15" s="22" t="n">
+        <v>158</v>
+      </c>
+      <c r="H15" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="I15" s="22" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J15" s="26" t="inlineStr">
+        <is>
+          <t>W1 Sat. 6:51/km; cadence 167 (4th straight 165+ easy); 96%Z2; 0 walk breaks (2nd continuous); shin clean during+after = check #8; RPE 7 + general discomfort on week-low sleep 7:32 (2nd straight post-midnight bed) — sleep tax read, watch not flag</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="35" t="n"/>

</xml_diff>

<commit_message>
xlsx: extend Weekly Summary to week 24 (race week Oct 11)
Tab was built for Block 1 weeks 1-11 only; current week (13) had no row.
Week column is anchored to 2026-04-27, so Block 2 W1 = workbook week 13.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -32695,7 +32695,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K12"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -33260,6 +33260,591 @@
       </c>
       <c r="K12" s="36">
         <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A12),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A13-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A13*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C13" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A13)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D13" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A13)</f>
+        <v/>
+      </c>
+      <c r="E13" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A13)</f>
+        <v/>
+      </c>
+      <c r="F13" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A13),"")</f>
+        <v/>
+      </c>
+      <c r="G13" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A13)</f>
+        <v/>
+      </c>
+      <c r="H13" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A13)</f>
+        <v/>
+      </c>
+      <c r="J13" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A13),"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A13),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="16" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A14-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A14*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C14" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A14)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D14" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A14)</f>
+        <v/>
+      </c>
+      <c r="E14" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A14)</f>
+        <v/>
+      </c>
+      <c r="F14" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A14),"")</f>
+        <v/>
+      </c>
+      <c r="G14" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A14)</f>
+        <v/>
+      </c>
+      <c r="H14" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A14)</f>
+        <v/>
+      </c>
+      <c r="J14" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A14),"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A14),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A15-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A15*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C15" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A15)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D15" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A15)</f>
+        <v/>
+      </c>
+      <c r="E15" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A15)</f>
+        <v/>
+      </c>
+      <c r="F15" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A15),"")</f>
+        <v/>
+      </c>
+      <c r="G15" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A15)</f>
+        <v/>
+      </c>
+      <c r="H15" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A15)</f>
+        <v/>
+      </c>
+      <c r="J15" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A15),"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A15),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A16-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A16*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C16" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A16)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D16" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A16)</f>
+        <v/>
+      </c>
+      <c r="E16" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A16)</f>
+        <v/>
+      </c>
+      <c r="F16" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A16),"")</f>
+        <v/>
+      </c>
+      <c r="G16" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A16)</f>
+        <v/>
+      </c>
+      <c r="H16" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A16)</f>
+        <v/>
+      </c>
+      <c r="J16" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A16),"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A16),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="16" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A17-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A17*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C17" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A17)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D17" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A17)</f>
+        <v/>
+      </c>
+      <c r="E17" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A17),"")</f>
+        <v/>
+      </c>
+      <c r="G17" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A17)</f>
+        <v/>
+      </c>
+      <c r="H17" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A17)</f>
+        <v/>
+      </c>
+      <c r="J17" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A17),"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A17),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A18-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A18*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C18" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A18)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D18" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A18)</f>
+        <v/>
+      </c>
+      <c r="E18" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A18),"")</f>
+        <v/>
+      </c>
+      <c r="G18" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A18)</f>
+        <v/>
+      </c>
+      <c r="H18" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A18)</f>
+        <v/>
+      </c>
+      <c r="J18" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A18),"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A18),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A19-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A19*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C19" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A19)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D19" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A19)</f>
+        <v/>
+      </c>
+      <c r="E19" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A19),"")</f>
+        <v/>
+      </c>
+      <c r="G19" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A19)</f>
+        <v/>
+      </c>
+      <c r="H19" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A19)</f>
+        <v/>
+      </c>
+      <c r="J19" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A19),"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A19),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A20-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A20*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C20" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A20)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D20" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A20)</f>
+        <v/>
+      </c>
+      <c r="E20" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A20),"")</f>
+        <v/>
+      </c>
+      <c r="G20" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A20)</f>
+        <v/>
+      </c>
+      <c r="H20" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A20)</f>
+        <v/>
+      </c>
+      <c r="J20" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A20),"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A20),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A21-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A21*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C21" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A21)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D21" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A21)</f>
+        <v/>
+      </c>
+      <c r="E21" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A21),"")</f>
+        <v/>
+      </c>
+      <c r="G21" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A21)</f>
+        <v/>
+      </c>
+      <c r="H21" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A21)</f>
+        <v/>
+      </c>
+      <c r="I21" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A21),"")</f>
+        <v/>
+      </c>
+      <c r="K21" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A21),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="16" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A22-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A22*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C22" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A22)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D22" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A22)</f>
+        <v/>
+      </c>
+      <c r="E22" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A22)</f>
+        <v/>
+      </c>
+      <c r="F22" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A22),"")</f>
+        <v/>
+      </c>
+      <c r="G22" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A22)</f>
+        <v/>
+      </c>
+      <c r="H22" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A22)</f>
+        <v/>
+      </c>
+      <c r="J22" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A22),"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A22),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="16" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A23-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A23*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C23" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A23)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D23" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A23)</f>
+        <v/>
+      </c>
+      <c r="E23" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A23)</f>
+        <v/>
+      </c>
+      <c r="F23" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A23),"")</f>
+        <v/>
+      </c>
+      <c r="G23" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A23)</f>
+        <v/>
+      </c>
+      <c r="H23" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A23)</f>
+        <v/>
+      </c>
+      <c r="J23" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A23),"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A23),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="16" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A24-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A24*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C24" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A24)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D24" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A24)</f>
+        <v/>
+      </c>
+      <c r="E24" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A24)</f>
+        <v/>
+      </c>
+      <c r="F24" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A24),"")</f>
+        <v/>
+      </c>
+      <c r="G24" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A24)</f>
+        <v/>
+      </c>
+      <c r="H24" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A24)</f>
+        <v/>
+      </c>
+      <c r="J24" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A24),"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A24),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="16" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A25-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A25*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C25" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A25)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D25" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A25)</f>
+        <v/>
+      </c>
+      <c r="E25" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A25)</f>
+        <v/>
+      </c>
+      <c r="F25" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A25),"")</f>
+        <v/>
+      </c>
+      <c r="G25" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A25)</f>
+        <v/>
+      </c>
+      <c r="H25" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A25)</f>
+        <v/>
+      </c>
+      <c r="I25" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A25)</f>
+        <v/>
+      </c>
+      <c r="J25" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A25),"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A25),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
log: close Mon 9/7 run, sync workbook, add Bike km column
5k easy shakeout: 7:18/km @ HR 147, 97% Z2, RPE 3 (lowest in log),
cadence 167 (4th straight cued hit), 0 walk breaks, shin check #17.
Ran ~20s/km faster than the 7:35-7:50 prescription; HR gate held but
the pattern is noted for Sunday's 12k.

Workbook backfilled to 9/7 (Running Log, Body Metrics). Running Log
gains a Bike km column now that the commute is tracked as load.

BW 75.85 flat for a third day closes the fuel-drift flag opened 9/5.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -26906,7 +26906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J151"/>
+  <dimension ref="A1:K151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26972,6 +26972,11 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="K1" s="14" t="inlineStr">
+        <is>
+          <t>Bike km</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="35" t="n">
@@ -27620,22 +27625,45 @@
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="A19" s="37" t="n"/>
+      <c r="A19" s="37" t="n">
+        <v>46272</v>
+      </c>
       <c r="B19" s="22">
         <f>IF(A19="","",IFERROR(INT((A19-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C19" s="28" t="n"/>
-      <c r="D19" s="38" t="n"/>
+      <c r="C19" s="28" t="n">
+        <v>5</v>
+      </c>
+      <c r="D19" s="38" t="n">
+        <v>36.5</v>
+      </c>
       <c r="E19" s="22">
         <f>IF(OR(C19="",D19=""),"",TEXT(D19/C19/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F19" s="22" t="n"/>
-      <c r="G19" s="22" t="n"/>
-      <c r="H19" s="22" t="n"/>
-      <c r="I19" s="22" t="n"/>
-      <c r="J19" s="26" t="n"/>
+      <c r="F19" s="22" t="n">
+        <v>147</v>
+      </c>
+      <c r="G19" s="22" t="n">
+        <v>162</v>
+      </c>
+      <c r="H19" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="I19" s="22" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J19" s="26" t="inlineStr">
+        <is>
+          <t>Blk2 Wk B Mon - 5k easy shakeout, 24h after Sun's 10k long. Monday was a REST day until two same-day schedule swaps (cali #3 Mon-&gt;Wed, cali #4 Fri-&gt;Sat) would have left 6 consecutive loaded days on one rest day; rebalanced by spending Monday's rest on the week's shortest run and making Thursday the rest day. 7:18/km @ HR 147, 97%Z2, RPE 3 = LOWEST RUN RPE IN THE LOG. Prescription was 7:35-7:50/km -&gt; ran ~20 s/km HOT. Allowed to stand because HR 147 held under the 150 ceiling, but it is the block's recurring pattern: feeling good becomes FASTER, not EASIER. On Sunday's 12k that costs the back half - open at 7:50 and mean it. EFFICIENCY: 7:18 @ 147 vs the clean rested comparable 7:08 @ 145 on 9/4 = 10 s/km slower at +2 bpm on a day-after-long shakeout = chassis recovering FASTER than the ramp assumed. CADENCE 167 = 4th straight cued run on target (166/166/167/167); metronome stays mandatory. 0 walk breaks, 3rd run running. SHIN CLEAN check #17. Fuel 2566 vs corrected uni-day ~2650-2700 = ~100 under, noise. Protein 169 (band 155-165). Creatine Y. Steps 9100. BIKE 24 km - uni-day commute, DISCLOSED TODAY as Tier 1 load (12 km each way, Mon-Thu = 96 km/wk, ~4-5 h, MORE clock time than the running). Zero bone cost (non-impact, does not spend the tibia budget) and it partly explains why the audits keep finding the engine ahead of the chassis. Makes the ~2400 kcal maintenance figure STALE: uni days 2650-2700, non-uni 2400, Sun long 2700. Sat+Sun are bike-free - that is what protects the long run. Wk B compliance: run 1 of 4.</t>
+        </is>
+      </c>
+      <c r="K19" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="35" t="n"/>
@@ -30888,18 +30916,28 @@
       </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="35" t="n"/>
+      <c r="A36" s="35" t="n">
+        <v>46272</v>
+      </c>
       <c r="B36" s="16">
         <f>IF(A36="","",IFERROR(INT((A36-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C36" s="36" t="n"/>
-      <c r="D36" s="36" t="n"/>
+      <c r="C36" s="36" t="n">
+        <v>75.84999999999999</v>
+      </c>
+      <c r="D36" s="36" t="n">
+        <v>9</v>
+      </c>
       <c r="E36" s="36" t="n"/>
       <c r="F36" s="36" t="n"/>
       <c r="G36" s="36" t="n"/>
       <c r="H36" s="36" t="n"/>
-      <c r="I36" s="20" t="n"/>
+      <c r="I36" s="20" t="inlineStr">
+        <is>
+          <t>Wk B Mon - 5k easy shakeout (was a rest day; converted after two cali swaps). AM FULL GREEN: sleep 9:00 q10, RHR 46 delta -2, motivation 10, energy 10, stress 2, joints all clear. SHIN PERFECT check #16 (pre) and #17 (post-run). DOMS legs ALL 1 (quad/ham/glute/calf) at 2 days post-cali = RPE 6 leg cap validated a 3rd time. Upper: shoulder 3, chest 2, back 1, arm 1 = 9/5 pressing residue at 48h; this is WHY moving cali Mon-&gt;Wed is a net positive (shoulders get 4 days instead of 2). BW 75.85 = THIRD CONSECUTIVE FLAT READING (9/5, 9/6, 9/7) after +937 and +93 kcal days. TREND CALL MADE: the +0.85 over the 8/31 close of 75.0 is glycogen + water, NOT fat - fuel-drift flag CLOSED. Second explanation landed same day: the 96 km/wk bike commute was unlogged, so ~2400 'maintenance' was never maintenance. CORRECTED: uni days (Mon-Thu) 2650-2700, non-uni 2400, Sun long 2700, protein 155-165. Fuel today 2566 = ~100 under, noise. Protein 169. Creatine Y. Alcohol 0. Steps 9100. Bike 24 km.</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="37" t="n"/>

</xml_diff>

<commit_message>
log: close Tue 9/8 run — pace obeyed, cadence misses at slow pace
6 km at 8:01/km, HR 140 and RPE 1, both block lows, with the pace
instruction followed for the first time this block after 9/7 ran
20 s/km hot. Shin clean, check 19.

Cadence came in at 163 and breaks a 166/166/167/167 cued streak.
The cue has only ever been tested at 7:08-7:18/km; at 8:01 the
stride overrode it, which re-opens the pace-linkage item that 9/6
recorded as closed. Sunday's 12 km opens at exactly that pace, so
the metronome stays at 166 and the beat gets matched by shortening
stride rather than by running faster.

Bike ridden at 24 km against a 12 km mitigation target, so
Wednesday's AM read becomes the unmitigated answer to the leg-DOMS
question and the trigger stays armed. Protein 178 g is a third
straight day over the 155-165 band; pull to 160.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -27666,22 +27666,45 @@
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="A20" s="35" t="n"/>
+      <c r="A20" s="35" t="n">
+        <v>46273</v>
+      </c>
       <c r="B20" s="16">
         <f>IF(A20="","",IFERROR(INT((A20-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C20" s="27" t="n"/>
-      <c r="D20" s="36" t="n"/>
+      <c r="C20" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D20" s="36" t="n">
+        <v>48.22</v>
+      </c>
       <c r="E20" s="16">
         <f>IF(OR(C20="",D20=""),"",TEXT(D20/C20/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F20" s="16" t="n"/>
-      <c r="G20" s="16" t="n"/>
-      <c r="H20" s="16" t="n"/>
-      <c r="I20" s="16" t="n"/>
-      <c r="J20" s="20" t="n"/>
+      <c r="F20" s="16" t="n">
+        <v>140</v>
+      </c>
+      <c r="G20" s="16" t="n">
+        <v>153</v>
+      </c>
+      <c r="H20" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="I20" s="16" t="inlineStr">
+        <is>
+          <t>Easy Z2</t>
+        </is>
+      </c>
+      <c r="J20" s="20" t="inlineStr">
+        <is>
+          <t>97% Z2, cadence 163 (first cued miss), 0 walk breaks, light rain, shin clean #19. Pace obeyed prescription 8:01 vs 7:45-8:00.</t>
+        </is>
+      </c>
+      <c r="K20" t="n">
+        <v>24</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="37" t="n"/>
@@ -30940,18 +30963,28 @@
       </c>
     </row>
     <row r="37" ht="18" customHeight="1">
-      <c r="A37" s="37" t="n"/>
+      <c r="A37" s="37" t="n">
+        <v>46273</v>
+      </c>
       <c r="B37" s="22">
         <f>IF(A37="","",IFERROR(INT((A37-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C37" s="38" t="n"/>
-      <c r="D37" s="38" t="n"/>
+      <c r="C37" s="38" t="n">
+        <v>75.2</v>
+      </c>
+      <c r="D37" s="38" t="n">
+        <v>7</v>
+      </c>
       <c r="E37" s="38" t="n"/>
       <c r="F37" s="38" t="n"/>
       <c r="G37" s="38" t="n"/>
       <c r="H37" s="38" t="n"/>
-      <c r="I37" s="26" t="n"/>
+      <c r="I37" s="26" t="inlineStr">
+        <is>
+          <t>RHR 46 (-1). Mot 10/En 8/Str 2. DOMS quad2 ham2 glute2 calf2 - first 4-way, bike flag tripped. Shin clean #18.</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="35" t="n"/>

</xml_diff>

<commit_message>
log: sync 9/11 AM, backfill 9/7-9/10 session files, sync workbook
Workbook: Body Metrics gets 9/11 (BW 76.20, sleep 10h, full AM read).
9/9 and 9/10 notes rewritten to record the data as unrecoverable rather
than outstanding.

Backfilled logs/sessions/ files that were never written: 9/7 run, 9/8 run,
9/10 rest (data-loss record), plus the 9/11 run prescription.

Memory updated: Fri 9/11 AM read, the data-loss rule, and the BW 76.20
water call.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -31490,7 +31490,7 @@
       <c r="H38" s="36" t="n"/>
       <c r="I38" s="20" t="inlineStr">
         <is>
-          <t>Wk B Wed - Cali Full Body #3 (14:10-15:00, 50 min, 28/28 sets, 293 reps, avg set RPE 7.0). AM CLEANEST OF THE BLOCK: sleep 7:30 q8 (bed 22:30 wake 06:35), RHR 46 delta -1, motivation 10, energy 10, stress 3, joints clear, ZERO DOMS above 1 anywhere (chest/back/shldr/arm all 0; quad/ham/glute/calf all 1). SHIN CLEAN check #20 (AM) and #21 (post-session). BIKE TRIGGER DID NOT FIRE, AND IT WAS ANSWERED UNMITIGATED: Tuesday's first-of-block 4-way leg DOMS 2 cleared to 1 across all four groups in 24 h while the full 24 km commute was ridden AND a 6 k run was run. The 9/8 read was right - local fatigue, not accumulation. Bike stays 24 km on uni days; Wed cali ran in full, BSS + SL-RDL NOT cut. Trigger disarmed for Wk B, re-arms on any future two consecutive mornings at &gt;=2. Shoulders 3 -&gt; 1 -&gt; 0 in three days off cali = the 9/7 Mon-&gt;Wed swap fully vindicated, pressing landed on recovered delts. BW 75.20 second flat day off the -0.65 drop = noise, not a plateau; no kcal change (uni day 2650-2700). Protein: pull to ~160 after three straight high days (227 -&gt; 169 -&gt; 178). PM data outstanding: kcal, protein, Bike km (uni day, expect 24), steps.</t>
+          <t>Wk B Wed - Cali Full Body #3 (14:10-15:00, 50 min, 28/28 sets, 293 reps, avg set RPE 7.0). AM CLEANEST OF THE BLOCK: sleep 7:30 q8 (bed 22:30 wake 06:35), RHR 46 delta -1, motivation 10, energy 10, stress 3, joints clear, ZERO DOMS above 1 anywhere (chest/back/shldr/arm all 0; quad/ham/glute/calf all 1). SHIN CLEAN check #20 (AM) and #21 (post-session). BIKE TRIGGER DID NOT FIRE, AND IT WAS ANSWERED UNMITIGATED: Tuesday's first-of-block 4-way leg DOMS 2 cleared to 1 across all four groups in 24 h while the full 24 km commute was ridden AND a 6 k run was run. The 9/8 read was right - local fatigue, not accumulation. Bike stays 24 km on uni days; Wed cali ran in full, BSS + SL-RDL NOT cut. Trigger disarmed for Wk B, re-arms on any future two consecutive mornings at &gt;=2. Shoulders 3 -&gt; 1 -&gt; 0 in three days off cali = the 9/7 Mon-&gt;Wed swap fully vindicated, pressing landed on recovered delts. BW 75.20 second flat day off the -0.65 drop = noise, not a plateau; no kcal change (uni day 2650-2700). Protein: pull to ~160 after three straight high days (227 -&gt; 169 -&gt; 178). PM DATA NOT RECOVERABLE (confirmed 9/11): kcal, protein, Bike km and steps for 9/9 do not exist. Uni day so the bike was 24 km by routine, but it is NOT logged as measured. Not chased, not reconstructed - an invented number is worse than a gap. Wk B fuel/bike compliance is therefore a 5-day week, not 7.</t>
         </is>
       </c>
     </row>
@@ -31510,23 +31510,33 @@
       <c r="H39" s="38" t="n"/>
       <c r="I39" s="26" t="inlineStr">
         <is>
-          <t>Wk B Thu - REST (full), as prescribed. This is the rest day created by the 9/7 double-swap (cali #3 Mon-&gt;Wed, cali #4 Fri-&gt;Sat, Monday's rest spent on the week's shortest run). ZERO runs missed - the revised week never had a Thursday run. Uni day, bike 24 km expected. AM and PM blocks NOT captured (blanks genuine): sleep, BW AM, RHR, DOMS, shin check #22, kcal, protein, Bike km, steps all outstanding. Remaining Wk B: Fri 9/11 run easy 6 k PM, Sat 9/12 Cali #4, Sun 9/13 LONG 12 k AM = 18 km to close 29 km and 4 runs of 4.</t>
+          <t>Wk B Thu - REST (full), as prescribed. The rest day created by the 9/7 double-swap (cali #3 Mon-&gt;Wed, cali #4 Fri-&gt;Sat, Monday's rest spent on the week's shortest run). ZERO runs missed - the revised week never had a Thursday run. Uni day, bike 24 km by routine but unmeasured. AM + PM BLOCKS NOT RECOVERABLE (confirmed by user 9/11): no sleep, BW, RHR, DOMS, shin check, kcal, protein, bike km or steps exist for this day. A full dark day of data on a rest day. NOT reconstructed. Two consequences: (1) the BW series has a hole between 75.20 (9/9) and 76.20 (9/11), so the +1.00 kg jump is measured across 48 h, not 24 - which makes the water/glycogen read MORE likely, not less; (2) the shin-check count loses a day - Thu took none, so Fri 9/11 AM is check #22, not #23. Numbering corrected downstream; the clean streak itself is unbroken, the count is simply one lower than previously stated. Countermeasure is the one this block already named: two-touch logging ON the day.</t>
         </is>
       </c>
     </row>
     <row r="40" ht="18" customHeight="1">
-      <c r="A40" s="35" t="n"/>
+      <c r="A40" s="35" t="n">
+        <v>46276</v>
+      </c>
       <c r="B40" s="16">
         <f>IF(A40="","",IFERROR(INT((A40-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C40" s="36" t="n"/>
-      <c r="D40" s="36" t="n"/>
+      <c r="C40" s="36" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="D40" s="36" t="n">
+        <v>10</v>
+      </c>
       <c r="E40" s="36" t="n"/>
       <c r="F40" s="36" t="n"/>
       <c r="G40" s="36" t="n"/>
       <c r="H40" s="36" t="n"/>
-      <c r="I40" s="20" t="n"/>
+      <c r="I40" s="20" t="inlineStr">
+        <is>
+          <t>Wk B Fri - run easy 6 k PM (cali #4 sits Sat after the 9/7 swap). AM: sleep 10:00 q10 = longest sleep in the log, RHR 45 (delta +1 vs 7 d, baseline 44, trending down off 46), motivation 10, energy 10, stress 3, tendons clean. SHIN CLEAN check #22 (renumbered: Thu 9/10 took no check). DOMS chest 2 / back 2 / shldr 2 / arm 1 = 48 h off cali #3, the first session carrying the B2 second push-up block, so a mild press+pull bump is the seed working. Zero impact on a run; Sat cali #4 lands at 72 h, clear, no cuts owed. LEGS 1/1/1/1 for the SECOND consecutive morning -&gt; bike trigger stays DISARMED (needs two consecutive mornings at &gt;=2). Bike holds 24 km on uni days; Friday is bike-free regardless. BW 76.20 = +1.00 kg off two flat days at 75.20, and measured across 48 h because 9/10 was not logged. NOT FAT: +1 kg of fat needs +7700 kcal against days that ran ~2400-2700. Water/glycogen/sodium. The block already ran this exact experiment - 75.85 held flat three days under a +937 kcal day, then dropped 0.65 overnight. Same noise band, same answer. NO KCAL CHANGE. 7-day picture 75.85/75.85/75.85/75.20/75.20/(hole)/76.20 = avg 75.69, still inside the 8/31 close +1. MON 9/14 AM MAKES THE TREND CALL, not today. Non-uni day -&gt; ~2400 kcal, protein pull to ~160 (227 -&gt; 169 -&gt; 178 run must stop). Cleanest readiness of the week; nothing to autoregulate, run goes full 6 k. Rules: open ~7:50/km, avg HR 140-145, HARD ceiling 150, metronome 166 matched by SHORTENING STRIDE. This run is Sunday's rehearsal - Tue's 8:01/km produced cadence 163 and the 12 k opens at exactly this pace.</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="37" t="n"/>

</xml_diff>

<commit_message>
log: close Wk B at 3/4 runs after illness, sync workbook and memory
Fri 9/11 session file filled with result. Added 9/12 (cali #4) and
9/13 (long 12k) illness skip files. Workbook: Running Log +9/11,
Body Metrics +9/12,9/13 — both tabs now current.

CLAUDE.md: added the neck-check illness rule (fever = hard stop,
illness is not drift, re-entry is one easy short run at HR<=140,
checkpoints are moveable and the bone is not) and scoped the cadence
item — a cadence hit only counts if the pace instruction was obeyed,
which 9/11 was not.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -28191,22 +28191,45 @@
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="A21" s="37" t="n"/>
-      <c r="B21" s="22">
+      <c r="A21" s="35" t="n">
+        <v>46276</v>
+      </c>
+      <c r="B21" s="16">
         <f>IF(A21="","",IFERROR(INT((A21-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C21" s="28" t="n"/>
-      <c r="D21" s="38" t="n"/>
-      <c r="E21" s="22">
+      <c r="C21" s="27" t="n">
+        <v>6</v>
+      </c>
+      <c r="D21" s="36" t="n">
+        <v>44.3</v>
+      </c>
+      <c r="E21" s="16">
         <f>IF(OR(C21="",D21=""),"",TEXT(D21/C21/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F21" s="22" t="n"/>
-      <c r="G21" s="22" t="n"/>
-      <c r="H21" s="22" t="n"/>
-      <c r="I21" s="22" t="n"/>
-      <c r="J21" s="26" t="n"/>
+      <c r="F21" s="16" t="n">
+        <v>146</v>
+      </c>
+      <c r="G21" s="16" t="n">
+        <v>158</v>
+      </c>
+      <c r="H21" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="I21" s="16" t="inlineStr">
+        <is>
+          <t>Easy Z2</t>
+        </is>
+      </c>
+      <c r="J21" s="20" t="inlineStr">
+        <is>
+          <t>Blk2 Wk B Fri - run easy 6 k, LAST SESSION OF WK B. 7:22/km @ HR 146, 98% Z2 = HIGHEST Z2 SHARE OF THE BLOCK, max 158, RPE 2, 0 walk breaks (streak 4), chilly cloudy, 'It was a chill day.' SHIN CLEAN check #23. Fri is bike-free. ENGINE READ EXCELLENT: clean comparable is 9/4 (7:08/km @ HR 145, fully rested) -&gt; 7:22 @ 146 shows NO drift; third consecutive run at RPE &lt;=3. CADENCE 166 HIT BUT BOUGHT WITH SPEED - THIS RUN DOES NOT ANSWER THE OPEN QUESTION. Prescription was open ~7:50/km; actual 7:22 = 28 s/km HOT, landing back in the 7:08-7:18 band where the cue has always worked. The session's own rule called it in advance: pace under 7:40 means cadence was bought with speed, not turnover. The metronome still has ZERO successful reps below ~7:20/km; the only honest test remains 9/8 (8:01/km -&gt; 163). THIRD REPEAT OF THE PATTERN: 9/7 ran 7:18 vs 7:35-7:50, 9/8 obeyed at 8:01, 9/11 ran 7:22 vs 7:50. The correction lands for exactly one run, then decays. Costs nothing on a 6 k; costs the back half on a 12-22 k, the only place opening pace matters. Carried forward and now overdue. PM NOT SUPPLIED - kcal, protein, creatine, steps, Friday-night symptoms written off, not reconstructed. Illness surfaced Saturday so this run was likely made on an incubating bug; HR 146 at RPE 2 shows no prodrome, so noted not weighted. WK B CLOSES HERE: runs 3 of 4, 17 of 29 km, cali 1 of 2 - Sat cali #4 and Sun long 12 k both LOST TO ILLNESS.</t>
+        </is>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="35" t="n"/>
@@ -31539,7 +31562,9 @@
       </c>
     </row>
     <row r="41" ht="18" customHeight="1">
-      <c r="A41" s="37" t="n"/>
+      <c r="A41" s="37" t="n">
+        <v>46277</v>
+      </c>
       <c r="B41" s="22">
         <f>IF(A41="","",IFERROR(INT((A41-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
@@ -31550,21 +31575,31 @@
       <c r="F41" s="38" t="n"/>
       <c r="G41" s="38" t="n"/>
       <c r="H41" s="38" t="n"/>
-      <c r="I41" s="26" t="n"/>
+      <c r="I41" s="26" t="inlineStr">
+        <is>
+          <t>Wk B Sat - CALI #4 MISSED, ILLNESS. User sick Sat + Sun, reported 9/13. No AM block, no PM block, no session, no shin check. NOT reconstructed - missing data is written off, never back-filled from memory; an invented number is worse than an honest gap. WHAT WAS LOST: the second cali day of Wk B, which would have carried the first bumps off the 9/9 gate clears - tibialis to SLOW-ECCENTRIC 3x20 and side plank to 2x45 s/side, with A1 push-up holding all four sets at setting 3. Those advancements are UNRUN, not cancelled: they carry forward intact to the next cali session, gates stay cleared, nothing regresses on one missed session. Cali frequency for Wk B closes at 1 of 2. NO MAKE-UP SESSION - stacking cali into a re-entry week would put loaded legs in front of the first post-illness run, which is backwards: the run is the session that matters and the bone is the gate.</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="18" customHeight="1">
-      <c r="A42" s="35" t="n"/>
-      <c r="B42" s="16">
+      <c r="A42" s="37" t="n">
+        <v>46278</v>
+      </c>
+      <c r="B42" s="22">
         <f>IF(A42="","",IFERROR(INT((A42-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C42" s="36" t="n"/>
-      <c r="D42" s="36" t="n"/>
-      <c r="E42" s="36" t="n"/>
-      <c r="F42" s="36" t="n"/>
-      <c r="G42" s="36" t="n"/>
-      <c r="H42" s="36" t="n"/>
-      <c r="I42" s="20" t="n"/>
+      <c r="C42" s="38" t="n"/>
+      <c r="D42" s="38" t="n"/>
+      <c r="E42" s="38" t="n"/>
+      <c r="F42" s="38" t="n"/>
+      <c r="G42" s="38" t="n"/>
+      <c r="H42" s="38" t="n"/>
+      <c r="I42" s="26" t="inlineStr">
+        <is>
+          <t>Wk B Sun - LONG 12 k MISSED, ILLNESS, second consecutive day. User reported 16:13: still symptomatic but IMPROVING vs Saturday. No AM block, no PM block, no BW, no shin check. NOT reconstructed. THE LONG IS GONE AND IS NOT CHASED - not moved to Monday, not compressed into next week. Reported at 16:13 and the long is an AM session by design; two sick days sat in front of it; a 12 k off illness on bone only 5 weeks past a 34-day layoff spends the tibia budget for nothing. 'Better than yesterday' is not 'clear'. SICK RULE - NECK CHECK: above neck only (nose/throat/sneeze) = easy run permitted at reduced distance, HR ceiling 140. Below neck (fever/chest/body aches/GI) = ZERO training until 24 h FULLY symptom-free, then one easy short run before anything loaded. Fever is a hard stop; myocarditis risk is not traded for a session. WK B FINAL: runs 3 of 4, 17 of 29 km, cali 1 of 2, 2 rest as planned + 2 lost. First missed sessions of Block 2. THIS IS ILLNESS, NOT DRIFT - categorically different from the Jul 29 - Aug 30 dark month and not treated the same way. Two days do not move the block; panic-compressing them would. BW TREND CALL VOID: 76.20 (9/11) is confounded by the 9/10 data hole plus two illness days (appetite, hydration, glycogen swing). Mon 9/14 AM reads nothing useful. Next real BW call ~9/17. No kcal change made on illness data. FRI SEP 18 BENCHMARK AT RISK - the decision Wk C turns on. The 8 k benchmark gates the whole goal-pace addendum (sub-3:00 vs sub-3:10; the 3 k @ 6:20 inside the Sep 27 long). A benchmark on a post-illness engine reads falsely slow and would retire the stretch goal for the wrong reason. The benchmark is moveable; the bone is not. Call made off the first clean AM, not before. WK C DEFERRED to the first symptom-free morning. Re-entry shape: one easy short run first, HR ceiling 140, distance set by bone - not a jump back onto the ramp where it was interrupted.</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="18" customHeight="1">
       <c r="A43" s="37" t="n"/>

</xml_diff>

<commit_message>
log: set Wk C illness re-entry, defer 8k benchmark to Sep 25
Mon 9/14 + Tue 9/15 logged as illness rest (bike only, no data).
Clear <24h as of Tue, so re-entry run is Wed 9/16, not today.

Wk C: 21 km / 3 runs / 1 cali / 2 rest. Wed 4k re-entry HR ceiling
140 (gated on a clear Wed AM), Thu rest, Fri cali #4 + 5k, Sat rest,
Sun long 12k — reuses Wk B's lost long rather than compressing.

8k benchmark moved Fri Sep 18 -> Fri Sep 25: a post-illness benchmark
reads falsely slow and would retire sub-3:00 for the wrong reason.
Sep 25 still precedes the Sep 27 long, so the goal-pace addendum is
intact. Nothing above HR 150 until then.

Also flags the decision due Sun 9/20 on the 12->18->22 ramp.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -31602,7 +31602,9 @@
       </c>
     </row>
     <row r="43" ht="18" customHeight="1">
-      <c r="A43" s="37" t="n"/>
+      <c r="A43" s="37" t="n">
+        <v>46279</v>
+      </c>
       <c r="B43" s="22">
         <f>IF(A43="","",IFERROR(INT((A43-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
@@ -31613,10 +31615,16 @@
       <c r="F43" s="38" t="n"/>
       <c r="G43" s="38" t="n"/>
       <c r="H43" s="38" t="n"/>
-      <c r="I43" s="26" t="n"/>
+      <c r="I43" s="26" t="inlineStr">
+        <is>
+          <t>Wk B/C gap Mon - REST, ILLNESS day 3. No run, no cali, no AM block, no PM block, no BW, no shin check. NOT reconstructed. Uni day, bike commute ridden but unmeasured - not logged as a number. MONDAY AM CALI SLOT LOST and NOT made up: stacking a cali session into a re-entry week would put loaded legs in front of the first post-illness run, which is backwards - the run is the session that matters and the bone is the gate. BW TREND CALL THAT WAS SCHEDULED FOR TODAY IS VOID: no weigh-in taken, and 9/11's 76.20 is already confounded by the 9/10 data hole plus illness (appetite, hydration, glycogen). First honest BW reading is Thu 9/17; trend call Sun 9/20. NO KCAL CHANGE ON ILLNESS DATA.</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="35" t="n"/>
+      <c r="A44" s="35" t="n">
+        <v>46280</v>
+      </c>
       <c r="B44" s="16">
         <f>IF(A44="","",IFERROR(INT((A44-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
@@ -31627,7 +31635,11 @@
       <c r="F44" s="36" t="n"/>
       <c r="G44" s="36" t="n"/>
       <c r="H44" s="36" t="n"/>
-      <c r="I44" s="20" t="n"/>
+      <c r="I44" s="20" t="inlineStr">
+        <is>
+          <t>Wk C eve Tue - REST, illness clearing. SYMPTOM-FREE FROM THIS MORNING ONLY = under 24 h, so the neck-check gate is NOT met and there is NO re-entry run today. Below-neck rule governs: zero training until 24 h FULLY symptom-free, then ONE easy short run before anything loaded. 'Better than yesterday' is not 'clear'. Uni day, bike commute ridden, nothing else. WED 9/16 AM IS THE 24 H MARK. Run gap now 5 days (last run Fri 9/11, 6 k). THIS IS ILLNESS, NOT DRIFT - no make-ups, no clawed-back km, repeat don't compress. WK C SET TONIGHT: 21 km / 3 runs / 1 cali / 2 rest - Wed 4 k re-entry HR CEILING 140 (gated on a still-clear Wed AM), Thu REST, Fri cali #4 + 5 k, Sat REST, Sun LONG 12 k (reuses Wk B's lost long rather than jumping to where the ramp stopped). FRI SEP 18 8 K BENCHMARK DEFERRED TO FRI SEP 25: an 8 k all-out off two sick days and a 5-day run gap reads falsely slow and would retire sub-3:00 for the wrong reason - the benchmark is moveable, the bone is not. Sep 25 still sits 2 days before the Sep 27 long so the goal-pace addendum survives intact; gate thresholds unchanged. Consequence: NOTHING ABOVE HR 150 THROUGH FRI SEP 25 - Wk C is 100% easy. DECISION DUE SUN 9/20: the 12-&gt;18-&gt;22 long-run ramp is +50% in one week on bone that will have run 21 km in three weeks; recommendation is 16 k on 9/27 and 20 k on 10/4, decided off the 9/20 shin check and back-half pace.</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="37" t="n"/>

</xml_diff>

<commit_message>
sync: workbook + memory through 2026-09-21
Running Log row 23 and Body Metrics row 47 appended for Mon 9/21
(6 k, 7:56/km, HR 145, cadence 170, shin clean #26, bike 0).

Memory: cadence item closed for good; workbook sync state recorded;
BW series flagged dark since 9/11 (10-day hole, no trend call, no
kcal change off it).

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -28273,22 +28273,45 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="A23" s="37" t="n"/>
+      <c r="A23" s="37" t="n">
+        <v>46286</v>
+      </c>
       <c r="B23" s="22">
         <f>IF(A23="","",IFERROR(INT((A23-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C23" s="28" t="n"/>
-      <c r="D23" s="38" t="n"/>
+      <c r="C23" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D23" s="38" t="n">
+        <v>47.7</v>
+      </c>
       <c r="E23" s="22">
         <f>IF(OR(C23="",D23=""),"",TEXT(D23/C23/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F23" s="22" t="n"/>
-      <c r="G23" s="22" t="n"/>
-      <c r="H23" s="22" t="n"/>
-      <c r="I23" s="22" t="n"/>
-      <c r="J23" s="26" t="n"/>
+      <c r="F23" s="22" t="n">
+        <v>145</v>
+      </c>
+      <c r="G23" s="22" t="n">
+        <v>154</v>
+      </c>
+      <c r="H23" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="I23" s="22" t="inlineStr">
+        <is>
+          <t>Easy Z2</t>
+        </is>
+      </c>
+      <c r="J23" s="26" t="inlineStr">
+        <is>
+          <t>Wk D Mon - run easy 6 k AM (Mon&lt;-&gt;Tue swap; cali #5 moved to Tue 9/22). 7:56/km, 99% Z2, CADENCE 170, 0 walk breaks, RPE 4, 'chill run'. SLOW-PACE CADENCE TEST - PASSED, ITEM CLOSED. Prescription was hold 7:45-8:00/km and hit 166 by SHORTENING STRIDE; pace came in at 7:56 = INSIDE the band, so the data point is VALID (no sub-7:40 void, nothing bought with speed) - the first obeyed opening pace in four tries (9/7 hot, 9/11 hot, 9/16 hot, 9/21 obeyed). Cadence 170 vs the only prior honest slow-pace test, 9/8 at 8:01/km -&gt; 163: same pace, +7 spm, and 4 ABOVE the 166 target. The cue does NOT break at slow pace; 9/8 was one failed rep, not a pace ceiling. NEW STANDING RULE: metronome 166 is a FLOOR at every pace, held by shortening stride; overshoot to 170 is welcome, do not chase it back down. Never re-test uncued (9/2 ran that: 160). Bone lever, not cosmetic - 163-&gt;170 across Sunday's 12 k easy portion is real reduction in impact per strike, and that is exactly where the tibia budget is spent. SHIN CLEAN - check #26, 26/26 this block. HR 145 @ 7:56 vs 140 @ 8:01 on 9/8 = +5 bpm at the same pace; NOT called as drift - 9/8 was RPE 1 in light rain, today RPE 4, and a shorter quicker stride carries a small metabolic cost. Noise band. Recheck Thu 9/24. BIKE 0 km on a uni day (class 12:00-17:00, run went AM) - zero training consequence, bike has no bone value; consequence is fuel only: Monday target drops from 2650-2700 to ~2400. Creatine Y. Loaded-day count intact: Mon run (1) -&gt; Tue cali #5 (2) -&gt; Wed full rest; max-2 holds, and the swap now gives the RPE-6 leg cap 48 h in front of Thu's 4 k. STILL OPEN: 9/18, 9/19, 9/20 unlogged - Sun 9/27 stays provisional at 15 k if the 9/20 long happened, 13 k if it was missed or cut short. Fri 9/25 benchmark unaffected.</t>
+        </is>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="24" ht="18" customHeight="1">
       <c r="A24" s="35" t="n"/>
@@ -31705,7 +31728,9 @@
       </c>
     </row>
     <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="37" t="n"/>
+      <c r="A47" s="37" t="n">
+        <v>46286</v>
+      </c>
       <c r="B47" s="22">
         <f>IF(A47="","",IFERROR(INT((A47-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
@@ -31716,7 +31741,11 @@
       <c r="F47" s="38" t="n"/>
       <c r="G47" s="38" t="n"/>
       <c r="H47" s="38" t="n"/>
-      <c r="I47" s="26" t="n"/>
+      <c r="I47" s="26" t="inlineStr">
+        <is>
+          <t>Wk D Mon - run easy 6 k AM, DONE (see Running Log 9/21). AM BLOCK NOT SUPPLIED - no BW, no sleep, no RHR, no DOMS, no motivation/energy/stress. NOT reconstructed. Shin CLEAN check #26 reported with the run. BW TREND STILL VOID: the last weigh-in is 9/11's confounded 76.20, and 9/14, 9/17 and 9/20 were all missed - the series now has a 10-day hole and no kcal decision can be made off it. NEXT REAL BW CALL NEEDS A CLEAN AM WEIGH-IN; earliest useful trend read is a week of consecutive mornings. Macros not counted - written off, not re-asked (user directive 2026-09-17). Creatine Y. Bike 0 km on a uni day -&gt; fuel target for the day is ~2400, not 2650-2700.</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Tue 9/22 cali #5 — row cap broken, ladder updated, workbook synced
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -18616,17 +18616,33 @@
       <c r="K403" s="26" t="n"/>
     </row>
     <row r="404" ht="18" customHeight="1">
-      <c r="A404" s="35" t="n"/>
+      <c r="A404" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B404" s="16">
         <f>IF(A404="","",IFERROR(INT((A404-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C404" s="16" t="n"/>
-      <c r="D404" s="17" t="n"/>
-      <c r="E404" s="16" t="n"/>
-      <c r="F404" s="16" t="n"/>
+      <c r="C404" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D404" s="17" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E404" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F404" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="G404" s="36" t="n"/>
-      <c r="H404" s="16" t="n"/>
+      <c r="H404" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I404" s="19">
         <f>IF(OR(F404="",G404=""),"",F404*G404)</f>
         <v/>
@@ -18635,20 +18651,40 @@
         <f>IF(OR(F404="",G404=""),"",ROUND(G404*(1+F404/30),1))</f>
         <v/>
       </c>
-      <c r="K404" s="20" t="n"/>
+      <c r="K404" s="20" t="inlineStr">
+        <is>
+          <t>Cali #5 (Wk D Tue, swapped from Mon). Setting 3, prescribed 4x8 -&gt; ran 4x10 @ 6/7/7/9 off a 13-day layoff. S4 RPE 9 -&gt; setting-2 gate not cleared. Next: setting 3 4x10; setting 2 opens at 4x10 @ &lt;=8. Session 45 min vs 60 planned - rests compressed.</t>
+        </is>
+      </c>
     </row>
     <row r="405" ht="18" customHeight="1">
-      <c r="A405" s="37" t="n"/>
+      <c r="A405" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B405" s="22">
         <f>IF(A405="","",IFERROR(INT((A405-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C405" s="22" t="n"/>
-      <c r="D405" s="23" t="n"/>
-      <c r="E405" s="22" t="n"/>
-      <c r="F405" s="22" t="n"/>
+      <c r="C405" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D405" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E405" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F405" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="G405" s="38" t="n"/>
-      <c r="H405" s="22" t="n"/>
+      <c r="H405" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I405" s="25">
         <f>IF(OR(F405="",G405=""),"",F405*G405)</f>
         <v/>
@@ -18660,17 +18696,33 @@
       <c r="K405" s="26" t="n"/>
     </row>
     <row r="406" ht="18" customHeight="1">
-      <c r="A406" s="35" t="n"/>
+      <c r="A406" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B406" s="16">
         <f>IF(A406="","",IFERROR(INT((A406-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C406" s="16" t="n"/>
-      <c r="D406" s="17" t="n"/>
-      <c r="E406" s="16" t="n"/>
-      <c r="F406" s="16" t="n"/>
+      <c r="C406" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D406" s="17" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E406" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F406" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="G406" s="36" t="n"/>
-      <c r="H406" s="16" t="n"/>
+      <c r="H406" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I406" s="19">
         <f>IF(OR(F406="",G406=""),"",F406*G406)</f>
         <v/>
@@ -18682,17 +18734,33 @@
       <c r="K406" s="20" t="n"/>
     </row>
     <row r="407" ht="18" customHeight="1">
-      <c r="A407" s="37" t="n"/>
+      <c r="A407" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B407" s="22">
         <f>IF(A407="","",IFERROR(INT((A407-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C407" s="22" t="n"/>
-      <c r="D407" s="23" t="n"/>
-      <c r="E407" s="22" t="n"/>
-      <c r="F407" s="22" t="n"/>
+      <c r="C407" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D407" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E407" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F407" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="G407" s="38" t="n"/>
-      <c r="H407" s="22" t="n"/>
+      <c r="H407" s="22" t="n">
+        <v>9</v>
+      </c>
       <c r="I407" s="25">
         <f>IF(OR(F407="",G407=""),"",F407*G407)</f>
         <v/>
@@ -18704,17 +18772,33 @@
       <c r="K407" s="26" t="n"/>
     </row>
     <row r="408" ht="18" customHeight="1">
-      <c r="A408" s="35" t="n"/>
+      <c r="A408" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B408" s="16">
         <f>IF(A408="","",IFERROR(INT((A408-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C408" s="16" t="n"/>
-      <c r="D408" s="17" t="n"/>
-      <c r="E408" s="16" t="n"/>
-      <c r="F408" s="16" t="n"/>
+      <c r="C408" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D408" s="17" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E408" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F408" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="G408" s="36" t="n"/>
-      <c r="H408" s="16" t="n"/>
+      <c r="H408" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I408" s="19">
         <f>IF(OR(F408="",G408=""),"",F408*G408)</f>
         <v/>
@@ -18723,20 +18807,40 @@
         <f>IF(OR(F408="",G408=""),"",ROUND(G408*(1+F408/30),1))</f>
         <v/>
       </c>
-      <c r="K408" s="20" t="n"/>
+      <c r="K408" s="20" t="inlineStr">
+        <is>
+          <t>Setting 3. 8-REP CAP BROKEN -&gt; 10/9/9/7 @ 8/9/9/10, decay returned exactly as 9/5. Push/pull RPE gap 0.0 -&gt; 1.14 from this alone. Next: 4x8 HARD STOP.</t>
+        </is>
+      </c>
     </row>
     <row r="409" ht="18" customHeight="1">
-      <c r="A409" s="37" t="n"/>
+      <c r="A409" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B409" s="22">
         <f>IF(A409="","",IFERROR(INT((A409-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C409" s="22" t="n"/>
-      <c r="D409" s="23" t="n"/>
-      <c r="E409" s="22" t="n"/>
-      <c r="F409" s="22" t="n"/>
+      <c r="C409" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D409" s="23" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E409" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F409" s="22" t="n">
+        <v>9</v>
+      </c>
       <c r="G409" s="38" t="n"/>
-      <c r="H409" s="22" t="n"/>
+      <c r="H409" s="22" t="n">
+        <v>9</v>
+      </c>
       <c r="I409" s="25">
         <f>IF(OR(F409="",G409=""),"",F409*G409)</f>
         <v/>
@@ -18748,17 +18852,33 @@
       <c r="K409" s="26" t="n"/>
     </row>
     <row r="410" ht="18" customHeight="1">
-      <c r="A410" s="35" t="n"/>
+      <c r="A410" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B410" s="16">
         <f>IF(A410="","",IFERROR(INT((A410-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C410" s="16" t="n"/>
-      <c r="D410" s="17" t="n"/>
-      <c r="E410" s="16" t="n"/>
-      <c r="F410" s="16" t="n"/>
+      <c r="C410" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D410" s="17" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E410" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F410" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="G410" s="36" t="n"/>
-      <c r="H410" s="16" t="n"/>
+      <c r="H410" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="I410" s="19">
         <f>IF(OR(F410="",G410=""),"",F410*G410)</f>
         <v/>
@@ -18770,17 +18890,33 @@
       <c r="K410" s="20" t="n"/>
     </row>
     <row r="411" ht="18" customHeight="1">
-      <c r="A411" s="37" t="n"/>
+      <c r="A411" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B411" s="22">
         <f>IF(A411="","",IFERROR(INT((A411-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C411" s="22" t="n"/>
-      <c r="D411" s="23" t="n"/>
-      <c r="E411" s="22" t="n"/>
-      <c r="F411" s="22" t="n"/>
+      <c r="C411" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D411" s="23" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E411" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F411" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="G411" s="38" t="n"/>
-      <c r="H411" s="22" t="n"/>
+      <c r="H411" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="I411" s="25">
         <f>IF(OR(F411="",G411=""),"",F411*G411)</f>
         <v/>
@@ -18792,17 +18928,33 @@
       <c r="K411" s="26" t="n"/>
     </row>
     <row r="412" ht="18" customHeight="1">
-      <c r="A412" s="35" t="n"/>
+      <c r="A412" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B412" s="16">
         <f>IF(A412="","",IFERROR(INT((A412-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C412" s="16" t="n"/>
-      <c r="D412" s="17" t="n"/>
-      <c r="E412" s="16" t="n"/>
-      <c r="F412" s="16" t="n"/>
+      <c r="C412" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D412" s="17" t="inlineStr">
+        <is>
+          <t>Pull-up (negatives)</t>
+        </is>
+      </c>
+      <c r="E412" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F412" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="G412" s="36" t="n"/>
-      <c r="H412" s="16" t="n"/>
+      <c r="H412" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I412" s="19">
         <f>IF(OR(F412="",G412=""),"",F412*G412)</f>
         <v/>
@@ -18811,20 +18963,40 @@
         <f>IF(OR(F412="",G412=""),"",ROUND(G412*(1+F412/30),1))</f>
         <v/>
       </c>
-      <c r="K412" s="20" t="n"/>
+      <c r="K412" s="20" t="inlineStr">
+        <is>
+          <t>Variation switched from feet-assisted to negatives by athlete. S1 overshoot (9) spent S3 (RPE 10). Next: negatives 3x5, stop at 5.</t>
+        </is>
+      </c>
     </row>
     <row r="413" ht="18" customHeight="1">
-      <c r="A413" s="37" t="n"/>
+      <c r="A413" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B413" s="22">
         <f>IF(A413="","",IFERROR(INT((A413-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C413" s="22" t="n"/>
-      <c r="D413" s="23" t="n"/>
-      <c r="E413" s="22" t="n"/>
-      <c r="F413" s="22" t="n"/>
+      <c r="C413" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D413" s="23" t="inlineStr">
+        <is>
+          <t>Pull-up (negatives)</t>
+        </is>
+      </c>
+      <c r="E413" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F413" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="G413" s="38" t="n"/>
-      <c r="H413" s="22" t="n"/>
+      <c r="H413" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I413" s="25">
         <f>IF(OR(F413="",G413=""),"",F413*G413)</f>
         <v/>
@@ -18836,17 +19008,33 @@
       <c r="K413" s="26" t="n"/>
     </row>
     <row r="414" ht="18" customHeight="1">
-      <c r="A414" s="35" t="n"/>
+      <c r="A414" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B414" s="16">
         <f>IF(A414="","",IFERROR(INT((A414-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C414" s="16" t="n"/>
-      <c r="D414" s="17" t="n"/>
-      <c r="E414" s="16" t="n"/>
-      <c r="F414" s="16" t="n"/>
+      <c r="C414" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D414" s="17" t="inlineStr">
+        <is>
+          <t>Pull-up (negatives)</t>
+        </is>
+      </c>
+      <c r="E414" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F414" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="G414" s="36" t="n"/>
-      <c r="H414" s="16" t="n"/>
+      <c r="H414" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="I414" s="19">
         <f>IF(OR(F414="",G414=""),"",F414*G414)</f>
         <v/>
@@ -18858,17 +19046,33 @@
       <c r="K414" s="20" t="n"/>
     </row>
     <row r="415" ht="18" customHeight="1">
-      <c r="A415" s="37" t="n"/>
+      <c r="A415" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B415" s="22">
         <f>IF(A415="","",IFERROR(INT((A415-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C415" s="22" t="n"/>
-      <c r="D415" s="23" t="n"/>
-      <c r="E415" s="22" t="n"/>
-      <c r="F415" s="22" t="n"/>
+      <c r="C415" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D415" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (2nd block, incline)</t>
+        </is>
+      </c>
+      <c r="E415" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F415" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="G415" s="38" t="n"/>
-      <c r="H415" s="22" t="n"/>
+      <c r="H415" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I415" s="25">
         <f>IF(OR(F415="",G415=""),"",F415*G415)</f>
         <v/>
@@ -18877,20 +19081,40 @@
         <f>IF(OR(F415="",G415=""),"",ROUND(G415*(1+F415/30),1))</f>
         <v/>
       </c>
-      <c r="K415" s="26" t="n"/>
+      <c r="K415" s="26" t="inlineStr">
+        <is>
+          <t>Setting 3, prescribed 3x6. S3 to failure. Next: hold 3x6.</t>
+        </is>
+      </c>
     </row>
     <row r="416" ht="18" customHeight="1">
-      <c r="A416" s="35" t="n"/>
+      <c r="A416" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B416" s="16">
         <f>IF(A416="","",IFERROR(INT((A416-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C416" s="16" t="n"/>
-      <c r="D416" s="17" t="n"/>
-      <c r="E416" s="16" t="n"/>
-      <c r="F416" s="16" t="n"/>
+      <c r="C416" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D416" s="17" t="inlineStr">
+        <is>
+          <t>Push-up (2nd block, incline)</t>
+        </is>
+      </c>
+      <c r="E416" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F416" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="G416" s="36" t="n"/>
-      <c r="H416" s="16" t="n"/>
+      <c r="H416" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I416" s="19">
         <f>IF(OR(F416="",G416=""),"",F416*G416)</f>
         <v/>
@@ -18902,17 +19126,33 @@
       <c r="K416" s="20" t="n"/>
     </row>
     <row r="417" ht="18" customHeight="1">
-      <c r="A417" s="37" t="n"/>
+      <c r="A417" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B417" s="22">
         <f>IF(A417="","",IFERROR(INT((A417-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C417" s="22" t="n"/>
-      <c r="D417" s="23" t="n"/>
-      <c r="E417" s="22" t="n"/>
-      <c r="F417" s="22" t="n"/>
+      <c r="C417" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D417" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (2nd block, incline)</t>
+        </is>
+      </c>
+      <c r="E417" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F417" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="G417" s="38" t="n"/>
-      <c r="H417" s="22" t="n"/>
+      <c r="H417" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="I417" s="25">
         <f>IF(OR(F417="",G417=""),"",F417*G417)</f>
         <v/>
@@ -18924,17 +19164,33 @@
       <c r="K417" s="26" t="n"/>
     </row>
     <row r="418" ht="18" customHeight="1">
-      <c r="A418" s="35" t="n"/>
+      <c r="A418" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B418" s="16">
         <f>IF(A418="","",IFERROR(INT((A418-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C418" s="16" t="n"/>
-      <c r="D418" s="17" t="n"/>
-      <c r="E418" s="16" t="n"/>
-      <c r="F418" s="16" t="n"/>
+      <c r="C418" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D418" s="17" t="inlineStr">
+        <is>
+          <t>Bulgarian Split Squat (BW)</t>
+        </is>
+      </c>
+      <c r="E418" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F418" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="G418" s="36" t="n"/>
-      <c r="H418" s="16" t="n"/>
+      <c r="H418" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I418" s="19">
         <f>IF(OR(F418="",G418=""),"",F418*G418)</f>
         <v/>
@@ -18943,20 +19199,40 @@
         <f>IF(OR(F418="",G418=""),"",ROUND(G418*(1+F418/30),1))</f>
         <v/>
       </c>
-      <c r="K418" s="20" t="n"/>
+      <c r="K418" s="20" t="inlineStr">
+        <is>
+          <t>reps per leg. RPE 6 cap held every set. Cut Fri 9/25 (benchmark); next Mon 9/28 3x8.</t>
+        </is>
+      </c>
     </row>
     <row r="419" ht="18" customHeight="1">
-      <c r="A419" s="37" t="n"/>
+      <c r="A419" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B419" s="22">
         <f>IF(A419="","",IFERROR(INT((A419-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C419" s="22" t="n"/>
-      <c r="D419" s="23" t="n"/>
-      <c r="E419" s="22" t="n"/>
-      <c r="F419" s="22" t="n"/>
+      <c r="C419" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D419" s="23" t="inlineStr">
+        <is>
+          <t>Bulgarian Split Squat (BW)</t>
+        </is>
+      </c>
+      <c r="E419" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F419" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G419" s="38" t="n"/>
-      <c r="H419" s="22" t="n"/>
+      <c r="H419" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I419" s="25">
         <f>IF(OR(F419="",G419=""),"",F419*G419)</f>
         <v/>
@@ -18968,17 +19244,33 @@
       <c r="K419" s="26" t="n"/>
     </row>
     <row r="420" ht="18" customHeight="1">
-      <c r="A420" s="35" t="n"/>
+      <c r="A420" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B420" s="16">
         <f>IF(A420="","",IFERROR(INT((A420-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C420" s="16" t="n"/>
-      <c r="D420" s="17" t="n"/>
-      <c r="E420" s="16" t="n"/>
-      <c r="F420" s="16" t="n"/>
+      <c r="C420" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D420" s="17" t="inlineStr">
+        <is>
+          <t>Bulgarian Split Squat (BW)</t>
+        </is>
+      </c>
+      <c r="E420" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F420" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="G420" s="36" t="n"/>
-      <c r="H420" s="16" t="n"/>
+      <c r="H420" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I420" s="19">
         <f>IF(OR(F420="",G420=""),"",F420*G420)</f>
         <v/>
@@ -18990,17 +19282,33 @@
       <c r="K420" s="20" t="n"/>
     </row>
     <row r="421" ht="18" customHeight="1">
-      <c r="A421" s="37" t="n"/>
+      <c r="A421" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B421" s="22">
         <f>IF(A421="","",IFERROR(INT((A421-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C421" s="22" t="n"/>
-      <c r="D421" s="23" t="n"/>
-      <c r="E421" s="22" t="n"/>
-      <c r="F421" s="22" t="n"/>
+      <c r="C421" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D421" s="23" t="inlineStr">
+        <is>
+          <t>Single-Leg RDL (BW)</t>
+        </is>
+      </c>
+      <c r="E421" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F421" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="G421" s="38" t="n"/>
-      <c r="H421" s="22" t="n"/>
+      <c r="H421" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I421" s="25">
         <f>IF(OR(F421="",G421=""),"",F421*G421)</f>
         <v/>
@@ -19009,20 +19317,40 @@
         <f>IF(OR(F421="",G421=""),"",ROUND(G421*(1+F421/30),1))</f>
         <v/>
       </c>
-      <c r="K421" s="26" t="n"/>
+      <c r="K421" s="26" t="inlineStr">
+        <is>
+          <t>reps per leg. RPE 6 cap held every set.</t>
+        </is>
+      </c>
     </row>
     <row r="422" ht="18" customHeight="1">
-      <c r="A422" s="35" t="n"/>
+      <c r="A422" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B422" s="16">
         <f>IF(A422="","",IFERROR(INT((A422-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C422" s="16" t="n"/>
-      <c r="D422" s="17" t="n"/>
-      <c r="E422" s="16" t="n"/>
-      <c r="F422" s="16" t="n"/>
+      <c r="C422" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D422" s="17" t="inlineStr">
+        <is>
+          <t>Single-Leg RDL (BW)</t>
+        </is>
+      </c>
+      <c r="E422" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F422" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="G422" s="36" t="n"/>
-      <c r="H422" s="16" t="n"/>
+      <c r="H422" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I422" s="19">
         <f>IF(OR(F422="",G422=""),"",F422*G422)</f>
         <v/>
@@ -19034,17 +19362,33 @@
       <c r="K422" s="20" t="n"/>
     </row>
     <row r="423" ht="18" customHeight="1">
-      <c r="A423" s="37" t="n"/>
+      <c r="A423" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B423" s="22">
         <f>IF(A423="","",IFERROR(INT((A423-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C423" s="22" t="n"/>
-      <c r="D423" s="23" t="n"/>
-      <c r="E423" s="22" t="n"/>
-      <c r="F423" s="22" t="n"/>
+      <c r="C423" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D423" s="23" t="inlineStr">
+        <is>
+          <t>Single-Leg RDL (BW)</t>
+        </is>
+      </c>
+      <c r="E423" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F423" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G423" s="38" t="n"/>
-      <c r="H423" s="22" t="n"/>
+      <c r="H423" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I423" s="25">
         <f>IF(OR(F423="",G423=""),"",F423*G423)</f>
         <v/>
@@ -19056,17 +19400,33 @@
       <c r="K423" s="26" t="n"/>
     </row>
     <row r="424" ht="18" customHeight="1">
-      <c r="A424" s="35" t="n"/>
+      <c r="A424" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B424" s="16">
         <f>IF(A424="","",IFERROR(INT((A424-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C424" s="16" t="n"/>
-      <c r="D424" s="17" t="n"/>
-      <c r="E424" s="16" t="n"/>
-      <c r="F424" s="16" t="n"/>
+      <c r="C424" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D424" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise (slow ecc, BW)</t>
+        </is>
+      </c>
+      <c r="E424" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F424" s="16" t="n">
+        <v>15</v>
+      </c>
       <c r="G424" s="36" t="n"/>
-      <c r="H424" s="16" t="n"/>
+      <c r="H424" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="I424" s="19">
         <f>IF(OR(F424="",G424=""),"",F424*G424)</f>
         <v/>
@@ -19075,20 +19435,40 @@
         <f>IF(OR(F424="",G424=""),"",ROUND(G424*(1+F424/30),1))</f>
         <v/>
       </c>
-      <c r="K424" s="20" t="n"/>
+      <c r="K424" s="20" t="inlineStr">
+        <is>
+          <t>First session slow eccentric 3 s. Prescribed 3x20 - ran 15s at RPE 5-5.5, far under target. Next: full 3x20, Fri PM post-run.</t>
+        </is>
+      </c>
     </row>
     <row r="425" ht="18" customHeight="1">
-      <c r="A425" s="37" t="n"/>
+      <c r="A425" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B425" s="22">
         <f>IF(A425="","",IFERROR(INT((A425-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C425" s="22" t="n"/>
-      <c r="D425" s="23" t="n"/>
-      <c r="E425" s="22" t="n"/>
-      <c r="F425" s="22" t="n"/>
+      <c r="C425" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D425" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise (slow ecc, BW)</t>
+        </is>
+      </c>
+      <c r="E425" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F425" s="22" t="n">
+        <v>15</v>
+      </c>
       <c r="G425" s="38" t="n"/>
-      <c r="H425" s="22" t="n"/>
+      <c r="H425" s="22" t="n">
+        <v>5.5</v>
+      </c>
       <c r="I425" s="25">
         <f>IF(OR(F425="",G425=""),"",F425*G425)</f>
         <v/>
@@ -19100,17 +19480,33 @@
       <c r="K425" s="26" t="n"/>
     </row>
     <row r="426" ht="18" customHeight="1">
-      <c r="A426" s="35" t="n"/>
+      <c r="A426" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B426" s="16">
         <f>IF(A426="","",IFERROR(INT((A426-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C426" s="16" t="n"/>
-      <c r="D426" s="17" t="n"/>
-      <c r="E426" s="16" t="n"/>
-      <c r="F426" s="16" t="n"/>
+      <c r="C426" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D426" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise (slow ecc, BW)</t>
+        </is>
+      </c>
+      <c r="E426" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F426" s="16" t="n">
+        <v>15</v>
+      </c>
       <c r="G426" s="36" t="n"/>
-      <c r="H426" s="16" t="n"/>
+      <c r="H426" s="16" t="n">
+        <v>5.5</v>
+      </c>
       <c r="I426" s="19">
         <f>IF(OR(F426="",G426=""),"",F426*G426)</f>
         <v/>
@@ -19122,17 +19518,33 @@
       <c r="K426" s="20" t="n"/>
     </row>
     <row r="427" ht="18" customHeight="1">
-      <c r="A427" s="37" t="n"/>
+      <c r="A427" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B427" s="22">
         <f>IF(A427="","",IFERROR(INT((A427-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C427" s="22" t="n"/>
-      <c r="D427" s="23" t="n"/>
-      <c r="E427" s="22" t="n"/>
-      <c r="F427" s="22" t="n"/>
+      <c r="C427" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D427" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E427" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F427" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="G427" s="38" t="n"/>
-      <c r="H427" s="22" t="n"/>
+      <c r="H427" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I427" s="25">
         <f>IF(OR(F427="",G427=""),"",F427*G427)</f>
         <v/>
@@ -19141,20 +19553,40 @@
         <f>IF(OR(F427="",G427=""),"",ROUND(G427*(1+F427/30),1))</f>
         <v/>
       </c>
-      <c r="K427" s="26" t="n"/>
+      <c r="K427" s="26" t="inlineStr">
+        <is>
+          <t>Down from 8/8/8 on 9/9 - grip spent after B1 RPE 10. Next: 3x6, rebuild to 8.</t>
+        </is>
+      </c>
     </row>
     <row r="428" ht="18" customHeight="1">
-      <c r="A428" s="35" t="n"/>
+      <c r="A428" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B428" s="16">
         <f>IF(A428="","",IFERROR(INT((A428-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C428" s="16" t="n"/>
-      <c r="D428" s="17" t="n"/>
-      <c r="E428" s="16" t="n"/>
-      <c r="F428" s="16" t="n"/>
+      <c r="C428" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D428" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E428" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F428" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="G428" s="36" t="n"/>
-      <c r="H428" s="16" t="n"/>
+      <c r="H428" s="16" t="n">
+        <v>7.5</v>
+      </c>
       <c r="I428" s="19">
         <f>IF(OR(F428="",G428=""),"",F428*G428)</f>
         <v/>
@@ -19166,17 +19598,33 @@
       <c r="K428" s="20" t="n"/>
     </row>
     <row r="429" ht="18" customHeight="1">
-      <c r="A429" s="37" t="n"/>
+      <c r="A429" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B429" s="22">
         <f>IF(A429="","",IFERROR(INT((A429-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C429" s="22" t="n"/>
-      <c r="D429" s="23" t="n"/>
-      <c r="E429" s="22" t="n"/>
-      <c r="F429" s="22" t="n"/>
+      <c r="C429" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D429" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E429" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F429" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="G429" s="38" t="n"/>
-      <c r="H429" s="22" t="n"/>
+      <c r="H429" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I429" s="25">
         <f>IF(OR(F429="",G429=""),"",F429*G429)</f>
         <v/>
@@ -19188,17 +19636,33 @@
       <c r="K429" s="26" t="n"/>
     </row>
     <row r="430" ht="18" customHeight="1">
-      <c r="A430" s="35" t="n"/>
+      <c r="A430" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B430" s="16">
         <f>IF(A430="","",IFERROR(INT((A430-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C430" s="16" t="n"/>
-      <c r="D430" s="17" t="n"/>
-      <c r="E430" s="16" t="n"/>
-      <c r="F430" s="16" t="n"/>
+      <c r="C430" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D430" s="17" t="inlineStr">
+        <is>
+          <t>Side Plank (BW)</t>
+        </is>
+      </c>
+      <c r="E430" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F430" s="16" t="n">
+        <v>20</v>
+      </c>
       <c r="G430" s="36" t="n"/>
-      <c r="H430" s="16" t="n"/>
+      <c r="H430" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I430" s="19">
         <f>IF(OR(F430="",G430=""),"",F430*G430)</f>
         <v/>
@@ -19207,20 +19671,40 @@
         <f>IF(OR(F430="",G430=""),"",ROUND(G430*(1+F430/30),1))</f>
         <v/>
       </c>
-      <c r="K430" s="20" t="n"/>
+      <c r="K430" s="20" t="inlineStr">
+        <is>
+          <t>reps col = seconds PER SIDE. 45 s rung FAILED -&gt; 20 s @ 8/9. REGRESS to 2x30 s.</t>
+        </is>
+      </c>
     </row>
     <row r="431" ht="18" customHeight="1">
-      <c r="A431" s="37" t="n"/>
+      <c r="A431" s="37" t="n">
+        <v>46287</v>
+      </c>
       <c r="B431" s="22">
         <f>IF(A431="","",IFERROR(INT((A431-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C431" s="22" t="n"/>
-      <c r="D431" s="23" t="n"/>
-      <c r="E431" s="22" t="n"/>
-      <c r="F431" s="22" t="n"/>
+      <c r="C431" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D431" s="23" t="inlineStr">
+        <is>
+          <t>Side Plank (BW)</t>
+        </is>
+      </c>
+      <c r="E431" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F431" s="22" t="n">
+        <v>20</v>
+      </c>
       <c r="G431" s="38" t="n"/>
-      <c r="H431" s="22" t="n"/>
+      <c r="H431" s="22" t="n">
+        <v>9</v>
+      </c>
       <c r="I431" s="25">
         <f>IF(OR(F431="",G431=""),"",F431*G431)</f>
         <v/>
@@ -31748,7 +32232,9 @@
       </c>
     </row>
     <row r="48" ht="18" customHeight="1">
-      <c r="A48" s="35" t="n"/>
+      <c r="A48" s="35" t="n">
+        <v>46287</v>
+      </c>
       <c r="B48" s="16">
         <f>IF(A48="","",IFERROR(INT((A48-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
@@ -31759,7 +32245,11 @@
       <c r="F48" s="36" t="n"/>
       <c r="G48" s="36" t="n"/>
       <c r="H48" s="36" t="n"/>
-      <c r="I48" s="20" t="n"/>
+      <c r="I48" s="20" t="inlineStr">
+        <is>
+          <t>Wk D Tue - Cali #5 full, DONE (see Lifting Log 9/22). AM BLOCK NOT SUPPLIED - no BW; series dark since 9/11 (11 days). Shin CLEAN #27. Bike 24 km (uni day). Kcal 2772 (target 2650-2700, +72). Protein 161 g on target. Creatine Y. Pain none.</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="18" customHeight="1">
       <c r="A49" s="37" t="n"/>

</xml_diff>

<commit_message>
sync: workbook + memory through 2026-09-23
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -32252,18 +32252,28 @@
       </c>
     </row>
     <row r="49" ht="18" customHeight="1">
-      <c r="A49" s="37" t="n"/>
+      <c r="A49" s="37" t="n">
+        <v>46288</v>
+      </c>
       <c r="B49" s="22">
         <f>IF(A49="","",IFERROR(INT((A49-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C49" s="38" t="n"/>
-      <c r="D49" s="38" t="n"/>
+      <c r="C49" s="38" t="n">
+        <v>76.40000000000001</v>
+      </c>
+      <c r="D49" s="38" t="n">
+        <v>8</v>
+      </c>
       <c r="E49" s="38" t="n"/>
       <c r="F49" s="38" t="n"/>
       <c r="G49" s="38" t="n"/>
       <c r="H49" s="38" t="n"/>
-      <c r="I49" s="26" t="n"/>
+      <c r="I49" s="26" t="inlineStr">
+        <is>
+          <t>Wk D Wed - REST, FULL. AM: sleep 8 h (02:00-10:00) q8, RHR 46 (-2), mot 10/energy 10/stress 2, DOMS back/shldr/arm 3 (9/22 RPE-10 sets + compressed rests), legs 1, shin CLEAN #28. BW 76.40 = first reading in 12 days, single point, NO kcal change. SUN 9/20 LONG MISSED (user 9/23) -&gt; Sun 9/27 cut to 13 k (10 easy + 3 @ 6:20), Wk D 35 -&gt; 33 km; Wk E peak long 20 k off (~16-17 k, decide off 9/27 shin). PM: bike 0 (uni day -&gt; target ~2400), kcal 2933 (+530), protein 169, creatine Y.</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Thu 9/24 PM — 4k @ 6:35 off-prescription, shin #30, workbook synced
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -28798,22 +28798,45 @@
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="A24" s="35" t="n"/>
+      <c r="A24" s="35" t="n">
+        <v>46289</v>
+      </c>
       <c r="B24" s="16">
         <f>IF(A24="","",IFERROR(INT((A24-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C24" s="27" t="n"/>
-      <c r="D24" s="36" t="n"/>
+      <c r="C24" s="27" t="n">
+        <v>4</v>
+      </c>
+      <c r="D24" s="36" t="n">
+        <v>26.38</v>
+      </c>
       <c r="E24" s="16">
         <f>IF(OR(C24="",D24=""),"",TEXT(D24/C24/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F24" s="16" t="n"/>
-      <c r="G24" s="16" t="n"/>
-      <c r="H24" s="16" t="n"/>
-      <c r="I24" s="16" t="n"/>
-      <c r="J24" s="20" t="n"/>
+      <c r="F24" s="16" t="n">
+        <v>154</v>
+      </c>
+      <c r="G24" s="16" t="n">
+        <v>167</v>
+      </c>
+      <c r="H24" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="I24" s="16" t="inlineStr">
+        <is>
+          <t>Easy Z2</t>
+        </is>
+      </c>
+      <c r="J24" s="20" t="inlineStr">
+        <is>
+          <t>Wk D Thu - run easy 4 k, day before Fri 9/25 8 k benchmark. OFF-PRESCRIPTION: prescribed open 8:00/km, never under 7:40, HR ceiling 150. ACTUAL 6:35/km @ avg HR 154, max 167, Z1 7 / Z2 80 / Z3 13, cadence 165, 0 walk breaks, RPE 4, outdoor sunny. 'All good I felt really good.' Pace floor missed ~1:05/km, HR cap broken. Pace-obedience decay: 9/7 hot, 9/8 obeyed, 9/11 hot, 9/16 hot, 9/21 obeyed, 9/24 hot. CADENCE 165 VOID (pace &lt;7:40); note 170 @ 7:56 vs 165 @ 6:35 = longer stride at speed - metronome on for benchmark. HR drift check VOID (pace not matched to 9/21 145 @ 7:56); engine consistent with 9/16 (6:14 @ 159). SHIN CLEAN #30 (same-night; Fri AM is the gate). Benchmark cost small, Fri stands.</t>
+        </is>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="37" t="n"/>
@@ -32276,18 +32299,28 @@
       </c>
     </row>
     <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="35" t="n"/>
+      <c r="A50" s="35" t="n">
+        <v>46289</v>
+      </c>
       <c r="B50" s="16">
         <f>IF(A50="","",IFERROR(INT((A50-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C50" s="36" t="n"/>
-      <c r="D50" s="36" t="n"/>
+      <c r="C50" s="36" t="n">
+        <v>77.05</v>
+      </c>
+      <c r="D50" s="36" t="n">
+        <v>8.75</v>
+      </c>
       <c r="E50" s="36" t="n"/>
       <c r="F50" s="36" t="n"/>
       <c r="G50" s="36" t="n"/>
       <c r="H50" s="36" t="n"/>
-      <c r="I50" s="20" t="n"/>
+      <c r="I50" s="20" t="inlineStr">
+        <is>
+          <t>Wk D Thu - Run easy 4 k (see Running Log 9/24). AM: sleep 8:45 (23:45-08:30) q8, RHR 45 (-2), mot 10/energy 10/stress 2, DOMS chest/back/shldr/arm 3 (48 h peak of 9/22 RPE-10 sets), quad/ham 2, glute/calf 1, shin CLEAN #29. BW 77.05 (+0.65 d/d) - 2nd reading, NO kcal change, trend call Sun 9/27 on &gt;=3. PM: bike 0 (uni day -&gt; ~2400), kcal 2596 (+196), protein 175 (+10 over 155-165), creatine Y, alcohol 0, steps 9891, shin CLEAN #30.</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Fri 9/25 — 8k benchmark 5:42 moving/5:58 elapsed, sub-3:10 confirmed
Strava pull: core km 3-8 5:57 @ HR ~175, max 198, RPE 9, shin #32.
sub-3:00 stays closed. Workbook synced through 9/25. Sat cali #6 staged,
Sun long AM gate added.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -28839,22 +28839,45 @@
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="A25" s="37" t="n"/>
+      <c r="A25" s="37" t="n">
+        <v>46290</v>
+      </c>
       <c r="B25" s="22">
         <f>IF(A25="","",IFERROR(INT((A25-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C25" s="28" t="n"/>
-      <c r="D25" s="38" t="n"/>
+      <c r="C25" s="28" t="n">
+        <v>9.01</v>
+      </c>
+      <c r="D25" s="38" t="n">
+        <v>52.43</v>
+      </c>
       <c r="E25" s="22">
         <f>IF(OR(C25="",D25=""),"",TEXT(D25/C25/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F25" s="22" t="n"/>
-      <c r="G25" s="22" t="n"/>
-      <c r="H25" s="22" t="n"/>
-      <c r="I25" s="22" t="n"/>
-      <c r="J25" s="26" t="n"/>
+      <c r="F25" s="22" t="n">
+        <v>173</v>
+      </c>
+      <c r="G25" s="22" t="n">
+        <v>198</v>
+      </c>
+      <c r="H25" s="22" t="n">
+        <v>9</v>
+      </c>
+      <c r="I25" s="22" t="inlineStr">
+        <is>
+          <t>Benchmark</t>
+        </is>
+      </c>
+      <c r="J25" s="26" t="inlineStr">
+        <is>
+          <t>Wk D Fri - 8 K BENCHMARK, AM 09:34 (flipped from PM). Total 9.01 km moving 52:26, elapsed 54:43. WU 1 k (not 2) 6:46 @ 146, cadence 159. 8 k (km 2-9): 5:42/km moving, 5:58 elapsed. Splits 5:21 @179 (hero opener) / 6:05 @172 (+42 s traffic light) / 5:59 @174 / 5:52 @177 / 5:53 @177 / 6:03 @174 / 5:48 @177 / 4:37 @190 max 198 (+44 s traffic light). Even-effort core km 3-8 = 5:57 @ HR ~175. Cadence ~166 over the 8 k (laps 163-170). No CD. RPE 9. SHIN CLEAN #32. VERDICT: sub-3:10 CONFIRMED, sub-3:00 NOT opened (opener + stops + kick inflate moving avg; longest run 10 k). Race-pace HR model holds: 6:20 ~ HR 163-168. Tibialis moved to Sat.</t>
+        </is>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="35" t="n"/>
@@ -32323,18 +32346,28 @@
       </c>
     </row>
     <row r="51" ht="18" customHeight="1">
-      <c r="A51" s="37" t="n"/>
+      <c r="A51" s="37" t="n">
+        <v>46290</v>
+      </c>
       <c r="B51" s="22">
         <f>IF(A51="","",IFERROR(INT((A51-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C51" s="38" t="n"/>
-      <c r="D51" s="38" t="n"/>
+      <c r="C51" s="38" t="n">
+        <v>77.05</v>
+      </c>
+      <c r="D51" s="38" t="n">
+        <v>8.5</v>
+      </c>
       <c r="E51" s="38" t="n"/>
       <c r="F51" s="38" t="n"/>
       <c r="G51" s="38" t="n"/>
       <c r="H51" s="38" t="n"/>
-      <c r="I51" s="26" t="n"/>
+      <c r="I51" s="26" t="inlineStr">
+        <is>
+          <t>Wk D Fri - 8 K BENCHMARK (see Running Log 9/25). AM: sleep 8:30 (00:30-09:00) q10, RHR 46 (-1), mot 10/energy 10/stress 1, DOMS chest 1 / back 2 / shldr 2 / arm 2, quad 1 / ham 1 / glute 0 / calf 0, shin CLEAN #31. BW 77.05 flat d/d (3rd reading), NO kcal change, trend call Sun 9/27. Cali #6 moved to Sat 9/26 AM. PM: bike 0, kcal 2706 (+306, 3rd day over; 684 kcal benchmark), protein 178, creatine Y, alcohol 0, steps 14538, shin CLEAN #32, RPE 9.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="35" t="n"/>

</xml_diff>

<commit_message>
log: sync xlsx thru 9/26 (cali #6 rows 432-453, body row 52), stage Sun 9/27 13k long
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -19716,17 +19716,33 @@
       <c r="K431" s="26" t="n"/>
     </row>
     <row r="432" ht="18" customHeight="1">
-      <c r="A432" s="35" t="n"/>
+      <c r="A432" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B432" s="16">
         <f>IF(A432="","",IFERROR(INT((A432-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C432" s="16" t="n"/>
-      <c r="D432" s="17" t="n"/>
-      <c r="E432" s="16" t="n"/>
-      <c r="F432" s="16" t="n"/>
+      <c r="C432" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D432" s="17" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E432" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F432" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="G432" s="36" t="n"/>
-      <c r="H432" s="16" t="n"/>
+      <c r="H432" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I432" s="19">
         <f>IF(OR(F432="",G432=""),"",F432*G432)</f>
         <v/>
@@ -19735,20 +19751,40 @@
         <f>IF(OR(F432="",G432=""),"",ROUND(G432*(1+F432/30),1))</f>
         <v/>
       </c>
-      <c r="K432" s="20" t="n"/>
+      <c r="K432" s="20" t="inlineStr">
+        <is>
+          <t>Cali #6 UPPER ONLY (Sat, day before long), setting 3. S4 9-&gt;8 vs 9/22. Not all &lt;=7 -&gt; HOLD 4x10.</t>
+        </is>
+      </c>
     </row>
     <row r="433" ht="18" customHeight="1">
-      <c r="A433" s="37" t="n"/>
+      <c r="A433" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B433" s="22">
         <f>IF(A433="","",IFERROR(INT((A433-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C433" s="22" t="n"/>
-      <c r="D433" s="23" t="n"/>
-      <c r="E433" s="22" t="n"/>
-      <c r="F433" s="22" t="n"/>
+      <c r="C433" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D433" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E433" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F433" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="G433" s="38" t="n"/>
-      <c r="H433" s="22" t="n"/>
+      <c r="H433" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I433" s="25">
         <f>IF(OR(F433="",G433=""),"",F433*G433)</f>
         <v/>
@@ -19760,17 +19796,33 @@
       <c r="K433" s="26" t="n"/>
     </row>
     <row r="434" ht="18" customHeight="1">
-      <c r="A434" s="35" t="n"/>
+      <c r="A434" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B434" s="16">
         <f>IF(A434="","",IFERROR(INT((A434-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C434" s="16" t="n"/>
-      <c r="D434" s="17" t="n"/>
-      <c r="E434" s="16" t="n"/>
-      <c r="F434" s="16" t="n"/>
+      <c r="C434" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D434" s="17" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E434" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F434" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="G434" s="36" t="n"/>
-      <c r="H434" s="16" t="n"/>
+      <c r="H434" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I434" s="19">
         <f>IF(OR(F434="",G434=""),"",F434*G434)</f>
         <v/>
@@ -19782,17 +19834,33 @@
       <c r="K434" s="20" t="n"/>
     </row>
     <row r="435" ht="18" customHeight="1">
-      <c r="A435" s="37" t="n"/>
+      <c r="A435" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B435" s="22">
         <f>IF(A435="","",IFERROR(INT((A435-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C435" s="22" t="n"/>
-      <c r="D435" s="23" t="n"/>
-      <c r="E435" s="22" t="n"/>
-      <c r="F435" s="22" t="n"/>
+      <c r="C435" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D435" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E435" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F435" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="G435" s="38" t="n"/>
-      <c r="H435" s="22" t="n"/>
+      <c r="H435" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I435" s="25">
         <f>IF(OR(F435="",G435=""),"",F435*G435)</f>
         <v/>
@@ -19804,17 +19872,33 @@
       <c r="K435" s="26" t="n"/>
     </row>
     <row r="436" ht="18" customHeight="1">
-      <c r="A436" s="35" t="n"/>
+      <c r="A436" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B436" s="16">
         <f>IF(A436="","",IFERROR(INT((A436-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C436" s="16" t="n"/>
-      <c r="D436" s="17" t="n"/>
-      <c r="E436" s="16" t="n"/>
-      <c r="F436" s="16" t="n"/>
+      <c r="C436" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D436" s="17" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E436" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F436" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="G436" s="36" t="n"/>
-      <c r="H436" s="16" t="n"/>
+      <c r="H436" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I436" s="19">
         <f>IF(OR(F436="",G436=""),"",F436*G436)</f>
         <v/>
@@ -19823,20 +19907,40 @@
         <f>IF(OR(F436="",G436=""),"",ROUND(G436*(1+F436/30),1))</f>
         <v/>
       </c>
-      <c r="K436" s="20" t="n"/>
+      <c r="K436" s="20" t="inlineStr">
+        <is>
+          <t>Setting 3, 8-rep HARD STOP OBEYED (9/22: 10/9/9/7 @ ..10). Hold 4x8 cap.</t>
+        </is>
+      </c>
     </row>
     <row r="437" ht="18" customHeight="1">
-      <c r="A437" s="37" t="n"/>
+      <c r="A437" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B437" s="22">
         <f>IF(A437="","",IFERROR(INT((A437-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C437" s="22" t="n"/>
-      <c r="D437" s="23" t="n"/>
-      <c r="E437" s="22" t="n"/>
-      <c r="F437" s="22" t="n"/>
+      <c r="C437" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D437" s="23" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E437" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F437" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="G437" s="38" t="n"/>
-      <c r="H437" s="22" t="n"/>
+      <c r="H437" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I437" s="25">
         <f>IF(OR(F437="",G437=""),"",F437*G437)</f>
         <v/>
@@ -19848,17 +19952,33 @@
       <c r="K437" s="26" t="n"/>
     </row>
     <row r="438" ht="18" customHeight="1">
-      <c r="A438" s="35" t="n"/>
+      <c r="A438" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B438" s="16">
         <f>IF(A438="","",IFERROR(INT((A438-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C438" s="16" t="n"/>
-      <c r="D438" s="17" t="n"/>
-      <c r="E438" s="16" t="n"/>
-      <c r="F438" s="16" t="n"/>
+      <c r="C438" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D438" s="17" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E438" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F438" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="G438" s="36" t="n"/>
-      <c r="H438" s="16" t="n"/>
+      <c r="H438" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I438" s="19">
         <f>IF(OR(F438="",G438=""),"",F438*G438)</f>
         <v/>
@@ -19870,17 +19990,33 @@
       <c r="K438" s="20" t="n"/>
     </row>
     <row r="439" ht="18" customHeight="1">
-      <c r="A439" s="37" t="n"/>
+      <c r="A439" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B439" s="22">
         <f>IF(A439="","",IFERROR(INT((A439-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C439" s="22" t="n"/>
-      <c r="D439" s="23" t="n"/>
-      <c r="E439" s="22" t="n"/>
-      <c r="F439" s="22" t="n"/>
+      <c r="C439" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D439" s="23" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E439" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F439" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="G439" s="38" t="n"/>
-      <c r="H439" s="22" t="n"/>
+      <c r="H439" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I439" s="25">
         <f>IF(OR(F439="",G439=""),"",F439*G439)</f>
         <v/>
@@ -19892,17 +20028,33 @@
       <c r="K439" s="26" t="n"/>
     </row>
     <row r="440" ht="18" customHeight="1">
-      <c r="A440" s="35" t="n"/>
+      <c r="A440" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B440" s="16">
         <f>IF(A440="","",IFERROR(INT((A440-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C440" s="16" t="n"/>
-      <c r="D440" s="17" t="n"/>
-      <c r="E440" s="16" t="n"/>
-      <c r="F440" s="16" t="n"/>
+      <c r="C440" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D440" s="17" t="inlineStr">
+        <is>
+          <t>Pull-up (negatives)</t>
+        </is>
+      </c>
+      <c r="E440" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F440" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="G440" s="36" t="n"/>
-      <c r="H440" s="16" t="n"/>
+      <c r="H440" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I440" s="19">
         <f>IF(OR(F440="",G440=""),"",F440*G440)</f>
         <v/>
@@ -19911,20 +20063,40 @@
         <f>IF(OR(F440="",G440=""),"",ROUND(G440*(1+F440/30),1))</f>
         <v/>
       </c>
-      <c r="K440" s="20" t="n"/>
+      <c r="K440" s="20" t="inlineStr">
+        <is>
+          <t>Cap 5 held. S2 RPE 9 over &lt;=8 cap. Hold 3x5.</t>
+        </is>
+      </c>
     </row>
     <row r="441" ht="18" customHeight="1">
-      <c r="A441" s="37" t="n"/>
+      <c r="A441" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B441" s="22">
         <f>IF(A441="","",IFERROR(INT((A441-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C441" s="22" t="n"/>
-      <c r="D441" s="23" t="n"/>
-      <c r="E441" s="22" t="n"/>
-      <c r="F441" s="22" t="n"/>
+      <c r="C441" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D441" s="23" t="inlineStr">
+        <is>
+          <t>Pull-up (negatives)</t>
+        </is>
+      </c>
+      <c r="E441" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F441" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="G441" s="38" t="n"/>
-      <c r="H441" s="22" t="n"/>
+      <c r="H441" s="22" t="n">
+        <v>9</v>
+      </c>
       <c r="I441" s="25">
         <f>IF(OR(F441="",G441=""),"",F441*G441)</f>
         <v/>
@@ -19936,17 +20108,33 @@
       <c r="K441" s="26" t="n"/>
     </row>
     <row r="442" ht="18" customHeight="1">
-      <c r="A442" s="35" t="n"/>
+      <c r="A442" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B442" s="16">
         <f>IF(A442="","",IFERROR(INT((A442-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C442" s="16" t="n"/>
-      <c r="D442" s="17" t="n"/>
-      <c r="E442" s="16" t="n"/>
-      <c r="F442" s="16" t="n"/>
+      <c r="C442" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D442" s="17" t="inlineStr">
+        <is>
+          <t>Pull-up (negatives)</t>
+        </is>
+      </c>
+      <c r="E442" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F442" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="G442" s="36" t="n"/>
-      <c r="H442" s="16" t="n"/>
+      <c r="H442" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I442" s="19">
         <f>IF(OR(F442="",G442=""),"",F442*G442)</f>
         <v/>
@@ -19958,17 +20146,33 @@
       <c r="K442" s="20" t="n"/>
     </row>
     <row r="443" ht="18" customHeight="1">
-      <c r="A443" s="37" t="n"/>
+      <c r="A443" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B443" s="22">
         <f>IF(A443="","",IFERROR(INT((A443-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C443" s="22" t="n"/>
-      <c r="D443" s="23" t="n"/>
-      <c r="E443" s="22" t="n"/>
-      <c r="F443" s="22" t="n"/>
+      <c r="C443" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D443" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (2nd block, incline)</t>
+        </is>
+      </c>
+      <c r="E443" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F443" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G443" s="38" t="n"/>
-      <c r="H443" s="22" t="n"/>
+      <c r="H443" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I443" s="25">
         <f>IF(OR(F443="",G443=""),"",F443*G443)</f>
         <v/>
@@ -19977,20 +20181,40 @@
         <f>IF(OR(F443="",G443=""),"",ROUND(G443*(1+F443/30),1))</f>
         <v/>
       </c>
-      <c r="K443" s="26" t="n"/>
+      <c r="K443" s="26" t="inlineStr">
+        <is>
+          <t>Setting 3. Gate cleared -&gt; 3x7 next.</t>
+        </is>
+      </c>
     </row>
     <row r="444" ht="18" customHeight="1">
-      <c r="A444" s="35" t="n"/>
+      <c r="A444" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B444" s="16">
         <f>IF(A444="","",IFERROR(INT((A444-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C444" s="16" t="n"/>
-      <c r="D444" s="17" t="n"/>
-      <c r="E444" s="16" t="n"/>
-      <c r="F444" s="16" t="n"/>
+      <c r="C444" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D444" s="17" t="inlineStr">
+        <is>
+          <t>Push-up (2nd block, incline)</t>
+        </is>
+      </c>
+      <c r="E444" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F444" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="G444" s="36" t="n"/>
-      <c r="H444" s="16" t="n"/>
+      <c r="H444" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I444" s="19">
         <f>IF(OR(F444="",G444=""),"",F444*G444)</f>
         <v/>
@@ -20002,17 +20226,33 @@
       <c r="K444" s="20" t="n"/>
     </row>
     <row r="445" ht="18" customHeight="1">
-      <c r="A445" s="37" t="n"/>
+      <c r="A445" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B445" s="22">
         <f>IF(A445="","",IFERROR(INT((A445-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C445" s="22" t="n"/>
-      <c r="D445" s="23" t="n"/>
-      <c r="E445" s="22" t="n"/>
-      <c r="F445" s="22" t="n"/>
+      <c r="C445" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D445" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (2nd block, incline)</t>
+        </is>
+      </c>
+      <c r="E445" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F445" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G445" s="38" t="n"/>
-      <c r="H445" s="22" t="n"/>
+      <c r="H445" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I445" s="25">
         <f>IF(OR(F445="",G445=""),"",F445*G445)</f>
         <v/>
@@ -20024,17 +20264,33 @@
       <c r="K445" s="26" t="n"/>
     </row>
     <row r="446" ht="18" customHeight="1">
-      <c r="A446" s="35" t="n"/>
+      <c r="A446" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B446" s="16">
         <f>IF(A446="","",IFERROR(INT((A446-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C446" s="16" t="n"/>
-      <c r="D446" s="17" t="n"/>
-      <c r="E446" s="16" t="n"/>
-      <c r="F446" s="16" t="n"/>
+      <c r="C446" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D446" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E446" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F446" s="16" t="n">
+        <v>20</v>
+      </c>
       <c r="G446" s="36" t="n"/>
-      <c r="H446" s="16" t="n"/>
+      <c r="H446" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I446" s="19">
         <f>IF(OR(F446="",G446=""),"",F446*G446)</f>
         <v/>
@@ -20043,20 +20299,40 @@
         <f>IF(OR(F446="",G446=""),"",ROUND(G446*(1+F446/30),1))</f>
         <v/>
       </c>
-      <c r="K446" s="20" t="n"/>
+      <c r="K446" s="20" t="inlineStr">
+        <is>
+          <t>NORMAL tempo (carried from Fri, no slow ecc pre-long). Over &lt;=6 cap on DOMS-2 legs. Next: slow ecc 3x20.</t>
+        </is>
+      </c>
     </row>
     <row r="447" ht="18" customHeight="1">
-      <c r="A447" s="37" t="n"/>
+      <c r="A447" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B447" s="22">
         <f>IF(A447="","",IFERROR(INT((A447-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C447" s="22" t="n"/>
-      <c r="D447" s="23" t="n"/>
-      <c r="E447" s="22" t="n"/>
-      <c r="F447" s="22" t="n"/>
+      <c r="C447" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D447" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E447" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F447" s="22" t="n">
+        <v>20</v>
+      </c>
       <c r="G447" s="38" t="n"/>
-      <c r="H447" s="22" t="n"/>
+      <c r="H447" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I447" s="25">
         <f>IF(OR(F447="",G447=""),"",F447*G447)</f>
         <v/>
@@ -20068,17 +20344,33 @@
       <c r="K447" s="26" t="n"/>
     </row>
     <row r="448" ht="18" customHeight="1">
-      <c r="A448" s="35" t="n"/>
+      <c r="A448" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B448" s="16">
         <f>IF(A448="","",IFERROR(INT((A448-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C448" s="16" t="n"/>
-      <c r="D448" s="17" t="n"/>
-      <c r="E448" s="16" t="n"/>
-      <c r="F448" s="16" t="n"/>
+      <c r="C448" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D448" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E448" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F448" s="16" t="n">
+        <v>20</v>
+      </c>
       <c r="G448" s="36" t="n"/>
-      <c r="H448" s="16" t="n"/>
+      <c r="H448" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I448" s="19">
         <f>IF(OR(F448="",G448=""),"",F448*G448)</f>
         <v/>
@@ -20090,17 +20382,33 @@
       <c r="K448" s="20" t="n"/>
     </row>
     <row r="449" ht="18" customHeight="1">
-      <c r="A449" s="37" t="n"/>
+      <c r="A449" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B449" s="22">
         <f>IF(A449="","",IFERROR(INT((A449-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C449" s="22" t="n"/>
-      <c r="D449" s="23" t="n"/>
-      <c r="E449" s="22" t="n"/>
-      <c r="F449" s="22" t="n"/>
+      <c r="C449" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D449" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E449" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F449" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G449" s="38" t="n"/>
-      <c r="H449" s="22" t="n"/>
+      <c r="H449" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I449" s="25">
         <f>IF(OR(F449="",G449=""),"",F449*G449)</f>
         <v/>
@@ -20109,20 +20417,40 @@
         <f>IF(OR(F449="",G449=""),"",ROUND(G449*(1+F449/30),1))</f>
         <v/>
       </c>
-      <c r="K449" s="26" t="n"/>
+      <c r="K449" s="26" t="inlineStr">
+        <is>
+          <t>Rebuilding. Hold 3x6.</t>
+        </is>
+      </c>
     </row>
     <row r="450" ht="18" customHeight="1">
-      <c r="A450" s="35" t="n"/>
+      <c r="A450" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B450" s="16">
         <f>IF(A450="","",IFERROR(INT((A450-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C450" s="16" t="n"/>
-      <c r="D450" s="17" t="n"/>
-      <c r="E450" s="16" t="n"/>
-      <c r="F450" s="16" t="n"/>
+      <c r="C450" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D450" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E450" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F450" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="G450" s="36" t="n"/>
-      <c r="H450" s="16" t="n"/>
+      <c r="H450" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I450" s="19">
         <f>IF(OR(F450="",G450=""),"",F450*G450)</f>
         <v/>
@@ -20134,17 +20462,33 @@
       <c r="K450" s="20" t="n"/>
     </row>
     <row r="451" ht="18" customHeight="1">
-      <c r="A451" s="37" t="n"/>
+      <c r="A451" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B451" s="22">
         <f>IF(A451="","",IFERROR(INT((A451-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C451" s="22" t="n"/>
-      <c r="D451" s="23" t="n"/>
-      <c r="E451" s="22" t="n"/>
-      <c r="F451" s="22" t="n"/>
+      <c r="C451" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D451" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E451" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F451" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G451" s="38" t="n"/>
-      <c r="H451" s="22" t="n"/>
+      <c r="H451" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I451" s="25">
         <f>IF(OR(F451="",G451=""),"",F451*G451)</f>
         <v/>
@@ -20156,17 +20500,33 @@
       <c r="K451" s="26" t="n"/>
     </row>
     <row r="452" ht="18" customHeight="1">
-      <c r="A452" s="35" t="n"/>
+      <c r="A452" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B452" s="16">
         <f>IF(A452="","",IFERROR(INT((A452-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C452" s="16" t="n"/>
-      <c r="D452" s="17" t="n"/>
-      <c r="E452" s="16" t="n"/>
-      <c r="F452" s="16" t="n"/>
+      <c r="C452" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D452" s="17" t="inlineStr">
+        <is>
+          <t>Side Plank (BW)</t>
+        </is>
+      </c>
+      <c r="E452" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F452" s="16" t="n">
+        <v>30</v>
+      </c>
       <c r="G452" s="36" t="n"/>
-      <c r="H452" s="16" t="n"/>
+      <c r="H452" s="16" t="n">
+        <v>9</v>
+      </c>
       <c r="I452" s="19">
         <f>IF(OR(F452="",G452=""),"",F452*G452)</f>
         <v/>
@@ -20175,20 +20535,40 @@
         <f>IF(OR(F452="",G452=""),"",ROUND(G452*(1+F452/30),1))</f>
         <v/>
       </c>
-      <c r="K452" s="20" t="n"/>
+      <c r="K452" s="20" t="inlineStr">
+        <is>
+          <t>reps col = seconds PER SIDE. 30 s rung FAILED (30/20 @ 9). REGRESS to 2x20 s.</t>
+        </is>
+      </c>
     </row>
     <row r="453" ht="18" customHeight="1">
-      <c r="A453" s="37" t="n"/>
+      <c r="A453" s="37" t="n">
+        <v>46291</v>
+      </c>
       <c r="B453" s="22">
         <f>IF(A453="","",IFERROR(INT((A453-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C453" s="22" t="n"/>
-      <c r="D453" s="23" t="n"/>
-      <c r="E453" s="22" t="n"/>
-      <c r="F453" s="22" t="n"/>
+      <c r="C453" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D453" s="23" t="inlineStr">
+        <is>
+          <t>Side Plank (BW)</t>
+        </is>
+      </c>
+      <c r="E453" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F453" s="22" t="n">
+        <v>20</v>
+      </c>
       <c r="G453" s="38" t="n"/>
-      <c r="H453" s="22" t="n"/>
+      <c r="H453" s="22" t="n">
+        <v>9</v>
+      </c>
       <c r="I453" s="25">
         <f>IF(OR(F453="",G453=""),"",F453*G453)</f>
         <v/>
@@ -32370,18 +32750,28 @@
       </c>
     </row>
     <row r="52" ht="18" customHeight="1">
-      <c r="A52" s="35" t="n"/>
+      <c r="A52" s="35" t="n">
+        <v>46291</v>
+      </c>
       <c r="B52" s="16">
         <f>IF(A52="","",IFERROR(INT((A52-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C52" s="36" t="n"/>
-      <c r="D52" s="36" t="n"/>
+      <c r="C52" s="36" t="n">
+        <v>76.7</v>
+      </c>
+      <c r="D52" s="36" t="n">
+        <v>9.25</v>
+      </c>
       <c r="E52" s="36" t="n"/>
       <c r="F52" s="36" t="n"/>
       <c r="G52" s="36" t="n"/>
       <c r="H52" s="36" t="n"/>
-      <c r="I52" s="20" t="n"/>
+      <c r="I52" s="20" t="inlineStr">
+        <is>
+          <t>Wk D Sat - CALI #6 UPPER ONLY (see Lifting Log 9/26). AM: sleep 9:15 (23:45-09:00) q10, RHR 45 (-1), mot 10/energy 10/stress 2, DOMS chest 0 / back 1 / shldr 1 / arm 1, quad/ham/glute/calf 2 (benchmark hangover), shin CLEAN #33. BW 76.70 (-0.35 d/d), 4th reading, trend call Sun 9/27. PM: 22/22 sets 55 min avg RPE 7.6, 0 RPE-10 sets, row cap held, bike 0, kcal 2485 (+85), protein 171, creatine Y, shin CLEAN #34.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="37" t="n"/>

</xml_diff>

<commit_message>
log: sync xlsx thru 9/27, stage Wk E (32 km, 16k long) + Mon cali #7
- Running row 26 (9/27 long), Body row 53; wk 22 recalc = 4 runs, 32.02 km, BW 76.64
- Addendum table: 9/27 actuals, Oct 4 long 22k -> 16k (11 easy + 5k @ 6:20 hold)
- cali_fullbody: 9/26 #6 delta (B2 3x7, side plank 2x20s)
- CLAUDE.md: sub-3:00 stretch closed, addendum updated

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -29260,22 +29260,45 @@
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="A26" s="35" t="n"/>
+      <c r="A26" s="35" t="n">
+        <v>46292</v>
+      </c>
       <c r="B26" s="16">
         <f>IF(A26="","",IFERROR(INT((A26-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C26" s="27" t="n"/>
-      <c r="D26" s="36" t="n"/>
+      <c r="C26" s="27" t="n">
+        <v>13.01</v>
+      </c>
+      <c r="D26" s="36" t="n">
+        <v>98.92</v>
+      </c>
       <c r="E26" s="16">
         <f>IF(OR(C26="",D26=""),"",TEXT(D26/C26/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F26" s="16" t="n"/>
-      <c r="G26" s="16" t="n"/>
-      <c r="H26" s="16" t="n"/>
-      <c r="I26" s="16" t="n"/>
-      <c r="J26" s="20" t="n"/>
+      <c r="F26" s="16" t="n">
+        <v>153</v>
+      </c>
+      <c r="G26" s="16" t="n">
+        <v>179</v>
+      </c>
+      <c r="H26" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I26" s="16" t="inlineStr">
+        <is>
+          <t>Long</t>
+        </is>
+      </c>
+      <c r="J26" s="20" t="inlineStr">
+        <is>
+          <t>Wk D Sun - LONG 13 k, PM 15:43 (moved from AM). Moving 1:38:55, elapsed 1:46:38 (7.7 min stopped, 4.5 min at ~1.3 k). Gate 3 (legs 1 AM): 10 easy + 3 @ 6:20. Easy 10 k 8:03/km @ HR ~148, cadence ~164 (2 under floor). OPENING MISSED: km1-2 6:45/6:58 vs 7:50; km 3-9 8:15-8:36 under HR cap. Final 3 k 6:19 @171 / 6:06 @169 / 5:54 @171 = 6:06 avg @ HR 170, max 179 - kicked, not held; HR&gt;172 rule not obeyed. Race-pace HR on fatigue ~171 (model said 163-168). Easy HR ~149 @ 8:24 vs 145 @ 7:56 (9/21) - Tue 9/29 drift check. Fuel 80 g. RPE 6. SHIN CLEAN #36. Quad/calf post 3. Wk D closed 4/4 runs, 32 km. Strava 20353804584.</t>
+        </is>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="37" t="n"/>
@@ -32774,18 +32797,28 @@
       </c>
     </row>
     <row r="53" ht="18" customHeight="1">
-      <c r="A53" s="37" t="n"/>
+      <c r="A53" s="37" t="n">
+        <v>46292</v>
+      </c>
       <c r="B53" s="22">
         <f>IF(A53="","",IFERROR(INT((A53-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C53" s="38" t="n"/>
-      <c r="D53" s="38" t="n"/>
+      <c r="C53" s="38" t="n">
+        <v>76</v>
+      </c>
+      <c r="D53" s="38" t="n">
+        <v>9</v>
+      </c>
       <c r="E53" s="38" t="n"/>
       <c r="F53" s="38" t="n"/>
       <c r="G53" s="38" t="n"/>
       <c r="H53" s="38" t="n"/>
-      <c r="I53" s="26" t="n"/>
+      <c r="I53" s="26" t="inlineStr">
+        <is>
+          <t>Wk D Sun - LONG 13 k (see Running Log 9/27). AM: sleep 9:00 (00:00-09:00) q10, RHR 45 (-1), mot 10/energy 10/stress 2, DOMS chest/back/shldr/arm 2 (cali #6), quad/ham/glute/calf 1, shin CLEAN #35. BW 76.00 (-0.70 d/d). 5-reading avg 76.64 (76.40/77.05/77.05/76.70/76.00) - no kcal change, stop overshoot. PM: 13 k done, kcal 2800 (+100 vs ~2700), protein 180, creatine Y, bike 0, shin CLEAN #36, quad/calf post 3.</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Mon 9/28 cali #7 — 26/26, D2 gate cleared, tib slow ecc 20/20/14, shin #38; xlsx synced
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -20580,17 +20580,33 @@
       <c r="K453" s="26" t="n"/>
     </row>
     <row r="454" ht="18" customHeight="1">
-      <c r="A454" s="35" t="n"/>
+      <c r="A454" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B454" s="16">
         <f>IF(A454="","",IFERROR(INT((A454-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C454" s="16" t="n"/>
-      <c r="D454" s="17" t="n"/>
-      <c r="E454" s="16" t="n"/>
-      <c r="F454" s="16" t="n"/>
+      <c r="C454" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D454" s="17" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E454" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F454" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="G454" s="36" t="n"/>
-      <c r="H454" s="16" t="n"/>
+      <c r="H454" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I454" s="19">
         <f>IF(OR(F454="",G454=""),"",F454*G454)</f>
         <v/>
@@ -20599,20 +20615,40 @@
         <f>IF(OR(F454="",G454=""),"",ROUND(G454*(1+F454/30),1))</f>
         <v/>
       </c>
-      <c r="K454" s="20" t="n"/>
+      <c r="K454" s="20" t="inlineStr">
+        <is>
+          <t>Cali #7 FULL BODY (Mon, day after 13 k long), setting 3. S4 8-&gt;7 vs 9/26. S2 8 -&gt; HOLD 4x10.</t>
+        </is>
+      </c>
     </row>
     <row r="455" ht="18" customHeight="1">
-      <c r="A455" s="37" t="n"/>
+      <c r="A455" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B455" s="22">
         <f>IF(A455="","",IFERROR(INT((A455-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C455" s="22" t="n"/>
-      <c r="D455" s="23" t="n"/>
-      <c r="E455" s="22" t="n"/>
-      <c r="F455" s="22" t="n"/>
+      <c r="C455" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D455" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E455" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F455" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="G455" s="38" t="n"/>
-      <c r="H455" s="22" t="n"/>
+      <c r="H455" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I455" s="25">
         <f>IF(OR(F455="",G455=""),"",F455*G455)</f>
         <v/>
@@ -20624,17 +20660,33 @@
       <c r="K455" s="26" t="n"/>
     </row>
     <row r="456" ht="18" customHeight="1">
-      <c r="A456" s="35" t="n"/>
+      <c r="A456" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B456" s="16">
         <f>IF(A456="","",IFERROR(INT((A456-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C456" s="16" t="n"/>
-      <c r="D456" s="17" t="n"/>
-      <c r="E456" s="16" t="n"/>
-      <c r="F456" s="16" t="n"/>
+      <c r="C456" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D456" s="17" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E456" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F456" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="G456" s="36" t="n"/>
-      <c r="H456" s="16" t="n"/>
+      <c r="H456" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I456" s="19">
         <f>IF(OR(F456="",G456=""),"",F456*G456)</f>
         <v/>
@@ -20646,17 +20698,33 @@
       <c r="K456" s="20" t="n"/>
     </row>
     <row r="457" ht="18" customHeight="1">
-      <c r="A457" s="37" t="n"/>
+      <c r="A457" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B457" s="22">
         <f>IF(A457="","",IFERROR(INT((A457-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C457" s="22" t="n"/>
-      <c r="D457" s="23" t="n"/>
-      <c r="E457" s="22" t="n"/>
-      <c r="F457" s="22" t="n"/>
+      <c r="C457" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D457" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (incline)</t>
+        </is>
+      </c>
+      <c r="E457" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F457" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="G457" s="38" t="n"/>
-      <c r="H457" s="22" t="n"/>
+      <c r="H457" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I457" s="25">
         <f>IF(OR(F457="",G457=""),"",F457*G457)</f>
         <v/>
@@ -20668,17 +20736,33 @@
       <c r="K457" s="26" t="n"/>
     </row>
     <row r="458" ht="18" customHeight="1">
-      <c r="A458" s="35" t="n"/>
+      <c r="A458" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B458" s="16">
         <f>IF(A458="","",IFERROR(INT((A458-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C458" s="16" t="n"/>
-      <c r="D458" s="17" t="n"/>
-      <c r="E458" s="16" t="n"/>
-      <c r="F458" s="16" t="n"/>
+      <c r="C458" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D458" s="17" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E458" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F458" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="G458" s="36" t="n"/>
-      <c r="H458" s="16" t="n"/>
+      <c r="H458" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I458" s="19">
         <f>IF(OR(F458="",G458=""),"",F458*G458)</f>
         <v/>
@@ -20687,20 +20771,40 @@
         <f>IF(OR(F458="",G458=""),"",ROUND(G458*(1+F458/30),1))</f>
         <v/>
       </c>
-      <c r="K458" s="20" t="n"/>
+      <c r="K458" s="20" t="inlineStr">
+        <is>
+          <t>Setting 3, 8-rep HARD STOP held. S1 8 -&gt; hold 4x8 cap.</t>
+        </is>
+      </c>
     </row>
     <row r="459" ht="18" customHeight="1">
-      <c r="A459" s="37" t="n"/>
+      <c r="A459" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B459" s="22">
         <f>IF(A459="","",IFERROR(INT((A459-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C459" s="22" t="n"/>
-      <c r="D459" s="23" t="n"/>
-      <c r="E459" s="22" t="n"/>
-      <c r="F459" s="22" t="n"/>
+      <c r="C459" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D459" s="23" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E459" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F459" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="G459" s="38" t="n"/>
-      <c r="H459" s="22" t="n"/>
+      <c r="H459" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I459" s="25">
         <f>IF(OR(F459="",G459=""),"",F459*G459)</f>
         <v/>
@@ -20712,17 +20816,33 @@
       <c r="K459" s="26" t="n"/>
     </row>
     <row r="460" ht="18" customHeight="1">
-      <c r="A460" s="35" t="n"/>
+      <c r="A460" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B460" s="16">
         <f>IF(A460="","",IFERROR(INT((A460-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C460" s="16" t="n"/>
-      <c r="D460" s="17" t="n"/>
-      <c r="E460" s="16" t="n"/>
-      <c r="F460" s="16" t="n"/>
+      <c r="C460" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D460" s="17" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E460" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F460" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="G460" s="36" t="n"/>
-      <c r="H460" s="16" t="n"/>
+      <c r="H460" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I460" s="19">
         <f>IF(OR(F460="",G460=""),"",F460*G460)</f>
         <v/>
@@ -20734,17 +20854,33 @@
       <c r="K460" s="20" t="n"/>
     </row>
     <row r="461" ht="18" customHeight="1">
-      <c r="A461" s="37" t="n"/>
+      <c r="A461" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B461" s="22">
         <f>IF(A461="","",IFERROR(INT((A461-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C461" s="22" t="n"/>
-      <c r="D461" s="23" t="n"/>
-      <c r="E461" s="22" t="n"/>
-      <c r="F461" s="22" t="n"/>
+      <c r="C461" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D461" s="23" t="inlineStr">
+        <is>
+          <t>Inverted Row</t>
+        </is>
+      </c>
+      <c r="E461" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F461" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="G461" s="38" t="n"/>
-      <c r="H461" s="22" t="n"/>
+      <c r="H461" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I461" s="25">
         <f>IF(OR(F461="",G461=""),"",F461*G461)</f>
         <v/>
@@ -20756,17 +20892,33 @@
       <c r="K461" s="26" t="n"/>
     </row>
     <row r="462" ht="18" customHeight="1">
-      <c r="A462" s="35" t="n"/>
+      <c r="A462" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B462" s="16">
         <f>IF(A462="","",IFERROR(INT((A462-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C462" s="16" t="n"/>
-      <c r="D462" s="17" t="n"/>
-      <c r="E462" s="16" t="n"/>
-      <c r="F462" s="16" t="n"/>
+      <c r="C462" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D462" s="17" t="inlineStr">
+        <is>
+          <t>Pull-up (negatives)</t>
+        </is>
+      </c>
+      <c r="E462" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F462" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="G462" s="36" t="n"/>
-      <c r="H462" s="16" t="n"/>
+      <c r="H462" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I462" s="19">
         <f>IF(OR(F462="",G462=""),"",F462*G462)</f>
         <v/>
@@ -20775,20 +20927,40 @@
         <f>IF(OR(F462="",G462=""),"",ROUND(G462*(1+F462/30),1))</f>
         <v/>
       </c>
-      <c r="K462" s="20" t="n"/>
+      <c r="K462" s="20" t="inlineStr">
+        <is>
+          <t>S3 RPE 10 over &lt;=8 cap (3rd session w/ set &gt;=9). Hold 3x5.</t>
+        </is>
+      </c>
     </row>
     <row r="463" ht="18" customHeight="1">
-      <c r="A463" s="37" t="n"/>
+      <c r="A463" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B463" s="22">
         <f>IF(A463="","",IFERROR(INT((A463-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C463" s="22" t="n"/>
-      <c r="D463" s="23" t="n"/>
-      <c r="E463" s="22" t="n"/>
-      <c r="F463" s="22" t="n"/>
+      <c r="C463" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D463" s="23" t="inlineStr">
+        <is>
+          <t>Pull-up (negatives)</t>
+        </is>
+      </c>
+      <c r="E463" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F463" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="G463" s="38" t="n"/>
-      <c r="H463" s="22" t="n"/>
+      <c r="H463" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I463" s="25">
         <f>IF(OR(F463="",G463=""),"",F463*G463)</f>
         <v/>
@@ -20800,17 +20972,33 @@
       <c r="K463" s="26" t="n"/>
     </row>
     <row r="464" ht="18" customHeight="1">
-      <c r="A464" s="35" t="n"/>
+      <c r="A464" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B464" s="16">
         <f>IF(A464="","",IFERROR(INT((A464-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C464" s="16" t="n"/>
-      <c r="D464" s="17" t="n"/>
-      <c r="E464" s="16" t="n"/>
-      <c r="F464" s="16" t="n"/>
+      <c r="C464" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D464" s="17" t="inlineStr">
+        <is>
+          <t>Pull-up (negatives)</t>
+        </is>
+      </c>
+      <c r="E464" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F464" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="G464" s="36" t="n"/>
-      <c r="H464" s="16" t="n"/>
+      <c r="H464" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="I464" s="19">
         <f>IF(OR(F464="",G464=""),"",F464*G464)</f>
         <v/>
@@ -20822,17 +21010,33 @@
       <c r="K464" s="20" t="n"/>
     </row>
     <row r="465" ht="18" customHeight="1">
-      <c r="A465" s="37" t="n"/>
+      <c r="A465" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B465" s="22">
         <f>IF(A465="","",IFERROR(INT((A465-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C465" s="22" t="n"/>
-      <c r="D465" s="23" t="n"/>
-      <c r="E465" s="22" t="n"/>
-      <c r="F465" s="22" t="n"/>
+      <c r="C465" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D465" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (2nd block, incline)</t>
+        </is>
+      </c>
+      <c r="E465" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F465" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="G465" s="38" t="n"/>
-      <c r="H465" s="22" t="n"/>
+      <c r="H465" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I465" s="25">
         <f>IF(OR(F465="",G465=""),"",F465*G465)</f>
         <v/>
@@ -20841,20 +21045,40 @@
         <f>IF(OR(F465="",G465=""),"",ROUND(G465*(1+F465/30),1))</f>
         <v/>
       </c>
-      <c r="K465" s="26" t="n"/>
+      <c r="K465" s="26" t="inlineStr">
+        <is>
+          <t>Setting 3, first session at 7 reps. Hold 3x7.</t>
+        </is>
+      </c>
     </row>
     <row r="466" ht="18" customHeight="1">
-      <c r="A466" s="35" t="n"/>
+      <c r="A466" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B466" s="16">
         <f>IF(A466="","",IFERROR(INT((A466-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C466" s="16" t="n"/>
-      <c r="D466" s="17" t="n"/>
-      <c r="E466" s="16" t="n"/>
-      <c r="F466" s="16" t="n"/>
+      <c r="C466" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D466" s="17" t="inlineStr">
+        <is>
+          <t>Push-up (2nd block, incline)</t>
+        </is>
+      </c>
+      <c r="E466" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F466" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="G466" s="36" t="n"/>
-      <c r="H466" s="16" t="n"/>
+      <c r="H466" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I466" s="19">
         <f>IF(OR(F466="",G466=""),"",F466*G466)</f>
         <v/>
@@ -20866,17 +21090,33 @@
       <c r="K466" s="20" t="n"/>
     </row>
     <row r="467" ht="18" customHeight="1">
-      <c r="A467" s="37" t="n"/>
+      <c r="A467" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B467" s="22">
         <f>IF(A467="","",IFERROR(INT((A467-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C467" s="22" t="n"/>
-      <c r="D467" s="23" t="n"/>
-      <c r="E467" s="22" t="n"/>
-      <c r="F467" s="22" t="n"/>
+      <c r="C467" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D467" s="23" t="inlineStr">
+        <is>
+          <t>Push-up (2nd block, incline)</t>
+        </is>
+      </c>
+      <c r="E467" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F467" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="G467" s="38" t="n"/>
-      <c r="H467" s="22" t="n"/>
+      <c r="H467" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I467" s="25">
         <f>IF(OR(F467="",G467=""),"",F467*G467)</f>
         <v/>
@@ -20888,17 +21128,33 @@
       <c r="K467" s="26" t="n"/>
     </row>
     <row r="468" ht="18" customHeight="1">
-      <c r="A468" s="35" t="n"/>
+      <c r="A468" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B468" s="16">
         <f>IF(A468="","",IFERROR(INT((A468-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C468" s="16" t="n"/>
-      <c r="D468" s="17" t="n"/>
-      <c r="E468" s="16" t="n"/>
-      <c r="F468" s="16" t="n"/>
+      <c r="C468" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D468" s="17" t="inlineStr">
+        <is>
+          <t>Bulgarian Split Squat (BW)</t>
+        </is>
+      </c>
+      <c r="E468" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F468" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="G468" s="36" t="n"/>
-      <c r="H468" s="16" t="n"/>
+      <c r="H468" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I468" s="19">
         <f>IF(OR(F468="",G468=""),"",F468*G468)</f>
         <v/>
@@ -20907,20 +21163,40 @@
         <f>IF(OR(F468="",G468=""),"",ROUND(G468*(1+F468/30),1))</f>
         <v/>
       </c>
-      <c r="K468" s="20" t="n"/>
+      <c r="K468" s="20" t="inlineStr">
+        <is>
+          <t>reps PER LEG. Gate 1 (calf 2) -&gt; 2x8 RPE 6 cap; S2 stopped at cap.</t>
+        </is>
+      </c>
     </row>
     <row r="469" ht="18" customHeight="1">
-      <c r="A469" s="37" t="n"/>
+      <c r="A469" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B469" s="22">
         <f>IF(A469="","",IFERROR(INT((A469-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C469" s="22" t="n"/>
-      <c r="D469" s="23" t="n"/>
-      <c r="E469" s="22" t="n"/>
-      <c r="F469" s="22" t="n"/>
+      <c r="C469" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D469" s="23" t="inlineStr">
+        <is>
+          <t>Bulgarian Split Squat (BW)</t>
+        </is>
+      </c>
+      <c r="E469" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F469" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G469" s="38" t="n"/>
-      <c r="H469" s="22" t="n"/>
+      <c r="H469" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I469" s="25">
         <f>IF(OR(F469="",G469=""),"",F469*G469)</f>
         <v/>
@@ -20932,17 +21208,33 @@
       <c r="K469" s="26" t="n"/>
     </row>
     <row r="470" ht="18" customHeight="1">
-      <c r="A470" s="35" t="n"/>
+      <c r="A470" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B470" s="16">
         <f>IF(A470="","",IFERROR(INT((A470-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C470" s="16" t="n"/>
-      <c r="D470" s="17" t="n"/>
-      <c r="E470" s="16" t="n"/>
-      <c r="F470" s="16" t="n"/>
+      <c r="C470" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D470" s="17" t="inlineStr">
+        <is>
+          <t>Single-Leg RDL (BW)</t>
+        </is>
+      </c>
+      <c r="E470" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F470" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="G470" s="36" t="n"/>
-      <c r="H470" s="16" t="n"/>
+      <c r="H470" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I470" s="19">
         <f>IF(OR(F470="",G470=""),"",F470*G470)</f>
         <v/>
@@ -20951,20 +21243,40 @@
         <f>IF(OR(F470="",G470=""),"",ROUND(G470*(1+F470/30),1))</f>
         <v/>
       </c>
-      <c r="K470" s="20" t="n"/>
+      <c r="K470" s="20" t="inlineStr">
+        <is>
+          <t>reps PER LEG. RPE 6 cap on ham/glute DOMS 2; S2 stopped at cap.</t>
+        </is>
+      </c>
     </row>
     <row r="471" ht="18" customHeight="1">
-      <c r="A471" s="37" t="n"/>
+      <c r="A471" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B471" s="22">
         <f>IF(A471="","",IFERROR(INT((A471-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C471" s="22" t="n"/>
-      <c r="D471" s="23" t="n"/>
-      <c r="E471" s="22" t="n"/>
-      <c r="F471" s="22" t="n"/>
+      <c r="C471" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D471" s="23" t="inlineStr">
+        <is>
+          <t>Single-Leg RDL (BW)</t>
+        </is>
+      </c>
+      <c r="E471" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F471" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G471" s="38" t="n"/>
-      <c r="H471" s="22" t="n"/>
+      <c r="H471" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I471" s="25">
         <f>IF(OR(F471="",G471=""),"",F471*G471)</f>
         <v/>
@@ -20976,17 +21288,33 @@
       <c r="K471" s="26" t="n"/>
     </row>
     <row r="472" ht="18" customHeight="1">
-      <c r="A472" s="35" t="n"/>
+      <c r="A472" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B472" s="16">
         <f>IF(A472="","",IFERROR(INT((A472-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C472" s="16" t="n"/>
-      <c r="D472" s="17" t="n"/>
-      <c r="E472" s="16" t="n"/>
-      <c r="F472" s="16" t="n"/>
+      <c r="C472" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D472" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise (slow ecc, BW)</t>
+        </is>
+      </c>
+      <c r="E472" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F472" s="16" t="n">
+        <v>20</v>
+      </c>
       <c r="G472" s="36" t="n"/>
-      <c r="H472" s="16" t="n"/>
+      <c r="H472" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I472" s="19">
         <f>IF(OR(F472="",G472=""),"",F472*G472)</f>
         <v/>
@@ -20995,20 +21323,40 @@
         <f>IF(OR(F472="",G472=""),"",ROUND(G472*(1+F472/30),1))</f>
         <v/>
       </c>
-      <c r="K472" s="20" t="n"/>
+      <c r="K472" s="20" t="inlineStr">
+        <is>
+          <t>SLOW ECC 3 s. Jumped 15-&gt;20 (9/22 15s @&lt;=5.5); S3 failed 14 @10. Next slow ecc 3x18.</t>
+        </is>
+      </c>
     </row>
     <row r="473" ht="18" customHeight="1">
-      <c r="A473" s="37" t="n"/>
+      <c r="A473" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B473" s="22">
         <f>IF(A473="","",IFERROR(INT((A473-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C473" s="22" t="n"/>
-      <c r="D473" s="23" t="n"/>
-      <c r="E473" s="22" t="n"/>
-      <c r="F473" s="22" t="n"/>
+      <c r="C473" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D473" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise (slow ecc, BW)</t>
+        </is>
+      </c>
+      <c r="E473" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F473" s="22" t="n">
+        <v>20</v>
+      </c>
       <c r="G473" s="38" t="n"/>
-      <c r="H473" s="22" t="n"/>
+      <c r="H473" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I473" s="25">
         <f>IF(OR(F473="",G473=""),"",F473*G473)</f>
         <v/>
@@ -21020,17 +21368,33 @@
       <c r="K473" s="26" t="n"/>
     </row>
     <row r="474" ht="18" customHeight="1">
-      <c r="A474" s="35" t="n"/>
+      <c r="A474" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B474" s="16">
         <f>IF(A474="","",IFERROR(INT((A474-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C474" s="16" t="n"/>
-      <c r="D474" s="17" t="n"/>
-      <c r="E474" s="16" t="n"/>
-      <c r="F474" s="16" t="n"/>
+      <c r="C474" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D474" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise (slow ecc, BW)</t>
+        </is>
+      </c>
+      <c r="E474" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F474" s="16" t="n">
+        <v>14</v>
+      </c>
       <c r="G474" s="36" t="n"/>
-      <c r="H474" s="16" t="n"/>
+      <c r="H474" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="I474" s="19">
         <f>IF(OR(F474="",G474=""),"",F474*G474)</f>
         <v/>
@@ -21042,17 +21406,33 @@
       <c r="K474" s="20" t="n"/>
     </row>
     <row r="475" ht="18" customHeight="1">
-      <c r="A475" s="37" t="n"/>
+      <c r="A475" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B475" s="22">
         <f>IF(A475="","",IFERROR(INT((A475-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C475" s="22" t="n"/>
-      <c r="D475" s="23" t="n"/>
-      <c r="E475" s="22" t="n"/>
-      <c r="F475" s="22" t="n"/>
+      <c r="C475" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D475" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E475" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F475" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G475" s="38" t="n"/>
-      <c r="H475" s="22" t="n"/>
+      <c r="H475" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I475" s="25">
         <f>IF(OR(F475="",G475=""),"",F475*G475)</f>
         <v/>
@@ -21061,20 +21441,40 @@
         <f>IF(OR(F475="",G475=""),"",ROUND(G475*(1+F475/30),1))</f>
         <v/>
       </c>
-      <c r="K475" s="26" t="n"/>
+      <c r="K475" s="26" t="inlineStr">
+        <is>
+          <t>All top of range &amp; &lt;=7 -&gt; GATE CLEARED, 3x7.</t>
+        </is>
+      </c>
     </row>
     <row r="476" ht="18" customHeight="1">
-      <c r="A476" s="35" t="n"/>
+      <c r="A476" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B476" s="16">
         <f>IF(A476="","",IFERROR(INT((A476-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C476" s="16" t="n"/>
-      <c r="D476" s="17" t="n"/>
-      <c r="E476" s="16" t="n"/>
-      <c r="F476" s="16" t="n"/>
+      <c r="C476" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D476" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E476" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F476" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="G476" s="36" t="n"/>
-      <c r="H476" s="16" t="n"/>
+      <c r="H476" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I476" s="19">
         <f>IF(OR(F476="",G476=""),"",F476*G476)</f>
         <v/>
@@ -21086,17 +21486,33 @@
       <c r="K476" s="20" t="n"/>
     </row>
     <row r="477" ht="18" customHeight="1">
-      <c r="A477" s="37" t="n"/>
+      <c r="A477" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B477" s="22">
         <f>IF(A477="","",IFERROR(INT((A477-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C477" s="22" t="n"/>
-      <c r="D477" s="23" t="n"/>
-      <c r="E477" s="22" t="n"/>
-      <c r="F477" s="22" t="n"/>
+      <c r="C477" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D477" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E477" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F477" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="G477" s="38" t="n"/>
-      <c r="H477" s="22" t="n"/>
+      <c r="H477" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I477" s="25">
         <f>IF(OR(F477="",G477=""),"",F477*G477)</f>
         <v/>
@@ -21108,17 +21524,33 @@
       <c r="K477" s="26" t="n"/>
     </row>
     <row r="478" ht="18" customHeight="1">
-      <c r="A478" s="35" t="n"/>
+      <c r="A478" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B478" s="16">
         <f>IF(A478="","",IFERROR(INT((A478-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C478" s="16" t="n"/>
-      <c r="D478" s="17" t="n"/>
-      <c r="E478" s="16" t="n"/>
-      <c r="F478" s="16" t="n"/>
+      <c r="C478" s="16" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D478" s="17" t="inlineStr">
+        <is>
+          <t>Side Plank (BW)</t>
+        </is>
+      </c>
+      <c r="E478" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F478" s="16" t="n">
+        <v>20</v>
+      </c>
       <c r="G478" s="36" t="n"/>
-      <c r="H478" s="16" t="n"/>
+      <c r="H478" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I478" s="19">
         <f>IF(OR(F478="",G478=""),"",F478*G478)</f>
         <v/>
@@ -21127,20 +21559,40 @@
         <f>IF(OR(F478="",G478=""),"",ROUND(G478*(1+F478/30),1))</f>
         <v/>
       </c>
-      <c r="K478" s="20" t="n"/>
+      <c r="K478" s="20" t="inlineStr">
+        <is>
+          <t>reps col = seconds PER SIDE. 20 s regression landed. Hold 2x20 s.</t>
+        </is>
+      </c>
     </row>
     <row r="479" ht="18" customHeight="1">
-      <c r="A479" s="37" t="n"/>
+      <c r="A479" s="37" t="n">
+        <v>46293</v>
+      </c>
       <c r="B479" s="22">
         <f>IF(A479="","",IFERROR(INT((A479-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C479" s="22" t="n"/>
-      <c r="D479" s="23" t="n"/>
-      <c r="E479" s="22" t="n"/>
-      <c r="F479" s="22" t="n"/>
+      <c r="C479" s="22" t="inlineStr">
+        <is>
+          <t>Cali Full Body</t>
+        </is>
+      </c>
+      <c r="D479" s="23" t="inlineStr">
+        <is>
+          <t>Side Plank (BW)</t>
+        </is>
+      </c>
+      <c r="E479" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F479" s="22" t="n">
+        <v>20</v>
+      </c>
       <c r="G479" s="38" t="n"/>
-      <c r="H479" s="22" t="n"/>
+      <c r="H479" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I479" s="25">
         <f>IF(OR(F479="",G479=""),"",F479*G479)</f>
         <v/>
@@ -32821,18 +33273,28 @@
       </c>
     </row>
     <row r="54" ht="18" customHeight="1">
-      <c r="A54" s="35" t="n"/>
+      <c r="A54" s="35" t="n">
+        <v>46293</v>
+      </c>
       <c r="B54" s="16">
         <f>IF(A54="","",IFERROR(INT((A54-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C54" s="36" t="n"/>
-      <c r="D54" s="36" t="n"/>
+      <c r="C54" s="36" t="n">
+        <v>76.45</v>
+      </c>
+      <c r="D54" s="36" t="n">
+        <v>8.33</v>
+      </c>
       <c r="E54" s="36" t="n"/>
       <c r="F54" s="36" t="n"/>
       <c r="G54" s="36" t="n"/>
       <c r="H54" s="36" t="n"/>
-      <c r="I54" s="20" t="n"/>
+      <c r="I54" s="20" t="inlineStr">
+        <is>
+          <t>Wk E Mon - CALI #7 FULL BODY, legs 2x8 (see Lifting Log 9/28). AM: sleep 8:20 (00:05-08:25) q10, RHR 45 (-1), mot 10/energy 10/stress 2, DOMS upper 1/1/1/1, quad 1 / ham 2 / glute 2 / calf 2, shin CLEAN #37. BW 76.45, 6-reading avg 76.61 - flat, no kcal change. PM: 26/26 sets 50 min avg RPE 7.27, 2 RPE-10 sets (B1 S3, tib S3), bike 0, kcal 2541 (+141 vs no-bike 2400), protein 174, creatine Y, shin CLEAN #38.</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Tue 9/29 6k — 6:57 @ HR 142, drift check void but no drift, shin #40; xlsx synced
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -29753,22 +29753,45 @@
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="A27" s="37" t="n"/>
+      <c r="A27" s="37" t="n">
+        <v>46294</v>
+      </c>
       <c r="B27" s="22">
         <f>IF(A27="","",IFERROR(INT((A27-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C27" s="28" t="n"/>
-      <c r="D27" s="38" t="n"/>
+      <c r="C27" s="28" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" s="38" t="n">
+        <v>41.77</v>
+      </c>
       <c r="E27" s="22">
         <f>IF(OR(C27="",D27=""),"",TEXT(D27/C27/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F27" s="22" t="n"/>
-      <c r="G27" s="22" t="n"/>
-      <c r="H27" s="22" t="n"/>
-      <c r="I27" s="22" t="n"/>
-      <c r="J27" s="26" t="n"/>
+      <c r="F27" s="22" t="n">
+        <v>142</v>
+      </c>
+      <c r="G27" s="22" t="n">
+        <v>155</v>
+      </c>
+      <c r="H27" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="I27" s="22" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J27" s="26" t="inlineStr">
+        <is>
+          <t>Wk E Tue - EASY 6 k DRIFT CHECK, PM 15:31. Moving 41:46 (6:57/km), elapsed 46:37 (4.3 min stop ~0.7 k). Splits 6:43@127 / 6:42@146 / 6:45@148 / 7:13@144 / 7:27@144 / 6:55@145. Km 2-6 = 7:00/km @ HR 145.5 vs 145 @ 7:56 (9/21) -&gt; check technically void (pace under 7:40) but NO DRIFT: same HR 56 s/km faster. Thu run stays. Opening missed 4th straight (6:43 vs 7:50). Cadence 164 (laps 165/166/166/164/163 - fades late, 2 under floor 2nd run running). RPE 4, 0 walk breaks. SHIN CLEAN #40. Quad/calf post 2. Strava 20378851247.</t>
+        </is>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="35" t="n"/>
@@ -33297,18 +33320,28 @@
       </c>
     </row>
     <row r="55" ht="18" customHeight="1">
-      <c r="A55" s="37" t="n"/>
+      <c r="A55" s="37" t="n">
+        <v>46294</v>
+      </c>
       <c r="B55" s="22">
         <f>IF(A55="","",IFERROR(INT((A55-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C55" s="38" t="n"/>
-      <c r="D55" s="38" t="n"/>
+      <c r="C55" s="38" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="D55" s="38" t="n">
+        <v>7.42</v>
+      </c>
       <c r="E55" s="38" t="n"/>
       <c r="F55" s="38" t="n"/>
       <c r="G55" s="38" t="n"/>
       <c r="H55" s="38" t="n"/>
-      <c r="I55" s="26" t="n"/>
+      <c r="I55" s="26" t="inlineStr">
+        <is>
+          <t>Wk E Tue - EASY 6 k (see Running Log 9/29). AM: sleep 7:25 (23:00-06:30) q8, RHR 43 (-2), mot 10/energy 9/stress 2, DOMS chest 2/back 2/shldr 3/arm 2 (cali #7), quad/ham/glute/calf 1, tib-ant 0, shin CLEAN #39. BW 76.60, 7-reading avg 76.61 - flat, no kcal change. PM: 6 k done, bike 0, kcal 2883 (+483 vs no-bike 2400), protein 170, creatine Y, shin CLEAN #40, quad/calf post 2.</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="18" customHeight="1">
       <c r="A56" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Mon 10/5 Gym #1 done (24 WS, 3595 kg, RPE 6.92); bumps for Fri upper; xlsx synced
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -21604,17 +21604,35 @@
       <c r="K479" s="26" t="n"/>
     </row>
     <row r="480" ht="18" customHeight="1">
-      <c r="A480" s="35" t="n"/>
+      <c r="A480" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B480" s="16">
         <f>IF(A480="","",IFERROR(INT((A480-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C480" s="16" t="n"/>
-      <c r="D480" s="17" t="n"/>
-      <c r="E480" s="16" t="n"/>
-      <c r="F480" s="16" t="n"/>
-      <c r="G480" s="36" t="n"/>
-      <c r="H480" s="16" t="n"/>
+      <c r="C480" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D480" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E480" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F480" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G480" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="H480" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I480" s="19">
         <f>IF(OR(F480="",G480=""),"",F480*G480)</f>
         <v/>
@@ -21623,20 +21641,42 @@
         <f>IF(OR(F480="",G480=""),"",ROUND(G480*(1+F480/30),1))</f>
         <v/>
       </c>
-      <c r="K480" s="20" t="n"/>
+      <c r="K480" s="20" t="inlineStr">
+        <is>
+          <t>Gym #1, first barbell since Jun. Seeded 32.5, ran 25. Hold 25.</t>
+        </is>
+      </c>
     </row>
     <row r="481" ht="18" customHeight="1">
-      <c r="A481" s="37" t="n"/>
+      <c r="A481" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B481" s="22">
         <f>IF(A481="","",IFERROR(INT((A481-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C481" s="22" t="n"/>
-      <c r="D481" s="23" t="n"/>
-      <c r="E481" s="22" t="n"/>
-      <c r="F481" s="22" t="n"/>
-      <c r="G481" s="38" t="n"/>
-      <c r="H481" s="22" t="n"/>
+      <c r="C481" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D481" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E481" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F481" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G481" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H481" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I481" s="25">
         <f>IF(OR(F481="",G481=""),"",F481*G481)</f>
         <v/>
@@ -21648,17 +21688,35 @@
       <c r="K481" s="26" t="n"/>
     </row>
     <row r="482" ht="18" customHeight="1">
-      <c r="A482" s="35" t="n"/>
+      <c r="A482" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B482" s="16">
         <f>IF(A482="","",IFERROR(INT((A482-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C482" s="16" t="n"/>
-      <c r="D482" s="17" t="n"/>
-      <c r="E482" s="16" t="n"/>
-      <c r="F482" s="16" t="n"/>
-      <c r="G482" s="36" t="n"/>
-      <c r="H482" s="16" t="n"/>
+      <c r="C482" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D482" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E482" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F482" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G482" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="H482" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I482" s="19">
         <f>IF(OR(F482="",G482=""),"",F482*G482)</f>
         <v/>
@@ -21670,17 +21728,35 @@
       <c r="K482" s="20" t="n"/>
     </row>
     <row r="483" ht="18" customHeight="1">
-      <c r="A483" s="37" t="n"/>
+      <c r="A483" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B483" s="22">
         <f>IF(A483="","",IFERROR(INT((A483-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C483" s="22" t="n"/>
-      <c r="D483" s="23" t="n"/>
-      <c r="E483" s="22" t="n"/>
-      <c r="F483" s="22" t="n"/>
-      <c r="G483" s="38" t="n"/>
-      <c r="H483" s="22" t="n"/>
+      <c r="C483" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D483" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E483" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F483" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G483" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H483" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I483" s="25">
         <f>IF(OR(F483="",G483=""),"",F483*G483)</f>
         <v/>
@@ -21692,17 +21768,35 @@
       <c r="K483" s="26" t="n"/>
     </row>
     <row r="484" ht="18" customHeight="1">
-      <c r="A484" s="35" t="n"/>
+      <c r="A484" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B484" s="16">
         <f>IF(A484="","",IFERROR(INT((A484-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C484" s="16" t="n"/>
-      <c r="D484" s="17" t="n"/>
-      <c r="E484" s="16" t="n"/>
-      <c r="F484" s="16" t="n"/>
-      <c r="G484" s="36" t="n"/>
-      <c r="H484" s="16" t="n"/>
+      <c r="C484" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D484" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E484" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F484" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G484" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="H484" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I484" s="19">
         <f>IF(OR(F484="",G484=""),"",F484*G484)</f>
         <v/>
@@ -21711,20 +21805,42 @@
         <f>IF(OR(F484="",G484=""),"",ROUND(G484*(1+F484/30),1))</f>
         <v/>
       </c>
-      <c r="K484" s="20" t="n"/>
+      <c r="K484" s="20" t="inlineStr">
+        <is>
+          <t>S4 RPE 8 -&gt; hold 25.</t>
+        </is>
+      </c>
     </row>
     <row r="485" ht="18" customHeight="1">
-      <c r="A485" s="37" t="n"/>
+      <c r="A485" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B485" s="22">
         <f>IF(A485="","",IFERROR(INT((A485-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C485" s="22" t="n"/>
-      <c r="D485" s="23" t="n"/>
-      <c r="E485" s="22" t="n"/>
-      <c r="F485" s="22" t="n"/>
-      <c r="G485" s="38" t="n"/>
-      <c r="H485" s="22" t="n"/>
+      <c r="C485" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D485" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E485" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F485" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G485" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H485" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I485" s="25">
         <f>IF(OR(F485="",G485=""),"",F485*G485)</f>
         <v/>
@@ -21736,17 +21852,35 @@
       <c r="K485" s="26" t="n"/>
     </row>
     <row r="486" ht="18" customHeight="1">
-      <c r="A486" s="35" t="n"/>
+      <c r="A486" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B486" s="16">
         <f>IF(A486="","",IFERROR(INT((A486-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C486" s="16" t="n"/>
-      <c r="D486" s="17" t="n"/>
-      <c r="E486" s="16" t="n"/>
-      <c r="F486" s="16" t="n"/>
-      <c r="G486" s="36" t="n"/>
-      <c r="H486" s="16" t="n"/>
+      <c r="C486" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D486" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E486" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F486" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G486" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="H486" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I486" s="19">
         <f>IF(OR(F486="",G486=""),"",F486*G486)</f>
         <v/>
@@ -21758,17 +21892,35 @@
       <c r="K486" s="20" t="n"/>
     </row>
     <row r="487" ht="18" customHeight="1">
-      <c r="A487" s="37" t="n"/>
+      <c r="A487" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B487" s="22">
         <f>IF(A487="","",IFERROR(INT((A487-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C487" s="22" t="n"/>
-      <c r="D487" s="23" t="n"/>
-      <c r="E487" s="22" t="n"/>
-      <c r="F487" s="22" t="n"/>
-      <c r="G487" s="38" t="n"/>
-      <c r="H487" s="22" t="n"/>
+      <c r="C487" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D487" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E487" s="22" t="n">
+        <v>4</v>
+      </c>
+      <c r="F487" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G487" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H487" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I487" s="25">
         <f>IF(OR(F487="",G487=""),"",F487*G487)</f>
         <v/>
@@ -21780,17 +21932,35 @@
       <c r="K487" s="26" t="n"/>
     </row>
     <row r="488" ht="18" customHeight="1">
-      <c r="A488" s="35" t="n"/>
+      <c r="A488" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B488" s="16">
         <f>IF(A488="","",IFERROR(INT((A488-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C488" s="16" t="n"/>
-      <c r="D488" s="17" t="n"/>
-      <c r="E488" s="16" t="n"/>
-      <c r="F488" s="16" t="n"/>
-      <c r="G488" s="36" t="n"/>
-      <c r="H488" s="16" t="n"/>
+      <c r="C488" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D488" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E488" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F488" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G488" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="H488" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I488" s="19">
         <f>IF(OR(F488="",G488=""),"",F488*G488)</f>
         <v/>
@@ -21799,20 +21969,42 @@
         <f>IF(OR(F488="",G488=""),"",ROUND(G488*(1+F488/30),1))</f>
         <v/>
       </c>
-      <c r="K488" s="20" t="n"/>
+      <c r="K488" s="20" t="inlineStr">
+        <is>
+          <t>per-DB. Gate cleared -&gt; 6/DB.</t>
+        </is>
+      </c>
     </row>
     <row r="489" ht="18" customHeight="1">
-      <c r="A489" s="37" t="n"/>
+      <c r="A489" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B489" s="22">
         <f>IF(A489="","",IFERROR(INT((A489-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C489" s="22" t="n"/>
-      <c r="D489" s="23" t="n"/>
-      <c r="E489" s="22" t="n"/>
-      <c r="F489" s="22" t="n"/>
-      <c r="G489" s="38" t="n"/>
-      <c r="H489" s="22" t="n"/>
+      <c r="C489" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D489" s="23" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E489" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F489" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G489" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="H489" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I489" s="25">
         <f>IF(OR(F489="",G489=""),"",F489*G489)</f>
         <v/>
@@ -21824,17 +22016,35 @@
       <c r="K489" s="26" t="n"/>
     </row>
     <row r="490" ht="18" customHeight="1">
-      <c r="A490" s="35" t="n"/>
+      <c r="A490" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B490" s="16">
         <f>IF(A490="","",IFERROR(INT((A490-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C490" s="16" t="n"/>
-      <c r="D490" s="17" t="n"/>
-      <c r="E490" s="16" t="n"/>
-      <c r="F490" s="16" t="n"/>
-      <c r="G490" s="36" t="n"/>
-      <c r="H490" s="16" t="n"/>
+      <c r="C490" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D490" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E490" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F490" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G490" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="H490" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I490" s="19">
         <f>IF(OR(F490="",G490=""),"",F490*G490)</f>
         <v/>
@@ -21846,17 +22056,35 @@
       <c r="K490" s="20" t="n"/>
     </row>
     <row r="491" ht="18" customHeight="1">
-      <c r="A491" s="37" t="n"/>
+      <c r="A491" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B491" s="22">
         <f>IF(A491="","",IFERROR(INT((A491-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C491" s="22" t="n"/>
-      <c r="D491" s="23" t="n"/>
-      <c r="E491" s="22" t="n"/>
-      <c r="F491" s="22" t="n"/>
-      <c r="G491" s="38" t="n"/>
-      <c r="H491" s="22" t="n"/>
+      <c r="C491" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D491" s="23" t="inlineStr">
+        <is>
+          <t>Barbell Lying Row</t>
+        </is>
+      </c>
+      <c r="E491" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F491" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G491" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="H491" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I491" s="25">
         <f>IF(OR(F491="",G491=""),"",F491*G491)</f>
         <v/>
@@ -21865,20 +22093,42 @@
         <f>IF(OR(F491="",G491=""),"",ROUND(G491*(1+F491/30),1))</f>
         <v/>
       </c>
-      <c r="K491" s="26" t="n"/>
+      <c r="K491" s="26" t="inlineStr">
+        <is>
+          <t>Sub for cable row. Gate cleared -&gt; 32.5.</t>
+        </is>
+      </c>
     </row>
     <row r="492" ht="18" customHeight="1">
-      <c r="A492" s="35" t="n"/>
+      <c r="A492" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B492" s="16">
         <f>IF(A492="","",IFERROR(INT((A492-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C492" s="16" t="n"/>
-      <c r="D492" s="17" t="n"/>
-      <c r="E492" s="16" t="n"/>
-      <c r="F492" s="16" t="n"/>
-      <c r="G492" s="36" t="n"/>
-      <c r="H492" s="16" t="n"/>
+      <c r="C492" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D492" s="17" t="inlineStr">
+        <is>
+          <t>Barbell Lying Row</t>
+        </is>
+      </c>
+      <c r="E492" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F492" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G492" s="36" t="n">
+        <v>30</v>
+      </c>
+      <c r="H492" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I492" s="19">
         <f>IF(OR(F492="",G492=""),"",F492*G492)</f>
         <v/>
@@ -21890,17 +22140,35 @@
       <c r="K492" s="20" t="n"/>
     </row>
     <row r="493" ht="18" customHeight="1">
-      <c r="A493" s="37" t="n"/>
+      <c r="A493" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B493" s="22">
         <f>IF(A493="","",IFERROR(INT((A493-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C493" s="22" t="n"/>
-      <c r="D493" s="23" t="n"/>
-      <c r="E493" s="22" t="n"/>
-      <c r="F493" s="22" t="n"/>
-      <c r="G493" s="38" t="n"/>
-      <c r="H493" s="22" t="n"/>
+      <c r="C493" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D493" s="23" t="inlineStr">
+        <is>
+          <t>Barbell Lying Row</t>
+        </is>
+      </c>
+      <c r="E493" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F493" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G493" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="H493" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I493" s="25">
         <f>IF(OR(F493="",G493=""),"",F493*G493)</f>
         <v/>
@@ -21912,17 +22180,35 @@
       <c r="K493" s="26" t="n"/>
     </row>
     <row r="494" ht="18" customHeight="1">
-      <c r="A494" s="35" t="n"/>
+      <c r="A494" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B494" s="16">
         <f>IF(A494="","",IFERROR(INT((A494-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C494" s="16" t="n"/>
-      <c r="D494" s="17" t="n"/>
-      <c r="E494" s="16" t="n"/>
-      <c r="F494" s="16" t="n"/>
-      <c r="G494" s="36" t="n"/>
-      <c r="H494" s="16" t="n"/>
+      <c r="C494" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D494" s="17" t="inlineStr">
+        <is>
+          <t>Leg Extension</t>
+        </is>
+      </c>
+      <c r="E494" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F494" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G494" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="H494" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="I494" s="19">
         <f>IF(OR(F494="",G494=""),"",F494*G494)</f>
         <v/>
@@ -21931,20 +22217,42 @@
         <f>IF(OR(F494="",G494=""),"",ROUND(G494*(1+F494/30),1))</f>
         <v/>
       </c>
-      <c r="K494" s="20" t="n"/>
+      <c r="K494" s="20" t="inlineStr">
+        <is>
+          <t>Sub for leg press. RPE 6 cap (track Tue). -&gt; 12.5.</t>
+        </is>
+      </c>
     </row>
     <row r="495" ht="18" customHeight="1">
-      <c r="A495" s="37" t="n"/>
+      <c r="A495" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B495" s="22">
         <f>IF(A495="","",IFERROR(INT((A495-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C495" s="22" t="n"/>
-      <c r="D495" s="23" t="n"/>
-      <c r="E495" s="22" t="n"/>
-      <c r="F495" s="22" t="n"/>
-      <c r="G495" s="38" t="n"/>
-      <c r="H495" s="22" t="n"/>
+      <c r="C495" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D495" s="23" t="inlineStr">
+        <is>
+          <t>Leg Extension</t>
+        </is>
+      </c>
+      <c r="E495" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F495" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G495" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="H495" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="I495" s="25">
         <f>IF(OR(F495="",G495=""),"",F495*G495)</f>
         <v/>
@@ -21956,17 +22264,35 @@
       <c r="K495" s="26" t="n"/>
     </row>
     <row r="496" ht="18" customHeight="1">
-      <c r="A496" s="35" t="n"/>
+      <c r="A496" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B496" s="16">
         <f>IF(A496="","",IFERROR(INT((A496-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C496" s="16" t="n"/>
-      <c r="D496" s="17" t="n"/>
-      <c r="E496" s="16" t="n"/>
-      <c r="F496" s="16" t="n"/>
-      <c r="G496" s="36" t="n"/>
-      <c r="H496" s="16" t="n"/>
+      <c r="C496" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D496" s="17" t="inlineStr">
+        <is>
+          <t>Lying Leg Curl</t>
+        </is>
+      </c>
+      <c r="E496" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F496" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G496" s="36" t="n">
+        <v>10</v>
+      </c>
+      <c r="H496" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I496" s="19">
         <f>IF(OR(F496="",G496=""),"",F496*G496)</f>
         <v/>
@@ -21975,20 +22301,42 @@
         <f>IF(OR(F496="",G496=""),"",ROUND(G496*(1+F496/30),1))</f>
         <v/>
       </c>
-      <c r="K496" s="20" t="n"/>
+      <c r="K496" s="20" t="inlineStr">
+        <is>
+          <t>At RPE 6 cap -&gt; hold 10.</t>
+        </is>
+      </c>
     </row>
     <row r="497" ht="18" customHeight="1">
-      <c r="A497" s="37" t="n"/>
+      <c r="A497" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B497" s="22">
         <f>IF(A497="","",IFERROR(INT((A497-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C497" s="22" t="n"/>
-      <c r="D497" s="23" t="n"/>
-      <c r="E497" s="22" t="n"/>
-      <c r="F497" s="22" t="n"/>
-      <c r="G497" s="38" t="n"/>
-      <c r="H497" s="22" t="n"/>
+      <c r="C497" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D497" s="23" t="inlineStr">
+        <is>
+          <t>Lying Leg Curl</t>
+        </is>
+      </c>
+      <c r="E497" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F497" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G497" s="38" t="n">
+        <v>10</v>
+      </c>
+      <c r="H497" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I497" s="25">
         <f>IF(OR(F497="",G497=""),"",F497*G497)</f>
         <v/>
@@ -22000,17 +22348,35 @@
       <c r="K497" s="26" t="n"/>
     </row>
     <row r="498" ht="18" customHeight="1">
-      <c r="A498" s="35" t="n"/>
+      <c r="A498" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B498" s="16">
         <f>IF(A498="","",IFERROR(INT((A498-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C498" s="16" t="n"/>
-      <c r="D498" s="17" t="n"/>
-      <c r="E498" s="16" t="n"/>
-      <c r="F498" s="16" t="n"/>
-      <c r="G498" s="36" t="n"/>
-      <c r="H498" s="16" t="n"/>
+      <c r="C498" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D498" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E498" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F498" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G498" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="H498" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I498" s="19">
         <f>IF(OR(F498="",G498=""),"",F498*G498)</f>
         <v/>
@@ -22019,20 +22385,42 @@
         <f>IF(OR(F498="",G498=""),"",ROUND(G498*(1+F498/30),1))</f>
         <v/>
       </c>
-      <c r="K498" s="20" t="n"/>
+      <c r="K498" s="20" t="inlineStr">
+        <is>
+          <t>Prescribed BW 3x20, ran 5 kg 3x15: reps fell 15/10/8. -&gt; 2.5 kg 3x15.</t>
+        </is>
+      </c>
     </row>
     <row r="499" ht="18" customHeight="1">
-      <c r="A499" s="37" t="n"/>
+      <c r="A499" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B499" s="22">
         <f>IF(A499="","",IFERROR(INT((A499-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C499" s="22" t="n"/>
-      <c r="D499" s="23" t="n"/>
-      <c r="E499" s="22" t="n"/>
-      <c r="F499" s="22" t="n"/>
-      <c r="G499" s="38" t="n"/>
-      <c r="H499" s="22" t="n"/>
+      <c r="C499" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D499" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E499" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F499" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G499" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="H499" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I499" s="25">
         <f>IF(OR(F499="",G499=""),"",F499*G499)</f>
         <v/>
@@ -22044,17 +22432,35 @@
       <c r="K499" s="26" t="n"/>
     </row>
     <row r="500" ht="18" customHeight="1">
-      <c r="A500" s="35" t="n"/>
+      <c r="A500" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B500" s="16">
         <f>IF(A500="","",IFERROR(INT((A500-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C500" s="16" t="n"/>
-      <c r="D500" s="17" t="n"/>
-      <c r="E500" s="16" t="n"/>
-      <c r="F500" s="16" t="n"/>
-      <c r="G500" s="36" t="n"/>
-      <c r="H500" s="16" t="n"/>
+      <c r="C500" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D500" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E500" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F500" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G500" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="H500" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I500" s="19">
         <f>IF(OR(F500="",G500=""),"",F500*G500)</f>
         <v/>
@@ -22066,17 +22472,33 @@
       <c r="K500" s="20" t="n"/>
     </row>
     <row r="501" ht="18" customHeight="1">
-      <c r="A501" s="37" t="n"/>
+      <c r="A501" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B501" s="22">
         <f>IF(A501="","",IFERROR(INT((A501-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C501" s="22" t="n"/>
-      <c r="D501" s="23" t="n"/>
-      <c r="E501" s="22" t="n"/>
-      <c r="F501" s="22" t="n"/>
+      <c r="C501" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D501" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E501" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F501" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="G501" s="38" t="n"/>
-      <c r="H501" s="22" t="n"/>
+      <c r="H501" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I501" s="25">
         <f>IF(OR(F501="",G501=""),"",F501*G501)</f>
         <v/>
@@ -22085,20 +22507,40 @@
         <f>IF(OR(F501="",G501=""),"",ROUND(G501*(1+F501/30),1))</f>
         <v/>
       </c>
-      <c r="K501" s="26" t="n"/>
+      <c r="K501" s="26" t="inlineStr">
+        <is>
+          <t>Hold 3x8.</t>
+        </is>
+      </c>
     </row>
     <row r="502" ht="18" customHeight="1">
-      <c r="A502" s="35" t="n"/>
+      <c r="A502" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B502" s="16">
         <f>IF(A502="","",IFERROR(INT((A502-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C502" s="16" t="n"/>
-      <c r="D502" s="17" t="n"/>
-      <c r="E502" s="16" t="n"/>
-      <c r="F502" s="16" t="n"/>
+      <c r="C502" s="16" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D502" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E502" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F502" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="G502" s="36" t="n"/>
-      <c r="H502" s="16" t="n"/>
+      <c r="H502" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I502" s="19">
         <f>IF(OR(F502="",G502=""),"",F502*G502)</f>
         <v/>
@@ -22110,17 +22552,33 @@
       <c r="K502" s="20" t="n"/>
     </row>
     <row r="503" ht="18" customHeight="1">
-      <c r="A503" s="37" t="n"/>
+      <c r="A503" s="37" t="n">
+        <v>46300</v>
+      </c>
       <c r="B503" s="22">
         <f>IF(A503="","",IFERROR(INT((A503-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C503" s="22" t="n"/>
-      <c r="D503" s="23" t="n"/>
-      <c r="E503" s="22" t="n"/>
-      <c r="F503" s="22" t="n"/>
+      <c r="C503" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D503" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E503" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F503" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="G503" s="38" t="n"/>
-      <c r="H503" s="22" t="n"/>
+      <c r="H503" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I503" s="25">
         <f>IF(OR(F503="",G503=""),"",F503*G503)</f>
         <v/>
@@ -33344,18 +33802,28 @@
       </c>
     </row>
     <row r="56" ht="18" customHeight="1">
-      <c r="A56" s="35" t="n"/>
+      <c r="A56" s="35" t="n">
+        <v>46300</v>
+      </c>
       <c r="B56" s="16">
         <f>IF(A56="","",IFERROR(INT((A56-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C56" s="36" t="n"/>
-      <c r="D56" s="36" t="n"/>
+      <c r="C56" s="36" t="n">
+        <v>77.59999999999999</v>
+      </c>
+      <c r="D56" s="36" t="n">
+        <v>8.5</v>
+      </c>
       <c r="E56" s="36" t="n"/>
       <c r="F56" s="36" t="n"/>
       <c r="G56" s="36" t="n"/>
       <c r="H56" s="36" t="n"/>
-      <c r="I56" s="20" t="n"/>
+      <c r="I56" s="20" t="inlineStr">
+        <is>
+          <t>5K Wk 1 Mon - GYM #1 full body (joined normal gym; replaces cali). AM: sleep 8:30 (00:05-08:35) q10, RHR 40 (-3, block low), mot 10/energy 10/stress 2, DOMS all 0, tendons clean. BW 77.60 = +1.0 vs 7-reading avg 76.61 after 6 unlogged days, single point, no kcal change. PM: bike 0, kcal 2858 (+458 vs no-bike 2400), protein 170, creatine Y, shin CLEAN.</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="18" customHeight="1">
       <c r="A57" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Tue 10/6 AM (RHR 40, BW 77.20, upper DOMS 3); 6x400 gate green; xlsx Body 57
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -33826,18 +33826,28 @@
       </c>
     </row>
     <row r="57" ht="18" customHeight="1">
-      <c r="A57" s="37" t="n"/>
+      <c r="A57" s="37" t="n">
+        <v>46301</v>
+      </c>
       <c r="B57" s="22">
         <f>IF(A57="","",IFERROR(INT((A57-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C57" s="38" t="n"/>
-      <c r="D57" s="38" t="n"/>
+      <c r="C57" s="38" t="n">
+        <v>77.2</v>
+      </c>
+      <c r="D57" s="38" t="n">
+        <v>7.5</v>
+      </c>
       <c r="E57" s="38" t="n"/>
       <c r="F57" s="38" t="n"/>
       <c r="G57" s="38" t="n"/>
       <c r="H57" s="38" t="n"/>
-      <c r="I57" s="26" t="n"/>
+      <c r="I57" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 1 Tue - TRACK 6x400 staged. AM: sleep 7:30 (23:05-06:35) q8, RHR 40 (-3), mot 10/energy 8/stress 3, DOMS chest 3/back 3/shldr 3/arm 2 (Gym #1), quad/ham/glute/calf 1, tendons clean. BW 77.20 (-0.40 vs 10/5), no kcal change. Legs &lt;2 -&gt; 6x400 stays.</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="18" customHeight="1">
       <c r="A58" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Tue 10/6 road 5 k done (4 k @ 5:34, RPE 6); Fri threshold -> 5:35-5:40; xlsx Running 28, Body 57
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -30252,22 +30252,45 @@
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="A28" s="35" t="n"/>
+      <c r="A28" s="35" t="n">
+        <v>46301</v>
+      </c>
       <c r="B28" s="16">
         <f>IF(A28="","",IFERROR(INT((A28-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C28" s="27" t="n"/>
-      <c r="D28" s="36" t="n"/>
+      <c r="C28" s="27" t="n">
+        <v>5</v>
+      </c>
+      <c r="D28" s="36" t="n">
+        <v>28.3</v>
+      </c>
       <c r="E28" s="16">
         <f>IF(OR(C28="",D28=""),"",TEXT(D28/C28/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F28" s="16" t="n"/>
-      <c r="G28" s="16" t="n"/>
-      <c r="H28" s="16" t="n"/>
-      <c r="I28" s="16" t="n"/>
-      <c r="J28" s="20" t="n"/>
+      <c r="F28" s="16" t="n">
+        <v>160</v>
+      </c>
+      <c r="G28" s="16" t="n">
+        <v>176</v>
+      </c>
+      <c r="H28" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I28" s="16" t="inlineStr">
+        <is>
+          <t>Steady</t>
+        </is>
+      </c>
+      <c r="J28" s="20" t="inlineStr">
+        <is>
+          <t>5K Wk 1 Tue - ROAD 5 k (track 6x400 swapped, user). PM 12:40. Moving 28:18 (5:39), elapsed 35:44 (6.5 min stop ~0.65 k). Splits 5:59@133 / 5:34@163 / 5:34@167 / 5:32@171 / 5:38@168. Main 4 k @ 5:34 HR ~167 max 176 vs prescribed 3 k @ 6:00 cap 172 - RAN HOT. No strides visible, no CD. Cadence 163. RPE 6. Engine: 9/25 5:57@175 RPE 9 -&gt; 5:34@167 RPE 6; 5K est ~26:30-27:00. Shin not reported. Fri threshold up to 5:35-5:40. Strava 20472528970.</t>
+        </is>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29" ht="18" customHeight="1">
       <c r="A29" s="37" t="n"/>
@@ -33845,7 +33868,7 @@
       <c r="H57" s="38" t="n"/>
       <c r="I57" s="26" t="inlineStr">
         <is>
-          <t>5K Wk 1 Tue - TRACK 6x400 staged. AM: sleep 7:30 (23:05-06:35) q8, RHR 40 (-3), mot 10/energy 8/stress 3, DOMS chest 3/back 3/shldr 3/arm 2 (Gym #1), quad/ham/glute/calf 1, tendons clean. BW 77.20 (-0.40 vs 10/5), no kcal change. Legs &lt;2 -&gt; 6x400 stays.</t>
+          <t>5K Wk 1 Tue - TRACK 6x400 staged. AM: sleep 7:30 (23:05-06:35) q8, RHR 40 (-3), mot 10/energy 8/stress 3, DOMS chest 3/back 3/shldr 3/arm 2 (Gym #1), quad/ham/glute/calf 1, tendons clean. BW 77.20 (-0.40 vs 10/5), no kcal change. Legs &lt;2 -&gt; 6x400 stays. PM: road 5 k (4 k @ 5:34, RPE 6), bike 0, kcal 2375 (on ~2400), protein 164, creatine Y.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
log: 10/6 shin clean #41; Fri threshold 5:35-5:40 confirmed
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -30285,7 +30285,7 @@
       </c>
       <c r="J28" s="20" t="inlineStr">
         <is>
-          <t>5K Wk 1 Tue - ROAD 5 k (track 6x400 swapped, user). PM 12:40. Moving 28:18 (5:39), elapsed 35:44 (6.5 min stop ~0.65 k). Splits 5:59@133 / 5:34@163 / 5:34@167 / 5:32@171 / 5:38@168. Main 4 k @ 5:34 HR ~167 max 176 vs prescribed 3 k @ 6:00 cap 172 - RAN HOT. No strides visible, no CD. Cadence 163. RPE 6. Engine: 9/25 5:57@175 RPE 9 -&gt; 5:34@167 RPE 6; 5K est ~26:30-27:00. Shin not reported. Fri threshold up to 5:35-5:40. Strava 20472528970.</t>
+          <t>5K Wk 1 Tue - ROAD 5 k (track 6x400 swapped, user). PM 12:40. Moving 28:18 (5:39), elapsed 35:44 (6.5 min stop ~0.65 k). Splits 5:59@133 / 5:34@163 / 5:34@167 / 5:32@171 / 5:38@168. Main 4 k @ 5:34 HR ~167 max 176 vs prescribed 3 k @ 6:00 cap 172 - RAN HOT. No strides visible, no CD. Cadence 163. RPE 6. Engine: 9/25 5:57@175 RPE 9 -&gt; 5:34@167 RPE 6; 5K est ~26:30-27:00. SHIN CLEAN #41. Fri threshold up to 5:35-5:40. Strava 20472528970.</t>
         </is>
       </c>
       <c r="K28" t="n">
@@ -33868,7 +33868,7 @@
       <c r="H57" s="38" t="n"/>
       <c r="I57" s="26" t="inlineStr">
         <is>
-          <t>5K Wk 1 Tue - TRACK 6x400 staged. AM: sleep 7:30 (23:05-06:35) q8, RHR 40 (-3), mot 10/energy 8/stress 3, DOMS chest 3/back 3/shldr 3/arm 2 (Gym #1), quad/ham/glute/calf 1, tendons clean. BW 77.20 (-0.40 vs 10/5), no kcal change. Legs &lt;2 -&gt; 6x400 stays. PM: road 5 k (4 k @ 5:34, RPE 6), bike 0, kcal 2375 (on ~2400), protein 164, creatine Y.</t>
+          <t>5K Wk 1 Tue - TRACK 6x400 staged. AM: sleep 7:30 (23:05-06:35) q8, RHR 40 (-3), mot 10/energy 8/stress 3, DOMS chest 3/back 3/shldr 3/arm 2 (Gym #1), quad/ham/glute/calf 1, tendons clean. BW 77.20 (-0.40 vs 10/5), no kcal change. Legs &lt;2 -&gt; 6x400 stays. PM: road 5 k (4 k @ 5:34, RPE 6), bike 0, kcal 2375 (on ~2400), protein 164, creatine Y. SHIN CLEAN #41.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
log: Wed 10/7 AM (BW 76.30, RHR 43, shin clean #42); Fri 2x2 k gate green; xlsx Body 58
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -33873,18 +33873,28 @@
       </c>
     </row>
     <row r="58" ht="18" customHeight="1">
-      <c r="A58" s="35" t="n"/>
+      <c r="A58" s="35" t="n">
+        <v>46302</v>
+      </c>
       <c r="B58" s="16">
         <f>IF(A58="","",IFERROR(INT((A58-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C58" s="36" t="n"/>
-      <c r="D58" s="36" t="n"/>
+      <c r="C58" s="36" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="D58" s="36" t="n">
+        <v>8.58</v>
+      </c>
       <c r="E58" s="36" t="n"/>
       <c r="F58" s="36" t="n"/>
       <c r="G58" s="36" t="n"/>
       <c r="H58" s="36" t="n"/>
-      <c r="I58" s="20" t="n"/>
+      <c r="I58" s="20" t="inlineStr">
+        <is>
+          <t>5K Wk 1 Wed - REST, full. AM: sleep 8:35 (23:45-08:20) q8, RHR 43 (0 vs 7d), mot 10/energy 10/stress 3, DOMS chest 2/back 1/shldr 2/arm 1 (Gym #1, falling), quad/ham/glute/calf 1, tendons clean, SHIN CLEAN #42. BW 76.30 (-0.90 d/d), 7-reading avg 76.69, no kcal change. Gates: Fri 2x2 k ON, Thu strides stay, upper recheck Fri AM.</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="18" customHeight="1">
       <c r="A59" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Thu 10/8 easy 5 k + strides done (strides hot, shin clean #45); xlsx Running 29, Body 59
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -30293,22 +30293,45 @@
       </c>
     </row>
     <row r="29" ht="18" customHeight="1">
-      <c r="A29" s="37" t="n"/>
+      <c r="A29" s="37" t="n">
+        <v>46303</v>
+      </c>
       <c r="B29" s="22">
         <f>IF(A29="","",IFERROR(INT((A29-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C29" s="28" t="n"/>
-      <c r="D29" s="38" t="n"/>
+      <c r="C29" s="28" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="D29" s="38" t="n">
+        <v>36.48</v>
+      </c>
       <c r="E29" s="22">
         <f>IF(OR(C29="",D29=""),"",TEXT(D29/C29/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F29" s="22" t="n"/>
-      <c r="G29" s="22" t="n"/>
-      <c r="H29" s="22" t="n"/>
-      <c r="I29" s="22" t="n"/>
-      <c r="J29" s="26" t="n"/>
+      <c r="F29" s="22" t="n">
+        <v>146</v>
+      </c>
+      <c r="G29" s="22" t="n">
+        <v>166</v>
+      </c>
+      <c r="H29" s="22" t="n">
+        <v>5</v>
+      </c>
+      <c r="I29" s="22" t="inlineStr">
+        <is>
+          <t>Easy+Strides</t>
+        </is>
+      </c>
+      <c r="J29" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 1 Thu - EASY 5 k + 6x20 s STRIDES. PM 18:23, light rain. Moving 36:29 (7:08), elapsed 41:39 (~4.7 min stop ~0.67 k). Laps 6:19@130 (GPS start) / 6:51@152 / 7:10@149 / 7:39@148 / 7:39@149 (strides) / 0.12 k. Easy km 2-4 = 7:13 @ ~150, pace obeyed. Cadence easy km 164/166/166/167 (floor back). Strides 6/6 smooth but GPS ~3:55-4:58, mostly 4:10-4:30 vs prescribed 5:10-5:20 = ran hot. RPE 5. SHIN CLEAN #45. Strava 20505117221.</t>
+        </is>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="35" t="n"/>
@@ -33897,18 +33920,28 @@
       </c>
     </row>
     <row r="59" ht="18" customHeight="1">
-      <c r="A59" s="37" t="n"/>
+      <c r="A59" s="37" t="n">
+        <v>46303</v>
+      </c>
       <c r="B59" s="22">
         <f>IF(A59="","",IFERROR(INT((A59-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C59" s="38" t="n"/>
-      <c r="D59" s="38" t="n"/>
+      <c r="C59" s="38" t="n">
+        <v>76.3</v>
+      </c>
+      <c r="D59" s="38" t="n">
+        <v>8.369999999999999</v>
+      </c>
       <c r="E59" s="38" t="n"/>
       <c r="F59" s="38" t="n"/>
       <c r="G59" s="38" t="n"/>
       <c r="H59" s="38" t="n"/>
-      <c r="I59" s="26" t="n"/>
+      <c r="I59" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 1 Thu - EASY 5 k + strides. AM: sleep 8:22 (23:45-08:10) q10, RHR 42 (0 vs 7d), mot 10/energy 10/stress 2, DOMS chest/back/shldr/arm 1, quad 1, ham/glute/calf 0, joints clean, SHIN CLEAN #44. BW 76.30 flat d/d, no kcal change. Gates all green. PM: 5.12 k easy + 6 strides (ran hot ~4:10-4:30), bike 0, kcal 2325 (-75 vs 2400), protein 174, creatine Y, alcohol 0, SHIN CLEAN #45.</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="18" customHeight="1">
       <c r="A60" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Wed 10/14 easy 5 k + strides done (shin clean #46, strides ~4:40-5:00); xlsx Running 30, Body 60
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -30334,22 +30334,45 @@
       </c>
     </row>
     <row r="30" ht="18" customHeight="1">
-      <c r="A30" s="35" t="n"/>
+      <c r="A30" s="35" t="n">
+        <v>46309</v>
+      </c>
       <c r="B30" s="16">
         <f>IF(A30="","",IFERROR(INT((A30-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C30" s="27" t="n"/>
-      <c r="D30" s="36" t="n"/>
+      <c r="C30" s="27" t="n">
+        <v>5.03</v>
+      </c>
+      <c r="D30" s="36" t="n">
+        <v>37.53</v>
+      </c>
       <c r="E30" s="16">
         <f>IF(OR(C30="",D30=""),"",TEXT(D30/C30/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F30" s="16" t="n"/>
-      <c r="G30" s="16" t="n"/>
-      <c r="H30" s="16" t="n"/>
-      <c r="I30" s="16" t="n"/>
-      <c r="J30" s="20" t="n"/>
+      <c r="F30" s="16" t="n">
+        <v>149</v>
+      </c>
+      <c r="G30" s="16" t="n">
+        <v>170</v>
+      </c>
+      <c r="H30" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="I30" s="16" t="inlineStr">
+        <is>
+          <t>Easy+Strides</t>
+        </is>
+      </c>
+      <c r="J30" s="20" t="inlineStr">
+        <is>
+          <t>5K Wk 2 Wed - EASY 5 k + 6x20 s STRIDES, re-entry after 6 run-free days (10/9-10/13 dark). PM 16:55, sunny. Moving = elapsed 37:32 (7:28), no stops. Laps 7:00@138 / 7:20@152 / 7:16@152 / 8:11@148 (+8 m) / 7:37@152 (strides). Cadence easy km 165/166/164/163 (under floor km 3-4). Strides 6/6, GPS ~5:00/4:23/4:46/4:38/5:08/4:54 - closer to 5:10-5:20 than 10/8. RPE 5, walk 0. SHIN CLEAN #46. Strava 20583383940.</t>
+        </is>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="37" t="n"/>
@@ -33944,7 +33967,9 @@
       </c>
     </row>
     <row r="60" ht="18" customHeight="1">
-      <c r="A60" s="35" t="n"/>
+      <c r="A60" s="35" t="n">
+        <v>46309</v>
+      </c>
       <c r="B60" s="16">
         <f>IF(A60="","",IFERROR(INT((A60-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
@@ -33955,7 +33980,11 @@
       <c r="F60" s="36" t="n"/>
       <c r="G60" s="36" t="n"/>
       <c r="H60" s="36" t="n"/>
-      <c r="I60" s="20" t="n"/>
+      <c r="I60" s="20" t="inlineStr">
+        <is>
+          <t>5K Wk 2 Wed - first run after 10/9-10/13 dark gap. AM not captured (BW/sleep/RHR blank). PM: 5.03 k easy + 6 strides, bike 0, kcal 2448 (+48 vs 2400), protein 172, creatine Y, alcohol 0, steps 14190, SHIN CLEAN #46.</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="18" customHeight="1">
       <c r="A61" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Thu 10/15 AM (BW 76.60, RHR 41, shin #47, back DOMS 3); Gym #2 re-cut pulls out, push -1 set; xlsx Body 61
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -33987,18 +33987,28 @@
       </c>
     </row>
     <row r="61" ht="18" customHeight="1">
-      <c r="A61" s="37" t="n"/>
+      <c r="A61" s="37" t="n">
+        <v>46310</v>
+      </c>
       <c r="B61" s="22">
         <f>IF(A61="","",IFERROR(INT((A61-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C61" s="38" t="n"/>
-      <c r="D61" s="38" t="n"/>
+      <c r="C61" s="38" t="n">
+        <v>76.59999999999999</v>
+      </c>
+      <c r="D61" s="38" t="n">
+        <v>7.67</v>
+      </c>
       <c r="E61" s="38" t="n"/>
       <c r="F61" s="38" t="n"/>
       <c r="G61" s="38" t="n"/>
       <c r="H61" s="38" t="n"/>
-      <c r="I61" s="26" t="n"/>
+      <c r="I61" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 2 Thu - AM: sleep 7:40 (23:45-07:25) q8, RHR 41 (-3 vs 7d), mot 10/energy 10/stress 3, DOMS chest 0/back 3/shldr 2/arm 2, quad/ham/glute/calf 1, tendons clean, SHIN CLEAN #47. BW 76.60 (+0.30 vs 10/8) single point after 6-day hole, no kcal change. Back DOMS 3 = Wed 10/14 back session (unlogged) -&gt; Gym #2 pulls out, push -1 set.</t>
+        </is>
+      </c>
     </row>
     <row r="62" ht="18" customHeight="1">
       <c r="A62" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Thu 10/15 easy 4 k done (7:11, HR 142, cadence 162 under floor, shin #48); xlsx Running 31
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -30375,22 +30375,43 @@
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="37" t="n"/>
+      <c r="A31" s="37" t="n">
+        <v>46310</v>
+      </c>
       <c r="B31" s="22">
         <f>IF(A31="","",IFERROR(INT((A31-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C31" s="28" t="n"/>
-      <c r="D31" s="38" t="n"/>
+      <c r="C31" s="28" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="D31" s="38" t="n">
+        <v>28.85</v>
+      </c>
       <c r="E31" s="22">
         <f>IF(OR(C31="",D31=""),"",TEXT(D31/C31/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F31" s="22" t="n"/>
-      <c r="G31" s="22" t="n"/>
+      <c r="F31" s="22" t="n">
+        <v>142</v>
+      </c>
+      <c r="G31" s="22" t="n">
+        <v>157</v>
+      </c>
       <c r="H31" s="22" t="n"/>
-      <c r="I31" s="22" t="n"/>
-      <c r="J31" s="26" t="n"/>
+      <c r="I31" s="22" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J31" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 2 Thu - EASY 4 k, AM 07:49 before Gym #2. Moving 28:51 (7:11), elapsed 29:36 (35 s stop km 3). Laps 7:05@124 / 7:00@147 / 7:34@146 (+9 m) / 7:05@151. HR cap obeyed. Cadence 160/163/162/162 - under 166 floor all run. RPE n/r. SHIN CLEAN #48. Strava 20591443035.</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="35" t="n"/>

</xml_diff>

<commit_message>
Log 10/17 RPE/shin + xlsx sync (10/15 gym, 10/15 & 10/17 runs); stage Sun 10/18 long 10k; CLAUDE.md status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KSXruGLKV1VLWxJ3FNXk6x
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -22590,39 +22590,79 @@
       <c r="K503" s="26" t="n"/>
     </row>
     <row r="504" ht="18" customHeight="1">
-      <c r="A504" s="35" t="n"/>
-      <c r="B504" s="16">
+      <c r="A504" s="37" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B504" s="22">
         <f>IF(A504="","",IFERROR(INT((A504-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C504" s="16" t="n"/>
-      <c r="D504" s="17" t="n"/>
-      <c r="E504" s="16" t="n"/>
-      <c r="F504" s="16" t="n"/>
-      <c r="G504" s="36" t="n"/>
-      <c r="H504" s="16" t="n"/>
-      <c r="I504" s="19">
+      <c r="C504" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D504" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E504" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F504" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G504" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H504" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="I504" s="25">
         <f>IF(OR(F504="",G504=""),"",F504*G504)</f>
         <v/>
       </c>
-      <c r="J504" s="36">
+      <c r="J504" s="38">
         <f>IF(OR(F504="",G504=""),"",ROUND(G504*(1+F504/30),1))</f>
         <v/>
       </c>
-      <c r="K504" s="20" t="n"/>
+      <c r="K504" s="26" t="inlineStr">
+        <is>
+          <t>Gym #2. 3 of 4 sets. Hold 25 4x8.</t>
+        </is>
+      </c>
     </row>
     <row r="505" ht="18" customHeight="1">
-      <c r="A505" s="37" t="n"/>
+      <c r="A505" s="37" t="n">
+        <v>46310</v>
+      </c>
       <c r="B505" s="22">
         <f>IF(A505="","",IFERROR(INT((A505-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C505" s="22" t="n"/>
-      <c r="D505" s="23" t="n"/>
-      <c r="E505" s="22" t="n"/>
-      <c r="F505" s="22" t="n"/>
-      <c r="G505" s="38" t="n"/>
-      <c r="H505" s="22" t="n"/>
+      <c r="C505" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D505" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E505" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F505" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G505" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H505" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I505" s="25">
         <f>IF(OR(F505="",G505=""),"",F505*G505)</f>
         <v/>
@@ -22634,39 +22674,75 @@
       <c r="K505" s="26" t="n"/>
     </row>
     <row r="506" ht="18" customHeight="1">
-      <c r="A506" s="35" t="n"/>
-      <c r="B506" s="16">
+      <c r="A506" s="37" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B506" s="22">
         <f>IF(A506="","",IFERROR(INT((A506-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C506" s="16" t="n"/>
-      <c r="D506" s="17" t="n"/>
-      <c r="E506" s="16" t="n"/>
-      <c r="F506" s="16" t="n"/>
-      <c r="G506" s="36" t="n"/>
-      <c r="H506" s="16" t="n"/>
-      <c r="I506" s="19">
+      <c r="C506" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D506" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E506" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F506" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G506" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H506" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="I506" s="25">
         <f>IF(OR(F506="",G506=""),"",F506*G506)</f>
         <v/>
       </c>
-      <c r="J506" s="36">
+      <c r="J506" s="38">
         <f>IF(OR(F506="",G506=""),"",ROUND(G506*(1+F506/30),1))</f>
         <v/>
       </c>
-      <c r="K506" s="20" t="n"/>
+      <c r="K506" s="26" t="n"/>
     </row>
     <row r="507" ht="18" customHeight="1">
-      <c r="A507" s="37" t="n"/>
+      <c r="A507" s="37" t="n">
+        <v>46310</v>
+      </c>
       <c r="B507" s="22">
         <f>IF(A507="","",IFERROR(INT((A507-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C507" s="22" t="n"/>
-      <c r="D507" s="23" t="n"/>
-      <c r="E507" s="22" t="n"/>
-      <c r="F507" s="22" t="n"/>
-      <c r="G507" s="38" t="n"/>
-      <c r="H507" s="22" t="n"/>
+      <c r="C507" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D507" s="23" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E507" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F507" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G507" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="H507" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I507" s="25">
         <f>IF(OR(F507="",G507=""),"",F507*G507)</f>
         <v/>
@@ -22675,42 +22751,82 @@
         <f>IF(OR(F507="",G507=""),"",ROUND(G507*(1+F507/30),1))</f>
         <v/>
       </c>
-      <c r="K507" s="26" t="n"/>
+      <c r="K507" s="26" t="inlineStr">
+        <is>
+          <t>6/DB. 2 of 3 sets. Hold 3x10.</t>
+        </is>
+      </c>
     </row>
     <row r="508" ht="18" customHeight="1">
-      <c r="A508" s="35" t="n"/>
-      <c r="B508" s="16">
+      <c r="A508" s="37" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B508" s="22">
         <f>IF(A508="","",IFERROR(INT((A508-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C508" s="16" t="n"/>
-      <c r="D508" s="17" t="n"/>
-      <c r="E508" s="16" t="n"/>
-      <c r="F508" s="16" t="n"/>
-      <c r="G508" s="36" t="n"/>
-      <c r="H508" s="16" t="n"/>
-      <c r="I508" s="19">
+      <c r="C508" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D508" s="23" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E508" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F508" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G508" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="H508" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="I508" s="25">
         <f>IF(OR(F508="",G508=""),"",F508*G508)</f>
         <v/>
       </c>
-      <c r="J508" s="36">
+      <c r="J508" s="38">
         <f>IF(OR(F508="",G508=""),"",ROUND(G508*(1+F508/30),1))</f>
         <v/>
       </c>
-      <c r="K508" s="20" t="n"/>
+      <c r="K508" s="26" t="n"/>
     </row>
     <row r="509" ht="18" customHeight="1">
-      <c r="A509" s="37" t="n"/>
+      <c r="A509" s="37" t="n">
+        <v>46310</v>
+      </c>
       <c r="B509" s="22">
         <f>IF(A509="","",IFERROR(INT((A509-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C509" s="22" t="n"/>
-      <c r="D509" s="23" t="n"/>
-      <c r="E509" s="22" t="n"/>
-      <c r="F509" s="22" t="n"/>
-      <c r="G509" s="38" t="n"/>
-      <c r="H509" s="22" t="n"/>
+      <c r="C509" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D509" s="23" t="inlineStr">
+        <is>
+          <t>Leg Extension</t>
+        </is>
+      </c>
+      <c r="E509" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F509" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G509" s="38" t="n">
+        <v>15</v>
+      </c>
+      <c r="H509" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I509" s="25">
         <f>IF(OR(F509="",G509=""),"",F509*G509)</f>
         <v/>
@@ -22719,42 +22835,82 @@
         <f>IF(OR(F509="",G509=""),"",ROUND(G509*(1+F509/30),1))</f>
         <v/>
       </c>
-      <c r="K509" s="26" t="n"/>
+      <c r="K509" s="26" t="inlineStr">
+        <is>
+          <t>Above seed 12.5, legs cap RPE 6. Hold.</t>
+        </is>
+      </c>
     </row>
     <row r="510" ht="18" customHeight="1">
-      <c r="A510" s="35" t="n"/>
-      <c r="B510" s="16">
+      <c r="A510" s="37" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B510" s="22">
         <f>IF(A510="","",IFERROR(INT((A510-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C510" s="16" t="n"/>
-      <c r="D510" s="17" t="n"/>
-      <c r="E510" s="16" t="n"/>
-      <c r="F510" s="16" t="n"/>
-      <c r="G510" s="36" t="n"/>
-      <c r="H510" s="16" t="n"/>
-      <c r="I510" s="19">
+      <c r="C510" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D510" s="23" t="inlineStr">
+        <is>
+          <t>Leg Extension</t>
+        </is>
+      </c>
+      <c r="E510" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F510" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G510" s="38" t="n">
+        <v>15</v>
+      </c>
+      <c r="H510" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="I510" s="25">
         <f>IF(OR(F510="",G510=""),"",F510*G510)</f>
         <v/>
       </c>
-      <c r="J510" s="36">
+      <c r="J510" s="38">
         <f>IF(OR(F510="",G510=""),"",ROUND(G510*(1+F510/30),1))</f>
         <v/>
       </c>
-      <c r="K510" s="20" t="n"/>
+      <c r="K510" s="26" t="n"/>
     </row>
     <row r="511" ht="18" customHeight="1">
-      <c r="A511" s="37" t="n"/>
+      <c r="A511" s="37" t="n">
+        <v>46310</v>
+      </c>
       <c r="B511" s="22">
         <f>IF(A511="","",IFERROR(INT((A511-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C511" s="22" t="n"/>
-      <c r="D511" s="23" t="n"/>
-      <c r="E511" s="22" t="n"/>
-      <c r="F511" s="22" t="n"/>
-      <c r="G511" s="38" t="n"/>
-      <c r="H511" s="22" t="n"/>
+      <c r="C511" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D511" s="23" t="inlineStr">
+        <is>
+          <t>Lying Leg Curl</t>
+        </is>
+      </c>
+      <c r="E511" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F511" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G511" s="38" t="n">
+        <v>16</v>
+      </c>
+      <c r="H511" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I511" s="25">
         <f>IF(OR(F511="",G511=""),"",F511*G511)</f>
         <v/>
@@ -22763,42 +22919,82 @@
         <f>IF(OR(F511="",G511=""),"",ROUND(G511*(1+F511/30),1))</f>
         <v/>
       </c>
-      <c r="K511" s="26" t="n"/>
+      <c r="K511" s="26" t="inlineStr">
+        <is>
+          <t>Above seed 10. Hold.</t>
+        </is>
+      </c>
     </row>
     <row r="512" ht="18" customHeight="1">
-      <c r="A512" s="35" t="n"/>
-      <c r="B512" s="16">
+      <c r="A512" s="37" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B512" s="22">
         <f>IF(A512="","",IFERROR(INT((A512-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C512" s="16" t="n"/>
-      <c r="D512" s="17" t="n"/>
-      <c r="E512" s="16" t="n"/>
-      <c r="F512" s="16" t="n"/>
-      <c r="G512" s="36" t="n"/>
-      <c r="H512" s="16" t="n"/>
-      <c r="I512" s="19">
+      <c r="C512" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D512" s="23" t="inlineStr">
+        <is>
+          <t>Lying Leg Curl</t>
+        </is>
+      </c>
+      <c r="E512" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F512" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G512" s="38" t="n">
+        <v>16</v>
+      </c>
+      <c r="H512" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="I512" s="25">
         <f>IF(OR(F512="",G512=""),"",F512*G512)</f>
         <v/>
       </c>
-      <c r="J512" s="36">
+      <c r="J512" s="38">
         <f>IF(OR(F512="",G512=""),"",ROUND(G512*(1+F512/30),1))</f>
         <v/>
       </c>
-      <c r="K512" s="20" t="n"/>
+      <c r="K512" s="26" t="n"/>
     </row>
     <row r="513" ht="18" customHeight="1">
-      <c r="A513" s="37" t="n"/>
+      <c r="A513" s="37" t="n">
+        <v>46310</v>
+      </c>
       <c r="B513" s="22">
         <f>IF(A513="","",IFERROR(INT((A513-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C513" s="22" t="n"/>
-      <c r="D513" s="23" t="n"/>
-      <c r="E513" s="22" t="n"/>
-      <c r="F513" s="22" t="n"/>
-      <c r="G513" s="38" t="n"/>
-      <c r="H513" s="22" t="n"/>
+      <c r="C513" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D513" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E513" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F513" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G513" s="38" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H513" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I513" s="25">
         <f>IF(OR(F513="",G513=""),"",F513*G513)</f>
         <v/>
@@ -22807,42 +23003,82 @@
         <f>IF(OR(F513="",G513=""),"",ROUND(G513*(1+F513/30),1))</f>
         <v/>
       </c>
-      <c r="K513" s="26" t="n"/>
+      <c r="K513" s="26" t="inlineStr">
+        <is>
+          <t>6.8 kg (seed 2.5). Hold.</t>
+        </is>
+      </c>
     </row>
     <row r="514" ht="18" customHeight="1">
-      <c r="A514" s="35" t="n"/>
-      <c r="B514" s="16">
+      <c r="A514" s="37" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B514" s="22">
         <f>IF(A514="","",IFERROR(INT((A514-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C514" s="16" t="n"/>
-      <c r="D514" s="17" t="n"/>
-      <c r="E514" s="16" t="n"/>
-      <c r="F514" s="16" t="n"/>
-      <c r="G514" s="36" t="n"/>
-      <c r="H514" s="16" t="n"/>
-      <c r="I514" s="19">
+      <c r="C514" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D514" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E514" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F514" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G514" s="38" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H514" s="22" t="n">
+        <v>7</v>
+      </c>
+      <c r="I514" s="25">
         <f>IF(OR(F514="",G514=""),"",F514*G514)</f>
         <v/>
       </c>
-      <c r="J514" s="36">
+      <c r="J514" s="38">
         <f>IF(OR(F514="",G514=""),"",ROUND(G514*(1+F514/30),1))</f>
         <v/>
       </c>
-      <c r="K514" s="20" t="n"/>
+      <c r="K514" s="26" t="n"/>
     </row>
     <row r="515" ht="18" customHeight="1">
-      <c r="A515" s="37" t="n"/>
+      <c r="A515" s="37" t="n">
+        <v>46310</v>
+      </c>
       <c r="B515" s="22">
         <f>IF(A515="","",IFERROR(INT((A515-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C515" s="22" t="n"/>
-      <c r="D515" s="23" t="n"/>
-      <c r="E515" s="22" t="n"/>
-      <c r="F515" s="22" t="n"/>
-      <c r="G515" s="38" t="n"/>
-      <c r="H515" s="22" t="n"/>
+      <c r="C515" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D515" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E515" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F515" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G515" s="38" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H515" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I515" s="25">
         <f>IF(OR(F515="",G515=""),"",F515*G515)</f>
         <v/>
@@ -22854,39 +23090,75 @@
       <c r="K515" s="26" t="n"/>
     </row>
     <row r="516" ht="18" customHeight="1">
-      <c r="A516" s="35" t="n"/>
-      <c r="B516" s="16">
+      <c r="A516" s="37" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B516" s="22">
         <f>IF(A516="","",IFERROR(INT((A516-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C516" s="16" t="n"/>
-      <c r="D516" s="17" t="n"/>
-      <c r="E516" s="16" t="n"/>
-      <c r="F516" s="16" t="n"/>
-      <c r="G516" s="36" t="n"/>
-      <c r="H516" s="16" t="n"/>
-      <c r="I516" s="19">
+      <c r="C516" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D516" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E516" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F516" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G516" s="38" t="n"/>
+      <c r="H516" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="I516" s="25">
         <f>IF(OR(F516="",G516=""),"",F516*G516)</f>
         <v/>
       </c>
-      <c r="J516" s="36">
+      <c r="J516" s="38">
         <f>IF(OR(F516="",G516=""),"",ROUND(G516*(1+F516/30),1))</f>
         <v/>
       </c>
-      <c r="K516" s="20" t="n"/>
+      <c r="K516" s="26" t="inlineStr">
+        <is>
+          <t>Next 3x10.</t>
+        </is>
+      </c>
     </row>
     <row r="517" ht="18" customHeight="1">
-      <c r="A517" s="37" t="n"/>
+      <c r="A517" s="37" t="n">
+        <v>46310</v>
+      </c>
       <c r="B517" s="22">
         <f>IF(A517="","",IFERROR(INT((A517-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C517" s="22" t="n"/>
-      <c r="D517" s="23" t="n"/>
-      <c r="E517" s="22" t="n"/>
-      <c r="F517" s="22" t="n"/>
+      <c r="C517" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D517" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E517" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F517" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="G517" s="38" t="n"/>
-      <c r="H517" s="22" t="n"/>
+      <c r="H517" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I517" s="25">
         <f>IF(OR(F517="",G517=""),"",F517*G517)</f>
         <v/>
@@ -22898,26 +23170,42 @@
       <c r="K517" s="26" t="n"/>
     </row>
     <row r="518" ht="18" customHeight="1">
-      <c r="A518" s="35" t="n"/>
-      <c r="B518" s="16">
+      <c r="A518" s="37" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B518" s="22">
         <f>IF(A518="","",IFERROR(INT((A518-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C518" s="16" t="n"/>
-      <c r="D518" s="17" t="n"/>
-      <c r="E518" s="16" t="n"/>
-      <c r="F518" s="16" t="n"/>
-      <c r="G518" s="36" t="n"/>
-      <c r="H518" s="16" t="n"/>
-      <c r="I518" s="19">
+      <c r="C518" s="22" t="inlineStr">
+        <is>
+          <t>Gym Full Body</t>
+        </is>
+      </c>
+      <c r="D518" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E518" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F518" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G518" s="38" t="n"/>
+      <c r="H518" s="22" t="n">
+        <v>6</v>
+      </c>
+      <c r="I518" s="25">
         <f>IF(OR(F518="",G518=""),"",F518*G518)</f>
         <v/>
       </c>
-      <c r="J518" s="36">
+      <c r="J518" s="38">
         <f>IF(OR(F518="",G518=""),"",ROUND(G518*(1+F518/30),1))</f>
         <v/>
       </c>
-      <c r="K518" s="20" t="n"/>
+      <c r="K518" s="26" t="n"/>
     </row>
     <row r="519" ht="18" customHeight="1">
       <c r="A519" s="37" t="n"/>
@@ -30375,40 +30663,84 @@
       </c>
     </row>
     <row r="31" ht="18" customHeight="1">
-      <c r="A31" s="37" t="n"/>
-      <c r="B31" s="22">
+      <c r="A31" s="35" t="n">
+        <v>46310</v>
+      </c>
+      <c r="B31" s="16">
         <f>IF(A31="","",IFERROR(INT((A31-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C31" s="28" t="n"/>
-      <c r="D31" s="38" t="n"/>
-      <c r="E31" s="22">
+      <c r="C31" s="27" t="n">
+        <v>4.02</v>
+      </c>
+      <c r="D31" s="36" t="n">
+        <v>28.85</v>
+      </c>
+      <c r="E31" s="16">
         <f>IF(OR(C31="",D31=""),"",TEXT(D31/C31/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F31" s="22" t="n"/>
-      <c r="G31" s="22" t="n"/>
-      <c r="H31" s="22" t="n"/>
-      <c r="I31" s="22" t="n"/>
-      <c r="J31" s="26" t="n"/>
+      <c r="F31" s="16" t="n">
+        <v>142</v>
+      </c>
+      <c r="G31" s="16" t="n">
+        <v>157</v>
+      </c>
+      <c r="H31" s="16" t="n"/>
+      <c r="I31" s="16" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J31" s="20" t="inlineStr">
+        <is>
+          <t>5K Wk 2 Thu - EASY 4 k, AM 07:49 (gym 19:45). Moving 28:51 (7:11), elapsed 29:36. Laps 7:05@124 / 7:00@147 / 7:34@146 / 7:05@151. Cadence ~160-163 (under floor). No pain - SHIN CLEAN #47. Strava 20591443035.</t>
+        </is>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="35" t="n"/>
+      <c r="A32" s="35" t="n">
+        <v>46312</v>
+      </c>
       <c r="B32" s="16">
         <f>IF(A32="","",IFERROR(INT((A32-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C32" s="27" t="n"/>
-      <c r="D32" s="36" t="n"/>
+      <c r="C32" s="27" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="D32" s="36" t="n">
+        <v>42.5</v>
+      </c>
       <c r="E32" s="16">
         <f>IF(OR(C32="",D32=""),"",TEXT(D32/C32/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F32" s="16" t="n"/>
-      <c r="G32" s="16" t="n"/>
-      <c r="H32" s="16" t="n"/>
-      <c r="I32" s="16" t="n"/>
-      <c r="J32" s="20" t="n"/>
+      <c r="F32" s="16" t="n">
+        <v>161</v>
+      </c>
+      <c r="G32" s="16" t="n">
+        <v>184</v>
+      </c>
+      <c r="H32" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>Threshold</t>
+        </is>
+      </c>
+      <c r="J32" s="20" t="inlineStr">
+        <is>
+          <t>5K Wk 2 Sat - THRESHOLD 2x2 k, 13:51 Sonderborg flat road. Moving 42:30, elapsed 45:23. WU ~2.4 k + 3 strides. Rep 1 ~5:27, rep 2 ~5:29 (stream est., moving; ~35 s pause in each) vs 5:35-5:40 = RAN HOT. HR 177-184 vs cap 175 (~10 bpm over 10/6 at similar pace). CD skipped. Cadence reps 164-168. RPE 6, felt good. SHIN CLEAN #48. Strava 20620965276.</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Wed 10/21 AM (BW 77.35, RHR 45, shin #49, DOMS 0); Sat 10/17 threshold done (HR +10); Wk 3 re-cut to 3 runs, stage 3 K TT; xlsx Running 32, Body 62
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -30414,22 +30414,43 @@
       </c>
     </row>
     <row r="32" ht="18" customHeight="1">
-      <c r="A32" s="35" t="n"/>
+      <c r="A32" s="35" t="n">
+        <v>46312</v>
+      </c>
       <c r="B32" s="16">
         <f>IF(A32="","",IFERROR(INT((A32-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C32" s="27" t="n"/>
-      <c r="D32" s="36" t="n"/>
+      <c r="C32" s="27" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="D32" s="36" t="n">
+        <v>42.5</v>
+      </c>
       <c r="E32" s="16">
         <f>IF(OR(C32="",D32=""),"",TEXT(D32/C32/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F32" s="16" t="n"/>
-      <c r="G32" s="16" t="n"/>
+      <c r="F32" s="16" t="n">
+        <v>161</v>
+      </c>
+      <c r="G32" s="16" t="n">
+        <v>184</v>
+      </c>
       <c r="H32" s="16" t="n"/>
-      <c r="I32" s="16" t="n"/>
-      <c r="J32" s="20" t="n"/>
+      <c r="I32" s="16" t="inlineStr">
+        <is>
+          <t>Threshold</t>
+        </is>
+      </c>
+      <c r="J32" s="20" t="inlineStr">
+        <is>
+          <t>5K Wk 2 Sat - THRESHOLD 2x~1.9 k, Sonderborg (travel). PM 13:51. Moving 42:30 (6:14), elapsed 45:23. WU ~2 k 6:30-7:00 @145-155; 3 strides ~4:00-4:30 (hot); rep 1 ~1.9 k @ ~5:26-5:31 HR 177-182; ~2:15 jog; rep 2 ~1.9 k @ ~5:33 HR 176-184, faded last ~750 m; CD skipped. HR cap 175 broken both reps: +10 bpm vs 10/6 at same pace. Cadence reps 165/167. RPE n/r, shin n/r. Strava 20620965276.</t>
+        </is>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="37" t="n"/>
@@ -34032,18 +34053,28 @@
       </c>
     </row>
     <row r="62" ht="18" customHeight="1">
-      <c r="A62" s="35" t="n"/>
+      <c r="A62" s="35" t="n">
+        <v>46316</v>
+      </c>
       <c r="B62" s="16">
         <f>IF(A62="","",IFERROR(INT((A62-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C62" s="36" t="n"/>
-      <c r="D62" s="36" t="n"/>
+      <c r="C62" s="36" t="n">
+        <v>77.34999999999999</v>
+      </c>
+      <c r="D62" s="36" t="n">
+        <v>6.73</v>
+      </c>
       <c r="E62" s="36" t="n"/>
       <c r="F62" s="36" t="n"/>
       <c r="G62" s="36" t="n"/>
       <c r="H62" s="36" t="n"/>
-      <c r="I62" s="20" t="n"/>
+      <c r="I62" s="20" t="inlineStr">
+        <is>
+          <t>5K Wk 3 Wed - AM: sleep 6:44 (00:02-06:46) q7, RHR 45 (-1 vs 7d), mot 10/energy 9/stress 3, DOMS all 0, joints clean, SHIN CLEAN #49. BW 77.35 (+0.75 vs 10/15) single point after 6-day hole + travel weekend, no kcal change. 10/16-10/20: only Sat 10/17 run logged; Sun long, Mon gym, Tue 3 K TT not on Strava. Gates green -&gt; 3 K TT today PM or Thu.</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="18" customHeight="1">
       <c r="A63" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Wed 10/21 3 K TT done (15:00 moving / 15:42 elapsed, shin #50); sub-27 confirmed, PR decided by 4x1 k; xlsx Running 33
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -30453,22 +30453,45 @@
       </c>
     </row>
     <row r="33" ht="18" customHeight="1">
-      <c r="A33" s="37" t="n"/>
+      <c r="A33" s="37" t="n">
+        <v>46316</v>
+      </c>
       <c r="B33" s="22">
         <f>IF(A33="","",IFERROR(INT((A33-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C33" s="28" t="n"/>
-      <c r="D33" s="38" t="n"/>
+      <c r="C33" s="28" t="n">
+        <v>6.17</v>
+      </c>
+      <c r="D33" s="38" t="n">
+        <v>41</v>
+      </c>
       <c r="E33" s="22">
         <f>IF(OR(C33="",D33=""),"",TEXT(D33/C33/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F33" s="22" t="n"/>
-      <c r="G33" s="22" t="n"/>
-      <c r="H33" s="22" t="n"/>
-      <c r="I33" s="22" t="n"/>
-      <c r="J33" s="26" t="n"/>
+      <c r="F33" s="22" t="n">
+        <v>158</v>
+      </c>
+      <c r="G33" s="22" t="n">
+        <v>198</v>
+      </c>
+      <c r="H33" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="I33" s="22" t="inlineStr">
+        <is>
+          <t>3K TT</t>
+        </is>
+      </c>
+      <c r="J33" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 3 Wed - 3 K TIME TRIAL, road, Ballerup, AM 07:28. Total moving 41:00 / elapsed 41:56. WU 2 k 7:36@132 / 7:23@149 (cad 162/161), 4 strides ~4:20-4:35. TT 3.00 k GPS: km 5:00 / 5:00 (5:42 elapsed, ~43 s standing ~1.5 k, HR 190-&gt;150) / 5:01 = 15:00 moving / 15:42 elapsed. TT HR ~183-187, max 198, cad 166. RPE 8. CD skipped. GATE: sub-27 CONFIRMED, PR not opened (borderline + rest) -&gt; run 2 4x1 k @ 5:10-5:12 decides PR. SHIN CLEAN #50. Strava 20670617068.</t>
+        </is>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="35" t="n"/>
@@ -34072,7 +34095,7 @@
       <c r="H62" s="36" t="n"/>
       <c r="I62" s="20" t="inlineStr">
         <is>
-          <t>5K Wk 3 Wed - AM: sleep 6:44 (00:02-06:46) q7, RHR 45 (-1 vs 7d), mot 10/energy 9/stress 3, DOMS all 0, joints clean, SHIN CLEAN #49. BW 77.35 (+0.75 vs 10/15) single point after 6-day hole + travel weekend, no kcal change. 10/16-10/20: only Sat 10/17 run logged; Sun long, Mon gym, Tue 3 K TT not on Strava. Gates green -&gt; 3 K TT today PM or Thu.</t>
+          <t>5K Wk 3 Wed - AM: sleep 6:44 (00:02-06:46) q7, RHR 45 (-1 vs 7d), mot 10/energy 9/stress 3, DOMS all 0, joints clean, SHIN CLEAN #49. BW 77.35 (+0.75 vs 10/15) single point after 6-day hole + travel weekend, no kcal change. 10/16-10/20: only Sat 10/17 run logged; Sun long, Mon gym, Tue 3 K TT not on Strava. Gates green -&gt; 3 K TT today PM or Thu. PM: 3 K TT 15:00 moving / 15:42 elapsed (5:00/5:00/5:01), RPE 8, max HR 198, shin clean #50; bike 0, kcal 2272, protein 150, creatine Y, alcohol 0.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
sync: extend Weekly Summary to wk 27 (race week); stage Thu 10/22 rest + run 2 slot rule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -36649,7 +36649,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -37799,6 +37799,141 @@
       </c>
       <c r="K25" s="36">
         <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A25),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="16" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A26-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A26*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C26" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A26)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D26" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A26)</f>
+        <v/>
+      </c>
+      <c r="E26" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A26)</f>
+        <v/>
+      </c>
+      <c r="F26" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A26),"")</f>
+        <v/>
+      </c>
+      <c r="G26" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A26)</f>
+        <v/>
+      </c>
+      <c r="H26" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A26)</f>
+        <v/>
+      </c>
+      <c r="I26" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A26),"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A26),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="16" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A27-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A27*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C27" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A27)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D27" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A27)</f>
+        <v/>
+      </c>
+      <c r="E27" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A27)</f>
+        <v/>
+      </c>
+      <c r="F27" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A27),"")</f>
+        <v/>
+      </c>
+      <c r="G27" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A27)</f>
+        <v/>
+      </c>
+      <c r="H27" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A27)</f>
+        <v/>
+      </c>
+      <c r="I27" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A27)</f>
+        <v/>
+      </c>
+      <c r="J27" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A27),"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A27),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="16" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="16">
+        <f>TEXT(DATE(2026,4,27)+(A28-1)*7,"mmm d")&amp;" – "&amp;TEXT(DATE(2026,4,27)+A28*7-1,"mmm d")</f>
+        <v/>
+      </c>
+      <c r="C28" s="16">
+        <f>SUMPRODUCT(IFERROR((('Lifting Log'!B2:B801=A28)*('Lifting Log'!E2:E801=1))/COUNTIFS('Lifting Log'!A:A,'Lifting Log'!A2:A801,'Lifting Log'!E:E,1),0))</f>
+        <v/>
+      </c>
+      <c r="D28" s="16">
+        <f>COUNTIFS('Lifting Log'!B:B,A28)</f>
+        <v/>
+      </c>
+      <c r="E28" s="29">
+        <f>SUMIFS('Lifting Log'!I:I,'Lifting Log'!B:B,A28)</f>
+        <v/>
+      </c>
+      <c r="F28" s="36">
+        <f>IFERROR(AVERAGEIFS('Lifting Log'!H:H,'Lifting Log'!B:B,A28),"")</f>
+        <v/>
+      </c>
+      <c r="G28" s="16">
+        <f>COUNTIFS('Running Log'!B:B,A28)</f>
+        <v/>
+      </c>
+      <c r="H28" s="27">
+        <f>SUMIFS('Running Log'!C:C,'Running Log'!B:B,A28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="19">
+        <f>SUMIFS('Running Log'!D:D,'Running Log'!B:B,A28)</f>
+        <v/>
+      </c>
+      <c r="J28" s="19">
+        <f>IFERROR(AVERAGEIFS('Running Log'!F:F,'Running Log'!B:B,A28),"")</f>
+        <v/>
+      </c>
+      <c r="K28" s="36">
+        <f>IFERROR(AVERAGEIFS('Body Metrics'!C:C,'Body Metrics'!B:B,A28),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
log: Thu 10/22 AM (BW 77.35, RHR 44, calf DOMS 3); stage Gym #3 upper today; xlsx Body 63
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lifting Log" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Running Log" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Body Metrics" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personal Records" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Summary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Data" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Charts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Lifting Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Running Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Body Metrics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Personal Records" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Weekly Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Progression Data" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Reference" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -301,13 +301,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -330,7 +330,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -338,7 +338,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -364,7 +364,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -372,7 +372,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -398,7 +398,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -406,7 +406,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -432,7 +432,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -440,7 +440,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -466,7 +466,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -474,7 +474,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -500,7 +500,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -508,7 +508,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -534,7 +534,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -542,7 +542,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -568,7 +568,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -576,7 +576,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -605,8 +605,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -631,8 +631,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -658,13 +658,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -688,7 +688,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -719,8 +719,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -746,8 +746,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -770,13 +770,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -799,7 +799,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -807,7 +807,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -835,8 +835,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -863,8 +863,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -890,13 +890,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -919,7 +919,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -927,7 +927,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:ln>
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -960,8 +960,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,8 +987,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1014,13 +1014,13 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1044,7 +1044,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1075,8 +1075,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1102,8 +1102,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1126,13 +1126,13 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1156,7 +1156,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1187,8 +1187,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1214,8 +1214,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1238,7 +1238,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -1253,9 +1253,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1275,9 +1275,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+          <c:chart r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1297,9 +1297,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
+          <c:chart r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1319,9 +1319,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
+          <c:chart r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1341,9 +1341,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
+          <c:chart r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1363,9 +1363,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
+          <c:chart r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -34390,18 +34390,28 @@
       </c>
     </row>
     <row r="63" ht="18" customHeight="1">
-      <c r="A63" s="37" t="n"/>
+      <c r="A63" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B63" s="22">
         <f>IF(A63="","",IFERROR(INT((A63-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C63" s="38" t="n"/>
-      <c r="D63" s="38" t="n"/>
+      <c r="C63" s="38" t="n">
+        <v>77.34999999999999</v>
+      </c>
+      <c r="D63" s="38" t="n">
+        <v>7.58</v>
+      </c>
       <c r="E63" s="38" t="n"/>
       <c r="F63" s="38" t="n"/>
       <c r="G63" s="38" t="n"/>
       <c r="H63" s="38" t="n"/>
-      <c r="I63" s="26" t="n"/>
+      <c r="I63" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 3 Thu (TT +1) - AM: sleep 7:35 (00:05-07:40) q9, RHR 44 (-2 vs 7d), mot 10/energy 10/stress 2, DOMS upper 0, quad 2/ham 2/glute 1/calf 3, joints clean, shin not reported (asked). BW 77.35 = 10/21, flat 2nd post-travel reading, no kcal change. Calf 3 = TT cost -&gt; 4x1 k leans Sat 10/24 (Fri AM gate rules). Gym #3 upper moved Fri -&gt; today.</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="18" customHeight="1">
       <c r="A64" s="35" t="n"/>

</xml_diff>

<commit_message>
log: Thu 10/22 Gym #3 upper done (20 sets, 3006 kg, avg RPE 5.8, all gates met), shin #52; xlsx Lifting 519-538, Body 63 PM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -23208,17 +23208,35 @@
       <c r="K518" s="26" t="n"/>
     </row>
     <row r="519" ht="18" customHeight="1">
-      <c r="A519" s="37" t="n"/>
+      <c r="A519" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B519" s="22">
         <f>IF(A519="","",IFERROR(INT((A519-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C519" s="22" t="n"/>
-      <c r="D519" s="23" t="n"/>
-      <c r="E519" s="22" t="n"/>
-      <c r="F519" s="22" t="n"/>
-      <c r="G519" s="38" t="n"/>
-      <c r="H519" s="22" t="n"/>
+      <c r="C519" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D519" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E519" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F519" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G519" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H519" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I519" s="25">
         <f>IF(OR(F519="",G519=""),"",F519*G519)</f>
         <v/>
@@ -23227,20 +23245,42 @@
         <f>IF(OR(F519="",G519=""),"",ROUND(G519*(1+F519/30),1))</f>
         <v/>
       </c>
-      <c r="K519" s="26" t="n"/>
+      <c r="K519" s="26" t="inlineStr">
+        <is>
+          <t>Gym #3 upper. Gate met -&gt; 27.5 4x8.</t>
+        </is>
+      </c>
     </row>
     <row r="520" ht="18" customHeight="1">
-      <c r="A520" s="35" t="n"/>
+      <c r="A520" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B520" s="16">
         <f>IF(A520="","",IFERROR(INT((A520-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C520" s="16" t="n"/>
-      <c r="D520" s="17" t="n"/>
-      <c r="E520" s="16" t="n"/>
-      <c r="F520" s="16" t="n"/>
-      <c r="G520" s="36" t="n"/>
-      <c r="H520" s="16" t="n"/>
+      <c r="C520" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D520" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E520" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F520" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G520" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="H520" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I520" s="19">
         <f>IF(OR(F520="",G520=""),"",F520*G520)</f>
         <v/>
@@ -23252,17 +23292,35 @@
       <c r="K520" s="20" t="n"/>
     </row>
     <row r="521" ht="18" customHeight="1">
-      <c r="A521" s="37" t="n"/>
+      <c r="A521" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B521" s="22">
         <f>IF(A521="","",IFERROR(INT((A521-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C521" s="22" t="n"/>
-      <c r="D521" s="23" t="n"/>
-      <c r="E521" s="22" t="n"/>
-      <c r="F521" s="22" t="n"/>
-      <c r="G521" s="38" t="n"/>
-      <c r="H521" s="22" t="n"/>
+      <c r="C521" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D521" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E521" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F521" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G521" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H521" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I521" s="25">
         <f>IF(OR(F521="",G521=""),"",F521*G521)</f>
         <v/>
@@ -23274,17 +23332,35 @@
       <c r="K521" s="26" t="n"/>
     </row>
     <row r="522" ht="18" customHeight="1">
-      <c r="A522" s="35" t="n"/>
+      <c r="A522" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B522" s="16">
         <f>IF(A522="","",IFERROR(INT((A522-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C522" s="16" t="n"/>
-      <c r="D522" s="17" t="n"/>
-      <c r="E522" s="16" t="n"/>
-      <c r="F522" s="16" t="n"/>
-      <c r="G522" s="36" t="n"/>
-      <c r="H522" s="16" t="n"/>
+      <c r="C522" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D522" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E522" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F522" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G522" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="H522" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I522" s="19">
         <f>IF(OR(F522="",G522=""),"",F522*G522)</f>
         <v/>
@@ -23296,17 +23372,35 @@
       <c r="K522" s="20" t="n"/>
     </row>
     <row r="523" ht="18" customHeight="1">
-      <c r="A523" s="37" t="n"/>
+      <c r="A523" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B523" s="22">
         <f>IF(A523="","",IFERROR(INT((A523-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C523" s="22" t="n"/>
-      <c r="D523" s="23" t="n"/>
-      <c r="E523" s="22" t="n"/>
-      <c r="F523" s="22" t="n"/>
-      <c r="G523" s="38" t="n"/>
-      <c r="H523" s="22" t="n"/>
+      <c r="C523" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D523" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E523" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F523" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G523" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H523" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="I523" s="25">
         <f>IF(OR(F523="",G523=""),"",F523*G523)</f>
         <v/>
@@ -23315,20 +23409,42 @@
         <f>IF(OR(F523="",G523=""),"",ROUND(G523*(1+F523/30),1))</f>
         <v/>
       </c>
-      <c r="K523" s="26" t="n"/>
+      <c r="K523" s="26" t="inlineStr">
+        <is>
+          <t>Restored. Gate met -&gt; 27.5 4x10.</t>
+        </is>
+      </c>
     </row>
     <row r="524" ht="18" customHeight="1">
-      <c r="A524" s="35" t="n"/>
+      <c r="A524" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B524" s="16">
         <f>IF(A524="","",IFERROR(INT((A524-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C524" s="16" t="n"/>
-      <c r="D524" s="17" t="n"/>
-      <c r="E524" s="16" t="n"/>
-      <c r="F524" s="16" t="n"/>
-      <c r="G524" s="36" t="n"/>
-      <c r="H524" s="16" t="n"/>
+      <c r="C524" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D524" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E524" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F524" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G524" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="H524" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="I524" s="19">
         <f>IF(OR(F524="",G524=""),"",F524*G524)</f>
         <v/>
@@ -23340,17 +23456,35 @@
       <c r="K524" s="20" t="n"/>
     </row>
     <row r="525" ht="18" customHeight="1">
-      <c r="A525" s="37" t="n"/>
+      <c r="A525" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B525" s="22">
         <f>IF(A525="","",IFERROR(INT((A525-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C525" s="22" t="n"/>
-      <c r="D525" s="23" t="n"/>
-      <c r="E525" s="22" t="n"/>
-      <c r="F525" s="22" t="n"/>
-      <c r="G525" s="38" t="n"/>
-      <c r="H525" s="22" t="n"/>
+      <c r="C525" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D525" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E525" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F525" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G525" s="38" t="n">
+        <v>25</v>
+      </c>
+      <c r="H525" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="I525" s="25">
         <f>IF(OR(F525="",G525=""),"",F525*G525)</f>
         <v/>
@@ -23362,17 +23496,35 @@
       <c r="K525" s="26" t="n"/>
     </row>
     <row r="526" ht="18" customHeight="1">
-      <c r="A526" s="35" t="n"/>
+      <c r="A526" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B526" s="16">
         <f>IF(A526="","",IFERROR(INT((A526-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C526" s="16" t="n"/>
-      <c r="D526" s="17" t="n"/>
-      <c r="E526" s="16" t="n"/>
-      <c r="F526" s="16" t="n"/>
-      <c r="G526" s="36" t="n"/>
-      <c r="H526" s="16" t="n"/>
+      <c r="C526" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D526" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E526" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F526" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G526" s="36" t="n">
+        <v>25</v>
+      </c>
+      <c r="H526" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="I526" s="19">
         <f>IF(OR(F526="",G526=""),"",F526*G526)</f>
         <v/>
@@ -23384,17 +23536,35 @@
       <c r="K526" s="20" t="n"/>
     </row>
     <row r="527" ht="18" customHeight="1">
-      <c r="A527" s="37" t="n"/>
+      <c r="A527" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B527" s="22">
         <f>IF(A527="","",IFERROR(INT((A527-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C527" s="22" t="n"/>
-      <c r="D527" s="23" t="n"/>
-      <c r="E527" s="22" t="n"/>
-      <c r="F527" s="22" t="n"/>
-      <c r="G527" s="38" t="n"/>
-      <c r="H527" s="22" t="n"/>
+      <c r="C527" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D527" s="23" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E527" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F527" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G527" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="H527" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I527" s="25">
         <f>IF(OR(F527="",G527=""),"",F527*G527)</f>
         <v/>
@@ -23403,20 +23573,42 @@
         <f>IF(OR(F527="",G527=""),"",ROUND(G527*(1+F527/30),1))</f>
         <v/>
       </c>
-      <c r="K527" s="26" t="n"/>
+      <c r="K527" s="26" t="inlineStr">
+        <is>
+          <t>6/DB. Gate met -&gt; 7/DB 3x10.</t>
+        </is>
+      </c>
     </row>
     <row r="528" ht="18" customHeight="1">
-      <c r="A528" s="35" t="n"/>
+      <c r="A528" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B528" s="16">
         <f>IF(A528="","",IFERROR(INT((A528-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C528" s="16" t="n"/>
-      <c r="D528" s="17" t="n"/>
-      <c r="E528" s="16" t="n"/>
-      <c r="F528" s="16" t="n"/>
-      <c r="G528" s="36" t="n"/>
-      <c r="H528" s="16" t="n"/>
+      <c r="C528" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D528" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E528" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F528" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G528" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="H528" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I528" s="19">
         <f>IF(OR(F528="",G528=""),"",F528*G528)</f>
         <v/>
@@ -23428,17 +23620,35 @@
       <c r="K528" s="20" t="n"/>
     </row>
     <row r="529" ht="18" customHeight="1">
-      <c r="A529" s="37" t="n"/>
+      <c r="A529" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B529" s="22">
         <f>IF(A529="","",IFERROR(INT((A529-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C529" s="22" t="n"/>
-      <c r="D529" s="23" t="n"/>
-      <c r="E529" s="22" t="n"/>
-      <c r="F529" s="22" t="n"/>
-      <c r="G529" s="38" t="n"/>
-      <c r="H529" s="22" t="n"/>
+      <c r="C529" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D529" s="23" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E529" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F529" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G529" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="H529" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I529" s="25">
         <f>IF(OR(F529="",G529=""),"",F529*G529)</f>
         <v/>
@@ -23450,17 +23660,35 @@
       <c r="K529" s="26" t="n"/>
     </row>
     <row r="530" ht="18" customHeight="1">
-      <c r="A530" s="35" t="n"/>
+      <c r="A530" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B530" s="16">
         <f>IF(A530="","",IFERROR(INT((A530-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C530" s="16" t="n"/>
-      <c r="D530" s="17" t="n"/>
-      <c r="E530" s="16" t="n"/>
-      <c r="F530" s="16" t="n"/>
-      <c r="G530" s="36" t="n"/>
-      <c r="H530" s="16" t="n"/>
+      <c r="C530" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D530" s="17" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E530" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F530" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G530" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="H530" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I530" s="19">
         <f>IF(OR(F530="",G530=""),"",F530*G530)</f>
         <v/>
@@ -23469,20 +23697,42 @@
         <f>IF(OR(F530="",G530=""),"",ROUND(G530*(1+F530/30),1))</f>
         <v/>
       </c>
-      <c r="K530" s="20" t="n"/>
+      <c r="K530" s="20" t="inlineStr">
+        <is>
+          <t>Barbell Row 20 (staged Lying Row 32.5). Gate met -&gt; 22.5 3x12.</t>
+        </is>
+      </c>
     </row>
     <row r="531" ht="18" customHeight="1">
-      <c r="A531" s="37" t="n"/>
+      <c r="A531" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B531" s="22">
         <f>IF(A531="","",IFERROR(INT((A531-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C531" s="22" t="n"/>
-      <c r="D531" s="23" t="n"/>
-      <c r="E531" s="22" t="n"/>
-      <c r="F531" s="22" t="n"/>
-      <c r="G531" s="38" t="n"/>
-      <c r="H531" s="22" t="n"/>
+      <c r="C531" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D531" s="23" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E531" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F531" s="22" t="n">
+        <v>12</v>
+      </c>
+      <c r="G531" s="38" t="n">
+        <v>20</v>
+      </c>
+      <c r="H531" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I531" s="25">
         <f>IF(OR(F531="",G531=""),"",F531*G531)</f>
         <v/>
@@ -23494,17 +23744,35 @@
       <c r="K531" s="26" t="n"/>
     </row>
     <row r="532" ht="18" customHeight="1">
-      <c r="A532" s="35" t="n"/>
+      <c r="A532" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B532" s="16">
         <f>IF(A532="","",IFERROR(INT((A532-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C532" s="16" t="n"/>
-      <c r="D532" s="17" t="n"/>
-      <c r="E532" s="16" t="n"/>
-      <c r="F532" s="16" t="n"/>
-      <c r="G532" s="36" t="n"/>
-      <c r="H532" s="16" t="n"/>
+      <c r="C532" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D532" s="17" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E532" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F532" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G532" s="36" t="n">
+        <v>20</v>
+      </c>
+      <c r="H532" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I532" s="19">
         <f>IF(OR(F532="",G532=""),"",F532*G532)</f>
         <v/>
@@ -23516,17 +23784,35 @@
       <c r="K532" s="20" t="n"/>
     </row>
     <row r="533" ht="18" customHeight="1">
-      <c r="A533" s="37" t="n"/>
+      <c r="A533" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B533" s="22">
         <f>IF(A533="","",IFERROR(INT((A533-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C533" s="22" t="n"/>
-      <c r="D533" s="23" t="n"/>
-      <c r="E533" s="22" t="n"/>
-      <c r="F533" s="22" t="n"/>
-      <c r="G533" s="38" t="n"/>
-      <c r="H533" s="22" t="n"/>
+      <c r="C533" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D533" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E533" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F533" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G533" s="38" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H533" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I533" s="25">
         <f>IF(OR(F533="",G533=""),"",F533*G533)</f>
         <v/>
@@ -23535,20 +23821,42 @@
         <f>IF(OR(F533="",G533=""),"",ROUND(G533*(1+F533/30),1))</f>
         <v/>
       </c>
-      <c r="K533" s="26" t="n"/>
+      <c r="K533" s="26" t="inlineStr">
+        <is>
+          <t>Gate met 2nd session -&gt; reps first: 6.8 3x20.</t>
+        </is>
+      </c>
     </row>
     <row r="534" ht="18" customHeight="1">
-      <c r="A534" s="35" t="n"/>
+      <c r="A534" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B534" s="16">
         <f>IF(A534="","",IFERROR(INT((A534-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C534" s="16" t="n"/>
-      <c r="D534" s="17" t="n"/>
-      <c r="E534" s="16" t="n"/>
-      <c r="F534" s="16" t="n"/>
-      <c r="G534" s="36" t="n"/>
-      <c r="H534" s="16" t="n"/>
+      <c r="C534" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D534" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E534" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F534" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G534" s="36" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H534" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="I534" s="19">
         <f>IF(OR(F534="",G534=""),"",F534*G534)</f>
         <v/>
@@ -23560,17 +23868,35 @@
       <c r="K534" s="20" t="n"/>
     </row>
     <row r="535" ht="18" customHeight="1">
-      <c r="A535" s="37" t="n"/>
+      <c r="A535" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B535" s="22">
         <f>IF(A535="","",IFERROR(INT((A535-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C535" s="22" t="n"/>
-      <c r="D535" s="23" t="n"/>
-      <c r="E535" s="22" t="n"/>
-      <c r="F535" s="22" t="n"/>
-      <c r="G535" s="38" t="n"/>
-      <c r="H535" s="22" t="n"/>
+      <c r="C535" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D535" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E535" s="22" t="n">
+        <v>3</v>
+      </c>
+      <c r="F535" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G535" s="38" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H535" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="I535" s="25">
         <f>IF(OR(F535="",G535=""),"",F535*G535)</f>
         <v/>
@@ -23582,17 +23908,33 @@
       <c r="K535" s="26" t="n"/>
     </row>
     <row r="536" ht="18" customHeight="1">
-      <c r="A536" s="35" t="n"/>
+      <c r="A536" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B536" s="16">
         <f>IF(A536="","",IFERROR(INT((A536-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C536" s="16" t="n"/>
-      <c r="D536" s="17" t="n"/>
-      <c r="E536" s="16" t="n"/>
-      <c r="F536" s="16" t="n"/>
+      <c r="C536" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D536" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E536" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F536" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="G536" s="36" t="n"/>
-      <c r="H536" s="16" t="n"/>
+      <c r="H536" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I536" s="19">
         <f>IF(OR(F536="",G536=""),"",F536*G536)</f>
         <v/>
@@ -23601,20 +23943,40 @@
         <f>IF(OR(F536="",G536=""),"",ROUND(G536*(1+F536/30),1))</f>
         <v/>
       </c>
-      <c r="K536" s="20" t="n"/>
+      <c r="K536" s="20" t="inlineStr">
+        <is>
+          <t>Gate met -&gt; 3x12.</t>
+        </is>
+      </c>
     </row>
     <row r="537" ht="18" customHeight="1">
-      <c r="A537" s="37" t="n"/>
+      <c r="A537" s="37" t="n">
+        <v>46317</v>
+      </c>
       <c r="B537" s="22">
         <f>IF(A537="","",IFERROR(INT((A537-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C537" s="22" t="n"/>
-      <c r="D537" s="23" t="n"/>
-      <c r="E537" s="22" t="n"/>
-      <c r="F537" s="22" t="n"/>
+      <c r="C537" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D537" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E537" s="22" t="n">
+        <v>2</v>
+      </c>
+      <c r="F537" s="22" t="n">
+        <v>10</v>
+      </c>
       <c r="G537" s="38" t="n"/>
-      <c r="H537" s="22" t="n"/>
+      <c r="H537" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I537" s="25">
         <f>IF(OR(F537="",G537=""),"",F537*G537)</f>
         <v/>
@@ -23626,17 +23988,33 @@
       <c r="K537" s="26" t="n"/>
     </row>
     <row r="538" ht="18" customHeight="1">
-      <c r="A538" s="35" t="n"/>
+      <c r="A538" s="35" t="n">
+        <v>46317</v>
+      </c>
       <c r="B538" s="16">
         <f>IF(A538="","",IFERROR(INT((A538-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C538" s="16" t="n"/>
-      <c r="D538" s="17" t="n"/>
-      <c r="E538" s="16" t="n"/>
-      <c r="F538" s="16" t="n"/>
+      <c r="C538" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D538" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E538" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F538" s="16" t="n">
+        <v>10</v>
+      </c>
       <c r="G538" s="36" t="n"/>
-      <c r="H538" s="16" t="n"/>
+      <c r="H538" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I538" s="19">
         <f>IF(OR(F538="",G538=""),"",F538*G538)</f>
         <v/>
@@ -34409,7 +34787,7 @@
       <c r="H63" s="38" t="n"/>
       <c r="I63" s="26" t="inlineStr">
         <is>
-          <t>5K Wk 3 Thu (TT +1) - AM: sleep 7:35 (00:05-07:40) q9, RHR 44 (-2 vs 7d), mot 10/energy 10/stress 2, DOMS upper 0, quad 2/ham 2/glute 1/calf 3, joints clean, shin not reported (asked). BW 77.35 = 10/21, flat 2nd post-travel reading, no kcal change. Calf 3 = TT cost -&gt; 4x1 k leans Sat 10/24 (Fri AM gate rules). Gym #3 upper moved Fri -&gt; today.</t>
+          <t>5K Wk 3 Thu (TT +1) - AM: sleep 7:35 (00:05-07:40) q9, RHR 44 (-2 vs 7d), mot 10/energy 10/stress 2, DOMS upper 0, quad 2/ham 2/glute 1/calf 3, joints clean, shin not reported (asked). BW 77.35 = 10/21, flat 2nd post-travel reading, no kcal change. Calf 3 = TT cost -&gt; 4x1 k leans Sat 10/24 (Fri AM gate rules). Gym #3 upper moved Fri -&gt; today. PM: Gym #3 upper DONE 20 sets / 3006 kg / avg RPE 5.8, all gates met; shin clean #52; bike 0, kcal 2344, protein 176, creatine Y.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
log: Fri 10/23 AM (BW 76.90, RHR 44, calf 1, shin #53); 4x1 k gate green -> Fri PM, Sat fallback; xlsx Body 64
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -1,21 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Charts" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Lifting Log" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Running Log" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Body Metrics" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Personal Records" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Weekly Summary" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Progression Data" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Reference" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Charts" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Lifting Log" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Running Log" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Body Metrics" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Personal Records" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Weekly Summary" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Progression Data" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -301,13 +301,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -330,7 +330,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -338,7 +338,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -364,7 +364,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -372,7 +372,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -398,7 +398,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -406,7 +406,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -432,7 +432,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -440,7 +440,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -466,7 +466,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -474,7 +474,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -500,7 +500,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -508,7 +508,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -534,7 +534,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -542,7 +542,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -568,7 +568,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -576,7 +576,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -605,8 +605,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -631,8 +631,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -658,13 +658,13 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -688,7 +688,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -719,8 +719,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -746,8 +746,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -770,13 +770,13 @@
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -799,7 +799,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -807,7 +807,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -835,8 +835,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -863,8 +863,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -890,13 +890,13 @@
 </file>
 
 <file path=xl/charts/chart4.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -919,7 +919,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -927,7 +927,7 @@
             <symbol val="circle"/>
             <size val="6"/>
             <spPr>
-              <a:ln>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:prstDash val="solid"/>
               </a:ln>
             </spPr>
@@ -960,8 +960,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -987,8 +987,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1014,13 +1014,13 @@
 </file>
 
 <file path=xl/charts/chart5.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1044,7 +1044,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1075,8 +1075,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1102,8 +1102,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1126,13 +1126,13 @@
 </file>
 
 <file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -1156,7 +1156,7 @@
             </strRef>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -1187,8 +1187,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1214,8 +1214,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -1238,7 +1238,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>1</col>
@@ -1253,9 +1253,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1275,9 +1275,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId2"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1297,9 +1297,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId3"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1319,9 +1319,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId4"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId4"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1341,9 +1341,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId5"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId5"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1363,9 +1363,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId6"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId6"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -34792,18 +34792,28 @@
       </c>
     </row>
     <row r="64" ht="18" customHeight="1">
-      <c r="A64" s="35" t="n"/>
+      <c r="A64" s="37" t="n">
+        <v>46318</v>
+      </c>
       <c r="B64" s="16">
         <f>IF(A64="","",IFERROR(INT((A64-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C64" s="36" t="n"/>
-      <c r="D64" s="36" t="n"/>
+      <c r="C64" s="38" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="D64" s="38" t="n">
+        <v>8.130000000000001</v>
+      </c>
       <c r="E64" s="36" t="n"/>
       <c r="F64" s="36" t="n"/>
       <c r="G64" s="36" t="n"/>
       <c r="H64" s="36" t="n"/>
-      <c r="I64" s="20" t="n"/>
+      <c r="I64" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 3 Fri (TT +2) - AM: sleep 8:08 (23:35-07:43) q8, RHR 44 (-1 vs 7d), mot 10/energy 10/stress 3, DOMS chest 3/shldr 3/back 2/arm 0 (Gym #3), quad 1/ham 1/glute 1/calf 1, tendons clean, SHIN CLEAN #53. BW 76.90 (-0.45 vs 77.35x2) water, no kcal change. Gate green -&gt; 4x1 k PR decider Fri PM, Sat fallback.</t>
+        </is>
+      </c>
     </row>
     <row r="65" ht="18" customHeight="1">
       <c r="A65" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Fri 10/23 4x1 k PR decider PARTIAL (5:21/5:00/5:35 fade/DNF, RPE 10) -> PR closed, race sub-26:40; stage Sat rest, Sun 8 k, race week; xlsx Running 34, Body 64 PM
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -31162,22 +31162,45 @@
       </c>
     </row>
     <row r="34" ht="18" customHeight="1">
-      <c r="A34" s="35" t="n"/>
+      <c r="A34" s="37" t="n">
+        <v>46318</v>
+      </c>
       <c r="B34" s="16">
         <f>IF(A34="","",IFERROR(INT((A34-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C34" s="27" t="n"/>
-      <c r="D34" s="36" t="n"/>
-      <c r="E34" s="16">
+      <c r="C34" s="28" t="n">
+        <v>7.01</v>
+      </c>
+      <c r="D34" s="38" t="n">
+        <v>48.85</v>
+      </c>
+      <c r="E34" s="22">
         <f>IF(OR(C34="",D34=""),"",TEXT(D34/C34/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F34" s="16" t="n"/>
-      <c r="G34" s="16" t="n"/>
-      <c r="H34" s="16" t="n"/>
-      <c r="I34" s="16" t="n"/>
-      <c r="J34" s="20" t="n"/>
+      <c r="F34" s="22" t="n">
+        <v>155</v>
+      </c>
+      <c r="G34" s="22" t="n">
+        <v>191</v>
+      </c>
+      <c r="H34" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="I34" s="22" t="inlineStr">
+        <is>
+          <t>4x1 k PR decider</t>
+        </is>
+      </c>
+      <c r="J34" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 3 Fri - 4x1 k PR DECIDER, PARTIAL (3 of 4). Road, Ballerup, AM 08:18 (plan was PM; ~40 h post-TT). Moving 48:51 / elapsed 49:23. WU ~2.1 k 7:41@139 (cad 159-160), 3 strides ~5:10-5:50. Rep 1 5:21 (HR 171/184) · Rep 2 5:00 (HR 184/191, 8 s/km under the 5:08 ceiling) · Rep 3 ~980 m 5:35 (680 m @ 5:24 then 6:02 fade), stopped · Rep 4 not run. Jogs 2:54/2:59, HR ~170. CD walked. RPE 10, no pain. VERDICT: PR CLOSED -&gt; race sub-26:40 (laps 2:08). SHIN CLEAN #54. Strava 20697205297.</t>
+        </is>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="37" t="n"/>
@@ -34811,7 +34834,7 @@
       <c r="H64" s="36" t="n"/>
       <c r="I64" s="26" t="inlineStr">
         <is>
-          <t>5K Wk 3 Fri (TT +2) - AM: sleep 8:08 (23:35-07:43) q8, RHR 44 (-1 vs 7d), mot 10/energy 10/stress 3, DOMS chest 3/shldr 3/back 2/arm 0 (Gym #3), quad 1/ham 1/glute 1/calf 1, tendons clean, SHIN CLEAN #53. BW 76.90 (-0.45 vs 77.35x2) water, no kcal change. Gate green -&gt; 4x1 k PR decider Fri PM, Sat fallback.</t>
+          <t>5K Wk 3 Fri (TT +2) - AM: sleep 8:08 (23:35-07:43) q8, RHR 44 (-1 vs 7d), mot 10/energy 10/stress 3, DOMS chest 3/shldr 3/back 2/arm 0 (Gym #3), quad 1/ham 1/glute 1/calf 1, tendons clean, SHIN CLEAN #53. BW 76.90 (-0.45 vs 77.35x2) water, no kcal change. Gate green -&gt; 4x1 k PR decider Fri PM, Sat fallback. PM: 4x1 k PR decider ran 08:18 road - 5:21/5:00/5:35 fade/DNF, RPE 10, shin clean #54 -&gt; PR CLOSED, race sub-26:40; bike 0, kcal 2567, protein 175, creatine Y, alcohol 0.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
log: Sat 10/24 Gym #4 upper DONE (3376 kg, avg RPE 6.85); Sun 10/25 rest; stage Mon 10/26 easy 5 k
- Gym #4: Bench 27.5 4x8 (S4 RPE 8 -> hold), Lat PD ran 30 (gate met -> 32.5), Incline ran 6/DB (-> 7), Row 22.5 (-> 25), Tib 6.8 3x15, HKR 3x12 (8/9/8 -> hold). Shin clean #56.
- Sun 8 k moved to rest (user's call), no make-up. Wk 3 = 2 runs / 13.18 km.
- Mon 10/26 rest -> easy 5 k AM so Tue 3x1 k is not off a 4-day running gap; calf >=2 -> rest.
- xlsx: Lifting 539-558 (Gym #4), Body 65 PM note, Body 66 (10/25 rest).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -24026,39 +24026,79 @@
       <c r="K538" s="20" t="n"/>
     </row>
     <row r="539" ht="18" customHeight="1">
-      <c r="A539" s="37" t="n"/>
-      <c r="B539" s="22">
+      <c r="A539" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B539" s="16">
         <f>IF(A539="","",IFERROR(INT((A539-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C539" s="22" t="n"/>
-      <c r="D539" s="23" t="n"/>
-      <c r="E539" s="22" t="n"/>
-      <c r="F539" s="22" t="n"/>
-      <c r="G539" s="38" t="n"/>
-      <c r="H539" s="22" t="n"/>
-      <c r="I539" s="25">
+      <c r="C539" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D539" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E539" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F539" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G539" s="36" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H539" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I539" s="19">
         <f>IF(OR(F539="",G539=""),"",F539*G539)</f>
         <v/>
       </c>
-      <c r="J539" s="38">
+      <c r="J539" s="36">
         <f>IF(OR(F539="",G539=""),"",ROUND(G539*(1+F539/30),1))</f>
         <v/>
       </c>
-      <c r="K539" s="26" t="n"/>
+      <c r="K539" s="20" t="inlineStr">
+        <is>
+          <t>Gym #4 upper. S4 RPE 8 -&gt; HOLD 27.5 4x8.</t>
+        </is>
+      </c>
     </row>
     <row r="540" ht="18" customHeight="1">
-      <c r="A540" s="35" t="n"/>
+      <c r="A540" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B540" s="16">
         <f>IF(A540="","",IFERROR(INT((A540-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C540" s="16" t="n"/>
-      <c r="D540" s="17" t="n"/>
-      <c r="E540" s="16" t="n"/>
-      <c r="F540" s="16" t="n"/>
-      <c r="G540" s="36" t="n"/>
-      <c r="H540" s="16" t="n"/>
+      <c r="C540" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D540" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E540" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F540" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G540" s="36" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H540" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I540" s="19">
         <f>IF(OR(F540="",G540=""),"",F540*G540)</f>
         <v/>
@@ -24070,39 +24110,75 @@
       <c r="K540" s="20" t="n"/>
     </row>
     <row r="541" ht="18" customHeight="1">
-      <c r="A541" s="37" t="n"/>
-      <c r="B541" s="22">
+      <c r="A541" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B541" s="16">
         <f>IF(A541="","",IFERROR(INT((A541-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C541" s="22" t="n"/>
-      <c r="D541" s="23" t="n"/>
-      <c r="E541" s="22" t="n"/>
-      <c r="F541" s="22" t="n"/>
-      <c r="G541" s="38" t="n"/>
-      <c r="H541" s="22" t="n"/>
-      <c r="I541" s="25">
+      <c r="C541" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D541" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E541" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F541" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G541" s="36" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H541" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="I541" s="19">
         <f>IF(OR(F541="",G541=""),"",F541*G541)</f>
         <v/>
       </c>
-      <c r="J541" s="38">
+      <c r="J541" s="36">
         <f>IF(OR(F541="",G541=""),"",ROUND(G541*(1+F541/30),1))</f>
         <v/>
       </c>
-      <c r="K541" s="26" t="n"/>
+      <c r="K541" s="20" t="n"/>
     </row>
     <row r="542" ht="18" customHeight="1">
-      <c r="A542" s="35" t="n"/>
+      <c r="A542" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B542" s="16">
         <f>IF(A542="","",IFERROR(INT((A542-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C542" s="16" t="n"/>
-      <c r="D542" s="17" t="n"/>
-      <c r="E542" s="16" t="n"/>
-      <c r="F542" s="16" t="n"/>
-      <c r="G542" s="36" t="n"/>
-      <c r="H542" s="16" t="n"/>
+      <c r="C542" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D542" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E542" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F542" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G542" s="36" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H542" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I542" s="19">
         <f>IF(OR(F542="",G542=""),"",F542*G542)</f>
         <v/>
@@ -24114,39 +24190,79 @@
       <c r="K542" s="20" t="n"/>
     </row>
     <row r="543" ht="18" customHeight="1">
-      <c r="A543" s="37" t="n"/>
-      <c r="B543" s="22">
+      <c r="A543" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B543" s="16">
         <f>IF(A543="","",IFERROR(INT((A543-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C543" s="22" t="n"/>
-      <c r="D543" s="23" t="n"/>
-      <c r="E543" s="22" t="n"/>
-      <c r="F543" s="22" t="n"/>
-      <c r="G543" s="38" t="n"/>
-      <c r="H543" s="22" t="n"/>
-      <c r="I543" s="25">
+      <c r="C543" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D543" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E543" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F543" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G543" s="36" t="n">
+        <v>30</v>
+      </c>
+      <c r="H543" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I543" s="19">
         <f>IF(OR(F543="",G543=""),"",F543*G543)</f>
         <v/>
       </c>
-      <c r="J543" s="38">
+      <c r="J543" s="36">
         <f>IF(OR(F543="",G543=""),"",ROUND(G543*(1+F543/30),1))</f>
         <v/>
       </c>
-      <c r="K543" s="26" t="n"/>
+      <c r="K543" s="20" t="inlineStr">
+        <is>
+          <t>Ran 30 (staged 27.5). Gate met -&gt; 32.5 4x10.</t>
+        </is>
+      </c>
     </row>
     <row r="544" ht="18" customHeight="1">
-      <c r="A544" s="35" t="n"/>
+      <c r="A544" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B544" s="16">
         <f>IF(A544="","",IFERROR(INT((A544-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C544" s="16" t="n"/>
-      <c r="D544" s="17" t="n"/>
-      <c r="E544" s="16" t="n"/>
-      <c r="F544" s="16" t="n"/>
-      <c r="G544" s="36" t="n"/>
-      <c r="H544" s="16" t="n"/>
+      <c r="C544" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D544" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E544" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F544" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G544" s="36" t="n">
+        <v>30</v>
+      </c>
+      <c r="H544" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I544" s="19">
         <f>IF(OR(F544="",G544=""),"",F544*G544)</f>
         <v/>
@@ -24158,39 +24274,75 @@
       <c r="K544" s="20" t="n"/>
     </row>
     <row r="545" ht="18" customHeight="1">
-      <c r="A545" s="37" t="n"/>
-      <c r="B545" s="22">
+      <c r="A545" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B545" s="16">
         <f>IF(A545="","",IFERROR(INT((A545-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C545" s="22" t="n"/>
-      <c r="D545" s="23" t="n"/>
-      <c r="E545" s="22" t="n"/>
-      <c r="F545" s="22" t="n"/>
-      <c r="G545" s="38" t="n"/>
-      <c r="H545" s="22" t="n"/>
-      <c r="I545" s="25">
+      <c r="C545" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D545" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E545" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F545" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G545" s="36" t="n">
+        <v>30</v>
+      </c>
+      <c r="H545" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="I545" s="19">
         <f>IF(OR(F545="",G545=""),"",F545*G545)</f>
         <v/>
       </c>
-      <c r="J545" s="38">
+      <c r="J545" s="36">
         <f>IF(OR(F545="",G545=""),"",ROUND(G545*(1+F545/30),1))</f>
         <v/>
       </c>
-      <c r="K545" s="26" t="n"/>
+      <c r="K545" s="20" t="n"/>
     </row>
     <row r="546" ht="18" customHeight="1">
-      <c r="A546" s="35" t="n"/>
+      <c r="A546" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B546" s="16">
         <f>IF(A546="","",IFERROR(INT((A546-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C546" s="16" t="n"/>
-      <c r="D546" s="17" t="n"/>
-      <c r="E546" s="16" t="n"/>
-      <c r="F546" s="16" t="n"/>
-      <c r="G546" s="36" t="n"/>
-      <c r="H546" s="16" t="n"/>
+      <c r="C546" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D546" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E546" s="16" t="n">
+        <v>4</v>
+      </c>
+      <c r="F546" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G546" s="36" t="n">
+        <v>30</v>
+      </c>
+      <c r="H546" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I546" s="19">
         <f>IF(OR(F546="",G546=""),"",F546*G546)</f>
         <v/>
@@ -24202,39 +24354,79 @@
       <c r="K546" s="20" t="n"/>
     </row>
     <row r="547" ht="18" customHeight="1">
-      <c r="A547" s="37" t="n"/>
-      <c r="B547" s="22">
+      <c r="A547" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B547" s="16">
         <f>IF(A547="","",IFERROR(INT((A547-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C547" s="22" t="n"/>
-      <c r="D547" s="23" t="n"/>
-      <c r="E547" s="22" t="n"/>
-      <c r="F547" s="22" t="n"/>
-      <c r="G547" s="38" t="n"/>
-      <c r="H547" s="22" t="n"/>
-      <c r="I547" s="25">
+      <c r="C547" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D547" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E547" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F547" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G547" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="H547" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I547" s="19">
         <f>IF(OR(F547="",G547=""),"",F547*G547)</f>
         <v/>
       </c>
-      <c r="J547" s="38">
+      <c r="J547" s="36">
         <f>IF(OR(F547="",G547=""),"",ROUND(G547*(1+F547/30),1))</f>
         <v/>
       </c>
-      <c r="K547" s="26" t="n"/>
+      <c r="K547" s="20" t="inlineStr">
+        <is>
+          <t>6/DB (staged 7). Gate met -&gt; 7/DB 3x10.</t>
+        </is>
+      </c>
     </row>
     <row r="548" ht="18" customHeight="1">
-      <c r="A548" s="35" t="n"/>
+      <c r="A548" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B548" s="16">
         <f>IF(A548="","",IFERROR(INT((A548-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C548" s="16" t="n"/>
-      <c r="D548" s="17" t="n"/>
-      <c r="E548" s="16" t="n"/>
-      <c r="F548" s="16" t="n"/>
-      <c r="G548" s="36" t="n"/>
-      <c r="H548" s="16" t="n"/>
+      <c r="C548" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D548" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E548" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F548" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G548" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="H548" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I548" s="19">
         <f>IF(OR(F548="",G548=""),"",F548*G548)</f>
         <v/>
@@ -24246,39 +24438,75 @@
       <c r="K548" s="20" t="n"/>
     </row>
     <row r="549" ht="18" customHeight="1">
-      <c r="A549" s="37" t="n"/>
-      <c r="B549" s="22">
+      <c r="A549" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B549" s="16">
         <f>IF(A549="","",IFERROR(INT((A549-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C549" s="22" t="n"/>
-      <c r="D549" s="23" t="n"/>
-      <c r="E549" s="22" t="n"/>
-      <c r="F549" s="22" t="n"/>
-      <c r="G549" s="38" t="n"/>
-      <c r="H549" s="22" t="n"/>
-      <c r="I549" s="25">
+      <c r="C549" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D549" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E549" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F549" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G549" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="H549" s="16" t="n">
+        <v>5</v>
+      </c>
+      <c r="I549" s="19">
         <f>IF(OR(F549="",G549=""),"",F549*G549)</f>
         <v/>
       </c>
-      <c r="J549" s="38">
+      <c r="J549" s="36">
         <f>IF(OR(F549="",G549=""),"",ROUND(G549*(1+F549/30),1))</f>
         <v/>
       </c>
-      <c r="K549" s="26" t="n"/>
+      <c r="K549" s="20" t="n"/>
     </row>
     <row r="550" ht="18" customHeight="1">
-      <c r="A550" s="35" t="n"/>
+      <c r="A550" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B550" s="16">
         <f>IF(A550="","",IFERROR(INT((A550-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C550" s="16" t="n"/>
-      <c r="D550" s="17" t="n"/>
-      <c r="E550" s="16" t="n"/>
-      <c r="F550" s="16" t="n"/>
-      <c r="G550" s="36" t="n"/>
-      <c r="H550" s="16" t="n"/>
+      <c r="C550" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D550" s="17" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E550" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F550" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G550" s="36" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H550" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I550" s="19">
         <f>IF(OR(F550="",G550=""),"",F550*G550)</f>
         <v/>
@@ -24287,42 +24515,82 @@
         <f>IF(OR(F550="",G550=""),"",ROUND(G550*(1+F550/30),1))</f>
         <v/>
       </c>
-      <c r="K550" s="20" t="n"/>
+      <c r="K550" s="20" t="inlineStr">
+        <is>
+          <t>Gate met -&gt; 25 3x12.</t>
+        </is>
+      </c>
     </row>
     <row r="551" ht="18" customHeight="1">
-      <c r="A551" s="37" t="n"/>
-      <c r="B551" s="22">
+      <c r="A551" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B551" s="16">
         <f>IF(A551="","",IFERROR(INT((A551-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C551" s="22" t="n"/>
-      <c r="D551" s="23" t="n"/>
-      <c r="E551" s="22" t="n"/>
-      <c r="F551" s="22" t="n"/>
-      <c r="G551" s="38" t="n"/>
-      <c r="H551" s="22" t="n"/>
-      <c r="I551" s="25">
+      <c r="C551" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D551" s="17" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E551" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F551" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G551" s="36" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H551" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="I551" s="19">
         <f>IF(OR(F551="",G551=""),"",F551*G551)</f>
         <v/>
       </c>
-      <c r="J551" s="38">
+      <c r="J551" s="36">
         <f>IF(OR(F551="",G551=""),"",ROUND(G551*(1+F551/30),1))</f>
         <v/>
       </c>
-      <c r="K551" s="26" t="n"/>
+      <c r="K551" s="20" t="n"/>
     </row>
     <row r="552" ht="18" customHeight="1">
-      <c r="A552" s="35" t="n"/>
+      <c r="A552" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B552" s="16">
         <f>IF(A552="","",IFERROR(INT((A552-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C552" s="16" t="n"/>
-      <c r="D552" s="17" t="n"/>
-      <c r="E552" s="16" t="n"/>
-      <c r="F552" s="16" t="n"/>
-      <c r="G552" s="36" t="n"/>
-      <c r="H552" s="16" t="n"/>
+      <c r="C552" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D552" s="17" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E552" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F552" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G552" s="36" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H552" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I552" s="19">
         <f>IF(OR(F552="",G552=""),"",F552*G552)</f>
         <v/>
@@ -24334,39 +24602,79 @@
       <c r="K552" s="20" t="n"/>
     </row>
     <row r="553" ht="18" customHeight="1">
-      <c r="A553" s="37" t="n"/>
-      <c r="B553" s="22">
+      <c r="A553" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B553" s="16">
         <f>IF(A553="","",IFERROR(INT((A553-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C553" s="22" t="n"/>
-      <c r="D553" s="23" t="n"/>
-      <c r="E553" s="22" t="n"/>
-      <c r="F553" s="22" t="n"/>
-      <c r="G553" s="38" t="n"/>
-      <c r="H553" s="22" t="n"/>
-      <c r="I553" s="25">
+      <c r="C553" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D553" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E553" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F553" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G553" s="36" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H553" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="I553" s="19">
         <f>IF(OR(F553="",G553=""),"",F553*G553)</f>
         <v/>
       </c>
-      <c r="J553" s="38">
+      <c r="J553" s="36">
         <f>IF(OR(F553="",G553=""),"",ROUND(G553*(1+F553/30),1))</f>
         <v/>
       </c>
-      <c r="K553" s="26" t="n"/>
+      <c r="K553" s="20" t="inlineStr">
+        <is>
+          <t>Held 3x15 (race wk, calf 3 AM). Post-race -&gt; 6.8 3x20.</t>
+        </is>
+      </c>
     </row>
     <row r="554" ht="18" customHeight="1">
-      <c r="A554" s="35" t="n"/>
+      <c r="A554" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B554" s="16">
         <f>IF(A554="","",IFERROR(INT((A554-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C554" s="16" t="n"/>
-      <c r="D554" s="17" t="n"/>
-      <c r="E554" s="16" t="n"/>
-      <c r="F554" s="16" t="n"/>
-      <c r="G554" s="36" t="n"/>
-      <c r="H554" s="16" t="n"/>
+      <c r="C554" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D554" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E554" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F554" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G554" s="36" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H554" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I554" s="19">
         <f>IF(OR(F554="",G554=""),"",F554*G554)</f>
         <v/>
@@ -24378,39 +24686,73 @@
       <c r="K554" s="20" t="n"/>
     </row>
     <row r="555" ht="18" customHeight="1">
-      <c r="A555" s="37" t="n"/>
-      <c r="B555" s="22">
+      <c r="A555" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B555" s="16">
         <f>IF(A555="","",IFERROR(INT((A555-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C555" s="22" t="n"/>
-      <c r="D555" s="23" t="n"/>
-      <c r="E555" s="22" t="n"/>
-      <c r="F555" s="22" t="n"/>
-      <c r="G555" s="38" t="n"/>
-      <c r="H555" s="22" t="n"/>
-      <c r="I555" s="25">
+      <c r="C555" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D555" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E555" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F555" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G555" s="36" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="H555" s="16" t="n">
+        <v>7</v>
+      </c>
+      <c r="I555" s="19">
         <f>IF(OR(F555="",G555=""),"",F555*G555)</f>
         <v/>
       </c>
-      <c r="J555" s="38">
+      <c r="J555" s="36">
         <f>IF(OR(F555="",G555=""),"",ROUND(G555*(1+F555/30),1))</f>
         <v/>
       </c>
-      <c r="K555" s="26" t="n"/>
+      <c r="K555" s="20" t="n"/>
     </row>
     <row r="556" ht="18" customHeight="1">
-      <c r="A556" s="35" t="n"/>
+      <c r="A556" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B556" s="16">
         <f>IF(A556="","",IFERROR(INT((A556-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C556" s="16" t="n"/>
-      <c r="D556" s="17" t="n"/>
-      <c r="E556" s="16" t="n"/>
-      <c r="F556" s="16" t="n"/>
+      <c r="C556" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D556" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E556" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F556" s="16" t="n">
+        <v>12</v>
+      </c>
       <c r="G556" s="36" t="n"/>
-      <c r="H556" s="16" t="n"/>
+      <c r="H556" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I556" s="19">
         <f>IF(OR(F556="",G556=""),"",F556*G556)</f>
         <v/>
@@ -24419,42 +24761,78 @@
         <f>IF(OR(F556="",G556=""),"",ROUND(G556*(1+F556/30),1))</f>
         <v/>
       </c>
-      <c r="K556" s="20" t="n"/>
+      <c r="K556" s="20" t="inlineStr">
+        <is>
+          <t>RPE 8/9/8 -&gt; HOLD 3x12.</t>
+        </is>
+      </c>
     </row>
     <row r="557" ht="18" customHeight="1">
-      <c r="A557" s="37" t="n"/>
-      <c r="B557" s="22">
+      <c r="A557" s="35" t="n">
+        <v>46319</v>
+      </c>
+      <c r="B557" s="16">
         <f>IF(A557="","",IFERROR(INT((A557-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C557" s="22" t="n"/>
-      <c r="D557" s="23" t="n"/>
-      <c r="E557" s="22" t="n"/>
-      <c r="F557" s="22" t="n"/>
-      <c r="G557" s="38" t="n"/>
-      <c r="H557" s="22" t="n"/>
-      <c r="I557" s="25">
+      <c r="C557" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D557" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E557" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F557" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="G557" s="36" t="n"/>
+      <c r="H557" s="16" t="n">
+        <v>9</v>
+      </c>
+      <c r="I557" s="19">
         <f>IF(OR(F557="",G557=""),"",F557*G557)</f>
         <v/>
       </c>
-      <c r="J557" s="38">
+      <c r="J557" s="36">
         <f>IF(OR(F557="",G557=""),"",ROUND(G557*(1+F557/30),1))</f>
         <v/>
       </c>
-      <c r="K557" s="26" t="n"/>
+      <c r="K557" s="20" t="n"/>
     </row>
     <row r="558" ht="18" customHeight="1">
-      <c r="A558" s="35" t="n"/>
+      <c r="A558" s="35" t="n">
+        <v>46319</v>
+      </c>
       <c r="B558" s="16">
         <f>IF(A558="","",IFERROR(INT((A558-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C558" s="16" t="n"/>
-      <c r="D558" s="17" t="n"/>
-      <c r="E558" s="16" t="n"/>
-      <c r="F558" s="16" t="n"/>
+      <c r="C558" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D558" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E558" s="16" t="n">
+        <v>3</v>
+      </c>
+      <c r="F558" s="16" t="n">
+        <v>12</v>
+      </c>
       <c r="G558" s="36" t="n"/>
-      <c r="H558" s="16" t="n"/>
+      <c r="H558" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I558" s="19">
         <f>IF(OR(F558="",G558=""),"",F558*G558)</f>
         <v/>
@@ -34839,32 +35217,48 @@
       </c>
     </row>
     <row r="65" ht="18" customHeight="1">
-      <c r="A65" s="37" t="n"/>
+      <c r="A65" s="37" t="n">
+        <v>46319</v>
+      </c>
       <c r="B65" s="22">
         <f>IF(A65="","",IFERROR(INT((A65-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C65" s="38" t="n"/>
-      <c r="D65" s="38" t="n"/>
+      <c r="C65" s="38" t="n">
+        <v>76.09999999999999</v>
+      </c>
+      <c r="D65" s="38" t="n">
+        <v>8.050000000000001</v>
+      </c>
       <c r="E65" s="38" t="n"/>
       <c r="F65" s="38" t="n"/>
       <c r="G65" s="38" t="n"/>
       <c r="H65" s="38" t="n"/>
-      <c r="I65" s="26" t="n"/>
+      <c r="I65" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 3 Sat (4x1 k +1) - AM: sleep 8:03 (23:45-07:50) q10, RHR 44 (-1 vs 7d), mot 10/energy 10/stress 2, DOMS chest 1/back 0/shldr 1/arm 0, quad 1/ham 2/glute 1/calf 3 (4x1 k cost, same as post-TT), joints clean, SHIN CLEAN #55. BW 76.10 (-0.80) travel water gone, 7-reading avg 76.70 flat, no kcal change. Rest MOVED -&gt; Gym #4 upper. PM: Gym #4 upper DONE 20 sets / 3376 kg / avg RPE 6.85 (LPD ran 30, incline 6/DB); shin clean #56; bike 0, kcal/protein/creatine not tracked.</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="18" customHeight="1">
-      <c r="A66" s="35" t="n"/>
-      <c r="B66" s="16">
+      <c r="A66" s="37" t="n">
+        <v>46320</v>
+      </c>
+      <c r="B66" s="22">
         <f>IF(A66="","",IFERROR(INT((A66-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C66" s="36" t="n"/>
-      <c r="D66" s="36" t="n"/>
-      <c r="E66" s="36" t="n"/>
-      <c r="F66" s="36" t="n"/>
-      <c r="G66" s="36" t="n"/>
-      <c r="H66" s="36" t="n"/>
-      <c r="I66" s="20" t="n"/>
+      <c r="C66" s="38" t="n"/>
+      <c r="D66" s="38" t="n"/>
+      <c r="E66" s="38" t="n"/>
+      <c r="F66" s="38" t="n"/>
+      <c r="G66" s="38" t="n"/>
+      <c r="H66" s="38" t="n"/>
+      <c r="I66" s="26" t="inlineStr">
+        <is>
+          <t>5K Wk 3 Sun - easy 8 k MOVED -&gt; REST (user's call), no make-up. No AM check reported. Wk 3 = 2 runs / 13.18 km + Gym #3 + Gym #4. Mon 10/26 easy 5 k AM added (Tue reps off a 4-day gap otherwise; calf &gt;=2 -&gt; rest).</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="18" customHeight="1">
       <c r="A67" s="37" t="n"/>

</xml_diff>

<commit_message>
log: Thu 10/29 strides + 2x400 (~2:05/2:04, RPE 6) + Gym #5 upper DONE; stage Fri rest + Sat 10/31 race
- Mon 10/26 easy 5 k closed (7:35 @ HR 143, cadence 163)
- Tue 10/27 3x1 k skipped (assumed, not on Strava); Wed 10/28 rest
- Thu 10/29 track: 4.91 km, 400s ~2:05 / ~2:04 GPS vs 2:08 target, both opened
  ~4:45/km -> ran hot again; shin clean #57
- Gym #5: 12 sets / 1760 kg / avg RPE 6.75; LPD 30 ran RPE 9/8 -> post-race
  LPD bump cancelled, HOLD 30 4x10
- Stage Fri 10/30 race-eve rest and Sat 10/31 race (200 m start, first 200 = 1:04,
  laps 2:08, 3 k = 16:00, push from 3 k)
- xlsx: Running 36, Body 68, Lifting 559-570

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/logs/training_log.xlsx
+++ b/logs/training_log.xlsx
@@ -24844,17 +24844,35 @@
       <c r="K558" s="20" t="n"/>
     </row>
     <row r="559" ht="18" customHeight="1">
-      <c r="A559" s="37" t="n"/>
+      <c r="A559" s="37" t="n">
+        <v>46324</v>
+      </c>
       <c r="B559" s="22">
         <f>IF(A559="","",IFERROR(INT((A559-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C559" s="22" t="n"/>
-      <c r="D559" s="23" t="n"/>
-      <c r="E559" s="22" t="n"/>
-      <c r="F559" s="22" t="n"/>
-      <c r="G559" s="38" t="n"/>
-      <c r="H559" s="22" t="n"/>
+      <c r="C559" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D559" s="23" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E559" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F559" s="22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G559" s="38" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H559" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I559" s="25">
         <f>IF(OR(F559="",G559=""),"",F559*G559)</f>
         <v/>
@@ -24863,20 +24881,42 @@
         <f>IF(OR(F559="",G559=""),"",ROUND(G559*(1+F559/30),1))</f>
         <v/>
       </c>
-      <c r="K559" s="26" t="n"/>
+      <c r="K559" s="26" t="inlineStr">
+        <is>
+          <t>Gym #5 upper (race wk, 2 sets, ~8 min post-run). Post-race HOLD 27.5 4x8.</t>
+        </is>
+      </c>
     </row>
     <row r="560" ht="18" customHeight="1">
-      <c r="A560" s="35" t="n"/>
+      <c r="A560" s="35" t="n">
+        <v>46324</v>
+      </c>
       <c r="B560" s="16">
         <f>IF(A560="","",IFERROR(INT((A560-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C560" s="16" t="n"/>
-      <c r="D560" s="17" t="n"/>
-      <c r="E560" s="16" t="n"/>
-      <c r="F560" s="16" t="n"/>
-      <c r="G560" s="36" t="n"/>
-      <c r="H560" s="16" t="n"/>
+      <c r="C560" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D560" s="17" t="inlineStr">
+        <is>
+          <t>Bench Press</t>
+        </is>
+      </c>
+      <c r="E560" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F560" s="16" t="n">
+        <v>8</v>
+      </c>
+      <c r="G560" s="36" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H560" s="16" t="n">
+        <v>7</v>
+      </c>
       <c r="I560" s="19">
         <f>IF(OR(F560="",G560=""),"",F560*G560)</f>
         <v/>
@@ -24888,17 +24928,35 @@
       <c r="K560" s="20" t="n"/>
     </row>
     <row r="561" ht="18" customHeight="1">
-      <c r="A561" s="37" t="n"/>
+      <c r="A561" s="37" t="n">
+        <v>46324</v>
+      </c>
       <c r="B561" s="22">
         <f>IF(A561="","",IFERROR(INT((A561-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C561" s="22" t="n"/>
-      <c r="D561" s="23" t="n"/>
-      <c r="E561" s="22" t="n"/>
-      <c r="F561" s="22" t="n"/>
-      <c r="G561" s="38" t="n"/>
-      <c r="H561" s="22" t="n"/>
+      <c r="C561" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D561" s="23" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E561" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F561" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G561" s="38" t="n">
+        <v>30</v>
+      </c>
+      <c r="H561" s="22" t="n">
+        <v>9</v>
+      </c>
       <c r="I561" s="25">
         <f>IF(OR(F561="",G561=""),"",F561*G561)</f>
         <v/>
@@ -24907,20 +24965,42 @@
         <f>IF(OR(F561="",G561=""),"",ROUND(G561*(1+F561/30),1))</f>
         <v/>
       </c>
-      <c r="K561" s="26" t="n"/>
+      <c r="K561" s="26" t="inlineStr">
+        <is>
+          <t>RPE 9/8 (6/6/7/7 on 10/24) - post-400s. Post-race 32.5 cancelled -&gt; HOLD 30 4x10.</t>
+        </is>
+      </c>
     </row>
     <row r="562" ht="18" customHeight="1">
-      <c r="A562" s="35" t="n"/>
+      <c r="A562" s="35" t="n">
+        <v>46324</v>
+      </c>
       <c r="B562" s="16">
         <f>IF(A562="","",IFERROR(INT((A562-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C562" s="16" t="n"/>
-      <c r="D562" s="17" t="n"/>
-      <c r="E562" s="16" t="n"/>
-      <c r="F562" s="16" t="n"/>
-      <c r="G562" s="36" t="n"/>
-      <c r="H562" s="16" t="n"/>
+      <c r="C562" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D562" s="17" t="inlineStr">
+        <is>
+          <t>Lat Pulldown</t>
+        </is>
+      </c>
+      <c r="E562" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F562" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G562" s="36" t="n">
+        <v>30</v>
+      </c>
+      <c r="H562" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I562" s="19">
         <f>IF(OR(F562="",G562=""),"",F562*G562)</f>
         <v/>
@@ -24932,17 +25012,35 @@
       <c r="K562" s="20" t="n"/>
     </row>
     <row r="563" ht="18" customHeight="1">
-      <c r="A563" s="37" t="n"/>
+      <c r="A563" s="37" t="n">
+        <v>46324</v>
+      </c>
       <c r="B563" s="22">
         <f>IF(A563="","",IFERROR(INT((A563-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C563" s="22" t="n"/>
-      <c r="D563" s="23" t="n"/>
-      <c r="E563" s="22" t="n"/>
-      <c r="F563" s="22" t="n"/>
-      <c r="G563" s="38" t="n"/>
-      <c r="H563" s="22" t="n"/>
+      <c r="C563" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D563" s="23" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E563" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F563" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G563" s="38" t="n">
+        <v>6</v>
+      </c>
+      <c r="H563" s="22" t="n">
+        <v>5</v>
+      </c>
       <c r="I563" s="25">
         <f>IF(OR(F563="",G563=""),"",F563*G563)</f>
         <v/>
@@ -24951,20 +25049,42 @@
         <f>IF(OR(F563="",G563=""),"",ROUND(G563*(1+F563/30),1))</f>
         <v/>
       </c>
-      <c r="K563" s="26" t="n"/>
+      <c r="K563" s="26" t="inlineStr">
+        <is>
+          <t>6/DB. Post-race 7/DB 3x10.</t>
+        </is>
+      </c>
     </row>
     <row r="564" ht="18" customHeight="1">
-      <c r="A564" s="35" t="n"/>
+      <c r="A564" s="35" t="n">
+        <v>46324</v>
+      </c>
       <c r="B564" s="16">
         <f>IF(A564="","",IFERROR(INT((A564-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C564" s="16" t="n"/>
-      <c r="D564" s="17" t="n"/>
-      <c r="E564" s="16" t="n"/>
-      <c r="F564" s="16" t="n"/>
-      <c r="G564" s="36" t="n"/>
-      <c r="H564" s="16" t="n"/>
+      <c r="C564" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D564" s="17" t="inlineStr">
+        <is>
+          <t>Incline DB Press</t>
+        </is>
+      </c>
+      <c r="E564" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F564" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G564" s="36" t="n">
+        <v>6</v>
+      </c>
+      <c r="H564" s="16" t="n">
+        <v>5</v>
+      </c>
       <c r="I564" s="19">
         <f>IF(OR(F564="",G564=""),"",F564*G564)</f>
         <v/>
@@ -24976,17 +25096,35 @@
       <c r="K564" s="20" t="n"/>
     </row>
     <row r="565" ht="18" customHeight="1">
-      <c r="A565" s="37" t="n"/>
+      <c r="A565" s="37" t="n">
+        <v>46324</v>
+      </c>
       <c r="B565" s="22">
         <f>IF(A565="","",IFERROR(INT((A565-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C565" s="22" t="n"/>
-      <c r="D565" s="23" t="n"/>
-      <c r="E565" s="22" t="n"/>
-      <c r="F565" s="22" t="n"/>
-      <c r="G565" s="38" t="n"/>
-      <c r="H565" s="22" t="n"/>
+      <c r="C565" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D565" s="23" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E565" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F565" s="22" t="n">
+        <v>10</v>
+      </c>
+      <c r="G565" s="38" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H565" s="22" t="n">
+        <v>7</v>
+      </c>
       <c r="I565" s="25">
         <f>IF(OR(F565="",G565=""),"",F565*G565)</f>
         <v/>
@@ -24995,20 +25133,42 @@
         <f>IF(OR(F565="",G565=""),"",ROUND(G565*(1+F565/30),1))</f>
         <v/>
       </c>
-      <c r="K565" s="26" t="n"/>
+      <c r="K565" s="26" t="inlineStr">
+        <is>
+          <t>Post-race 25 3x12.</t>
+        </is>
+      </c>
     </row>
     <row r="566" ht="18" customHeight="1">
-      <c r="A566" s="35" t="n"/>
+      <c r="A566" s="35" t="n">
+        <v>46324</v>
+      </c>
       <c r="B566" s="16">
         <f>IF(A566="","",IFERROR(INT((A566-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C566" s="16" t="n"/>
-      <c r="D566" s="17" t="n"/>
-      <c r="E566" s="16" t="n"/>
-      <c r="F566" s="16" t="n"/>
-      <c r="G566" s="36" t="n"/>
-      <c r="H566" s="16" t="n"/>
+      <c r="C566" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D566" s="17" t="inlineStr">
+        <is>
+          <t>Barbell Row</t>
+        </is>
+      </c>
+      <c r="E566" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F566" s="16" t="n">
+        <v>10</v>
+      </c>
+      <c r="G566" s="36" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H566" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I566" s="19">
         <f>IF(OR(F566="",G566=""),"",F566*G566)</f>
         <v/>
@@ -25020,17 +25180,35 @@
       <c r="K566" s="20" t="n"/>
     </row>
     <row r="567" ht="18" customHeight="1">
-      <c r="A567" s="37" t="n"/>
+      <c r="A567" s="37" t="n">
+        <v>46324</v>
+      </c>
       <c r="B567" s="22">
         <f>IF(A567="","",IFERROR(INT((A567-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C567" s="22" t="n"/>
-      <c r="D567" s="23" t="n"/>
-      <c r="E567" s="22" t="n"/>
-      <c r="F567" s="22" t="n"/>
-      <c r="G567" s="38" t="n"/>
-      <c r="H567" s="22" t="n"/>
+      <c r="C567" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D567" s="23" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E567" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F567" s="22" t="n">
+        <v>15</v>
+      </c>
+      <c r="G567" s="38" t="n">
+        <v>5</v>
+      </c>
+      <c r="H567" s="22" t="n">
+        <v>6</v>
+      </c>
       <c r="I567" s="25">
         <f>IF(OR(F567="",G567=""),"",F567*G567)</f>
         <v/>
@@ -25039,20 +25217,42 @@
         <f>IF(OR(F567="",G567=""),"",ROUND(G567*(1+F567/30),1))</f>
         <v/>
       </c>
-      <c r="K567" s="26" t="n"/>
+      <c r="K567" s="26" t="inlineStr">
+        <is>
+          <t>Ran 5 kg (staged 6.8). Post-race 6.8 3x20.</t>
+        </is>
+      </c>
     </row>
     <row r="568" ht="18" customHeight="1">
-      <c r="A568" s="35" t="n"/>
+      <c r="A568" s="35" t="n">
+        <v>46324</v>
+      </c>
       <c r="B568" s="16">
         <f>IF(A568="","",IFERROR(INT((A568-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C568" s="16" t="n"/>
-      <c r="D568" s="17" t="n"/>
-      <c r="E568" s="16" t="n"/>
-      <c r="F568" s="16" t="n"/>
-      <c r="G568" s="36" t="n"/>
-      <c r="H568" s="16" t="n"/>
+      <c r="C568" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D568" s="17" t="inlineStr">
+        <is>
+          <t>Tibialis Raise</t>
+        </is>
+      </c>
+      <c r="E568" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F568" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="G568" s="36" t="n">
+        <v>5</v>
+      </c>
+      <c r="H568" s="16" t="n">
+        <v>6</v>
+      </c>
       <c r="I568" s="19">
         <f>IF(OR(F568="",G568=""),"",F568*G568)</f>
         <v/>
@@ -25064,17 +25264,33 @@
       <c r="K568" s="20" t="n"/>
     </row>
     <row r="569" ht="18" customHeight="1">
-      <c r="A569" s="37" t="n"/>
+      <c r="A569" s="37" t="n">
+        <v>46324</v>
+      </c>
       <c r="B569" s="22">
         <f>IF(A569="","",IFERROR(INT((A569-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C569" s="22" t="n"/>
-      <c r="D569" s="23" t="n"/>
-      <c r="E569" s="22" t="n"/>
-      <c r="F569" s="22" t="n"/>
+      <c r="C569" s="22" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D569" s="23" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E569" s="22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F569" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="G569" s="38" t="n"/>
-      <c r="H569" s="22" t="n"/>
+      <c r="H569" s="22" t="n">
+        <v>8</v>
+      </c>
       <c r="I569" s="25">
         <f>IF(OR(F569="",G569=""),"",F569*G569)</f>
         <v/>
@@ -25083,20 +25299,40 @@
         <f>IF(OR(F569="",G569=""),"",ROUND(G569*(1+F569/30),1))</f>
         <v/>
       </c>
-      <c r="K569" s="26" t="n"/>
+      <c r="K569" s="26" t="inlineStr">
+        <is>
+          <t>Post-race HOLD 3x12.</t>
+        </is>
+      </c>
     </row>
     <row r="570" ht="18" customHeight="1">
-      <c r="A570" s="35" t="n"/>
+      <c r="A570" s="35" t="n">
+        <v>46324</v>
+      </c>
       <c r="B570" s="16">
         <f>IF(A570="","",IFERROR(INT((A570-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C570" s="16" t="n"/>
-      <c r="D570" s="17" t="n"/>
-      <c r="E570" s="16" t="n"/>
-      <c r="F570" s="16" t="n"/>
+      <c r="C570" s="16" t="inlineStr">
+        <is>
+          <t>Gym Upper</t>
+        </is>
+      </c>
+      <c r="D570" s="17" t="inlineStr">
+        <is>
+          <t>Hanging Knee Raise (BW)</t>
+        </is>
+      </c>
+      <c r="E570" s="16" t="n">
+        <v>2</v>
+      </c>
+      <c r="F570" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="G570" s="36" t="n"/>
-      <c r="H570" s="16" t="n"/>
+      <c r="H570" s="16" t="n">
+        <v>8</v>
+      </c>
       <c r="I570" s="19">
         <f>IF(OR(F570="",G570=""),"",F570*G570)</f>
         <v/>
@@ -31581,40 +31817,81 @@
       </c>
     </row>
     <row r="35" ht="18" customHeight="1">
-      <c r="A35" s="37" t="n"/>
+      <c r="A35" s="37" t="n">
+        <v>46321</v>
+      </c>
       <c r="B35" s="22">
         <f>IF(A35="","",IFERROR(INT((A35-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C35" s="28" t="n"/>
-      <c r="D35" s="38" t="n"/>
+      <c r="C35" s="28" t="n">
+        <v>5.01</v>
+      </c>
+      <c r="D35" s="38" t="n">
+        <v>37.98</v>
+      </c>
       <c r="E35" s="22">
         <f>IF(OR(C35="",D35=""),"",TEXT(D35/C35/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F35" s="22" t="n"/>
-      <c r="G35" s="22" t="n"/>
+      <c r="F35" s="22" t="n">
+        <v>143</v>
+      </c>
+      <c r="G35" s="22" t="n">
+        <v>157</v>
+      </c>
       <c r="H35" s="22" t="n"/>
-      <c r="I35" s="22" t="n"/>
-      <c r="J35" s="26" t="n"/>
+      <c r="I35" s="22" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="J35" s="26" t="inlineStr">
+        <is>
+          <t>5K race wk Mon - easy 5 k, road, Ballerup, AM 08:02. Moving 37:59 / elapsed 38:28 (~29 s stop km 4). Splits 7:58/7:15/7:29/7:54/7:19, HR by km 129/145/146/147/149 (km 2 over the &lt;=140 cap), max 157 on km-4 climb. Cadence 163 (162-165), 3rd easy segment in a row under the 166 floor. 9 C, feels 3.5, wind 6.3 m/s. RPE/shin/metronome n/r (asked). Strava 20734026221.</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="18" customHeight="1">
-      <c r="A36" s="35" t="n"/>
+      <c r="A36" s="35" t="n">
+        <v>46324</v>
+      </c>
       <c r="B36" s="16">
         <f>IF(A36="","",IFERROR(INT((A36-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
       </c>
-      <c r="C36" s="27" t="n"/>
-      <c r="D36" s="36" t="n"/>
+      <c r="C36" s="27" t="n">
+        <v>4.91</v>
+      </c>
+      <c r="D36" s="36" t="n">
+        <v>33.9</v>
+      </c>
       <c r="E36" s="16">
         <f>IF(OR(C36="",D36=""),"",TEXT(D36/C36/1440,"m:ss"))</f>
         <v/>
       </c>
-      <c r="F36" s="16" t="n"/>
-      <c r="G36" s="16" t="n"/>
-      <c r="H36" s="16" t="n"/>
-      <c r="I36" s="16" t="n"/>
-      <c r="J36" s="20" t="n"/>
+      <c r="F36" s="16" t="n">
+        <v>148</v>
+      </c>
+      <c r="G36" s="16" t="n">
+        <v>174</v>
+      </c>
+      <c r="H36" s="16" t="n">
+        <v>6</v>
+      </c>
+      <c r="I36" s="16" t="inlineStr">
+        <is>
+          <t>Strides + 2x400</t>
+        </is>
+      </c>
+      <c r="J36" s="20" t="inlineStr">
+        <is>
+          <t>5K race wk Thu - 4 k + strides + 2x400 @ 2:08 (replaced missed Tue 3x1 k). Track, Ballerup Atletikbane, 11:12. Moving 33:54 / elapsed 34:34. WU 2.06 k (1.22 k 7:07@138 cad 162, ~43 s stop, 0.84 k 6:27@150 cad 169). 4 strides peak ~4:45 (ceiling 4:40 OK), walked after each. 400 #1 ~2:05 GPS (HR 160/172), 400 #2 ~2:04 (HR 169/173) - both under the 2:06 floor, both opened ~4:45-4:55/km. CD 0.97 k 7:26@153. RPE 6. SHIN CLEAN #57. 11.9 C, wind 3.7 m/s. Strava 20776417810.</t>
+        </is>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="37" t="n"/>
@@ -35261,7 +35538,9 @@
       </c>
     </row>
     <row r="67" ht="18" customHeight="1">
-      <c r="A67" s="37" t="n"/>
+      <c r="A67" s="37" t="n">
+        <v>46321</v>
+      </c>
       <c r="B67" s="22">
         <f>IF(A67="","",IFERROR(INT((A67-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
@@ -35272,10 +35551,16 @@
       <c r="F67" s="38" t="n"/>
       <c r="G67" s="38" t="n"/>
       <c r="H67" s="38" t="n"/>
-      <c r="I67" s="26" t="n"/>
+      <c r="I67" s="26" t="inlineStr">
+        <is>
+          <t>5K race wk Mon - no AM check reported (asked). PM: easy 5 k DONE 7:35/km @ HR 143, cadence 163; shin n/r. Bike/kcal/protein/creatine n/r. Next: Tue 10/27 3x1 k @ 5:20 (ceiling 5:18), track.</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="18" customHeight="1">
-      <c r="A68" s="35" t="n"/>
+      <c r="A68" s="35" t="n">
+        <v>46324</v>
+      </c>
       <c r="B68" s="16">
         <f>IF(A68="","",IFERROR(INT((A68-DATE(2026,4,27))/7)+1,""))</f>
         <v/>
@@ -35286,7 +35571,11 @@
       <c r="F68" s="36" t="n"/>
       <c r="G68" s="36" t="n"/>
       <c r="H68" s="36" t="n"/>
-      <c r="I68" s="20" t="n"/>
+      <c r="I68" s="20" t="inlineStr">
+        <is>
+          <t>5K race wk Thu - no AM check reported. PM: run 4.91 k (2x400 ~2:05/2:04, RPE 6) + Gym #5 upper DONE. Shin clean #57. Bike 0, kcal 2283, protein 187, creatine Y. Tue 10/27 3x1 k skipped (assumed), Wed 10/28 rest. Next: Fri REST, Sat 10/31 RACE.</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="18" customHeight="1">
       <c r="A69" s="37" t="n"/>

</xml_diff>